<commit_message>
fix(sk-hynix): One Resume page — PwC 제안 framing 제거, production 단계로 갱신
사용자 피드백: "'One Resume + AI 구성원 검색'은 PwC 제안이라는 표현은 빼자.
구현 이미 된거니까 추진계획이라는 표현도 없애고."

- 파일명 rename: sk-hynix-pwc-one-resume-employee-search → sk-hynix-one-resume-employee-search
- title·vendor·tags에서 PwC·planned-deployment 제거
- stage: announced → production
- confidence: 0.18 → 0.22 (외부 공개 0건 fact 유지)
- 본문 "PwC Korea가 제안한" / "추진 계획 단계" framing 전면 삭제
- Consulting Angle을 "SK하이닉스 자체 구축 reference"로 재작성
- "공개 1차 출처 0건" caveat은 유지 (factually 여전히 true)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/exports/hr-ai-usecase-collection.xlsx
+++ b/wiki/exports/hr-ai-usecase-collection.xlsx
@@ -611,7 +611,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>0.42</t>
+          <t>0.43</t>
         </is>
       </c>
     </row>
@@ -20260,22 +20260,176 @@
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
+          <t>EX·HR운영</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>SK하이닉스: One Resume + AI 구성원 검색 (통합 직원 프로필·내부 talent search)</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>SK하이닉스 One Resume + AI 구성원 검색 시스템. 직원 1인당 분산된 데이터 (HRMS·평가·교육·프로젝트·자격·관심사·skill)를 단일 통합 프로필 (One Resume)로 구성하고, 매니저가 자연어로 사내 talent를 검색·추천 받는 AI talent search 기능을 결합. 직원 self-service career path 시각화·내부 기회 추천 포함. 2026-05 시점: 내부 운영 중, 외부 공개 metric 미공개.</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr">
+        <is>
+          <t>• Before: SK하이닉스 38K 직원의 인사 데이터가 HRMS·평가·교육·프로젝트·자격증·외부 교육 등 다수 시스템에 분산. 매니저가 internal mobility·project staffing·후계자 후보 검색 시 여러 시스템 + 인적 네트워크 의존
+• Pain point:
+• 사내 talent visibility 부족: 매니저가 "양산공정 + 머신러닝 경험 5년+ 영어 가능자"를 사내에서 찾기 어려움
+• 직원 본인도 자기 career path·내부 기회 잘 모름
+• 핵심 인재 retention·project staffing·후계자 풀 식별 모두 동일한 root cause (skill·경력 visibi…</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="inlineStr">
+        <is>
+          <t>[Before]
+SK하이닉스 38K 직원의 인사 데이터가 HRMS·평가·교육·프로젝트·자격증·외부 교육 등 다수 시스템에 분산. 매니저가 internal mobility·project staffing·후계자 후보 검색 시 여러 시스템 + 인적 네트워크 의존 / Pain point: / 사내 talent visibility 부족: 매니저가 "양산공정 + 머신러닝 경험 5년…
+[After]
+1. : HRMS·평가·교육 LMS·프로젝트 시스템·자격 DB·외부 교육 이력 등에서 직원별 데이터 자동 수집 → ETL → 단일 직원 프로필
+2. :
+3. :
+4. : 본인 One Resume 검토·수정·career path 시각화·내부 기회 추천 받기
+5. HR·리더 분석 dashboard: skill gap·talent inventory·후계자 풀 분석</t>
+        </is>
+      </c>
+      <c r="H121" s="7" t="inlineStr"/>
+      <c r="I121" s="7" t="inlineStr"/>
+      <c r="J121" s="7" t="inlineStr">
+        <is>
+          <t>직원 1인당 단일 통합 프로필 (One Resume: 인사·평가·교육·프로젝트·자격·관심사·skill 통합) + 매니저용 자연어 talent search (예: '머신러닝 + 양산공정 경험 5년+ 한국어/영어 가능' 검색) + 직원 본인의 career path 시각화</t>
+        </is>
+      </c>
+      <c r="K121" s="7" t="inlineStr"/>
+      <c r="L121" s="7" t="inlineStr">
+        <is>
+          <t>직원 데이터를 분산 → 통합 + 매니저 검색을 수동 → AI 자연어로 전환. 외부 공개 production metric 0건: 내부 운영 효과 _미공개_.</t>
+        </is>
+      </c>
+      <c r="M121" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N121" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O121" s="9" t="inlineStr"/>
+      <c r="P121" s="9" t="inlineStr"/>
+      <c r="Q121" s="9" t="inlineStr"/>
+      <c r="R121" s="9" t="inlineStr"/>
+      <c r="S121" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T121" s="9" t="inlineStr"/>
+      <c r="U121" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V121" s="9" t="inlineStr"/>
+      <c r="W121" s="9" t="inlineStr"/>
+      <c r="X121" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y121" s="9" t="inlineStr"/>
+      <c r="Z121" s="9" t="inlineStr"/>
+      <c r="AA121" s="9" t="inlineStr"/>
+      <c r="AB121" s="9" t="inlineStr"/>
+      <c r="AC121" s="7" t="inlineStr">
+        <is>
+          <t>Core HR &amp; Employee Records</t>
+        </is>
+      </c>
+      <c r="AD121" s="7" t="inlineStr">
+        <is>
+          <t>SK하이닉스 internal</t>
+        </is>
+      </c>
+      <c r="AE121" s="7" t="inlineStr">
+        <is>
+          <t>internal-build</t>
+        </is>
+      </c>
+      <c r="AF121" s="7" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="AG121" s="7" t="inlineStr">
+        <is>
+          <t>🇰🇷 KR</t>
+        </is>
+      </c>
+      <c r="AH121" s="7" t="inlineStr">
+        <is>
+          <t>운영</t>
+        </is>
+      </c>
+      <c r="AI121" s="7" t="inlineStr">
+        <is>
+          <t>월</t>
+        </is>
+      </c>
+      <c r="AJ121" s="7" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AK121" s="7" t="inlineStr">
+        <is>
+          <t>• KR talent profile/search 컨설팅에서의 위치: "한국형 자체 구축 reference":
+• SK하이닉스가 글로벌 SaaS 벤더 (Gloat·Eightfold) 대신 자체 구축으로 talent profile/search를 운영: 한국 반도체·이차전지·바이오 그룹사 talent profile 컨설팅의 자체 구축 reference
+• 단 외부 공개 metric 0건 → "SK하이닉스 사례"로 인용 시 출처 한계 명시 필수
+• 글로벌 비교:</t>
+        </is>
+      </c>
+      <c r="AL121" s="7" t="inlineStr">
+        <is>
+          <t>sk-hynix, one-resume, employee-search, talent-profile, korean-conglomerate, korea, semiconductor, internal-build</t>
+        </is>
+      </c>
+      <c r="AM121" s="7" t="inlineStr"/>
+      <c r="AN121" s="7" t="inlineStr"/>
+      <c r="AO121" s="7" t="inlineStr"/>
+      <c r="AP121" s="7" t="inlineStr">
+        <is>
+          <t>sk-hynix-one-resume-employee-search</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="90" customHeight="1">
+      <c r="A122" s="7" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
           <t>채용</t>
         </is>
       </c>
-      <c r="C121" s="7" t="inlineStr">
+      <c r="C122" s="7" t="inlineStr">
         <is>
           <t>Cathay Pacific: HireVue AI 면접 (time-to-hire 90%↓, 3개월→2~3주)</t>
         </is>
       </c>
-      <c r="D121" s="7" t="inlineStr">
+      <c r="D122" s="7" t="inlineStr">
         <is>
           <t>Cathay Pacific</t>
         </is>
       </c>
-      <c r="E121" s="7" t="inlineStr"/>
-      <c r="F121" s="7" t="inlineStr"/>
-      <c r="G121" s="7" t="inlineStr">
+      <c r="E122" s="7" t="inlineStr"/>
+      <c r="F122" s="7" t="inlineStr"/>
+      <c r="G122" s="7" t="inlineStr">
         <is>
           <t>[Before]
 졸업생 trainee 채용에 3개월 소요, in-person 면접 no-show율 높음 /
@@ -20288,146 +20442,146 @@
 6. Cathay 채용 매니저의 인사말 영상으로 employer branding 강화</t>
         </is>
       </c>
-      <c r="H121" s="7" t="inlineStr"/>
-      <c r="I121" s="7" t="inlineStr"/>
-      <c r="J121" s="7" t="inlineStr">
+      <c r="H122" s="7" t="inlineStr"/>
+      <c r="I122" s="7" t="inlineStr"/>
+      <c r="J122" s="7" t="inlineStr">
         <is>
           <t>후보자 on-demand video 응답 점수 (언어/콜로키얼 평가 포함) + 채용팀 검토용 shortlist + in-person 최종평가 진출자 결정</t>
         </is>
       </c>
-      <c r="K121" s="7" t="inlineStr"/>
-      <c r="L121" s="7" t="inlineStr">
+      <c r="K122" s="7" t="inlineStr"/>
+      <c r="L122" s="7" t="inlineStr">
         <is>
           <t>Time-to-hire 3개월에서 2~3주로 90%+ 단축, no-show 30% 감소, 면접 참석 30% 증가 (벤더 주장).</t>
         </is>
       </c>
-      <c r="M121" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N121" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O121" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P121" s="9" t="inlineStr"/>
-      <c r="Q121" s="9" t="inlineStr"/>
-      <c r="R121" s="9" t="inlineStr"/>
-      <c r="S121" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T121" s="9" t="inlineStr"/>
-      <c r="U121" s="9" t="inlineStr"/>
-      <c r="V121" s="9" t="inlineStr"/>
-      <c r="W121" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X121" s="9" t="inlineStr"/>
-      <c r="Y121" s="9" t="inlineStr"/>
-      <c r="Z121" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA121" s="9" t="inlineStr"/>
-      <c r="AB121" s="9" t="inlineStr"/>
-      <c r="AC121" s="7" t="inlineStr">
+      <c r="M122" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N122" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O122" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P122" s="9" t="inlineStr"/>
+      <c r="Q122" s="9" t="inlineStr"/>
+      <c r="R122" s="9" t="inlineStr"/>
+      <c r="S122" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T122" s="9" t="inlineStr"/>
+      <c r="U122" s="9" t="inlineStr"/>
+      <c r="V122" s="9" t="inlineStr"/>
+      <c r="W122" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X122" s="9" t="inlineStr"/>
+      <c r="Y122" s="9" t="inlineStr"/>
+      <c r="Z122" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA122" s="9" t="inlineStr"/>
+      <c r="AB122" s="9" t="inlineStr"/>
+      <c r="AC122" s="7" t="inlineStr">
         <is>
           <t>Interview &amp; Selection</t>
         </is>
       </c>
-      <c r="AD121" s="7" t="inlineStr">
+      <c r="AD122" s="7" t="inlineStr">
         <is>
           <t>HireVue</t>
         </is>
       </c>
-      <c r="AE121" s="7" t="inlineStr">
+      <c r="AE122" s="7" t="inlineStr">
         <is>
           <t>point-solution</t>
         </is>
       </c>
-      <c r="AF121" s="7" t="inlineStr">
+      <c r="AF122" s="7" t="inlineStr">
         <is>
           <t>airline, aviation</t>
         </is>
       </c>
-      <c r="AG121" s="7" t="inlineStr">
+      <c r="AG122" s="7" t="inlineStr">
         <is>
           <t>APAC</t>
         </is>
       </c>
-      <c r="AH121" s="7" t="inlineStr">
+      <c r="AH122" s="7" t="inlineStr">
         <is>
           <t>운영</t>
         </is>
       </c>
-      <c r="AI121" s="7" t="inlineStr">
+      <c r="AI122" s="7" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="AJ121" s="7" t="n">
+      <c r="AJ122" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK121" s="7" t="inlineStr">
+      <c r="AK122" s="7" t="inlineStr">
         <is>
           <t>• APAC region 첫 사례: 한국·일본·싱가포르 클라이언트에 reference
 • HireVue wiki 고객 생태계: Goldman Sachs + Cathay Pacific + Emirates + Holcim + Great Southern Bank</t>
         </is>
       </c>
-      <c r="AL121" s="7" t="inlineStr">
+      <c r="AL122" s="7" t="inlineStr">
         <is>
           <t>hirevue, video-interview, airline, asia-pacific, volume-hiring</t>
         </is>
       </c>
-      <c r="AM121" s="11" t="inlineStr">
+      <c r="AM122" s="11" t="inlineStr">
         <is>
           <t>HireVue case study</t>
         </is>
       </c>
-      <c r="AN121" s="7" t="inlineStr"/>
-      <c r="AO121" s="7" t="inlineStr"/>
-      <c r="AP121" s="7" t="inlineStr">
+      <c r="AN122" s="7" t="inlineStr"/>
+      <c r="AO122" s="7" t="inlineStr"/>
+      <c r="AP122" s="7" t="inlineStr">
         <is>
           <t>cathay-pacific-hirevue</t>
         </is>
       </c>
     </row>
-    <row r="122" ht="90" customHeight="1">
-      <c r="A122" s="7" t="n">
-        <v>121</v>
-      </c>
-      <c r="B122" s="7" t="inlineStr">
+    <row r="123" ht="90" customHeight="1">
+      <c r="A123" s="7" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
         <is>
           <t>보상·복리후생</t>
         </is>
       </c>
-      <c r="C122" s="7" t="inlineStr">
+      <c r="C123" s="7" t="inlineStr">
         <is>
           <t>더존비즈온: ONE AI 연말정산 end-to-end 자동화</t>
         </is>
       </c>
-      <c r="D122" s="7" t="inlineStr">
+      <c r="D123" s="7" t="inlineStr">
         <is>
           <t>_N/A (product, 다수 중소·중견기업 대상)_</t>
         </is>
       </c>
-      <c r="E122" s="7" t="inlineStr">
+      <c r="E123" s="7" t="inlineStr">
         <is>
           <t>더존비즈온(국내 ERP·급여 dominant player)이 자사 ONE AI 제품군에 포함시킨 연말정산 end-to-end 자동화 서비스. 대상자 선정부터 결과 안내까지 전 과정을 자동화. 국세청 간소화 자료 자동 다운로드·세액 예측·홈택스 자동신고·총괄현황판 등 제공. 2024-12 기준 1,000개 기업 추가 계약 보고(⚠ 벤더 주장).</t>
         </is>
       </c>
-      <c r="F122" s="7" t="inlineStr">
+      <c r="F123" s="7" t="inlineStr">
         <is>
           <t>한국 HR의 연말정산은 다음과 같은 구조적 부담을 가짐:
 • 법정 프로세스: 매년 1~3월 연말정산 + 2월 지급명세서 신고 의무
@@ -20437,7 +20591,7 @@
 • 반복성: 수백~수천 명 기업에서는 HR 2~3명이 수 개월 투입되는 작업</t>
         </is>
       </c>
-      <c r="G122" s="7" t="inlineStr">
+      <c r="G123" s="7" t="inlineStr">
         <is>
           <t>[Before]
 _미공개 (기업별 상이)_. 일반적 한국 기업의 기존 연말정산 플로우는 HR 담당자가 직원별로 국세청 간소화 자료 수집·입력·검증하는 수작업이나, 소스에 기업별 구체 기술은 없음 (🚫 일반 지식) /
@@ -20452,7 +20606,7 @@
 8.: 총괄현황판으로 전사 진행상황 실시간 관리</t>
         </is>
       </c>
-      <c r="H122" s="7" t="inlineStr">
+      <c r="H123" s="7" t="inlineStr">
         <is>
           <t>• Core HRIS: 더존 Smart HR / 급여 (자사 ERP 통합, 새로 HR 시스템 도입 불필요)
 • AI 시스템 배치: 더존 ONE AI 플랫폼 (ERP 내장)
@@ -20460,155 +20614,155 @@
 • 사용자 접점: 더존 ERP UI + 직원 원챔버 포털</t>
         </is>
       </c>
-      <c r="I122" s="7" t="inlineStr">
+      <c r="I123" s="7" t="inlineStr">
         <is>
           <t>• 입력 데이터 소스: - 직원 급여·인사 데이터 (더존 ERP 내부)
 • 데이터 거버넌스: - 한국 개인정보보호법 준수 필수: 급여·세액은 민감 정보</t>
         </is>
       </c>
-      <c r="J122" s="7" t="inlineStr">
+      <c r="J123" s="7" t="inlineStr">
         <is>
           <t>연말정산 대상자 자동 식별 리스트 + 국세청 간소화 PDF 자동 다운로드·반영 + 세액 예측 결과·직원 안내문 + 홈택스 자동신고·지급명세서 + HR용 총괄현황판</t>
         </is>
       </c>
-      <c r="K122" s="7" t="inlineStr">
+      <c r="K123" s="7" t="inlineStr">
         <is>
           <t>• 모델 유형: 세액 예측은 deterministic 계산 (세법 rule) + 증빙 검증에 ML 사용 가능
 • 제공 방식: 더존 자체 플랫폼</t>
         </is>
       </c>
-      <c r="L122" s="7" t="inlineStr">
+      <c r="L123" s="7" t="inlineStr">
         <is>
           <t>Before: _미공개 (기존 연말정산 처리 소요 시간·오류율)_ → After: ⚠️ 벤더 주장 end-to-end 자동화로 1,000개 기업 추가 계약 (2024-12). 시간 절감·세액 정확도·오류율 등 정량 성과 _미공개_.</t>
         </is>
       </c>
-      <c r="M122" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N122" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O122" s="9" t="inlineStr"/>
-      <c r="P122" s="9" t="inlineStr"/>
-      <c r="Q122" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R122" s="9" t="inlineStr"/>
-      <c r="S122" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T122" s="9" t="inlineStr"/>
-      <c r="U122" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V122" s="9" t="inlineStr"/>
-      <c r="W122" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X122" s="9" t="inlineStr"/>
-      <c r="Y122" s="9" t="inlineStr"/>
-      <c r="Z122" s="9" t="inlineStr"/>
-      <c r="AA122" s="9" t="inlineStr"/>
-      <c r="AB122" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AC122" s="7" t="inlineStr">
+      <c r="M123" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N123" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O123" s="9" t="inlineStr"/>
+      <c r="P123" s="9" t="inlineStr"/>
+      <c r="Q123" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R123" s="9" t="inlineStr"/>
+      <c r="S123" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T123" s="9" t="inlineStr"/>
+      <c r="U123" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V123" s="9" t="inlineStr"/>
+      <c r="W123" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X123" s="9" t="inlineStr"/>
+      <c r="Y123" s="9" t="inlineStr"/>
+      <c r="Z123" s="9" t="inlineStr"/>
+      <c r="AA123" s="9" t="inlineStr"/>
+      <c r="AB123" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC123" s="7" t="inlineStr">
         <is>
           <t>Payroll Operations</t>
         </is>
       </c>
-      <c r="AD122" s="7" t="inlineStr">
+      <c r="AD123" s="7" t="inlineStr">
         <is>
           <t>Douzone Bizon</t>
         </is>
       </c>
-      <c r="AE122" s="7" t="inlineStr">
+      <c r="AE123" s="7" t="inlineStr">
         <is>
           <t>hrms</t>
         </is>
       </c>
-      <c r="AF122" s="7" t="inlineStr">
+      <c r="AF123" s="7" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="AG122" s="7" t="inlineStr">
+      <c r="AG123" s="7" t="inlineStr">
         <is>
           <t>🇰🇷 KR</t>
         </is>
       </c>
-      <c r="AH122" s="7" t="inlineStr">
+      <c r="AH123" s="7" t="inlineStr">
         <is>
           <t>운영</t>
         </is>
       </c>
-      <c r="AI122" s="7" t="inlineStr">
+      <c r="AI123" s="7" t="inlineStr">
         <is>
           <t>연</t>
         </is>
       </c>
-      <c r="AJ122" s="7" t="n">
+      <c r="AJ123" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK122" s="7" t="inlineStr"/>
-      <c r="AL122" s="7" t="inlineStr">
+      <c r="AK123" s="7" t="inlineStr"/>
+      <c r="AL123" s="7" t="inlineStr">
         <is>
           <t>year-end-tax, korean-payroll, automation, sme, compliance, mid-market, douzone</t>
         </is>
       </c>
-      <c r="AM122" s="7" t="inlineStr"/>
-      <c r="AN122" s="7" t="inlineStr"/>
-      <c r="AO122" s="7" t="inlineStr"/>
-      <c r="AP122" s="7" t="inlineStr">
+      <c r="AM123" s="7" t="inlineStr"/>
+      <c r="AN123" s="7" t="inlineStr"/>
+      <c r="AO123" s="7" t="inlineStr"/>
+      <c r="AP123" s="7" t="inlineStr">
         <is>
           <t>douzone-one-ai-year-end-tax</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="90" customHeight="1">
-      <c r="A123" s="7" t="n">
-        <v>122</v>
-      </c>
-      <c r="B123" s="7" t="inlineStr">
+    <row r="124" ht="90" customHeight="1">
+      <c r="A124" s="7" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
         <is>
           <t>채용</t>
         </is>
       </c>
-      <c r="C123" s="7" t="inlineStr">
+      <c r="C124" s="7" t="inlineStr">
         <is>
           <t>Eightfold AI: Talent Intelligence Platform + AI Interviewer</t>
         </is>
       </c>
-      <c r="D123" s="7" t="inlineStr">
+      <c r="D124" s="7" t="inlineStr">
         <is>
           <t>_다수 (specific names in vendor page)_</t>
         </is>
       </c>
-      <c r="E123" s="7" t="inlineStr">
+      <c r="E124" s="7" t="inlineStr">
         <is>
           <t>Eightfold AI는 skills-based talent intelligence 플랫폼으로, 채용·내부 이동·스킬 관리를 AI로 통합. 2025년 AI Interviewer (자동 1차 면접)과 Digital Twin (직원의 지식·스킬·경험을 캡처하는 개인화 LLM) 발표. ⚠️ 벤더 주장: AI Interviewer로 time to first interview 90% 감소, 3,000명 이상 후보자를 AI로 면접 처리. Deloitte…</t>
         </is>
       </c>
-      <c r="F123" s="7" t="inlineStr">
+      <c r="F124" s="7" t="inlineStr">
         <is>
           <t>벤더 제품이므로 특정 기업의 도입 배경은 고객별 상이. 일반적 pain point: skills-based hiring 전환 필요성, 기존 keyword 매칭의 한계, time-to-hire 병목.</t>
         </is>
       </c>
-      <c r="G123" s="7" t="inlineStr">
+      <c r="G124" s="7" t="inlineStr">
         <is>
           <t>[Before]
 채용·내부이동·후계 별도 시스템, 정적 직무 기술서·resume keyword 매칭 /
@@ -20621,90 +20775,90 @@
 6. 결과/feedback이 self-learning engine에 반영되어 매칭 정확도 개선</t>
         </is>
       </c>
-      <c r="H123" s="7" t="inlineStr"/>
-      <c r="I123" s="7" t="inlineStr"/>
-      <c r="J123" s="7" t="inlineStr">
+      <c r="H124" s="7" t="inlineStr"/>
+      <c r="I124" s="7" t="inlineStr"/>
+      <c r="J124" s="7" t="inlineStr">
         <is>
           <t>직원/후보 Capabilities Matrix 기반 채용·내부이동·후계 통합 매칭 점수 + AI Interviewer 1차 비동기 면접 결과 + Job Intelligence Engine의 자동 생성 role 정의·job architecture</t>
         </is>
       </c>
-      <c r="K123" s="7" t="inlineStr"/>
-      <c r="L123" s="7" t="inlineStr">
+      <c r="K124" s="7" t="inlineStr"/>
+      <c r="L124" s="7" t="inlineStr">
         <is>
           <t>Before: _미공개 (기존 first interview 소요 시간)_ → After: ⚠️ 벤더 주장 time to first interview 90% 감소, 3,000+ 후보자 AI 면접 처리 (자사 채용). Gartner Peer Insights 4.6/5 평점(Fact).</t>
         </is>
       </c>
-      <c r="M123" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N123" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O123" s="9" t="inlineStr"/>
-      <c r="P123" s="9" t="inlineStr"/>
-      <c r="Q123" s="9" t="inlineStr"/>
-      <c r="R123" s="9" t="inlineStr"/>
-      <c r="S123" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T123" s="9" t="inlineStr"/>
-      <c r="U123" s="9" t="inlineStr"/>
-      <c r="V123" s="9" t="inlineStr"/>
-      <c r="W123" s="9" t="inlineStr"/>
-      <c r="X123" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y123" s="9" t="inlineStr"/>
-      <c r="Z123" s="9" t="inlineStr"/>
-      <c r="AA123" s="9" t="inlineStr"/>
-      <c r="AB123" s="9" t="inlineStr"/>
-      <c r="AC123" s="7" t="inlineStr">
+      <c r="M124" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N124" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O124" s="9" t="inlineStr"/>
+      <c r="P124" s="9" t="inlineStr"/>
+      <c r="Q124" s="9" t="inlineStr"/>
+      <c r="R124" s="9" t="inlineStr"/>
+      <c r="S124" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T124" s="9" t="inlineStr"/>
+      <c r="U124" s="9" t="inlineStr"/>
+      <c r="V124" s="9" t="inlineStr"/>
+      <c r="W124" s="9" t="inlineStr"/>
+      <c r="X124" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y124" s="9" t="inlineStr"/>
+      <c r="Z124" s="9" t="inlineStr"/>
+      <c r="AA124" s="9" t="inlineStr"/>
+      <c r="AB124" s="9" t="inlineStr"/>
+      <c r="AC124" s="7" t="inlineStr">
         <is>
           <t>Screening &amp; Assessment</t>
         </is>
       </c>
-      <c r="AD123" s="7" t="inlineStr">
+      <c r="AD124" s="7" t="inlineStr">
         <is>
           <t>Eightfold AI</t>
         </is>
       </c>
-      <c r="AE123" s="7" t="inlineStr">
+      <c r="AE124" s="7" t="inlineStr">
         <is>
           <t>talent-marketplace</t>
         </is>
       </c>
-      <c r="AF123" s="7" t="inlineStr">
+      <c r="AF124" s="7" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="AG123" s="7" t="inlineStr">
+      <c r="AG124" s="7" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="AH123" s="7" t="inlineStr">
+      <c r="AH124" s="7" t="inlineStr">
         <is>
           <t>운영</t>
         </is>
       </c>
-      <c r="AI123" s="7" t="inlineStr">
+      <c r="AI124" s="7" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="AJ123" s="7" t="n">
+      <c r="AJ124" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK123" s="7" t="inlineStr">
+      <c r="AK124" s="7" t="inlineStr">
         <is>
           <t>• vs SAP SuccessFactors Talent Intelligence Hub: SAP는 Eightfold을 "대체 대상"으로 지목 (Delta/Pepsi 사례, bersin-successfactors-leapfrog-2024-10). 이 경쟁 구도가 컨설팅 vendor selection에서 핵심 질문
 • 🚫 Mastercard customer reference 정정 (2026-05-06):
@@ -20712,50 +20866,50 @@
 • 이전에 본 페이지에 등재했던 Mastercard 4개 메트릭 (93·42·1M·24h)은 Gloat 사례로 이관됨</t>
         </is>
       </c>
-      <c r="AL123" s="7" t="inlineStr">
+      <c r="AL124" s="7" t="inlineStr">
         <is>
           <t>talent-intelligence, skills-based-hiring, ai-interviewer, digital-twin, deloitte-alliance</t>
         </is>
       </c>
-      <c r="AM123" s="11" t="inlineStr">
+      <c r="AM124" s="11" t="inlineStr">
         <is>
           <t>Eightfold AI 공식</t>
         </is>
       </c>
-      <c r="AN123" s="11" t="inlineStr">
+      <c r="AN124" s="11" t="inlineStr">
         <is>
           <t>PR Newswire 2025</t>
         </is>
       </c>
-      <c r="AO123" s="7" t="inlineStr"/>
-      <c r="AP123" s="7" t="inlineStr">
+      <c r="AO124" s="7" t="inlineStr"/>
+      <c r="AP124" s="7" t="inlineStr">
         <is>
           <t>eightfold-ai-talent-intelligence</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="90" customHeight="1">
-      <c r="A124" s="7" t="n">
-        <v>123</v>
-      </c>
-      <c r="B124" s="7" t="inlineStr">
+    <row r="125" ht="90" customHeight="1">
+      <c r="A125" s="7" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="7" t="inlineStr">
         <is>
           <t>채용</t>
         </is>
       </c>
-      <c r="C124" s="7" t="inlineStr">
+      <c r="C125" s="7" t="inlineStr">
         <is>
           <t>Emirates: HireVue AI (60일→7일, 8k시간 절약, $500k 절감)</t>
         </is>
       </c>
-      <c r="D124" s="7" t="inlineStr">
+      <c r="D125" s="7" t="inlineStr">
         <is>
           <t>Emirates</t>
         </is>
       </c>
-      <c r="E124" s="7" t="inlineStr"/>
-      <c r="F124" s="7" t="inlineStr"/>
-      <c r="G124" s="7" t="inlineStr">
+      <c r="E125" s="7" t="inlineStr"/>
+      <c r="F125" s="7" t="inlineStr"/>
+      <c r="G125" s="7" t="inlineStr">
         <is>
           <t>[Before]
 Pandemic 후 1만 명 cabin crew 재채용 필요, 전통 face-to-face 채용으로는 timeline 불가 /
@@ -20768,134 +20922,134 @@
 6. 최종 채용 결정은 in-person assessor</t>
         </is>
       </c>
-      <c r="H124" s="7" t="inlineStr"/>
-      <c r="I124" s="7" t="inlineStr"/>
-      <c r="J124" s="7" t="inlineStr">
+      <c r="H125" s="7" t="inlineStr"/>
+      <c r="I125" s="7" t="inlineStr"/>
+      <c r="J125" s="7" t="inlineStr">
         <is>
           <t>영어 평가 점수 (15분 객관식) + situational video 응답 채점 결과 (verbal/written, 벤더 주장 non-verbal cues 포함) + assessment day 진출 후보 shortlist</t>
         </is>
       </c>
-      <c r="K124" s="7" t="inlineStr"/>
-      <c r="L124" s="7" t="inlineStr">
+      <c r="K125" s="7" t="inlineStr"/>
+      <c r="L125" s="7" t="inlineStr">
         <is>
           <t>Time-to-hire 60일에서 7일로 88% 단축, 채용팀 2/3 전략적 업무 재배치, 8,000시간 절약, $500k 비용 절감 (벤더 주장).</t>
         </is>
       </c>
-      <c r="M124" s="9" t="inlineStr"/>
-      <c r="N124" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O124" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P124" s="9" t="inlineStr"/>
-      <c r="Q124" s="9" t="inlineStr"/>
-      <c r="R124" s="9" t="inlineStr"/>
-      <c r="S124" s="9" t="inlineStr"/>
-      <c r="T124" s="9" t="inlineStr"/>
-      <c r="U124" s="9" t="inlineStr"/>
-      <c r="V124" s="9" t="inlineStr"/>
-      <c r="W124" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X124" s="9" t="inlineStr"/>
-      <c r="Y124" s="9" t="inlineStr"/>
-      <c r="Z124" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA124" s="9" t="inlineStr"/>
-      <c r="AB124" s="9" t="inlineStr"/>
-      <c r="AC124" s="7" t="inlineStr">
+      <c r="M125" s="9" t="inlineStr"/>
+      <c r="N125" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O125" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P125" s="9" t="inlineStr"/>
+      <c r="Q125" s="9" t="inlineStr"/>
+      <c r="R125" s="9" t="inlineStr"/>
+      <c r="S125" s="9" t="inlineStr"/>
+      <c r="T125" s="9" t="inlineStr"/>
+      <c r="U125" s="9" t="inlineStr"/>
+      <c r="V125" s="9" t="inlineStr"/>
+      <c r="W125" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X125" s="9" t="inlineStr"/>
+      <c r="Y125" s="9" t="inlineStr"/>
+      <c r="Z125" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA125" s="9" t="inlineStr"/>
+      <c r="AB125" s="9" t="inlineStr"/>
+      <c r="AC125" s="7" t="inlineStr">
         <is>
           <t>Interview &amp; Selection</t>
         </is>
       </c>
-      <c r="AD124" s="7" t="inlineStr">
+      <c r="AD125" s="7" t="inlineStr">
         <is>
           <t>HireVue</t>
         </is>
       </c>
-      <c r="AE124" s="7" t="inlineStr">
+      <c r="AE125" s="7" t="inlineStr">
         <is>
           <t>point-solution</t>
         </is>
       </c>
-      <c r="AF124" s="7" t="inlineStr">
+      <c r="AF125" s="7" t="inlineStr">
         <is>
           <t>airline, aviation</t>
         </is>
       </c>
-      <c r="AG124" s="7" t="inlineStr">
+      <c r="AG125" s="7" t="inlineStr">
         <is>
           <t>APAC</t>
         </is>
       </c>
-      <c r="AH124" s="7" t="inlineStr">
+      <c r="AH125" s="7" t="inlineStr">
         <is>
           <t>운영</t>
         </is>
       </c>
-      <c r="AI124" s="7" t="inlineStr">
+      <c r="AI125" s="7" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="AJ124" s="7" t="n">
+      <c r="AJ125" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK124" s="7" t="inlineStr"/>
-      <c r="AL124" s="7" t="inlineStr">
+      <c r="AK125" s="7" t="inlineStr"/>
+      <c r="AL125" s="7" t="inlineStr">
         <is>
           <t>hirevue, video-interview, airline, middle-east, volume-hiring</t>
         </is>
       </c>
-      <c r="AM124" s="11" t="inlineStr">
+      <c r="AM125" s="11" t="inlineStr">
         <is>
           <t>HireVue case study</t>
         </is>
       </c>
-      <c r="AN124" s="7" t="inlineStr"/>
-      <c r="AO124" s="7" t="inlineStr"/>
-      <c r="AP124" s="7" t="inlineStr">
+      <c r="AN125" s="7" t="inlineStr"/>
+      <c r="AO125" s="7" t="inlineStr"/>
+      <c r="AP125" s="7" t="inlineStr">
         <is>
           <t>emirates-hirevue-volume-hiring</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="90" customHeight="1">
-      <c r="A125" s="7" t="n">
-        <v>124</v>
-      </c>
-      <c r="B125" s="7" t="inlineStr">
+    <row r="126" ht="90" customHeight="1">
+      <c r="A126" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="7" t="inlineStr">
         <is>
           <t>온보딩·이동</t>
         </is>
       </c>
-      <c r="C125" s="7" t="inlineStr">
+      <c r="C126" s="7" t="inlineStr">
         <is>
           <t>Lennox: Fuel50 내부 이동 AI (4,800건 이동, 이동당 +5개월 근속)</t>
         </is>
       </c>
-      <c r="D125" s="7" t="inlineStr">
+      <c r="D126" s="7" t="inlineStr">
         <is>
           <t>Lennox</t>
         </is>
       </c>
-      <c r="E125" s="7" t="inlineStr"/>
-      <c r="F125" s="7" t="inlineStr">
+      <c r="E126" s="7" t="inlineStr"/>
+      <c r="F126" s="7" t="inlineStr">
         <is>
           <t>직원 이탈 시 기관 지식 손실이 핵심 pain point. 내부 이동으로 retention 개선 목표.</t>
         </is>
       </c>
-      <c r="G125" s="7" t="inlineStr">
+      <c r="G126" s="7" t="inlineStr">
         <is>
           <t>[Before]
 내부이동이 매니저 referral·HR 큐레이션에 의존, 직원 가시성·career path 불투명 /
@@ -20908,127 +21062,127 @@
 6. Lennox: 4,800건 internal move, 평균 +5개월 tenure</t>
         </is>
       </c>
-      <c r="H125" s="7" t="inlineStr"/>
-      <c r="I125" s="7" t="inlineStr"/>
-      <c r="J125" s="7" t="inlineStr">
+      <c r="H126" s="7" t="inlineStr"/>
+      <c r="I126" s="7" t="inlineStr"/>
+      <c r="J126" s="7" t="inlineStr">
         <is>
           <t>직원 Talent DNA 기반 gig·project·mentorship·lateral move 추천 매칭 + 매니저용 applicant 풀·project talent pool + 직원 career path·mentor 매칭</t>
         </is>
       </c>
-      <c r="K125" s="7" t="inlineStr"/>
-      <c r="L125" s="7" t="inlineStr">
+      <c r="K126" s="7" t="inlineStr"/>
+      <c r="L126" s="7" t="inlineStr">
         <is>
           <t>4,800건 내부 이동 추적, 이동당 평균 5개월 근속 연장으로 2,000년+ 기관 지식 보존 (벤더 주장). 내부 이동의 재무 가치를 근속 기간으로 정량화한 유일 사례.</t>
         </is>
       </c>
-      <c r="M125" s="9" t="inlineStr"/>
-      <c r="N125" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O125" s="9" t="inlineStr"/>
-      <c r="P125" s="9" t="inlineStr"/>
-      <c r="Q125" s="9" t="inlineStr"/>
-      <c r="R125" s="9" t="inlineStr"/>
-      <c r="S125" s="9" t="inlineStr"/>
-      <c r="T125" s="9" t="inlineStr"/>
-      <c r="U125" s="9" t="inlineStr"/>
-      <c r="V125" s="9" t="inlineStr"/>
-      <c r="W125" s="9" t="inlineStr"/>
-      <c r="X125" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y125" s="9" t="inlineStr"/>
-      <c r="Z125" s="9" t="inlineStr"/>
-      <c r="AA125" s="9" t="inlineStr"/>
-      <c r="AB125" s="9" t="inlineStr"/>
-      <c r="AC125" s="7" t="inlineStr">
+      <c r="M126" s="9" t="inlineStr"/>
+      <c r="N126" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O126" s="9" t="inlineStr"/>
+      <c r="P126" s="9" t="inlineStr"/>
+      <c r="Q126" s="9" t="inlineStr"/>
+      <c r="R126" s="9" t="inlineStr"/>
+      <c r="S126" s="9" t="inlineStr"/>
+      <c r="T126" s="9" t="inlineStr"/>
+      <c r="U126" s="9" t="inlineStr"/>
+      <c r="V126" s="9" t="inlineStr"/>
+      <c r="W126" s="9" t="inlineStr"/>
+      <c r="X126" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y126" s="9" t="inlineStr"/>
+      <c r="Z126" s="9" t="inlineStr"/>
+      <c r="AA126" s="9" t="inlineStr"/>
+      <c r="AB126" s="9" t="inlineStr"/>
+      <c r="AC126" s="7" t="inlineStr">
         <is>
           <t>Internal Mobility</t>
         </is>
       </c>
-      <c r="AD125" s="7" t="inlineStr">
+      <c r="AD126" s="7" t="inlineStr">
         <is>
           <t>Fuel50</t>
         </is>
       </c>
-      <c r="AE125" s="7" t="inlineStr">
+      <c r="AE126" s="7" t="inlineStr">
         <is>
           <t>talent-marketplace</t>
         </is>
       </c>
-      <c r="AF125" s="7" t="inlineStr">
+      <c r="AF126" s="7" t="inlineStr">
         <is>
           <t>manufacturing, hvac</t>
         </is>
       </c>
-      <c r="AG125" s="7" t="inlineStr">
+      <c r="AG126" s="7" t="inlineStr">
         <is>
           <t>N. America</t>
         </is>
       </c>
-      <c r="AH125" s="7" t="inlineStr">
+      <c r="AH126" s="7" t="inlineStr">
         <is>
           <t>운영</t>
         </is>
       </c>
-      <c r="AI125" s="7" t="inlineStr">
+      <c r="AI126" s="7" t="inlineStr">
         <is>
           <t>월</t>
         </is>
       </c>
-      <c r="AJ125" s="7" t="n">
+      <c r="AJ126" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK125" s="7" t="inlineStr">
+      <c r="AK126" s="7" t="inlineStr">
         <is>
           <t>• "내부 이동의 재무 가치를 정량화"한 유일 사례: 다른 talent marketplace(Gloat·Phenom)는 시간·비용으로 측정하지만 Fuel50은 근속 연장으로 측정
 • Onboarding &amp; Transitions 카테고리 4번째 사례: Unilever(Gloat) + Schneider(Gloat) + Merck KGaA(Phenom) + Lennox(Fuel50): 3개 벤더 비교 가능</t>
         </is>
       </c>
-      <c r="AL125" s="7" t="inlineStr">
+      <c r="AL126" s="7" t="inlineStr">
         <is>
           <t>career-pathing, internal-mobility, fuel50, retention, manufacturing</t>
         </is>
       </c>
-      <c r="AM125" s="11" t="inlineStr">
+      <c r="AM126" s="11" t="inlineStr">
         <is>
           <t>Fuel50 official</t>
         </is>
       </c>
-      <c r="AN125" s="7" t="inlineStr"/>
-      <c r="AO125" s="7" t="inlineStr"/>
-      <c r="AP125" s="7" t="inlineStr">
+      <c r="AN126" s="7" t="inlineStr"/>
+      <c r="AO126" s="7" t="inlineStr"/>
+      <c r="AP126" s="7" t="inlineStr">
         <is>
           <t>fuel50-lennox-internal-mobility</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="90" customHeight="1">
-      <c r="A126" s="7" t="n">
-        <v>125</v>
-      </c>
-      <c r="B126" s="7" t="inlineStr">
+    <row r="127" ht="90" customHeight="1">
+      <c r="A127" s="7" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
         <is>
           <t>채용</t>
         </is>
       </c>
-      <c r="C126" s="7" t="inlineStr">
+      <c r="C127" s="7" t="inlineStr">
         <is>
           <t>McDonald's: Paradox AI 채용 (21일→3일 미만 time-to-hire)</t>
         </is>
       </c>
-      <c r="D126" s="7" t="inlineStr">
+      <c r="D127" s="7" t="inlineStr">
         <is>
           <t>McDonald's</t>
         </is>
       </c>
-      <c r="E126" s="7" t="inlineStr"/>
-      <c r="F126" s="7" t="inlineStr"/>
-      <c r="G126" s="7" t="inlineStr">
+      <c r="E127" s="7" t="inlineStr"/>
+      <c r="F127" s="7" t="inlineStr"/>
+      <c r="G127" s="7" t="inlineStr">
         <is>
           <t>[Before]
 매장 매니저가 종이/이메일로 지원 처리, 지원 시간 10분, 시간 부족으로 채용 누수 /
@@ -21041,167 +21195,24 @@
 6. 매장 매니저가 in-person 인터뷰에서 hire 결정 (McHire 플랫폼 통합)</t>
         </is>
       </c>
-      <c r="H126" s="7" t="inlineStr"/>
-      <c r="I126" s="7" t="inlineStr"/>
-      <c r="J126" s="7" t="inlineStr">
-        <is>
-          <t>Olivia의 후보자 conversational 스크리닝 (work history·shift) 결과 + 매장 매니저 캘린더 기반 면접 slot 자동 제시 + McHire ATS 통합 hiring funnel 기록</t>
-        </is>
-      </c>
-      <c r="K126" s="7" t="inlineStr"/>
-      <c r="L126" s="7" t="inlineStr">
-        <is>
-          <t>Time-to-hire 21일에서 3일 미만으로 86% 단축 (벤더 주장). NBC News가 AI recruiter 사용을 독립 확인(Fact).</t>
-        </is>
-      </c>
-      <c r="M126" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N126" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O126" s="9" t="inlineStr"/>
-      <c r="P126" s="9" t="inlineStr"/>
-      <c r="Q126" s="9" t="inlineStr"/>
-      <c r="R126" s="9" t="inlineStr"/>
-      <c r="S126" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T126" s="9" t="inlineStr"/>
-      <c r="U126" s="9" t="inlineStr"/>
-      <c r="V126" s="9" t="inlineStr"/>
-      <c r="W126" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X126" s="9" t="inlineStr"/>
-      <c r="Y126" s="9" t="inlineStr"/>
-      <c r="Z126" s="9" t="inlineStr"/>
-      <c r="AA126" s="9" t="inlineStr"/>
-      <c r="AB126" s="9" t="inlineStr"/>
-      <c r="AC126" s="7" t="inlineStr">
-        <is>
-          <t>Screening &amp; Assessment</t>
-        </is>
-      </c>
-      <c r="AD126" s="7" t="inlineStr">
-        <is>
-          <t>Paradox</t>
-        </is>
-      </c>
-      <c r="AE126" s="7" t="inlineStr">
-        <is>
-          <t>point-solution</t>
-        </is>
-      </c>
-      <c r="AF126" s="7" t="inlineStr">
-        <is>
-          <t>restaurant, fast-food</t>
-        </is>
-      </c>
-      <c r="AG126" s="7" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="AH126" s="7" t="inlineStr">
-        <is>
-          <t>운영</t>
-        </is>
-      </c>
-      <c r="AI126" s="7" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="AJ126" s="7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AK126" s="7" t="inlineStr">
-        <is>
-          <t>• Paradox wiki 고객 생태계 6번째: Chipotle(75%↓) · Nestlé(600%↑) · 7-Eleven(40k hrs/wk) · GM($2M) · Workday(23k hrs) · McDonald's(21→3일)
-• 식음료·리테일 고볼륨 채용에서 Paradox의 market dominance가 데이터로 확실</t>
-        </is>
-      </c>
-      <c r="AL126" s="7" t="inlineStr">
-        <is>
-          <t>paradox, conversational-ai, high-volume, restaurant, fast-food</t>
-        </is>
-      </c>
-      <c r="AM126" s="11" t="inlineStr">
-        <is>
-          <t>Paradox clients + NBC News</t>
-        </is>
-      </c>
-      <c r="AN126" s="7" t="inlineStr"/>
-      <c r="AO126" s="7" t="inlineStr"/>
-      <c r="AP126" s="7" t="inlineStr">
-        <is>
-          <t>mcdonalds-paradox-recruiting</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="90" customHeight="1">
-      <c r="A127" s="7" t="n">
-        <v>126</v>
-      </c>
-      <c r="B127" s="7" t="inlineStr">
-        <is>
-          <t>보상·복리후생</t>
-        </is>
-      </c>
-      <c r="C127" s="7" t="inlineStr">
-        <is>
-          <t>Paychex/Paycor: Agentic Workforce Management (타임시트 자동승인·Auto-Shifts, 800K 고객)</t>
-        </is>
-      </c>
-      <c r="D127" s="7" t="inlineStr">
-        <is>
-          <t>_다수 (800K 고객)_</t>
-        </is>
-      </c>
-      <c r="E127" s="7" t="inlineStr">
-        <is>
-          <t>Paychex가 2026년 2월 Paycor 및 Paychex Flex 플랫폼에 에이전틱 AI 솔루션을 발표. Paycor Agentic Timesheet Approvals(타임카드 자동 스코어링·이상만 사람 검토), Paycor Auto-Shifts(근무시간 제한·휴식·공정근무법 기반 최적 교대 생성), Paychex Flex AI-Powered Time-Off(PTO 패턴 분석·반복 가용성 AI). 800,000 고객 규모. Nucleus…</t>
-        </is>
-      </c>
-      <c r="F127" s="7" t="inlineStr">
-        <is>
-          <t>• 매니저가 타임시트를 수동으로 하나씩 검토·승인 → 시간 낭비 + 오류 발생
-• 교대 스케줄을 수동 작성 → 노동법(공정근무법·52시간) 위반 리스크
-• PTO 관리가 반응적 → 피크 기간 인력 부족 사전 예측 불가
-• SMB(중소기업)는 HR 전담 인력이 적어 자동화 수요 특히 높음</t>
-        </is>
-      </c>
-      <c r="G127" s="7" t="inlineStr">
-        <is>
-          <t>[Before]
-매니저가 타임카드 수동 검토 → 교대표 수동 작성 → PTO 개별 승인 /
-[After]
-1. md]]</t>
-        </is>
-      </c>
       <c r="H127" s="7" t="inlineStr"/>
       <c r="I127" s="7" t="inlineStr"/>
       <c r="J127" s="7" t="inlineStr">
         <is>
-          <t>타임카드 자동 스코어링·승인 결과 (이상 케이스만 매니저 플래그) + 노동법·휴식·공정근무법 준수 최적 교대표 자동 생성 + PTO 패턴 분석·피크 기간 인력부족 예측 알림</t>
+          <t>Olivia의 후보자 conversational 스크리닝 (work history·shift) 결과 + 매장 매니저 캘린더 기반 면접 slot 자동 제시 + McHire ATS 통합 hiring funnel 기록</t>
         </is>
       </c>
       <c r="K127" s="7" t="inlineStr"/>
       <c r="L127" s="7" t="inlineStr">
         <is>
-          <t>타임시트 자동 승인 + 교대 최적화 + PTO 예측. 제품 발표 단계로 고객 outcome 미공개.</t>
-        </is>
-      </c>
-      <c r="M127" s="9" t="inlineStr"/>
+          <t>Time-to-hire 21일에서 3일 미만으로 86% 단축 (벤더 주장). NBC News가 AI recruiter 사용을 독립 확인(Fact).</t>
+        </is>
+      </c>
+      <c r="M127" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="N127" s="8" t="inlineStr">
         <is>
           <t>✓</t>
@@ -21211,14 +21222,14 @@
       <c r="P127" s="9" t="inlineStr"/>
       <c r="Q127" s="9" t="inlineStr"/>
       <c r="R127" s="9" t="inlineStr"/>
-      <c r="S127" s="9" t="inlineStr"/>
+      <c r="S127" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="T127" s="9" t="inlineStr"/>
       <c r="U127" s="9" t="inlineStr"/>
-      <c r="V127" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="V127" s="9" t="inlineStr"/>
       <c r="W127" s="10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -21231,32 +21242,32 @@
       <c r="AB127" s="9" t="inlineStr"/>
       <c r="AC127" s="7" t="inlineStr">
         <is>
-          <t>Payroll Operations</t>
+          <t>Screening &amp; Assessment</t>
         </is>
       </c>
       <c r="AD127" s="7" t="inlineStr">
         <is>
-          <t>Paychex</t>
+          <t>Paradox</t>
         </is>
       </c>
       <c r="AE127" s="7" t="inlineStr">
         <is>
-          <t>hrms</t>
+          <t>point-solution</t>
         </is>
       </c>
       <c r="AF127" s="7" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>restaurant, fast-food</t>
         </is>
       </c>
       <c r="AG127" s="7" t="inlineStr">
         <is>
-          <t>N. America, Europe</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="AH127" s="7" t="inlineStr">
         <is>
-          <t>발표·계획</t>
+          <t>운영</t>
         </is>
       </c>
       <c r="AI127" s="7" t="inlineStr">
@@ -21267,18 +21278,27 @@
       <c r="AJ127" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK127" s="7" t="inlineStr"/>
+      <c r="AK127" s="7" t="inlineStr">
+        <is>
+          <t>• Paradox wiki 고객 생태계 6번째: Chipotle(75%↓) · Nestlé(600%↑) · 7-Eleven(40k hrs/wk) · GM($2M) · Workday(23k hrs) · McDonald's(21→3일)
+• 식음료·리테일 고볼륨 채용에서 Paradox의 market dominance가 데이터로 확실</t>
+        </is>
+      </c>
       <c r="AL127" s="7" t="inlineStr">
         <is>
-          <t>payroll, timesheet, agentic-ai, shift-scheduling, time-off, auto-approval, smb, workforce-management</t>
-        </is>
-      </c>
-      <c r="AM127" s="7" t="inlineStr"/>
+          <t>paradox, conversational-ai, high-volume, restaurant, fast-food</t>
+        </is>
+      </c>
+      <c r="AM127" s="11" t="inlineStr">
+        <is>
+          <t>Paradox clients + NBC News</t>
+        </is>
+      </c>
       <c r="AN127" s="7" t="inlineStr"/>
       <c r="AO127" s="7" t="inlineStr"/>
       <c r="AP127" s="7" t="inlineStr">
         <is>
-          <t>paychex-flex-agentic-workforce</t>
+          <t>mcdonalds-paradox-recruiting</t>
         </is>
       </c>
     </row>
@@ -21288,35 +21308,36 @@
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>학습·육성</t>
+          <t>보상·복리후생</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>삼성 멀티캠퍼스: CIC AI 맞춤 교육 추천 (삼성전자 사내 교육)</t>
+          <t>Paychex/Paycor: Agentic Workforce Management (타임시트 자동승인·Auto-Shifts, 800K 고객)</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>_다수 (800K 고객)_</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>삼성 멀티캠퍼스의 CIC(Corporate Innovation Campus) 플랫폼은 삼성전자 사내 직원 대상 e-러닝 서비스로, 부서·직급·직무·관심 키워드·수강 이력을 분석해 맞춤형 교육 콘텐츠를 추천하는 AI 기능을 운영한다. 멀티캠퍼스는 별도로 외부 기업 대상 AI 직무 역량 교육 프로그램과 IT 업스킬링·리스킬링 서비스를 제공하며, 2025년 삼성청년SW·AI아카데미(SSAFY) 커리큘럼에서도 AI 역량 강화를 확대했다.</t>
+          <t>Paychex가 2026년 2월 Paycor 및 Paychex Flex 플랫폼에 에이전틱 AI 솔루션을 발표. Paycor Agentic Timesheet Approvals(타임카드 자동 스코어링·이상만 사람 검토), Paycor Auto-Shifts(근무시간 제한·휴식·공정근무법 기반 최적 교대 생성), Paychex Flex AI-Powered Time-Off(PTO 패턴 분석·반복 가용성 AI). 800,000 고객 규모. Nucleus…</t>
         </is>
       </c>
       <c r="F128" s="7" t="inlineStr">
         <is>
-          <t>• 삼성전자 규모(10만+ 직원)에서 개인별 교육 니즈가 극도로 다양: 부서·직급·직무·관심사 조합 수천 가지
-• 전통 LMS의 일률적 과정 목록은 직원 engagement 저하
-• AI·디지털 리스킬링 수요 폭증 → 맞춤형 추천 없이는 학습 효율 저하</t>
+          <t>• 매니저가 타임시트를 수동으로 하나씩 검토·승인 → 시간 낭비 + 오류 발생
+• 교대 스케줄을 수동 작성 → 노동법(공정근무법·52시간) 위반 리스크
+• PTO 관리가 반응적 → 피크 기간 인력 부족 사전 예측 불가
+• SMB(중소기업)는 HR 전담 인력이 적어 자동화 수요 특히 높음</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
         <is>
           <t>[Before]
-LMS에서 직원이 과정 목록을 수동 탐색 → 관련성 낮은 과정 수강 → 학습 효율 저하 /
+매니저가 타임카드 수동 검토 → 교대표 수동 작성 → PTO 개별 승인 /
 [After]
 1. md]]</t>
         </is>
@@ -21325,13 +21346,13 @@
       <c r="I128" s="7" t="inlineStr"/>
       <c r="J128" s="7" t="inlineStr">
         <is>
-          <t>직원 부서·직급·직무·관심 키워드·수강 이력 기반 맞춤형 사내 교육 콘텐츠 추천 목록 (삼성U 멀티캠퍼스 모바일·웹)</t>
+          <t>타임카드 자동 스코어링·승인 결과 (이상 케이스만 매니저 플래그) + 노동법·휴식·공정근무법 준수 최적 교대표 자동 생성 + PTO 패턴 분석·피크 기간 인력부족 예측 알림</t>
         </is>
       </c>
       <c r="K128" s="7" t="inlineStr"/>
       <c r="L128" s="7" t="inlineStr">
         <is>
-          <t>삼성전자 직원 대상 맞춤 교육 추천 → 학습 참여율·관련성 향상 기대. 구체 정량 지표 미공개.</t>
+          <t>타임시트 자동 승인 + 교대 최적화 + PTO 예측. 제품 발표 단계로 고객 outcome 미공개.</t>
         </is>
       </c>
       <c r="M128" s="9" t="inlineStr"/>
@@ -21347,45 +21368,49 @@
       <c r="S128" s="9" t="inlineStr"/>
       <c r="T128" s="9" t="inlineStr"/>
       <c r="U128" s="9" t="inlineStr"/>
-      <c r="V128" s="9" t="inlineStr"/>
-      <c r="W128" s="9" t="inlineStr"/>
-      <c r="X128" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="V128" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W128" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X128" s="9" t="inlineStr"/>
       <c r="Y128" s="9" t="inlineStr"/>
       <c r="Z128" s="9" t="inlineStr"/>
       <c r="AA128" s="9" t="inlineStr"/>
       <c r="AB128" s="9" t="inlineStr"/>
       <c r="AC128" s="7" t="inlineStr">
         <is>
-          <t>Content &amp; Delivery</t>
+          <t>Payroll Operations</t>
         </is>
       </c>
       <c r="AD128" s="7" t="inlineStr">
         <is>
-          <t>멀티캠퍼스</t>
+          <t>Paychex</t>
         </is>
       </c>
       <c r="AE128" s="7" t="inlineStr">
         <is>
-          <t>internal-build</t>
+          <t>hrms</t>
         </is>
       </c>
       <c r="AF128" s="7" t="inlineStr">
         <is>
-          <t>tech, manufacturing</t>
+          <t>all</t>
         </is>
       </c>
       <c r="AG128" s="7" t="inlineStr">
         <is>
-          <t>🇰🇷 KR</t>
+          <t>N. America, Europe</t>
         </is>
       </c>
       <c r="AH128" s="7" t="inlineStr">
         <is>
-          <t>운영</t>
+          <t>발표·계획</t>
         </is>
       </c>
       <c r="AI128" s="7" t="inlineStr">
@@ -21399,7 +21424,7 @@
       <c r="AK128" s="7" t="inlineStr"/>
       <c r="AL128" s="7" t="inlineStr">
         <is>
-          <t>korea, samsung, ai-recommendation, personalized-learning, corporate-education, upskilling, reskilling</t>
+          <t>payroll, timesheet, agentic-ai, shift-scheduling, time-off, auto-approval, smb, workforce-management</t>
         </is>
       </c>
       <c r="AM128" s="7" t="inlineStr"/>
@@ -21407,7 +21432,7 @@
       <c r="AO128" s="7" t="inlineStr"/>
       <c r="AP128" s="7" t="inlineStr">
         <is>
-          <t>samsung-multicampus-ai-learning</t>
+          <t>paychex-flex-agentic-workforce</t>
         </is>
       </c>
     </row>
@@ -21417,55 +21442,53 @@
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>전략기획·거버넌스</t>
+          <t>학습·육성</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>SK하이닉스: PwC 제안 5-Agent Agentic Retention 시스템 (추진 계획, Structura·Cognita·Chronos·Sentio·Agora)</t>
+          <t>삼성 멀티캠퍼스: CIC AI 맞춤 교육 추천 (삼성전자 사내 교육)</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>PwC Korea가 SK하이닉스에 제안한 5-Agent agentic retention prediction 시스템. 5개 specialist 에이전트가 각기 다른 데이터 영역을 분석하고 hybrid 가중치 (AHP + Bayesian) + LLM·XAI 기반 explainability로 통합. 각 에이전트는 라틴어/그리스어 어원 명명: Structura(정형) · Cognita(관계) · Chronos(시계열) · Sentio(텍스트) · A…</t>
+          <t>삼성 멀티캠퍼스의 CIC(Corporate Innovation Campus) 플랫폼은 삼성전자 사내 직원 대상 e-러닝 서비스로, 부서·직급·직무·관심 키워드·수강 이력을 분석해 맞춤형 교육 콘텐츠를 추천하는 AI 기능을 운영한다. 멀티캠퍼스는 별도로 외부 기업 대상 AI 직무 역량 교육 프로그램과 IT 업스킬링·리스킬링 서비스를 제공하며, 2025년 삼성청년SW·AI아카데미(SSAFY) 커리큘럼에서도 AI 역량 강화를 확대했다.</t>
         </is>
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
-          <t>• Before: 핵심 인재 이탈은 사후 면담 + 단편적 정형 데이터(근속·평가) 위주 분석. 미묘한 행동 변화·외부 시장 신호·관계 패턴 unintegrated. 매니저 "감"에 의존
-• Pain point: SK하이닉스 38K 직원 중 반도체 핵심 인재 (R&amp;D·tech 전문가) 이탈 비용 거대. 사후 대응으론 retention 불가
-• Trigger: 2024-25 SK 그룹 차원 AI 적극 도입 + PwC Korea 컨설팅 제안</t>
+          <t>• 삼성전자 규모(10만+ 직원)에서 개인별 교육 니즈가 극도로 다양: 부서·직급·직무·관심사 조합 수천 가지
+• 전통 LMS의 일률적 과정 목록은 직원 engagement 저하
+• AI·디지털 리스킬링 수요 폭증 → 맞춤형 추천 없이는 학습 효율 저하</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
         <is>
           <t>[Before]
-핵심 인재 이탈은 사후 면담 + 단편적 정형 데이터(근속·평가) 위주 분석. 미묘한 행동 변화·외부 시장 신호·관계 패턴 unintegrated. 매니저 "감"에 의존 / Pain point: SK하이닉스 38K 직원 중 반도체 핵심 인재 (R&amp;D·tech 전문가) 이탈 비용 거대. 사후 대응으론 retention 불가 / Trigger: 2024-25 …</t>
+LMS에서 직원이 과정 목록을 수동 탐색 → 관련성 낮은 과정 수강 → 학습 효율 저하 /
+[After]
+1. md]]</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr"/>
       <c r="I129" s="7" t="inlineStr"/>
       <c r="J129" s="7" t="inlineStr">
         <is>
-          <t>퇴사 위험 등급 (Green/Yellow/Red) + 위험 요인 Summary (LLM+XAI) + 5개 에이전트 (Structura/Cognita/Chronos/Sentio/Agora)별 상세 분석 + 등급별 맞춤 retention action 권고 (면담·보상·경력 개발)</t>
+          <t>직원 부서·직급·직무·관심 키워드·수강 이력 기반 맞춤형 사내 교육 콘텐츠 추천 목록 (삼성U 멀티캠퍼스 모바일·웹)</t>
         </is>
       </c>
       <c r="K129" s="7" t="inlineStr"/>
       <c r="L129" s="7" t="inlineStr">
         <is>
-          <t>이탈 예측을 단편적 사후 분석에서 5개 데이터 차원 통합 + 선제적 개입으로 전환 시도. 단, 추진 계획 단계로 actual production metric 0건.</t>
-        </is>
-      </c>
-      <c r="M129" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+          <t>삼성전자 직원 대상 맞춤 교육 추천 → 학습 참여율·관련성 향상 기대. 구체 정량 지표 미공개.</t>
+        </is>
+      </c>
+      <c r="M129" s="9" t="inlineStr"/>
       <c r="N129" s="8" t="inlineStr">
         <is>
           <t>✓</t>
@@ -21475,23 +21498,11 @@
       <c r="P129" s="9" t="inlineStr"/>
       <c r="Q129" s="9" t="inlineStr"/>
       <c r="R129" s="9" t="inlineStr"/>
-      <c r="S129" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="S129" s="9" t="inlineStr"/>
       <c r="T129" s="9" t="inlineStr"/>
       <c r="U129" s="9" t="inlineStr"/>
-      <c r="V129" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W129" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="V129" s="9" t="inlineStr"/>
+      <c r="W129" s="9" t="inlineStr"/>
       <c r="X129" s="10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -21503,22 +21514,22 @@
       <c r="AB129" s="9" t="inlineStr"/>
       <c r="AC129" s="7" t="inlineStr">
         <is>
-          <t>People Analytics</t>
+          <t>Content &amp; Delivery</t>
         </is>
       </c>
       <c r="AD129" s="7" t="inlineStr">
         <is>
-          <t>PwC, SK하이닉스 internal</t>
+          <t>멀티캠퍼스</t>
         </is>
       </c>
       <c r="AE129" s="7" t="inlineStr">
         <is>
-          <t>point-solution</t>
+          <t>internal-build</t>
         </is>
       </c>
       <c r="AF129" s="7" t="inlineStr">
         <is>
-          <t>semiconductor</t>
+          <t>tech, manufacturing</t>
         </is>
       </c>
       <c r="AG129" s="7" t="inlineStr">
@@ -21528,18 +21539,161 @@
       </c>
       <c r="AH129" s="7" t="inlineStr">
         <is>
-          <t>발표·계획</t>
+          <t>운영</t>
         </is>
       </c>
       <c r="AI129" s="7" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>일</t>
         </is>
       </c>
       <c r="AJ129" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK129" s="7" t="inlineStr">
+      <c r="AK129" s="7" t="inlineStr"/>
+      <c r="AL129" s="7" t="inlineStr">
+        <is>
+          <t>korea, samsung, ai-recommendation, personalized-learning, corporate-education, upskilling, reskilling</t>
+        </is>
+      </c>
+      <c r="AM129" s="7" t="inlineStr"/>
+      <c r="AN129" s="7" t="inlineStr"/>
+      <c r="AO129" s="7" t="inlineStr"/>
+      <c r="AP129" s="7" t="inlineStr">
+        <is>
+          <t>samsung-multicampus-ai-learning</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="90" customHeight="1">
+      <c r="A130" s="7" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>전략기획·거버넌스</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>SK하이닉스: PwC 제안 5-Agent Agentic Retention 시스템 (추진 계획, Structura·Cognita·Chronos·Sentio·Agora)</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>PwC Korea가 SK하이닉스에 제안한 5-Agent agentic retention prediction 시스템. 5개 specialist 에이전트가 각기 다른 데이터 영역을 분석하고 hybrid 가중치 (AHP + Bayesian) + LLM·XAI 기반 explainability로 통합. 각 에이전트는 라틴어/그리스어 어원 명명: Structura(정형) · Cognita(관계) · Chronos(시계열) · Sentio(텍스트) · A…</t>
+        </is>
+      </c>
+      <c r="F130" s="7" t="inlineStr">
+        <is>
+          <t>• Before: 핵심 인재 이탈은 사후 면담 + 단편적 정형 데이터(근속·평가) 위주 분석. 미묘한 행동 변화·외부 시장 신호·관계 패턴 unintegrated. 매니저 "감"에 의존
+• Pain point: SK하이닉스 38K 직원 중 반도체 핵심 인재 (R&amp;D·tech 전문가) 이탈 비용 거대. 사후 대응으론 retention 불가
+• Trigger: 2024-25 SK 그룹 차원 AI 적극 도입 + PwC Korea 컨설팅 제안</t>
+        </is>
+      </c>
+      <c r="G130" s="7" t="inlineStr">
+        <is>
+          <t>[Before]
+핵심 인재 이탈은 사후 면담 + 단편적 정형 데이터(근속·평가) 위주 분석. 미묘한 행동 변화·외부 시장 신호·관계 패턴 unintegrated. 매니저 "감"에 의존 / Pain point: SK하이닉스 38K 직원 중 반도체 핵심 인재 (R&amp;D·tech 전문가) 이탈 비용 거대. 사후 대응으론 retention 불가 / Trigger: 2024-25 …</t>
+        </is>
+      </c>
+      <c r="H130" s="7" t="inlineStr"/>
+      <c r="I130" s="7" t="inlineStr"/>
+      <c r="J130" s="7" t="inlineStr">
+        <is>
+          <t>퇴사 위험 등급 (Green/Yellow/Red) + 위험 요인 Summary (LLM+XAI) + 5개 에이전트 (Structura/Cognita/Chronos/Sentio/Agora)별 상세 분석 + 등급별 맞춤 retention action 권고 (면담·보상·경력 개발)</t>
+        </is>
+      </c>
+      <c r="K130" s="7" t="inlineStr"/>
+      <c r="L130" s="7" t="inlineStr">
+        <is>
+          <t>이탈 예측을 단편적 사후 분석에서 5개 데이터 차원 통합 + 선제적 개입으로 전환 시도. 단, 추진 계획 단계로 actual production metric 0건.</t>
+        </is>
+      </c>
+      <c r="M130" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N130" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O130" s="9" t="inlineStr"/>
+      <c r="P130" s="9" t="inlineStr"/>
+      <c r="Q130" s="9" t="inlineStr"/>
+      <c r="R130" s="9" t="inlineStr"/>
+      <c r="S130" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T130" s="9" t="inlineStr"/>
+      <c r="U130" s="9" t="inlineStr"/>
+      <c r="V130" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W130" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X130" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y130" s="9" t="inlineStr"/>
+      <c r="Z130" s="9" t="inlineStr"/>
+      <c r="AA130" s="9" t="inlineStr"/>
+      <c r="AB130" s="9" t="inlineStr"/>
+      <c r="AC130" s="7" t="inlineStr">
+        <is>
+          <t>People Analytics</t>
+        </is>
+      </c>
+      <c r="AD130" s="7" t="inlineStr">
+        <is>
+          <t>PwC, SK하이닉스 internal</t>
+        </is>
+      </c>
+      <c r="AE130" s="7" t="inlineStr">
+        <is>
+          <t>point-solution</t>
+        </is>
+      </c>
+      <c r="AF130" s="7" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="AG130" s="7" t="inlineStr">
+        <is>
+          <t>🇰🇷 KR</t>
+        </is>
+      </c>
+      <c r="AH130" s="7" t="inlineStr">
+        <is>
+          <t>발표·계획</t>
+        </is>
+      </c>
+      <c r="AI130" s="7" t="inlineStr">
+        <is>
+          <t>월</t>
+        </is>
+      </c>
+      <c r="AJ130" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AK130" s="7" t="inlineStr">
         <is>
           <t>• KR 컨설팅에서의 위치: "검증 후보 + 비교 reference":
 • 만약 SK하이닉스 deployment 성공 시 KR 반도체·이차전지·바이오 그룹사 retention 컨설팅의 reference architecture
@@ -21547,46 +21701,46 @@
 • 글로벌 비교:</t>
         </is>
       </c>
-      <c r="AL129" s="7" t="inlineStr">
+      <c r="AL130" s="7" t="inlineStr">
         <is>
           <t>sk-hynix, pwc, retention, multi-agent, agentic, ahp, bayesian-optimization, xai, korean-conglomerate, korea, planned-deployment, semiconductor</t>
         </is>
       </c>
-      <c r="AM129" s="7" t="inlineStr"/>
-      <c r="AN129" s="7" t="inlineStr"/>
-      <c r="AO129" s="7" t="inlineStr"/>
-      <c r="AP129" s="7" t="inlineStr">
+      <c r="AM130" s="7" t="inlineStr"/>
+      <c r="AN130" s="7" t="inlineStr"/>
+      <c r="AO130" s="7" t="inlineStr"/>
+      <c r="AP130" s="7" t="inlineStr">
         <is>
           <t>sk-hynix-pwc-5agent-retention</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="90" customHeight="1">
-      <c r="A130" s="7" t="n">
-        <v>129</v>
-      </c>
-      <c r="B130" s="7" t="inlineStr">
+    <row r="131" ht="90" customHeight="1">
+      <c r="A131" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="7" t="inlineStr">
         <is>
           <t>보상·복리후생</t>
         </is>
       </c>
-      <c r="C130" s="7" t="inlineStr">
+      <c r="C131" s="7" t="inlineStr">
         <is>
           <t>Syndio: Syndi Expert AI (보상 공정성 + EU AI Act 준수)</t>
         </is>
       </c>
-      <c r="D130" s="7" t="inlineStr">
+      <c r="D131" s="7" t="inlineStr">
         <is>
           <t>_다수 (300+ 고객, 30% Fortune Most Admired)_</t>
         </is>
       </c>
-      <c r="E130" s="7" t="inlineStr">
+      <c r="E131" s="7" t="inlineStr">
         <is>
           <t>Syndio는 보상 공정성(pay equity) 전문 AI 플랫폼. 2025년 3월 Syndi라는 expert AI를 출시해 급여 보고 규제(EU Pay Transparency Directive·미국 주별 법률 등) 준수를 자동화. ⚠️ 벤더 주장: 300+ 고객, Fortune Most Admired 30%. "10페이지 법률 메모를 단일 actionable 답변으로" 대체한 사례 보고.</t>
         </is>
       </c>
-      <c r="F130" s="7" t="inlineStr"/>
-      <c r="G130" s="7" t="inlineStr">
+      <c r="F131" s="7" t="inlineStr"/>
+      <c r="G131" s="7" t="inlineStr">
         <is>
           <t>[Before]
 보상 결정 시 매니저·HR이 spreadsheet·외부 market data로 ad-hoc 판단, equity 위반 사후 발견 /
@@ -21599,137 +21753,137 @@
 6. Expertise on Demand AI가 pay gap 보고·규제 컴플라이언스 가이드</t>
         </is>
       </c>
-      <c r="H130" s="7" t="inlineStr"/>
-      <c r="I130" s="7" t="inlineStr"/>
-      <c r="J130" s="7" t="inlineStr">
+      <c r="H131" s="7" t="inlineStr"/>
+      <c r="I131" s="7" t="inlineStr"/>
+      <c r="J131" s="7" t="inlineStr">
         <is>
           <t>protected class별 pay gap 분석 결과 + offer/raise/promotion 시점의 internal equity·budget·market 균형 추천 + 국가별 pay transparency 규제 컴플라이언스 가이드·법률 메모 답변</t>
         </is>
       </c>
-      <c r="K130" s="7" t="inlineStr"/>
-      <c r="L130" s="7" t="inlineStr">
+      <c r="K131" s="7" t="inlineStr"/>
+      <c r="L131" s="7" t="inlineStr">
         <is>
           <t>⚠️ 벤더 주장: 300+ 고객사, Fortune Most Admired 기업 30% 사용: 이는 시장 침투(market adoption) 수치이며 고객의 pay equity outcome(격차 해소율·감사 통과율·비용 절감) 아님. "10페이지 법률 메모→단일 답변" 1건 사례도 벤더 주장. 고객 outcome metric _미공개_.</t>
         </is>
       </c>
-      <c r="M130" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N130" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O130" s="9" t="inlineStr"/>
-      <c r="P130" s="9" t="inlineStr"/>
-      <c r="Q130" s="9" t="inlineStr"/>
-      <c r="R130" s="9" t="inlineStr"/>
-      <c r="S130" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T130" s="9" t="inlineStr"/>
-      <c r="U130" s="9" t="inlineStr"/>
-      <c r="V130" s="9" t="inlineStr"/>
-      <c r="W130" s="9" t="inlineStr"/>
-      <c r="X130" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y130" s="9" t="inlineStr"/>
-      <c r="Z130" s="9" t="inlineStr"/>
-      <c r="AA130" s="9" t="inlineStr"/>
-      <c r="AB130" s="9" t="inlineStr"/>
-      <c r="AC130" s="7" t="inlineStr">
+      <c r="M131" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N131" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O131" s="9" t="inlineStr"/>
+      <c r="P131" s="9" t="inlineStr"/>
+      <c r="Q131" s="9" t="inlineStr"/>
+      <c r="R131" s="9" t="inlineStr"/>
+      <c r="S131" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T131" s="9" t="inlineStr"/>
+      <c r="U131" s="9" t="inlineStr"/>
+      <c r="V131" s="9" t="inlineStr"/>
+      <c r="W131" s="9" t="inlineStr"/>
+      <c r="X131" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y131" s="9" t="inlineStr"/>
+      <c r="Z131" s="9" t="inlineStr"/>
+      <c r="AA131" s="9" t="inlineStr"/>
+      <c r="AB131" s="9" t="inlineStr"/>
+      <c r="AC131" s="7" t="inlineStr">
         <is>
           <t>Compensation</t>
         </is>
       </c>
-      <c r="AD130" s="7" t="inlineStr">
+      <c r="AD131" s="7" t="inlineStr">
         <is>
           <t>Syndio</t>
         </is>
       </c>
-      <c r="AE130" s="7" t="inlineStr">
+      <c r="AE131" s="7" t="inlineStr">
         <is>
           <t>point-solution</t>
         </is>
       </c>
-      <c r="AF130" s="7" t="inlineStr">
+      <c r="AF131" s="7" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="AG130" s="7" t="inlineStr">
+      <c r="AG131" s="7" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="AH130" s="7" t="inlineStr">
+      <c r="AH131" s="7" t="inlineStr">
         <is>
           <t>운영</t>
         </is>
       </c>
-      <c r="AI130" s="7" t="inlineStr">
+      <c r="AI131" s="7" t="inlineStr">
         <is>
           <t>월</t>
         </is>
       </c>
-      <c r="AJ130" s="7" t="n">
+      <c r="AJ131" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK130" s="7" t="inlineStr"/>
-      <c r="AL130" s="7" t="inlineStr">
+      <c r="AK131" s="7" t="inlineStr"/>
+      <c r="AL131" s="7" t="inlineStr">
         <is>
           <t>pay-equity, compliance, eu-ai-act, gdpr, pay-transparency, syndio</t>
         </is>
       </c>
-      <c r="AM130" s="11" t="inlineStr">
+      <c r="AM131" s="11" t="inlineStr">
         <is>
           <t>PR Newswire 2025-03-04</t>
         </is>
       </c>
-      <c r="AN130" s="11" t="inlineStr">
+      <c r="AN131" s="11" t="inlineStr">
         <is>
           <t>Syndio 공식</t>
         </is>
       </c>
-      <c r="AO130" s="7" t="inlineStr"/>
-      <c r="AP130" s="7" t="inlineStr">
+      <c r="AO131" s="7" t="inlineStr"/>
+      <c r="AP131" s="7" t="inlineStr">
         <is>
           <t>syndio-pay-equity-ai</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="90" customHeight="1">
-      <c r="A131" s="7" t="n">
-        <v>130</v>
-      </c>
-      <c r="B131" s="7" t="inlineStr">
+    <row r="132" ht="90" customHeight="1">
+      <c r="A132" s="7" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="7" t="inlineStr">
         <is>
           <t>채용</t>
         </is>
       </c>
-      <c r="C131" s="7" t="inlineStr">
+      <c r="C132" s="7" t="inlineStr">
         <is>
           <t>원티드랩: AI 채용 에이전트 (LLM 기반 자연어 인재 검색)</t>
         </is>
       </c>
-      <c r="D131" s="7" t="inlineStr">
+      <c r="D132" s="7" t="inlineStr">
         <is>
           <t>_N/A (product, no specific customer deployment yet)_</t>
         </is>
       </c>
-      <c r="E131" s="7" t="inlineStr">
+      <c r="E132" s="7" t="inlineStr">
         <is>
           <t>원티드랩(국내 최대급 HR tech 벤더, 상장)이 2025년 10월 21일 출시한 LLM 기반 AI 채용 에이전트. 기업 채용 담당자가 자연어로 인재를 검색할 수 있게 하는 B2B 제품. 복잡한 필터 설정 없이 "역량과 경험을 AI가 판단하여 추천 사유까지 제시"하는 것이 핵심 차별점.</t>
         </is>
       </c>
-      <c r="F131" s="7" t="inlineStr">
+      <c r="F132" s="7" t="inlineStr">
         <is>
           <t>• 기존 ATS·채용 플랫폼은 키워드·필터 기반 검색이어서 후보자의 "잠재 역량"이나 "정성적 경험"을 놓치기 쉬움
 • 자기소개서·프로젝트 경험 같은 비정형 텍스트 데이터가 검색에 제대로 반영되지 않음
@@ -21737,7 +21891,7 @@
 (원티드랩의 공식 problem statement를 전달하는 매체 요약 기반. 직접 인용 아님.)</t>
         </is>
       </c>
-      <c r="G131" s="7" t="inlineStr">
+      <c r="G132" s="7" t="inlineStr">
         <is>
           <t>[Before]
 채용 담당자가 키워드·필터로 후보자를 검색, 검색 결과를 수동으로 검토 /
@@ -21749,7 +21903,7 @@
 5. 담당자가 최종 판단 및 컨택</t>
         </is>
       </c>
-      <c r="H131" s="7" t="inlineStr">
+      <c r="H132" s="7" t="inlineStr">
         <is>
           <t>• Core HRIS: N/A (독립 플랫폼, 채용 담당자 B2B 제품)
 • AI 시스템 배치: 원티드 플랫폼 내부 (기존 원티드 서비스에 에이전트 기능으로 추가)
@@ -21758,169 +21912,28 @@
 • 사용자 접점: 원티드 웹 interface (별도 애플리케이션 여부 _미공개_)</t>
         </is>
       </c>
-      <c r="I131" s="7" t="inlineStr">
+      <c r="I132" s="7" t="inlineStr">
         <is>
           <t>• 입력 데이터 소스: (기존 원티드 플랫폼):
 • 데이터 규모: 국내 최대급 HR data pool (상장사 IR 기준)
 • 데이터 거버넌스: - 원티드랩은 국내 개인정보보호법 대상: 후보자 동의 기반 data 활용</t>
         </is>
       </c>
-      <c r="J131" s="7" t="inlineStr">
+      <c r="J132" s="7" t="inlineStr">
         <is>
           <t>자연어 쿼리 기반 후보자 검색 결과 (기본 탐색 풀 + 자기소개서·프로젝트 정성 분석 고급 탐색) + 후보별 역량·경험 판단 + 추천 사유 reasoning</t>
         </is>
       </c>
-      <c r="K131" s="7" t="inlineStr">
+      <c r="K132" s="7" t="inlineStr">
         <is>
           <t>• Foundation model: LLM 기반이라고만 명시. 구체 모델(자체 학습? OpenAI·Anthropic API 래핑?) _미공개_
 • 모델 유형: LLM 추론 + semantic search (추정되나 소스에 명시 없음)
 • 제공 방식: 원티드랩 자체 플랫폼</t>
         </is>
       </c>
-      <c r="L131" s="7" t="inlineStr">
+      <c r="L132" s="7" t="inlineStr">
         <is>
           <t>⚠️ 기대효과 수치 미공개. 아래 표 참조.</t>
-        </is>
-      </c>
-      <c r="M131" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N131" s="8" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O131" s="9" t="inlineStr"/>
-      <c r="P131" s="9" t="inlineStr"/>
-      <c r="Q131" s="9" t="inlineStr"/>
-      <c r="R131" s="9" t="inlineStr"/>
-      <c r="S131" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T131" s="9" t="inlineStr"/>
-      <c r="U131" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V131" s="9" t="inlineStr"/>
-      <c r="W131" s="9" t="inlineStr"/>
-      <c r="X131" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y131" s="9" t="inlineStr"/>
-      <c r="Z131" s="9" t="inlineStr"/>
-      <c r="AA131" s="9" t="inlineStr"/>
-      <c r="AB131" s="9" t="inlineStr"/>
-      <c r="AC131" s="7" t="inlineStr">
-        <is>
-          <t>Sourcing &amp; Attraction</t>
-        </is>
-      </c>
-      <c r="AD131" s="7" t="inlineStr">
-        <is>
-          <t>Wanted Lab</t>
-        </is>
-      </c>
-      <c r="AE131" s="7" t="inlineStr">
-        <is>
-          <t>ats</t>
-        </is>
-      </c>
-      <c r="AF131" s="7" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AG131" s="7" t="inlineStr">
-        <is>
-          <t>🇰🇷 KR</t>
-        </is>
-      </c>
-      <c r="AH131" s="7" t="inlineStr">
-        <is>
-          <t>파일럿</t>
-        </is>
-      </c>
-      <c r="AI131" s="7" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="AJ131" s="7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AK131" s="7" t="inlineStr"/>
-      <c r="AL131" s="7" t="inlineStr">
-        <is>
-          <t>ai-agent, llm, natural-language, recruiting, sourcing, korea, korean-vendor</t>
-        </is>
-      </c>
-      <c r="AM131" s="7" t="inlineStr"/>
-      <c r="AN131" s="7" t="inlineStr"/>
-      <c r="AO131" s="7" t="inlineStr"/>
-      <c r="AP131" s="7" t="inlineStr">
-        <is>
-          <t>wantedlab-ai-recruiting-agent</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="90" customHeight="1">
-      <c r="A132" s="7" t="n">
-        <v>131</v>
-      </c>
-      <c r="B132" s="7" t="inlineStr">
-        <is>
-          <t>EX·HR운영</t>
-        </is>
-      </c>
-      <c r="C132" s="7" t="inlineStr">
-        <is>
-          <t>SK하이닉스: PwC 제안 One Resume + AI 구성원 검색 (통합 직원 프로필·내부 talent search, 추진 계획)</t>
-        </is>
-      </c>
-      <c r="D132" s="7" t="inlineStr">
-        <is>
-          <t>SK하이닉스</t>
-        </is>
-      </c>
-      <c r="E132" s="7" t="inlineStr">
-        <is>
-          <t>PwC Korea가 SK하이닉스에 제안한 One Resume + AI 구성원 검색 시스템. 직원 1인당 분산된 데이터 (HRMS·평가·교육·프로젝트·자격·관심사·skill)를 단일 통합 프로필 (One Resume)로 구성하고, 매니저가 자연어로 사내 talent를 검색·추천 받는 AI talent search 기능을 결합. 동일한 PwC Korea 제안인 과 같은 SK하이닉스 추진 묶음. 2026-05 시점: 제안·검토 단계, 실제 depl…</t>
-        </is>
-      </c>
-      <c r="F132" s="7" t="inlineStr">
-        <is>
-          <t>• Before: SK하이닉스 38K 직원의 인사 데이터가 HRMS·평가·교육·프로젝트·자격증·외부 교육 등 다수 시스템에 분산. 매니저가 internal mobility·project staffing·후계자 후보 검색 시 여러 시스템 + 인적 네트워크 의존
-• Pain point:
-• 사내 talent visibility 부족: 매니저가 "양산공정 + 머신러닝 경험 5년+ 영어 가능자"를 사내에서 찾기 어려움
-• 직원 본인도 자기 career path·내부 기회 잘 모름
-• 핵심 인재 retention·project staffing·후계자 풀 식별 모두 동일한 root cause (skill·경력 visibi…</t>
-        </is>
-      </c>
-      <c r="G132" s="7" t="inlineStr">
-        <is>
-          <t>[Before]
-SK하이닉스 38K 직원의 인사 데이터가 HRMS·평가·교육·프로젝트·자격증·외부 교육 등 다수 시스템에 분산. 매니저가 internal mobility·project staffing·후계자 후보 검색 시 여러 시스템 + 인적 네트워크 의존 / Pain point: / 사내 talent visibility 부족: 매니저가 "양산공정 + 머신러닝 경험 5년…</t>
-        </is>
-      </c>
-      <c r="H132" s="7" t="inlineStr"/>
-      <c r="I132" s="7" t="inlineStr"/>
-      <c r="J132" s="7" t="inlineStr">
-        <is>
-          <t>직원 1인당 단일 통합 프로필 (One Resume: 인사·평가·교육·프로젝트·자격·관심사·skill 통합) + 매니저용 자연어 talent search (예: '머신러닝 + 양산공정 경험 5년+ 한국어/영어 가능' 검색) + 직원 본인의 career path 시각화</t>
-        </is>
-      </c>
-      <c r="K132" s="7" t="inlineStr"/>
-      <c r="L132" s="7" t="inlineStr">
-        <is>
-          <t>직원 데이터를 분산 → 통합 + 매니저 검색을 수동 → AI 자연어로 전환 시도. 단, 추진 계획 단계로 actual production metric 0건.</t>
         </is>
       </c>
       <c r="M132" s="8" t="inlineStr">
@@ -21961,22 +21974,22 @@
       <c r="AB132" s="9" t="inlineStr"/>
       <c r="AC132" s="7" t="inlineStr">
         <is>
-          <t>Core HR &amp; Employee Records</t>
+          <t>Sourcing &amp; Attraction</t>
         </is>
       </c>
       <c r="AD132" s="7" t="inlineStr">
         <is>
-          <t>PwC, SK하이닉스 internal</t>
+          <t>Wanted Lab</t>
         </is>
       </c>
       <c r="AE132" s="7" t="inlineStr">
         <is>
-          <t>internal-build</t>
+          <t>ats</t>
         </is>
       </c>
       <c r="AF132" s="7" t="inlineStr">
         <is>
-          <t>semiconductor</t>
+          <t>all</t>
         </is>
       </c>
       <c r="AG132" s="7" t="inlineStr">
@@ -21986,28 +21999,21 @@
       </c>
       <c r="AH132" s="7" t="inlineStr">
         <is>
-          <t>발표·계획</t>
+          <t>파일럿</t>
         </is>
       </c>
       <c r="AI132" s="7" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>일</t>
         </is>
       </c>
       <c r="AJ132" s="7" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="AK132" s="7" t="inlineStr">
-        <is>
-          <t>• KR talent profile/search 컨설팅에서의 위치: "검증 후보 + 비교 reference":
-• 만약 SK하이닉스 deployment 성공 시 KR 반도체·이차전지·바이오 그룹사 talent profile 컨설팅의 reference architecture
-• PwC Korea 제안 → 글로벌 PwC vs Deloitte Anjin (Zora AI) vs McKinsey/BCG의 KR talent search 컨설팅 시장 경쟁 신호
-• 글로벌 비교:</t>
-        </is>
-      </c>
+        <v>0.2</v>
+      </c>
+      <c r="AK132" s="7" t="inlineStr"/>
       <c r="AL132" s="7" t="inlineStr">
         <is>
-          <t>sk-hynix, pwc, one-resume, employee-search, talent-profile, korean-conglomerate, korea, planned-deployment, semiconductor, internal-build</t>
+          <t>ai-agent, llm, natural-language, recruiting, sourcing, korea, korean-vendor</t>
         </is>
       </c>
       <c r="AM132" s="7" t="inlineStr"/>
@@ -22015,7 +22021,7 @@
       <c r="AO132" s="7" t="inlineStr"/>
       <c r="AP132" s="7" t="inlineStr">
         <is>
-          <t>sk-hynix-pwc-one-resume-employee-search</t>
+          <t>wantedlab-ai-recruiting-agent</t>
         </is>
       </c>
     </row>
@@ -22266,14 +22272,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AN117" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM119" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AN119" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM121" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM123" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AN123" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM124" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM125" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM126" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM130" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AN130" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM122" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM124" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AN124" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM125" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM126" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM127" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM131" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AN131" r:id="rId83"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25697,17 +25703,17 @@
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
         <is>
-          <t>Cathay Pacific — HireVue AI 면접 (time-to-hire 90%↓, 3개월→2~3주)</t>
+          <t>SK하이닉스 — One Resume + AI 구성원 검색 (통합 직원 프로필·내부 talent search)</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Cathay Pacific</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C98" s="12" t="inlineStr">
         <is>
-          <t>채용</t>
+          <t>EX·HR운영</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -25721,28 +25727,28 @@
         </is>
       </c>
       <c r="F98" s="12" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>APAC</t>
+          <t>🇰🇷 KR</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t>더존비즈온 — ONE AI 연말정산 end-to-end 자동화</t>
+          <t>Cathay Pacific — HireVue AI 면접 (time-to-hire 90%↓, 3개월→2~3주)</t>
         </is>
       </c>
       <c r="B99" s="12" t="inlineStr">
         <is>
-          <t>_N/A (product, 다수 중소·중견기업 대상)_</t>
+          <t>Cathay Pacific</t>
         </is>
       </c>
       <c r="C99" s="12" t="inlineStr">
         <is>
-          <t>보상·복리후생</t>
+          <t>채용</t>
         </is>
       </c>
       <c r="D99" s="12" t="inlineStr">
@@ -25760,24 +25766,24 @@
       </c>
       <c r="G99" s="12" t="inlineStr">
         <is>
-          <t>🇰🇷 KR</t>
+          <t>APAC</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="12" t="inlineStr">
         <is>
-          <t>Eightfold AI — Talent Intelligence Platform + AI Interviewer</t>
+          <t>더존비즈온 — ONE AI 연말정산 end-to-end 자동화</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
         <is>
-          <t>_다수 (specific names in vendor page)_</t>
+          <t>_N/A (product, 다수 중소·중견기업 대상)_</t>
         </is>
       </c>
       <c r="C100" s="12" t="inlineStr">
         <is>
-          <t>채용</t>
+          <t>보상·복리후생</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -25795,19 +25801,19 @@
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>🇰🇷 KR</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="12" t="inlineStr">
         <is>
-          <t>McDonald's — Paradox AI 채용 (21일→3일 미만 time-to-hire)</t>
+          <t>Eightfold AI — Talent Intelligence Platform + AI Interviewer</t>
         </is>
       </c>
       <c r="B101" s="12" t="inlineStr">
         <is>
-          <t>McDonald's</t>
+          <t>_다수 (specific names in vendor page)_</t>
         </is>
       </c>
       <c r="C101" s="12" t="inlineStr">
@@ -25837,17 +25843,17 @@
     <row r="102">
       <c r="A102" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스 — PwC 제안 5-Agent Agentic Retention 시스템 (추진 계획, Structura·Cognita·Chronos·Sentio·Agora)</t>
+          <t>McDonald's — Paradox AI 채용 (21일→3일 미만 time-to-hire)</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>McDonald's</t>
         </is>
       </c>
       <c r="C102" s="12" t="inlineStr">
         <is>
-          <t>전략기획·거버넌스</t>
+          <t>채용</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -25865,24 +25871,24 @@
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>🇰🇷 KR</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t>Syndio — Syndi Expert AI (보상 공정성 + EU AI Act 준수)</t>
+          <t>SK하이닉스 — PwC 제안 5-Agent Agentic Retention 시스템 (추진 계획, Structura·Cognita·Chronos·Sentio·Agora)</t>
         </is>
       </c>
       <c r="B103" s="12" t="inlineStr">
         <is>
-          <t>_다수 (300+ 고객, 30% Fortune Most Admired)_</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C103" s="12" t="inlineStr">
         <is>
-          <t>보상·복리후생</t>
+          <t>전략기획·거버넌스</t>
         </is>
       </c>
       <c r="D103" s="12" t="inlineStr">
@@ -25900,24 +25906,24 @@
       </c>
       <c r="G103" s="12" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>🇰🇷 KR</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
         <is>
-          <t>원티드랩 — AI 채용 에이전트 (LLM 기반 자연어 인재 검색)</t>
+          <t>Syndio — Syndi Expert AI (보상 공정성 + EU AI Act 준수)</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>_N/A (product, no specific customer deployment yet)_</t>
+          <t>_다수 (300+ 고객, 30% Fortune Most Admired)_</t>
         </is>
       </c>
       <c r="C104" s="12" t="inlineStr">
         <is>
-          <t>채용</t>
+          <t>보상·복리후생</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -25935,24 +25941,24 @@
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>🇰🇷 KR</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스 — PwC 제안 One Resume + AI 구성원 검색 (통합 직원 프로필·내부 talent search, 추진 계획)</t>
+          <t>원티드랩 — AI 채용 에이전트 (LLM 기반 자연어 인재 검색)</t>
         </is>
       </c>
       <c r="B105" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>_N/A (product, no specific customer deployment yet)_</t>
         </is>
       </c>
       <c r="C105" s="12" t="inlineStr">
         <is>
-          <t>EX·HR운영</t>
+          <t>채용</t>
         </is>
       </c>
       <c r="D105" s="12" t="inlineStr">
@@ -25966,7 +25972,7 @@
         </is>
       </c>
       <c r="F105" s="12" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="G105" s="12" t="inlineStr">
         <is>
@@ -26502,17 +26508,17 @@
     <row r="121">
       <c r="A121" s="12" t="inlineStr">
         <is>
-          <t>더존비즈온 — ONE AI 연말정산 end-to-end 자동화</t>
+          <t>SK하이닉스 — One Resume + AI 구성원 검색 (통합 직원 프로필·내부 talent search)</t>
         </is>
       </c>
       <c r="B121" s="12" t="inlineStr">
         <is>
-          <t>_N/A (product, 다수 중소·중견기업 대상)_</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C121" s="12" t="inlineStr">
         <is>
-          <t>보상·복리후생</t>
+          <t>EX·HR운영</t>
         </is>
       </c>
       <c r="D121" s="12" t="inlineStr">
@@ -26526,7 +26532,7 @@
         </is>
       </c>
       <c r="F121" s="12" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="G121" s="12" t="inlineStr">
         <is>
@@ -26537,17 +26543,17 @@
     <row r="122">
       <c r="A122" s="12" t="inlineStr">
         <is>
-          <t>원티드랩 — AI 채용 에이전트 (LLM 기반 자연어 인재 검색)</t>
+          <t>더존비즈온 — ONE AI 연말정산 end-to-end 자동화</t>
         </is>
       </c>
       <c r="B122" s="12" t="inlineStr">
         <is>
-          <t>_N/A (product, no specific customer deployment yet)_</t>
+          <t>_N/A (product, 다수 중소·중견기업 대상)_</t>
         </is>
       </c>
       <c r="C122" s="12" t="inlineStr">
         <is>
-          <t>채용</t>
+          <t>보상·복리후생</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -26572,17 +26578,17 @@
     <row r="123">
       <c r="A123" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스 — PwC 제안 One Resume + AI 구성원 검색 (통합 직원 프로필·내부 talent search, 추진 계획)</t>
+          <t>원티드랩 — AI 채용 에이전트 (LLM 기반 자연어 인재 검색)</t>
         </is>
       </c>
       <c r="B123" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>_N/A (product, no specific customer deployment yet)_</t>
         </is>
       </c>
       <c r="C123" s="12" t="inlineStr">
         <is>
-          <t>EX·HR운영</t>
+          <t>채용</t>
         </is>
       </c>
       <c r="D123" s="12" t="inlineStr">
@@ -26596,7 +26602,7 @@
         </is>
       </c>
       <c r="F123" s="12" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="G123" s="12" t="inlineStr">
         <is>
@@ -31962,17 +31968,17 @@
     <row r="277">
       <c r="A277" s="12" t="inlineStr">
         <is>
-          <t>Eightfold AI — Talent Intelligence Platform + AI Interviewer</t>
+          <t>SK하이닉스 — One Resume + AI 구성원 검색 (통합 직원 프로필·내부 talent search)</t>
         </is>
       </c>
       <c r="B277" s="12" t="inlineStr">
         <is>
-          <t>_다수 (specific names in vendor page)_</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C277" s="12" t="inlineStr">
         <is>
-          <t>채용</t>
+          <t>EX·HR운영</t>
         </is>
       </c>
       <c r="D277" s="12" t="inlineStr">
@@ -31986,28 +31992,28 @@
         </is>
       </c>
       <c r="F277" s="12" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="G277" s="12" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>🇰🇷 KR</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="12" t="inlineStr">
         <is>
-          <t>Lennox — Fuel50 내부 이동 AI (4,800건 이동, 이동당 +5개월 근속)</t>
+          <t>Eightfold AI — Talent Intelligence Platform + AI Interviewer</t>
         </is>
       </c>
       <c r="B278" s="12" t="inlineStr">
         <is>
-          <t>Lennox</t>
+          <t>_다수 (specific names in vendor page)_</t>
         </is>
       </c>
       <c r="C278" s="12" t="inlineStr">
         <is>
-          <t>온보딩·이동</t>
+          <t>채용</t>
         </is>
       </c>
       <c r="D278" s="12" t="inlineStr">
@@ -32025,24 +32031,24 @@
       </c>
       <c r="G278" s="12" t="inlineStr">
         <is>
-          <t>N. America</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="12" t="inlineStr">
         <is>
-          <t>삼성 멀티캠퍼스 — CIC AI 맞춤 교육 추천 (삼성전자 사내 교육)</t>
+          <t>Lennox — Fuel50 내부 이동 AI (4,800건 이동, 이동당 +5개월 근속)</t>
         </is>
       </c>
       <c r="B279" s="12" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>Lennox</t>
         </is>
       </c>
       <c r="C279" s="12" t="inlineStr">
         <is>
-          <t>학습·육성</t>
+          <t>온보딩·이동</t>
         </is>
       </c>
       <c r="D279" s="12" t="inlineStr">
@@ -32060,24 +32066,24 @@
       </c>
       <c r="G279" s="12" t="inlineStr">
         <is>
-          <t>🇰🇷 KR</t>
+          <t>N. America</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스 — PwC 제안 5-Agent Agentic Retention 시스템 (추진 계획, Structura·Cognita·Chronos·Sentio·Agora)</t>
+          <t>삼성 멀티캠퍼스 — CIC AI 맞춤 교육 추천 (삼성전자 사내 교육)</t>
         </is>
       </c>
       <c r="B280" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="C280" s="12" t="inlineStr">
         <is>
-          <t>전략기획·거버넌스</t>
+          <t>학습·육성</t>
         </is>
       </c>
       <c r="D280" s="12" t="inlineStr">
@@ -32102,17 +32108,17 @@
     <row r="281">
       <c r="A281" s="12" t="inlineStr">
         <is>
-          <t>Syndio — Syndi Expert AI (보상 공정성 + EU AI Act 준수)</t>
+          <t>SK하이닉스 — PwC 제안 5-Agent Agentic Retention 시스템 (추진 계획, Structura·Cognita·Chronos·Sentio·Agora)</t>
         </is>
       </c>
       <c r="B281" s="12" t="inlineStr">
         <is>
-          <t>_다수 (300+ 고객, 30% Fortune Most Admired)_</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C281" s="12" t="inlineStr">
         <is>
-          <t>보상·복리후생</t>
+          <t>전략기획·거버넌스</t>
         </is>
       </c>
       <c r="D281" s="12" t="inlineStr">
@@ -32130,24 +32136,24 @@
       </c>
       <c r="G281" s="12" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>🇰🇷 KR</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="12" t="inlineStr">
         <is>
-          <t>원티드랩 — AI 채용 에이전트 (LLM 기반 자연어 인재 검색)</t>
+          <t>Syndio — Syndi Expert AI (보상 공정성 + EU AI Act 준수)</t>
         </is>
       </c>
       <c r="B282" s="12" t="inlineStr">
         <is>
-          <t>_N/A (product, no specific customer deployment yet)_</t>
+          <t>_다수 (300+ 고객, 30% Fortune Most Admired)_</t>
         </is>
       </c>
       <c r="C282" s="12" t="inlineStr">
         <is>
-          <t>채용</t>
+          <t>보상·복리후생</t>
         </is>
       </c>
       <c r="D282" s="12" t="inlineStr">
@@ -32165,24 +32171,24 @@
       </c>
       <c r="G282" s="12" t="inlineStr">
         <is>
-          <t>🇰🇷 KR</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스 — PwC 제안 One Resume + AI 구성원 검색 (통합 직원 프로필·내부 talent search, 추진 계획)</t>
+          <t>원티드랩 — AI 채용 에이전트 (LLM 기반 자연어 인재 검색)</t>
         </is>
       </c>
       <c r="B283" s="12" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>_N/A (product, no specific customer deployment yet)_</t>
         </is>
       </c>
       <c r="C283" s="12" t="inlineStr">
         <is>
-          <t>EX·HR운영</t>
+          <t>채용</t>
         </is>
       </c>
       <c r="D283" s="12" t="inlineStr">
@@ -32196,7 +32202,7 @@
         </is>
       </c>
       <c r="F283" s="12" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="G283" s="12" t="inlineStr">
         <is>
@@ -33112,7 +33118,7 @@
         <v>3</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: HTML process flow의 'md]]' 잔여 + Excel 개요 truncation·줄바꿈 누락 수정
사용자 피드백 2건:

1. HTML process flow에 'md]]'만 표시되는 use case 다수 (예: Betterworks/Colgate-Palmolive)
   원인: extract_v3.py의 numbered-step regex `\d+\.`가 wikilink
   `[[sources/betterworks-nextgen-2026-01.md]]` 안의 "01."을 잘못 매칭 →
   step 추출이 `md]]`만 남는 결과 → mermaid fallback 차단
   수정: numbered-step regex 실행 전에 wikilinks를 먼저 strip + ^ 앵커
   (MULTILINE)로 줄 시작에만 매칭 강제

2. Excel 개요 column이 '…'로 잘리고 bullet/줄바꿈 없어 가독성 불량
   수정: headline (250자 flat 텍스트) → summary (1500자 HTML 변환,
   strip_html이 <li>→•, <br>/</li>→줄바꿈 보존). Summary section
   max_lines 4 → 20. Column 폭 55 → 70. Row height 90 → 140

검증: 132건 중 'md]]' 잔여 0건. Betterworks 사례에서 mermaid 6노드 정상 추출.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/exports/hr-ai-usecase-collection.xlsx
+++ b/wiki/exports/hr-ai-usecase-collection.xlsx
@@ -1236,7 +1236,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="75" customWidth="1" min="7" max="7"/>
     <col width="38" customWidth="1" min="8" max="8"/>
@@ -1488,7 +1488,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="140" customHeight="1">
       <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>JPMorgan LLM Suite: 2024 여름 launch, model-agnostic gateway (OpenAI + Anthropic), ~230K 직원 대상 8개월 만에 200K+ 온보딩 (~2/3 workforce). ⚠️ 자사 보고: 30-40% efficiency, 직원당 3-6h/week saved, $1.5B/yr 추정 가치. 핵심 distinct feature: 직원이 LLM Suite로 annual performance …</t>
+          <t>JPMorgan LLM Suite: 2024 여름 launch, model-agnostic gateway (OpenAI + Anthropic), ~230K 직원 대상 8개월 만에 200K+ 온보딩 (~2/3 workforce). ⚠️ 자사 보고: 30-40% efficiency, 직원당 3-6h/week saved, $1.5B/yr 추정 가치. 핵심 distinct feature: 직원이 LLM Suite로 annual performance review 초안 drafting 가능. 동시에 Dimon Feb 2026: 백오피스/operations -4%/-2%, 클라이언트직 +4%: 총 318,512명 거의 flat 유지하며 AI 재배치. AI specialist 1,500 → 2,500 (+67%).</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="90" customHeight="1">
+    <row r="3" ht="140" customHeight="1">
       <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Workday가 2021-02 인수 (~$700M)한 Peakon Employee Voice: 지속적 pulse 서베이 + AI 감정·테마 분석. 2024-12-11에 Illuminate AI 기능 발표: open-end comment 자동 요약·테마 추출·driver 식별. ⚠️ 벤더 주장: 1B+ 응답 + 200M+ 텍스트 피드백 학습, 60+ 언어, 160개국 운영. ⚠️ 자사 보고: Workday 사내 활용 결과 직원 성장·커리어 만족…</t>
+          <t>Workday가 2021-02 인수 (~$700M)한 Peakon Employee Voice: 지속적 pulse 서베이 + AI 감정·테마 분석. 2024-12-11에 Illuminate AI 기능 발표: open-end comment 자동 요약·테마 추출·driver 식별. ⚠️ 벤더 주장: 1B+ 응답 + 200M+ 텍스트 피드백 학습, 60+ 언어, 160개국 운영. ⚠️ 자사 보고: Workday 사내 활용 결과 직원 성장·커리어 만족도 +35%.</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -1800,7 +1800,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="90" customHeight="1">
+    <row r="4" ht="140" customHeight="1">
       <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Accenture가 2022-11~2025-FY 사이 30명 → 550,000+ 직원 GenAI 교육. AI/data 전문 인력은 40,000(2023) → 77,000(2025) 증가. 연간 ~$1B L&amp;D 투자. CEO Julie Sweet (2026-03 발언): "AI를 사용하지 못하면 승진·고용이 위험" + "non-adaptable 직원은 compression timeline으로 exit".</t>
+          <t>Accenture가 2022-11~2025-FY 사이 30명 → 550,000+ 직원 GenAI 교육. AI/data 전문 인력은 40,000(2023) → 77,000(2025) 증가. 연간 ~$1B L&amp;D 투자. CEO Julie Sweet (2026-03 발언): "AI를 사용하지 못하면 승진·고용이 위험" + "non-adaptable 직원은 compression timeline으로 exit". 가장 강력한 mass reskilling reference.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -1960,7 +1960,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="90" customHeight="1">
+    <row r="5" ht="140" customHeight="1">
       <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Cisco가 anchor한 다자 컨소시엄 (Microsoft·Google·IBM·SAP·Accenture·Eightfold 등). 2025 보고서: 78% ICT 직무가 AI 기술 스킬 포함, top 10 fastest-growing ICT 직무 중 7개가 AI 관련. AI Workforce Playbook + 2025 AI Skills Glossary + 200+ curated learning recommendations 발간. multi-…</t>
+          <t>Cisco가 anchor한 다자 컨소시엄 (Microsoft·Google·IBM·SAP·Accenture·Eightfold 등). 2025 보고서: 78% ICT 직무가 AI 기술 스킬 포함, top 10 fastest-growing ICT 직무 중 7개가 AI 관련. AI Workforce Playbook + 2025 AI Skills Glossary + 200+ curated learning recommendations 발간. multi-vendor 방법론: Tier 1-equivalent 신뢰도.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -2129,7 +2129,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="90" customHeight="1">
+    <row r="6" ht="140" customHeight="1">
       <c r="A6" s="7" t="n">
         <v>5</v>
       </c>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>2025-05 IBM CEO Arvind Krishna 발언: AI agents (AskHR + watsonx Orchestrate stack)가 "a couple hundred HR roles" 대체. 전사 8,000명 layoff (~3% workforce). HR operating budget 4년간 40% 감소 (LaMoreaux). 단, 순 headcount는 증가: 절감액을 엔지니어·영업·마케팅 채용에 재투자.</t>
+          <t>2025-05 IBM CEO Arvind Krishna 발언: AI agents (AskHR + watsonx Orchestrate stack)가 "a couple hundred HR roles" 대체. 전사 8,000명 layoff (~3% workforce). HR operating budget 4년간 40% 감소 (LaMoreaux). 단, 순 headcount는 증가: 절감액을 엔지니어·영업·마케팅 채용에 재투자. "감원"이 아닌 "재배치 + 직무 전환" 패러다임의 canonical reference.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1">
+    <row r="7" ht="140" customHeight="1">
       <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>「인공지능 발전·신뢰 기반 조성 등에 관한 기본법」(통칭 'AI 기본법')이 2026-01-22 본격 시행. EU AI Act에 이은 세계 2번째 포괄규제. 고영향 AI(high-impact AI) 카테고리에 채용·인사평가·승진·해고 의사결정 AI가 명시적으로 포함됨. 영향평가·투명성 고지·인적 감독·이용자 권리 보장 의무.</t>
+          <t>「인공지능 발전·신뢰 기반 조성 등에 관한 기본법」(통칭 'AI 기본법')이 2026-01-22 본격 시행. EU AI Act에 이은 세계 2번째 포괄규제. 고영향 AI(high-impact AI) 카테고리에 채용·인사평가·승진·해고 의사결정 AI가 명시적으로 포함됨. 영향평가·투명성 고지·인적 감독·이용자 권리 보장 의무. 모든 KR HR AI 프로젝트의 legal foundation. 2026-08 EU AI Act high-risk 의무 발효와 결합되면 글로벌 KR 대기업은 dual compliance 운영 부담.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -2472,7 +2472,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="90" customHeight="1">
+    <row r="8" ht="140" customHeight="1">
       <c r="A8" s="7" t="n">
         <v>7</v>
       </c>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Walmart가 OpenAI와 파트너십: 미국 frontline + 사무 직원에게 OpenAI Certification 무료 access (2026 launch 시). 다층 (basics → prompt engineering). Walmart의 $1B 교육 commitment (2026까지)의 일부. ~50,000 직원이 AI/automation roles로 reskilling 진행.</t>
+          <t>Walmart가 OpenAI와 파트너십: 미국 frontline + 사무 직원에게 OpenAI Certification 무료 access (2026 launch 시). 다층 (basics → prompt engineering). Walmart의 $1B 교육 commitment (2026까지)의 일부. ~50,000 직원이 AI/automation roles로 reskilling 진행. 740K frontline에게 Me@Walmart 디바이스 (Samsung Galaxy XCover Pro) 배포로 학습 access 인프라 마련.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -2641,7 +2641,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="90" customHeight="1">
+    <row r="9" ht="140" customHeight="1">
       <c r="A9" s="7" t="n">
         <v>8</v>
       </c>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Anaplan이 2025-12-09 GA로 발표한 Role-Based AI Agents 제품군 중 Workforce Analyst. HR-finance 데이터 통합 + 자연어 query + 시나리오 시뮬레이션으로 인력 의사결정 가속. 검증된 고객 사례: healthcare provider $21M 연 절감 + time-to-market 20% 단축, Fresenius Medical Care planning time 30%+ 단축, Canada…</t>
+          <t>Anaplan이 2025-12-09 GA로 발표한 Role-Based AI Agents 제품군 중 Workforce Analyst. HR-finance 데이터 통합 + 자연어 query + 시나리오 시뮬레이션으로 인력 의사결정 가속. 검증된 고객 사례: healthcare provider $21M 연 절감 + time-to-market 20% 단축, Fresenius Medical Care planning time 30%+ 단축, Canada Goose planning cycle 60% 단축. 2026 H1에 autonomous AI 에이전트 (자율 이상 감지·워크플로 실행) 추가 예정.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -2814,7 +2814,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1">
+    <row r="10" ht="140" customHeight="1">
       <c r="A10" s="7" t="n">
         <v>9</v>
       </c>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Cisco의 사내 AI HR Assistant: HR 정책 Q&amp;A를 넘어 agentic 수준으로 진화. 직원 PTO 잔여 조회 + 매니저에게 보낼 time-off notification 메시지 자동 작성까지. HR case 열지 않고 처리. broader Cisco "AI agents + nudges" cut-bureaucracy 이니셔티브 일부.</t>
+          <t>Cisco의 사내 AI HR Assistant: HR 정책 Q&amp;A를 넘어 agentic 수준으로 진화. 직원 PTO 잔여 조회 + 매니저에게 보낼 time-off notification 메시지 자동 작성까지. HR case 열지 않고 처리. broader Cisco "AI agents + nudges" cut-bureaucracy 이니셔티브 일부. 35,000+ Cisco 직원이 2025-06까지 AI-upskilled (+121% YoY).</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -2974,7 +2974,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="90" customHeight="1">
+    <row r="11" ht="140" customHeight="1">
       <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>IBM이 2023년 launch한 cHaRlie (Cognitive HR Learning EM Assistant): Enterprise Learning Operations &amp; Administration 팀을 위한 watsonx Orchestrate 기반 백오피스 에이전트. 학습 enrollment 모니터링·저조 alert·event 홍보·pre-event comms·virtual class 출석 자동 로깅. ⚠️ 자사 보고: learner N…</t>
+          <t>IBM이 2023년 launch한 cHaRlie (Cognitive HR Learning EM Assistant): Enterprise Learning Operations &amp; Administration 팀을 위한 watsonx Orchestrate 기반 백오피스 에이전트. 학습 enrollment 모니터링·저조 alert·event 홍보·pre-event comms·virtual class 출석 자동 로깅. ⚠️ 자사 보고: learner NPS 15% 상승, 출석 캡처 100% 정확도, 출석부 turnaround 91% 단축, onboarding time 25% 감소.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -3155,7 +3155,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="90" customHeight="1">
+    <row r="12" ht="140" customHeight="1">
       <c r="A12" s="7" t="n">
         <v>11</v>
       </c>
@@ -3322,7 +3322,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="90" customHeight="1">
+    <row r="13" ht="140" customHeight="1">
       <c r="A13" s="7" t="n">
         <v>12</v>
       </c>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Microsoft People Skills + Skills Agent: M365 Copilot/Viva 데이터 레이어. OpenAI 모델로 직원 이메일·문서·미팅에서 스킬을 자동 추론해 dynamic 스킬 프로파일 생성. LinkedIn 공동 개발 16,000-skill taxonomy 기반. Skills Agent는 매니저에게 internal talent 매칭·workforce planning insight 제공.</t>
+          <t>Microsoft People Skills + Skills Agent: M365 Copilot/Viva 데이터 레이어. OpenAI 모델로 직원 이메일·문서·미팅에서 스킬을 자동 추론해 dynamic 스킬 프로파일 생성. LinkedIn 공동 개발 16,000-skill taxonomy 기반. Skills Agent는 매니저에게 internal talent 매칭·workforce planning insight 제공. 2025 GA. 2026-03 Skills Agent → Learning + Workforce Insights agents로 분리.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -3502,7 +3502,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="90" customHeight="1">
+    <row r="14" ht="140" customHeight="1">
       <c r="A14" s="7" t="n">
         <v>13</v>
       </c>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Moderna는 OpenAI ChatGPT Enterprise 위에 "Ask HR"이라는 centralized 커스텀 GPT를 구축해, 직원의 HR 문의를 performance·career·benefits 영역의 specialized GPT들로 분기(routing)시킨다. HR 도메인 전체에서 "front door" 역할을 수행. 이는 전사 3,000+ 커스텀 GPT 생태계 중 HR 특화 허브에 해당하며, 2025년 Moderna의 HR+IT…</t>
+          <t>Moderna는 OpenAI ChatGPT Enterprise 위에 "Ask HR"이라는 centralized 커스텀 GPT를 구축해, 직원의 HR 문의를 performance·career·benefits 영역의 specialized GPT들로 분기(routing)시킨다. HR 도메인 전체에서 "front door" 역할을 수행. 이는 전사 3,000+ 커스텀 GPT 생태계 중 HR 특화 허브에 해당하며, 2025년 Moderna의 HR+IT 부서 병합(단일 리더 Tracey Franklin CPDO)과 조직 구조 변화와 함께 전개된 사례라는 점에서 특히 주목된다.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -3658,7 +3658,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="90" customHeight="1">
+    <row r="15" ht="140" customHeight="1">
       <c r="A15" s="7" t="n">
         <v>14</v>
       </c>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Amazon Connections: 1.5M 직원에게 매일 로그인 시 1개 질문 pulse. 연 300M+ 응답이 People Science 팀의 ML 모델 입력: 행동·태도 변화로 attrition·engagement 예측. ⚠️ 자사 보고: 97% voluntary adoption (산업 평균 ~25%). Andie Baker (전 principal scientist)가 구축.</t>
+          <t>Amazon Connections: 1.5M 직원에게 매일 로그인 시 1개 질문 pulse. 연 300M+ 응답이 People Science 팀의 ML 모델 입력: 행동·태도 변화로 attrition·engagement 예측. ⚠️ 자사 보고: 97% voluntary adoption (산업 평균 ~25%). Andie Baker (전 principal scientist)가 구축. 단 Fortune Jun 2024 critical coverage: anonymity skepticism 보고.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -3828,7 +3828,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="90" customHeight="1">
+    <row r="16" ht="140" customHeight="1">
       <c r="A16" s="7" t="n">
         <v>15</v>
       </c>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Businessolver는 US 복리후생 어드민 SaaS 벤더로, 자체 AI 엔진 Sofia를 2010년대 후반부터 운영해왔으며 2025년 7월 agentic framework로 확장. 3개 specialist agent (Intake / Answer / Insights) 구조로 문서 자동 검증·24/7 직원 Q&amp;A·HR 운영 인사이트를 동시 처리. ⚠️ 자사 보고: 2024년 OE(Open Enrollment) 기준 document 자동 검…</t>
+          <t>Businessolver는 US 복리후생 어드민 SaaS 벤더로, 자체 AI 엔진 Sofia를 2010년대 후반부터 운영해왔으며 2025년 7월 agentic framework로 확장. 3개 specialist agent (Intake / Answer / Insights) 구조로 문서 자동 검증·24/7 직원 Q&amp;A·HR 운영 인사이트를 동시 처리. ⚠️ 자사 보고: 2024년 OE(Open Enrollment) 기준 document 자동 검증 62%·chat 당일 해결 92%·콜타임 7M minutes 절감·만족도 4.25/5. 2025년 마감 기준 client NPS 83·retention 97% (벤더 자사 발표).</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -3992,7 +3992,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="90" customHeight="1">
+    <row r="17" ht="140" customHeight="1">
       <c r="A17" s="7" t="n">
         <v>16</v>
       </c>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Deloitte의 Zora AI: agentic AI 플랫폼 (NVIDIA AI · Llama Nemotron · AI-Q Blueprint 기반). finance·human capital·supply chain·procurement·sales/marketing·customer service ready-to-deploy agents. 동시 launch한 Human Capital AI Solution Suite (2025-06): Workfor…</t>
+          <t>Deloitte의 Zora AI: agentic AI 플랫폼 (NVIDIA AI · Llama Nemotron · AI-Q Blueprint 기반). finance·human capital·supply chain·procurement·sales/marketing·customer service ready-to-deploy agents. 동시 launch한 Human Capital AI Solution Suite (2025-06): Workforce Analyzer (AI 워크포스 영향평가) + Workforce Planner+ + 300+ HR workflows reimagined library. Deloitte 13,000+ leader 서베이 기반 HR AI maturity model 동반.</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -4162,7 +4162,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="90" customHeight="1">
+    <row r="18" ht="140" customHeight="1">
       <c r="A18" s="7" t="n">
         <v>17</v>
       </c>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>IBM이 2015년 MVP로 시작한 사내 talent marketplace. opt-in 직원 280K+에게 AI로 추론한 스킬·경력·성과·근무지·디지털 footprint(블로그·코드·포럼 게시물) 기반 personalized 내부 직무 추천. peer 이동 패턴 continuous learning: A→B 이동이 5건 누적되면 유사 프로파일에게 동일 패턴 추천. ⚠️ 자사 보고: 40% 내부 채용 충원 증가, 1,000+ 측정 가능 plac…</t>
+          <t>IBM이 2015년 MVP로 시작한 사내 talent marketplace. opt-in 직원 280K+에게 AI로 추론한 스킬·경력·성과·근무지·디지털 footprint(블로그·코드·포럼 게시물) 기반 personalized 내부 직무 추천. peer 이동 패턴 continuous learning: A→B 이동이 5건 누적되면 유사 프로파일에게 동일 패턴 추천. ⚠️ 자사 보고: 40% 내부 채용 충원 증가, 1,000+ 측정 가능 placement.</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
@@ -4340,7 +4340,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="90" customHeight="1">
+    <row r="19" ht="140" customHeight="1">
       <c r="A19" s="7" t="n">
         <v>18</v>
       </c>
@@ -4496,7 +4496,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="90" customHeight="1">
+    <row r="20" ht="140" customHeight="1">
       <c r="A20" s="7" t="n">
         <v>19</v>
       </c>
@@ -4517,7 +4517,10 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Mastercard는 2022년 Gloat을 도입해 internal talent marketplace "Unlocked"를 출시: 이전 수동 운영하던 "Project Possible"의 AI 후속.</t>
+          <t>Mastercard는 2022년 Gloat을 도입해 internal talent marketplace "Unlocked"를 출시: 이전 수동 운영하던 "Project Possible"의 AI 후속. ⚠️ 자사 보고 (Gloat case study + Mastercard 2025 AI culture story 종합):
+• 2022 시점: $21M productivity 절감 (첫 1년), 24,000+ 직원 매칭, 62% 등록률, 100,000+ unlocked capacity hours, 3,000+ role/멘토십 매칭: cross-functional 62%·cross-regional 52%
+• 2025 시점: 93% 등록률, 42% 월간 engagement, 1M project hours 누적, 24h 내 인터뷰 스케줄링
+&gt; ⚠️ PwC 컨설팅 자료 정정: PwC 자료의 "$20M 절감"은 $21M의 오기/반올림 (Gloat 공식 case study 기준). "360,000 hours"는 Schneider Electric Open Talent Market 메트릭과 혼동된 것: Mastercard는 100K → 1M project hours.</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
@@ -4662,7 +4665,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="90" customHeight="1">
+    <row r="21" ht="140" customHeight="1">
       <c r="A21" s="7" t="n">
         <v>20</v>
       </c>
@@ -4810,7 +4813,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="90" customHeight="1">
+    <row r="22" ht="140" customHeight="1">
       <c r="A22" s="7" t="n">
         <v>21</v>
       </c>
@@ -4831,7 +4834,7 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Chipotle Mexican Grill(3,500+ 레스토랑, 110,000+ 직원)이 2024년 10월 22일 공식 발표한 AI 채용 플랫폼. Paradox의 대화형 AI 어시스턴트 Olivia 기반이며, Chipotle는 이를 "Ava Cado"라는 자사 브랜딩으로 배포. North America + Europe 전 매장 대상으로 영·스·불·독 4개 언어 지원. CHRO Ilene Eskenazi가 press release에서 직접 qu…</t>
+          <t>Chipotle Mexican Grill(3,500+ 레스토랑, 110,000+ 직원)이 2024년 10월 22일 공식 발표한 AI 채용 플랫폼. Paradox의 대화형 AI 어시스턴트 Olivia 기반이며, Chipotle는 이를 "Ava Cado"라는 자사 브랜딩으로 배포. North America + Europe 전 매장 대상으로 영·스·불·독 4개 언어 지원. CHRO Ilene Eskenazi가 press release에서 직접 quote 제공. ⚠️ 벤더+회사 공동 주장: time-to-hire 75% 감소.</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
@@ -4976,7 +4979,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="90" customHeight="1">
+    <row r="23" ht="140" customHeight="1">
       <c r="A23" s="7" t="n">
         <v>22</v>
       </c>
@@ -4997,7 +5000,7 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Commonwealth Bank of Australia(CBA)는 OpenAI ChatGPT Enterprise를 50,000명 직원에게 배포하고, Microsoft 365 Copilot을 17,500명에게 제공하며 AI 역량 구축을 전사적으로 추진하고 있다. ✅ Fact 2026년 2월에는 $90M(호주 달러) 3개년 "Future Workforce Program"을 발표하여 직원 스킬 개발과 커리어 전환 지원을 목표로 한다. 다만 AI 챗…</t>
+          <t>Commonwealth Bank of Australia(CBA)는 OpenAI ChatGPT Enterprise를 50,000명 직원에게 배포하고, Microsoft 365 Copilot을 17,500명에게 제공하며 AI 역량 구축을 전사적으로 추진하고 있다. ✅ Fact 2026년 2월에는 $90M(호주 달러) 3개년 "Future Workforce Program"을 발표하여 직원 스킬 개발과 커리어 전환 지원을 목표로 한다. 다만 AI 챗봇으로 45명 고객 서비스 직원을 대체하려다 노조 압박으로 결정을 번복한 사례도 주목된다. sources/openai-cba-case-study.md sources/cba-future-workforce-90m-2026.md</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -5125,7 +5128,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="90" customHeight="1">
+    <row r="24" ht="140" customHeight="1">
       <c r="A24" s="7" t="n">
         <v>23</v>
       </c>
@@ -5146,7 +5149,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Deloitte 2026 Global Human Capital Trends는 89개국·9,000명 임원 서베이 기반 capstone 리포트. 핵심 발견: 임원 60%가 AI를 의사결정에 사용하지만, 5%만 잘 관리한다. AI 도입 자체보다 work redesign과 거버넌스 격차가 ROI를 결정. "intentional work redesign" 조직은 AI ROI 기대치 초과 확률 2배.</t>
+          <t>Deloitte 2026 Global Human Capital Trends는 89개국·9,000명 임원 서베이 기반 capstone 리포트. 핵심 발견: 임원 60%가 AI를 의사결정에 사용하지만, 5%만 잘 관리한다. AI 도입 자체보다 work redesign과 거버넌스 격차가 ROI를 결정. "intentional work redesign" 조직은 AI ROI 기대치 초과 확률 2배. HR 기능이 "agent governance" 역할로 재정의되는 글로벌 trend 데이터: 모든 KR HR 임원 발표·제안서 첫 슬라이드 인용 가능.</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
@@ -5258,7 +5261,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="90" customHeight="1">
+    <row r="25" ht="140" customHeight="1">
       <c r="A25" s="7" t="n">
         <v>24</v>
       </c>
@@ -5279,7 +5282,7 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>IBM의 HiRo는 watsonx Orchestrate 기반 분기 승진 관리 specialist agent (digital worker). AskHR 생태계 (2.1M conversations/년·80+ HR tasks 자동화) 내 promotion 영역 자동화. ⚠️ 자사 보고: 분기 승진 cycle을 10주 → 자동화로 단축, HR Business Partner (HRBP) 시간 분기당 85% 절감. 매니저 10,000명에 promotio…</t>
+          <t>IBM의 HiRo는 watsonx Orchestrate 기반 분기 승진 관리 specialist agent (digital worker). AskHR 생태계 (2.1M conversations/년·80+ HR tasks 자동화) 내 promotion 영역 자동화. ⚠️ 자사 보고: 분기 승진 cycle을 10주 → 자동화로 단축, HR Business Partner (HRBP) 시간 분기당 85% 절감. 매니저 10,000명에 promotion criteria + eligible employees 리스트 자동 배포. IBM CHRO Nickle LaMoreaux가 HR Executive of the Year 2024 인터뷰·myHRfuture 팟캐스트·IBM 공식 case study에서 일관 언급.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -5428,7 +5431,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="90" customHeight="1">
+    <row r="26" ht="140" customHeight="1">
       <c r="A26" s="7" t="n">
         <v>25</v>
       </c>
@@ -5449,7 +5452,7 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>JPMorgan Chase는 2024년 여름 자체 개발 생성형 AI 플랫폼 LLM Suite를 출시하여, 2024년 9월 기준 140,000명 직원에게 배포하고 이후 200,000명 이상으로 확대했다. ✅ Fact 이 플랫폼은 문서 요약, 이메일 초안, 아이디어 생성 등 지식 노동자의 일상 업무 전반을 지원하며, HR 영역에서는 성과 리뷰 초안 작성 기능이 특히 주목된다. 월가 최대 규모 LLM 배포 사례 중 하나다.</t>
+          <t>JPMorgan Chase는 2024년 여름 자체 개발 생성형 AI 플랫폼 LLM Suite를 출시하여, 2024년 9월 기준 140,000명 직원에게 배포하고 이후 200,000명 이상으로 확대했다. ✅ Fact 이 플랫폼은 문서 요약, 이메일 초안, 아이디어 생성 등 지식 노동자의 일상 업무 전반을 지원하며, HR 영역에서는 성과 리뷰 초안 작성 기능이 특히 주목된다. 월가 최대 규모 LLM 배포 사례 중 하나다. sources/cnbc-jpmorgan-llm-suite-2024-08.md</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
@@ -5462,7 +5465,11 @@
           <t>[Before]
 직원이 개별적으로 외부 AI 도구 또는 전통적 검색·작성 도구를 사용. 성과 리뷰는 관리자가 수동으로 직접 작성. /
 [After]
-1. md]]</t>
+1. 직원 요청\n문서 요약·이메일·리뷰 초안 등
+2. LLM Suite\n내부 보안 포털
+3. AI 응답 생성
+4. 직원 검토·편집
+5. 최종 산출물 사용</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
@@ -5577,7 +5584,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="90" customHeight="1">
+    <row r="27" ht="140" customHeight="1">
       <c r="A27" s="7" t="n">
         <v>26</v>
       </c>
@@ -5598,7 +5605,10 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Legion Technologies (2016년 설립, Bay Area)는 AI-native WFM (workforce management) 벤더: 시급직 (retail·hospitality·restaurant·healthcare) 스케줄링·수요예측·노동 컴플라이언스 자동화. Forrester TEI 1,345% ROI / $13.35M NPV (2021-09 study, 9,000명·500개 매장 사례). 2022~2025 AI Breakt…</t>
+          <t>Legion Technologies (2016년 설립, Bay Area)는 AI-native WFM (workforce management) 벤더: 시급직 (retail·hospitality·restaurant·healthcare) 스케줄링·수요예측·노동 컴플라이언스 자동화. Forrester TEI 1,345% ROI / $13.35M NPV (2021-09 study, 9,000명·500개 매장 사례). 2022~2025 AI Breakthrough Awards "AI-based WFM Solution of the Year" 4년 연속. 2026년 1월 Agentic AI 90+ features 출시 발표 (벤더). 고객사: Dollar General·Cinemark·Five Below 등.
+&gt; ⚠️ Funding 정정 필수: 일부 자료(PwC 컨설팅 문서 포함)에서 "$195M Series C in 2024"로 기술되나, 실제로는 누적 funding 합계. 2024년 라운드는 (a) $50M growth round (Riverwood Capital, 2024-05) + (b) $50M debt financing (SVB, 2024-12). Series C는 2021년 5월 $50M이 별건. 컨설팅 deck 인용 시 정정.
+&gt;
+&gt; ⚠️ Mercy Health $30M misattribution: "Mercy Health 연 $30M travel nurse 절감" 사례는 Works/Trusted Health의 결과이지 Legion 아님. PwC 자료에 잘못 인용: wiki 등재 거부.</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -5747,7 +5757,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="90" customHeight="1">
+    <row r="28" ht="140" customHeight="1">
       <c r="A28" s="7" t="n">
         <v>27</v>
       </c>
@@ -5768,7 +5778,7 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>LG AI연구원이 자체 LLM EXAONE 기반 'ChatEXAONE' 정식 서비스 출시 (2026 Q1, 1년 베타 후). LG전자·LG이노텍·LG디스플레이 등 LG 그룹 5만+ 임직원 대상. 사무직 베타 활용률 65% 검증. 사내 규정·프로젝트 자료 검색·요약, PPTX·PDF·CSV·도표·수식 이해, SQL 생성, 22개 언어 코드 지원.</t>
+          <t>LG AI연구원이 자체 LLM EXAONE 기반 'ChatEXAONE' 정식 서비스 출시 (2026 Q1, 1년 베타 후). LG전자·LG이노텍·LG디스플레이 등 LG 그룹 5만+ 임직원 대상. 사무직 베타 활용률 65% 검증. 사내 규정·프로젝트 자료 검색·요약, PPTX·PDF·CSV·도표·수식 이해, SQL 생성, 22개 언어 코드 지원. 한국 자체 LLM 기반 그룹 전사 AI 챗봇 운영의 가장 큰 사례.</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
@@ -5920,7 +5930,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="90" customHeight="1">
+    <row r="29" ht="140" customHeight="1">
       <c r="A29" s="7" t="n">
         <v>28</v>
       </c>
@@ -5941,7 +5951,7 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>LinkedIn Learning이 Premium·Enterprise tier에 통합한 AI-Powered Coaching 기능. 2024 글로벌 출시 후 2025에 role-play scenario coaching으로 확장: 학습자가 AI coach와 가상 대화 (피드백 주고받기·어려운 대화 연습·인터뷰 모의 등)로 soft skill 학습. LinkedIn 16K+ skills taxonomy 위에서 작동.</t>
+          <t>LinkedIn Learning이 Premium·Enterprise tier에 통합한 AI-Powered Coaching 기능. 2024 글로벌 출시 후 2025에 role-play scenario coaching으로 확장: 학습자가 AI coach와 가상 대화 (피드백 주고받기·어려운 대화 연습·인터뷰 모의 등)로 soft skill 학습. LinkedIn 16K+ skills taxonomy 위에서 작동. ⚠️ 정량 metric은 LinkedIn 공식 KPI로 미공개: 시장에 자주 인용되는 "90% 만족·160% 학습시간 증가" 수치는 별도의 [MS-LinkedIn 2024 Work Trend Index](https://blogs.microsoft.com/blog/2024/05/08/microsoft-and-linkedin-release-the-2024-work-trend-index-on-the-state-of-ai-at-work/) 일반 통계: AI Coaching 자체 metric 아니므로 인용 시 주의.</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -6076,7 +6086,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="90" customHeight="1">
+    <row r="30" ht="140" customHeight="1">
       <c r="A30" s="7" t="n">
         <v>29</v>
       </c>
@@ -6097,7 +6107,7 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Lloyds Banking Group(67,000명)은 2018년 Workday HCM 도입, 2020년 Workday Skills Cloud를 추가 배포한 후, 2024년부터 HR 정책 Q&amp;A에 특화된 생성형 AI 파일럿을 운영 중이다. ✅ Fact 2025년 GenAI가 약 £50M 가치를 창출했으며, 2026년 £100M 이상을 목표로 GenAI·Agentic AI 확대를 추진 중이다. 2026년 1월에는 67,000명 전 직원 대상 A…</t>
+          <t>Lloyds Banking Group(67,000명)은 2018년 Workday HCM 도입, 2020년 Workday Skills Cloud를 추가 배포한 후, 2024년부터 HR 정책 Q&amp;A에 특화된 생성형 AI 파일럿을 운영 중이다. ✅ Fact 2025년 GenAI가 약 £50M 가치를 창출했으며, 2026년 £100M 이상을 목표로 GenAI·Agentic AI 확대를 추진 중이다. 2026년 1월에는 67,000명 전 직원 대상 AI Academy를 론칭했다. sources/ffnews-lloyds-100m-ai-2026.md sources/itpro-lloyds-ai-academy-2026.md</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -6222,7 +6232,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="90" customHeight="1">
+    <row r="31" ht="140" customHeight="1">
       <c r="A31" s="7" t="n">
         <v>30</v>
       </c>
@@ -6243,7 +6253,7 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Mercy(미국 5대 가톨릭 의료 시스템, 40개 병원)는 AI 기반 유연 인력 모델을 도입하여 계약직 간호사(Agency) 비중을 25%에서 8%로 줄이고, 2023년 $30M 비용 절감을 달성했다. ✅ Fact 핵심 전략은 AI 주도 스케줄링과 내부 유연 인력풀(Float Pool) 확대를 결합한 "혼합 인력 모델(Blended Workforce)"이다.</t>
+          <t>Mercy(미국 5대 가톨릭 의료 시스템, 40개 병원)는 AI 기반 유연 인력 모델을 도입하여 계약직 간호사(Agency) 비중을 25%에서 8%로 줄이고, 2023년 $30M 비용 절감을 달성했다. ✅ Fact 핵심 전략은 AI 주도 스케줄링과 내부 유연 인력풀(Float Pool) 확대를 결합한 "혼합 인력 모델(Blended Workforce)"이다. sources/healthcareitnews-mercy-30m-2023.md sources/beckershospitalreview-mercy-2024.md</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
@@ -6384,7 +6394,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="90" customHeight="1">
+    <row r="32" ht="140" customHeight="1">
       <c r="A32" s="7" t="n">
         <v>31</v>
       </c>
@@ -6405,7 +6415,7 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Microsoft Viva Glint에 Copilot 임베드: engagement 서베이 open-end 코멘트 대량 합성 + 반복 테마 탐지 + 속성별 sentiment slice + benchmark 비교. 2026-03 transition으로 default ON, 2026-04부터 Team/Executive 요약 리포트에 "Copilot Highlights" 자동 섹션 추가 (강점·기회·점수 변화·benchmark). Microsoft …</t>
+          <t>Microsoft Viva Glint에 Copilot 임베드: engagement 서베이 open-end 코멘트 대량 합성 + 반복 테마 탐지 + 속성별 sentiment slice + benchmark 비교. 2026-03 transition으로 default ON, 2026-04부터 Team/Executive 요약 리포트에 "Copilot Highlights" 자동 섹션 추가 (강점·기회·점수 변화·benchmark). Microsoft 자체 사용: 전사 "Employee Signals" twice-yearly.</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
@@ -6553,7 +6563,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="90" customHeight="1">
+    <row r="33" ht="140" customHeight="1">
       <c r="A33" s="7" t="n">
         <v>32</v>
       </c>
@@ -6574,7 +6584,7 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Siemens GBS(Global Business Services)는 360,000명 이상의 직원을 지원하는 HR·재무·구매 서비스를 통합 관리하기 위해 ServiceNow AI 플랫폼 기반의 "My Services" 포털을 구축했다. ✅ Fact 이 포털은 월 110,000건의 방문을 처리하며, 기존 100개 이상의 이메일 사서함을 단일 진입점으로 통합했다. 사용자 만족도 8.8/10, 직원의 87%가 업무를 즐기고 있다고 응답했다.</t>
+          <t>Siemens GBS(Global Business Services)는 360,000명 이상의 직원을 지원하는 HR·재무·구매 서비스를 통합 관리하기 위해 ServiceNow AI 플랫폼 기반의 "My Services" 포털을 구축했다. ✅ Fact 이 포털은 월 110,000건의 방문을 처리하며, 기존 100개 이상의 이메일 사서함을 단일 진입점으로 통합했다. 사용자 만족도 8.8/10, 직원의 87%가 업무를 즐기고 있다고 응답했다. sources/servicenow-siemens-case-study.md</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -6715,7 +6725,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="90" customHeight="1">
+    <row r="34" ht="140" customHeight="1">
       <c r="A34" s="7" t="n">
         <v>33</v>
       </c>
@@ -6736,7 +6746,7 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Walmart은 2025년 6월 1.5M 직원 대상의 AI 도구 모음을 공개하고, 2025년 9월 OpenAI와 AI 인증 교육 프로그램 파트너십을 발표했다. ✅ Fact "People-led, Tech-powered" 원칙 하에 AI를 인력 대체가 아닌 역할 전환(드론 기술자·로봇 감독관 등)의 도구로 활용하고 있다. Workday HCM을 전사 단일 HR 시스템으로 운영하며, Paradox의 대화형 ATS로 고볼륨 프론트라인 채용을 자동화…</t>
+          <t>Walmart은 2025년 6월 1.5M 직원 대상의 AI 도구 모음을 공개하고, 2025년 9월 OpenAI와 AI 인증 교육 프로그램 파트너십을 발표했다. ✅ Fact "People-led, Tech-powered" 원칙 하에 AI를 인력 대체가 아닌 역할 전환(드론 기술자·로봇 감독관 등)의 도구로 활용하고 있다. Workday HCM을 전사 단일 HR 시스템으로 운영하며, Paradox의 대화형 ATS로 고볼륨 프론트라인 채용을 자동화했다. sources/walmart-corporate-ai-tools-2025-06.md sources/hrdive-walmart-openai-2025-09.md</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
@@ -6877,7 +6887,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="90" customHeight="1">
+    <row r="35" ht="140" customHeight="1">
       <c r="A35" s="7" t="n">
         <v>34</v>
       </c>
@@ -6898,7 +6908,11 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Walmart(2.3M 직원, 10,500 매장)은 세 가지 HR AI 이니셔티브를 병행 운영: 1. Ask Sam: 매장 직원용 대화형 음성 AI 어시스턴트. 900,000명 직원이 사용하며 주 3,000,000+ 질문 처리. HR 정책·재고·가격·작업 절차 등 답변.</t>
+          <t>Walmart(2.3M 직원, 10,500 매장)은 세 가지 HR AI 이니셔티브를 병행 운영:
+1. Ask Sam: 매장 직원용 대화형 음성 AI 어시스턴트. 900,000명 직원이 사용하며 주 3,000,000+ 질문 처리. HR 정책·재고·가격·작업 절차 등 답변.
+2. AI Interview Coach: 2025-06 파일럿 공개. 직원의 승진 면접 준비를 AI가 코칭.
+3. 50,000명 리스킬링: 캐셔·매장 직원 → 드론 기술자·로봇 수퍼바이저로 역할 전환 계획.
+전략적 프레이밍: "People-led, tech-powered": AI를 "사람을 대체"가 아니라 "사람을 강화"로 포지셔닝.</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr"/>
@@ -7036,7 +7050,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="90" customHeight="1">
+    <row r="36" ht="140" customHeight="1">
       <c r="A36" s="7" t="n">
         <v>35</v>
       </c>
@@ -7057,7 +7071,7 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Bosch는 창업자 Robert Bosch의 이름을 딴 HR AI 디지털 어시스턴트 "ROB"를 25개국에 배포했다. ✅ Fact Cognigy.AI 플랫폼과 GPT 기반으로 구동되며, Microsoft Teams를 통해 직원에게 제공된다. 은행 계좌 정보 업데이트, 커리어 개발 정보 탐색, 회사 정책 안내, HR 셀프서비스 프로세스 안내 등을 처리하며, 감성 지능(emotional intelligence)을 활용해 추가 인간 지원이 필요한 …</t>
+          <t>Bosch는 창업자 Robert Bosch의 이름을 딴 HR AI 디지털 어시스턴트 "ROB"를 25개국에 배포했다. ✅ Fact Cognigy.AI 플랫폼과 GPT 기반으로 구동되며, Microsoft Teams를 통해 직원에게 제공된다. 은행 계좌 정보 업데이트, 커리어 개발 정보 탐색, 회사 정책 안내, HR 셀프서비스 프로세스 안내 등을 처리하며, 감성 지능(emotional intelligence)을 활용해 추가 인간 지원이 필요한 시점을 식별한다. sources/cognigy-bosch-case-study.md sources/hrgrapevine-bosch-rob-2025-01.md</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
@@ -7199,7 +7213,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="90" customHeight="1">
+    <row r="37" ht="140" customHeight="1">
       <c r="A37" s="7" t="n">
         <v>36</v>
       </c>
@@ -7220,7 +7234,7 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>싱가포르 최대 은행 DBS Bank는 인사 전 영역에 AI를 내재화한 아시아 금융권 선도 사례다. ✅ Fact 핵심 세 가지: (1) AI 채용 플랫폼 JIM(Jobs Intelligence Maestro): 이력서 스크리닝·면접 일정·초기 평가 자동화로 채용 소요시간을 32일→8일 단축, (2) 이탈 예측 모델: 학습·보상·휴가 패턴 등 다변수 분석으로 이탈 징후 조기 감지, (3) iGrow 커리어 어드바이저: 10,000개 이상 내부 과…</t>
+          <t>싱가포르 최대 은행 DBS Bank는 인사 전 영역에 AI를 내재화한 아시아 금융권 선도 사례다. ✅ Fact 핵심 세 가지: (1) AI 채용 플랫폼 JIM(Jobs Intelligence Maestro): 이력서 스크리닝·면접 일정·초기 평가 자동화로 채용 소요시간을 32일→8일 단축, (2) 이탈 예측 모델: 학습·보상·휴가 패턴 등 다변수 분석으로 이탈 징후 조기 감지, (3) iGrow 커리어 어드바이저: 10,000개 이상 내부 과정 기반 개인화 커리어 경로 추천. sources/emerj-dbs-ai-cases.md sources/adriantan-dbs-ai-recruiting.md</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
@@ -7360,7 +7374,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="90" customHeight="1">
+    <row r="38" ht="140" customHeight="1">
       <c r="A38" s="7" t="n">
         <v>37</v>
       </c>
@@ -7381,7 +7395,7 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Goldman Sachs는 2025년 1월 GS AI Assistant를 10,000명 파일럿으로 시작, 2025년 6월 전 지식노동자 대상 전사 배포를 완료했다. ✅ Fact 이 도구는 다수의 LLM(OpenAI GPT-4o/o3-mini, Google Gemini 2.0, Anthropic Claude 3.7 포함)을 단일 인터페이스로 접근하는 멀티모델 어시스턴트로, 문서 요약·리서치 노트 초안·규제 문서 분석·코드 생성·다국어 번역 등을…</t>
+          <t>Goldman Sachs는 2025년 1월 GS AI Assistant를 10,000명 파일럿으로 시작, 2025년 6월 전 지식노동자 대상 전사 배포를 완료했다. ✅ Fact 이 도구는 다수의 LLM(OpenAI GPT-4o/o3-mini, Google Gemini 2.0, Anthropic Claude 3.7 포함)을 단일 인터페이스로 접근하는 멀티모델 어시스턴트로, 문서 요약·리서치 노트 초안·규제 문서 분석·코드 생성·다국어 번역 등을 지원한다. sources/fortune-goldman-gs-ai-2025-06.md</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
@@ -7394,7 +7408,11 @@
           <t>[Before]
 지식노동자가 직접 문서 작성, 수동 검색, 개별 도구 사용. /
 [After]
-1. md]]</t>
+1. 직원 입력\n텍스트·문서
+2. GS AI Assistant\n사내 방화벽 내
+3. AI 응답 생성
+4. 직원 검토
+5. 사용</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
@@ -7507,7 +7525,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="90" customHeight="1">
+    <row r="39" ht="140" customHeight="1">
       <c r="A39" s="7" t="n">
         <v>38</v>
       </c>
@@ -7528,7 +7546,7 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>IBM이 2019년 공개한 Predictive Attrition Program: Watson 기반 patented ML 모델이 34+ 변수(overtime·salary·역할·성과·통근거리)를 분석해 6개월 flight risk를 예측. ⚠️ 자사 보고: 95% 정확도, $300M 누적 retention saving (2023까지). 동일 인프라가 AI Compensation Recommendation으로 확장: 매니저별 per-employee…</t>
+          <t>IBM이 2019년 공개한 Predictive Attrition Program: Watson 기반 patented ML 모델이 34+ 변수(overtime·salary·역할·성과·통근거리)를 분석해 6개월 flight risk를 예측. ⚠️ 자사 보고: 95% 정확도, $300M 누적 retention saving (2023까지). 동일 인프라가 AI Compensation Recommendation으로 확장: 매니저별 per-employee salary 추천 + 이유 설명. 매니저가 권고 무시 시 팀 attrition 2배.</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
@@ -7660,7 +7678,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="90" customHeight="1">
+    <row r="40" ht="140" customHeight="1">
       <c r="A40" s="7" t="n">
         <v>39</v>
       </c>
@@ -7681,7 +7699,7 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>마이다스아이티의 AI 역량검사 솔루션 inAIR은 성향파악·전략게임·영상면접 3개 과제로 구성된 시뮬레이션 기반 채용 평가 도구. 2025년 하반기 기준 기아·KB증권·신한은행·CJ그룹·LIG넥스원·GS리테일·비씨카드·티웨이항공·KT클라우드·유니클로 등 대기업과 오산시청·구미시청·경북도청·제주도청 등 공공기관이 도입. 2025-07 KAIST 연구진이 Nature 자매지 *Scientific Reports*에 발표한 논문에서 "기존 채용 방식…</t>
+          <t>마이다스아이티의 AI 역량검사 솔루션 inAIR은 성향파악·전략게임·영상면접 3개 과제로 구성된 시뮬레이션 기반 채용 평가 도구. 2025년 하반기 기준 기아·KB증권·신한은행·CJ그룹·LIG넥스원·GS리테일·비씨카드·티웨이항공·KT클라우드·유니클로 등 대기업과 오산시청·구미시청·경북도청·제주도청 등 공공기관이 도입. 2025-07 KAIST 연구진이 Nature 자매지 Scientific Reports에 발표한 논문에서 "기존 채용 방식 중 유일하게 채용 1년 후 실제 업무 성과를 통계적으로 유의미하게 예측"함을 확인: 국내 HR AI 중 최고 수준의 독립 검증.</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
@@ -7837,7 +7855,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="90" customHeight="1">
+    <row r="41" ht="140" customHeight="1">
       <c r="A41" s="7" t="n">
         <v>40</v>
       </c>
@@ -7858,7 +7876,8 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>Nayya는 2019년 설립 미국 startup, AI 기반 복리후생 의사결정 지원 platform. 직원이 OE(Open Enrollment) 시점에 의료·치과·생명·voluntary plan을 선택할 때 개인 청구이력·소득·가족 구성을 분석해 plan별 예상 본인부담을 시뮬레이션, 최적 plan 추천. 2023년 10월 MetLife 전략적 파트너십: MetLife가 1,000+ employer에 Nayya solution을 exclusi…</t>
+          <t>Nayya는 2019년 설립 미국 startup, AI 기반 복리후생 의사결정 지원 platform. 직원이 OE(Open Enrollment) 시점에 의료·치과·생명·voluntary plan을 선택할 때 개인 청구이력·소득·가족 구성을 분석해 plan별 예상 본인부담을 시뮬레이션, 최적 plan 추천. 2023년 10월 MetLife 전략적 파트너십: MetLife가 1,000+ employer에 Nayya solution을 exclusive 채널로 제공. 2024년 ADP·Workday Ventures 추가 strategic 라운드. ⚠️ 자사 보고: 평균 직원 $1,200 연간 절감.
+&gt; ⚠️ Funding 정정 필수: 일부 자료(PwC 컨설팅 문서 포함)에서 "$55M Series B (2022)"로 기술되나, 실제로는 $55M Series C (2022-03) + $37M Series B (2021-06). 컨설팅 deck에 인용 시 정정.</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
@@ -8000,7 +8019,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="90" customHeight="1">
+    <row r="42" ht="140" customHeight="1">
       <c r="A42" s="7" t="n">
         <v>41</v>
       </c>
@@ -8021,7 +8040,7 @@
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>풀무원이 2024-12-23 출시한 임직원 인적자원관리 전용 생성형 AI 챗봇 '두리번'. 근태·복리후생·학습·평가·승진·보상 6개 HR 영역에 대해 24/365 응답. 인사 정보 문서 기반 RAG로 hallucination 최소화. PC → 모바일 확장 계획.</t>
+          <t>풀무원이 2024-12-23 출시한 임직원 인적자원관리 전용 생성형 AI 챗봇 '두리번'. 근태·복리후생·학습·평가·승진·보상 6개 HR 영역에 대해 24/365 응답. 인사 정보 문서 기반 RAG로 hallucination 최소화. PC → 모바일 확장 계획. ★ KR 사례 중 순수 HR 챗봇으로 정의된 가장 selectoral 사례: 식품 중견기업이지만 KR HR 컨설팅의 가장 직접적 reference.</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
@@ -8164,7 +8183,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="90" customHeight="1">
+    <row r="43" ht="140" customHeight="1">
       <c r="A43" s="7" t="n">
         <v>42</v>
       </c>
@@ -8185,7 +8204,7 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>SAP가 2026-04에 발표한 SuccessFactors 1H 2026 Release에서 4개 신규 Joule Agent가 May 2026 GA 예정. 기존 Performance &amp; Goals Agent에 더해 Career &amp; Talent Development Agent(승계·커리어), HR Service Agent(self-service), People Intelligence Agent(매니저 분석), Payroll Agent(급여 Q&amp;A…</t>
+          <t>SAP가 2026-04에 발표한 SuccessFactors 1H 2026 Release에서 4개 신규 Joule Agent가 May 2026 GA 예정. 기존 Performance &amp; Goals Agent에 더해 Career &amp; Talent Development Agent(승계·커리어), HR Service Agent(self-service), People Intelligence Agent(매니저 분석), Payroll Agent(급여 Q&amp;A)가 추가됨. SAP 자사 표현으로 "the most comprehensive AI agent suite for HR". a2a/MCP 프로토콜 지원으로 3rd-party agent 호출 가능.</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
@@ -8340,7 +8359,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="90" customHeight="1">
+    <row r="44" ht="140" customHeight="1">
       <c r="A44" s="7" t="n">
         <v>43</v>
       </c>
@@ -8361,7 +8380,7 @@
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Schneider Electric(글로벌 에너지 관리·자동화 기업, 135,000+ 직원)은 Gloat 기반 "Open Talent Market"을 2020-04에 전사 big bang launch. 직원의 스킬·관심을 AI가 분석해 gig work·career transitions·mentorship 기회를 매칭. ⚠️ 벤더 주장: 360,000+ 시간 unlocked, $15M+ 생산성 향상 + 채용 비용 절감. Unilever FLEX와…</t>
+          <t>Schneider Electric(글로벌 에너지 관리·자동화 기업, 135,000+ 직원)은 Gloat 기반 "Open Talent Market"을 2020-04에 전사 big bang launch. 직원의 스킬·관심을 AI가 분석해 gig work·career transitions·mentorship 기회를 매칭. ⚠️ 벤더 주장: 360,000+ 시간 unlocked, $15M+ 생산성 향상 + 채용 비용 절감. Unilever FLEX와 함께 Gloat의 양대 레퍼런스. Josh Bersin(Tier 1)이 2019년 독립 분석에서 "가장 영리한 비즈니스 리더" CHRO Olivier Blum의 전략으로 소개 (bersin-schneider-unilever-talent-marketplace-2019-07). SHRM(Tier 2)이 2025년 현 CHRO Charise Le의 비전통적 인재 전략으로 재조명 (shrm-schneider-electric-chro-nontraditional-2025).</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
@@ -8505,7 +8524,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="90" customHeight="1">
+    <row r="45" ht="140" customHeight="1">
       <c r="A45" s="7" t="n">
         <v>44</v>
       </c>
@@ -8661,7 +8680,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="90" customHeight="1">
+    <row r="46" ht="140" customHeight="1">
       <c r="A46" s="7" t="n">
         <v>45</v>
       </c>
@@ -8834,7 +8853,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="90" customHeight="1">
+    <row r="47" ht="140" customHeight="1">
       <c r="A47" s="7" t="n">
         <v>46</v>
       </c>
@@ -8855,7 +8874,7 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>SK 그룹이 SKT-SK AX 합작 'A.Biz'를 그룹 단일 표준으로 25개 멤버사·약 8만 명에 배포 (2025 하반기 rollout). SK디스커버리 등 7개사 시작 → 2025년 말까지 SK하이닉스·SK이노베이션 포함 25개 멤버사 확산. HR 정책·절차 문의 응대용 AI 에이전트를 IT 전문 지식 없이 HR 담당자가 agent builder로 자체 구축 가능. 국가핵심기술 보유사 (SK하이닉스·SK온·SK실트론)에는 자체 LLM 'A…</t>
+          <t>SK 그룹이 SKT-SK AX 합작 'A.Biz'를 그룹 단일 표준으로 25개 멤버사·약 8만 명에 배포 (2025 하반기 rollout). SK디스커버리 등 7개사 시작 → 2025년 말까지 SK하이닉스·SK이노베이션 포함 25개 멤버사 확산. HR 정책·절차 문의 응대용 AI 에이전트를 IT 전문 지식 없이 HR 담당자가 agent builder로 자체 구축 가능. 국가핵심기술 보유사 (SK하이닉스·SK온·SK실트론)에는 자체 LLM 'A.X' + SK AX 산업특화 AI 적용으로 보안 보장.</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
@@ -8986,7 +9005,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="90" customHeight="1">
+    <row r="48" ht="140" customHeight="1">
       <c r="A48" s="7" t="n">
         <v>47</v>
       </c>
@@ -9007,7 +9026,7 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>우리은행이 금융권 최초 전사 AI 에이전트 도입 발표 (2026-03-05). 575개 후보 → 5대 영역(고객관계관리·자산관리·내부통제·고객상담·업무자동화) 29개 업무 175개 에이전트 선정. 2026-04-07 삼성SDS 우선협상대상자 선정. 12월 1차 97개, 2026 초 78개 추가 출시.</t>
+          <t>우리은행이 금융권 최초 전사 AI 에이전트 도입 발표 (2026-03-05). 575개 후보 → 5대 영역(고객관계관리·자산관리·내부통제·고객상담·업무자동화) 29개 업무 175개 에이전트 선정. 2026-04-07 삼성SDS 우선협상대상자 선정. 12월 1차 97개, 2026 초 78개 추가 출시. ⚠️ 자사 보고: 업무처리 속도 30% 향상 기대. AI 에이전트 portfolio management 컨설팅의 표준 reference architecture.</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
@@ -9020,7 +9039,7 @@
       <c r="G48" s="7" t="inlineStr">
         <is>
           <t>[Before]
-우리은행 ~13K 직원이 다수 산발 시스템 (코어뱅킹·CRM·콜센터·내부통제) 사용. AI 도입은 부서별 산발 PoC / Pain point: KB국민은행 kb-bank-ai-hr-deep-change (인사이동 AI), 신한 AI ONE shinhan-bank-ai-one-platform 등 경쟁 은행 AI 가속 → 우리은행 차별화 시급 / Trigge…
+우리은행 ~13K 직원이 다수 산발 시스템 (코어뱅킹·CRM·콜센터·내부통제) 사용. AI 도입은 부서별 산발 PoC / Pain point: KB국민은행 (인사이동 AI), 신한 AI ONE 등 경쟁 은행 AI 가속 → 우리은행 차별화 시급 / Trigger: 2026 신년 신경 그룹장 발표: 금융권 최초 전사 AI 에이전트 도입 결단
 [After]
 1. 575개 후보 사업부 nominate
 2. 5대 영역 29개 업무 175개 에이전트
@@ -9173,7 +9192,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="90" customHeight="1">
+    <row r="49" ht="140" customHeight="1">
       <c r="A49" s="7" t="n">
         <v>48</v>
       </c>
@@ -9194,7 +9213,7 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Workday가 2026-02-18에 GA 발표한 Agent System of Record (ASOR)는 AI 에이전트를 사람 직원과 동일한 방식으로 관리하는 거버넌스 레이어다. 1st-party Workday 에이전트(Illuminate 시리즈)와 3rd-party 에이전트(Salesforce·OpenAI·Microsoft 등)를 한 콘솔에서 권한·조직도·스킬·분석·보안으로 통합 관리. HR이 에이전트의 "owner of record"가 되…</t>
+          <t>Workday가 2026-02-18에 GA 발표한 Agent System of Record (ASOR)는 AI 에이전트를 사람 직원과 동일한 방식으로 관리하는 거버넌스 레이어다. 1st-party Workday 에이전트(Illuminate 시리즈)와 3rd-party 에이전트(Salesforce·OpenAI·Microsoft 등)를 한 콘솔에서 권한·조직도·스킬·분석·보안으로 통합 관리. HR이 에이전트의 "owner of record"가 되어 회사 인적자본의 일부로 책임을 가져간다는 패러다임.</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
@@ -9319,7 +9338,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="90" customHeight="1">
+    <row r="50" ht="140" customHeight="1">
       <c r="A50" s="7" t="n">
         <v>49</v>
       </c>
@@ -9495,7 +9514,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="90" customHeight="1">
+    <row r="51" ht="140" customHeight="1">
       <c r="A51" s="7" t="n">
         <v>50</v>
       </c>
@@ -9516,7 +9535,7 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>BetterUp은 AI 기반 리더십·매니저 코칭 플랫폼. 2025년 BetterUp Grow (AI-only 코칭 제품) 출시로 전통 human coaching 대비 비용 70% 절감 + 95% 사용자 만족을 주장. 가장 강력한 레퍼런스는 Twilio (8,000+ 직원): 코칭 받은 직원은 고성과 평가 32% 더 높고, 이탈 5배 낮음. 다수 고객에서 ROI 수치가 구체적으로 공개돼 wiki의 Performance 카테고리 가장 fact-r…</t>
+          <t>BetterUp은 AI 기반 리더십·매니저 코칭 플랫폼. 2025년 BetterUp Grow (AI-only 코칭 제품) 출시로 전통 human coaching 대비 비용 70% 절감 + 95% 사용자 만족을 주장. 가장 강력한 레퍼런스는 Twilio (8,000+ 직원): 코칭 받은 직원은 고성과 평가 32% 더 높고, 이탈 5배 낮음. 다수 고객에서 ROI 수치가 구체적으로 공개돼 wiki의 Performance 카테고리 가장 fact-rich 사례. Josh Bersin(Tier 1, 단 BetterUp advisor)이 BetterUp Manage를 "pioneering AI-powered platform for leaders"로 독립 분석 (bersin-betterup-manage-ai-coaching-2024-04). HR Executive(Tier 2)도 Bersin의 코칭 시장 분석을 보도 (hrexecutive-bersin-coaching-disruptions-2024).</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
@@ -9667,7 +9686,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="90" customHeight="1">
+    <row r="52" ht="140" customHeight="1">
       <c r="A52" s="7" t="n">
         <v>51</v>
       </c>
@@ -9828,7 +9847,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="90" customHeight="1">
+    <row r="53" ht="140" customHeight="1">
       <c r="A53" s="7" t="n">
         <v>52</v>
       </c>
@@ -9849,7 +9868,7 @@
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>현대모비스가 2025-10-21 본격 운영하는 사내 전용 GenAI 플랫폼 'MoAI(Mobis one AI)'. 온프레미스 배포로 1,000만 건 사내문서 RAG 기반 검색·요약. R&amp;D·IT·품질·영업·생산 등 7개 업무에 적용. 2025년 내 법무·경영지원(HR 포함)으로 확장 계획.</t>
+          <t>현대모비스가 2025-10-21 본격 운영하는 사내 전용 GenAI 플랫폼 'MoAI(Mobis one AI)'. 온프레미스 배포로 1,000만 건 사내문서 RAG 기반 검색·요약. R&amp;D·IT·품질·영업·생산 등 7개 업무에 적용. 2025년 내 법무·경영지원(HR 포함)으로 확장 계획. 변화관리로 프롬프트 템플릿 사전 탑재. 한국 제조 대기업의 "온프레미스 + 변화관리" 정석 사례.</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
@@ -9985,7 +10004,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="90" customHeight="1">
+    <row r="54" ht="140" customHeight="1">
       <c r="A54" s="7" t="n">
         <v>53</v>
       </c>
@@ -10006,7 +10025,7 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>IBM의 내부 HR 가상 에이전트 AskHR은 270,000 IBM 직원에게 HR 정책·보상·복리후생 등 전반적 질문에 답하는 AI 서비스. 초기 rule-based 챗봇에서 시작해, 2025년에 IBM watsonx Orchestrate를 통합하며 agentic automation 수준으로 진화. ⚠️ 자사 보고: 80+ HR 태스크 자동화, 연간 2.1M 대화 처리. IBM CEO Arvind Krishna가 "a couple hundre…</t>
+          <t>IBM의 내부 HR 가상 에이전트 AskHR은 270,000 IBM 직원에게 HR 정책·보상·복리후생 등 전반적 질문에 답하는 AI 서비스. 초기 rule-based 챗봇에서 시작해, 2025년에 IBM watsonx Orchestrate를 통합하며 agentic automation 수준으로 진화. ⚠️ 자사 보고: 80+ HR 태스크 자동화, 연간 2.1M 대화 처리. IBM CEO Arvind Krishna가 "a couple hundred HR workers의 업무가 AI로 대체됐고 프로그래머·영업 채용이 증가"했다고 공개 발언.</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
@@ -10151,7 +10170,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="90" customHeight="1">
+    <row r="55" ht="140" customHeight="1">
       <c r="A55" s="7" t="n">
         <v>54</v>
       </c>
@@ -10172,7 +10191,7 @@
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>IBM watsonx Orchestrate의 Talent Acquisition Agent: 2024-25 generation recruiter copilot. JD 템플릿 생성·hiring manager 공유·후보자 매칭·자격자 alert·intro 메시지·면접 일정·feedback 수집까지 multi-step 워크플로 자동화. ThisWay Global 통합으로 8,500+ diverse community sourcing. Knockri 파…</t>
+          <t>IBM watsonx Orchestrate의 Talent Acquisition Agent: 2024-25 generation recruiter copilot. JD 템플릿 생성·hiring manager 공유·후보자 매칭·자격자 alert·intro 메시지·면접 일정·feedback 수집까지 multi-step 워크플로 자동화. ThisWay Global 통합으로 8,500+ diverse community sourcing. Knockri 파트너십(2025-04)으로 면접 설계 워크플로 통합. ⚠️ 자사 보고: AskHR이 약 500K transactions 처리 (JD 생성 포함).</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -10318,7 +10337,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="90" customHeight="1">
+    <row r="56" ht="140" customHeight="1">
       <c r="A56" s="7" t="n">
         <v>55</v>
       </c>
@@ -10352,7 +10371,7 @@
       <c r="G56" s="7" t="inlineStr">
         <is>
           <t>[Before]
-잡코리아 채용 담당자는 공고 작성·후보자 search·매칭을 별도 도구·매뉴얼 process / Pain point: 한국 채용 시장 vendor 경쟁 (사람인·잡코리아·원티드): 차별화 압박 / Trigger: 2025-10 wantedlab-ai-recruiting-agent launch + 잡코리아 시장 점유 방어
+잡코리아 채용 담당자는 공고 작성·후보자 search·매칭을 별도 도구·매뉴얼 process / Pain point: 한국 채용 시장 vendor 경쟁 (사람인·잡코리아·원티드): 차별화 압박 / Trigger: 2025-10 launch + 잡코리아 시장 점유 방어
 [After]
 1. 채용 담당자가 탤런트 에이전트에 자연어로 의도 입력 ("Python backend 시니어 + 핀테크 경력 + 서울")
 2. 에이전트가 공고 맥락 분석 → 후보자 매칭 + 추천 사유
@@ -10484,7 +10503,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="90" customHeight="1">
+    <row r="57" ht="140" customHeight="1">
       <c r="A57" s="7" t="n">
         <v>56</v>
       </c>
@@ -10652,7 +10671,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="90" customHeight="1">
+    <row r="58" ht="140" customHeight="1">
       <c r="A58" s="7" t="n">
         <v>57</v>
       </c>
@@ -10816,7 +10835,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="90" customHeight="1">
+    <row r="59" ht="140" customHeight="1">
       <c r="A59" s="7" t="n">
         <v>58</v>
       </c>
@@ -10837,7 +10856,7 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>글로벌 제약사 Novartis는 Gloat의 AI 탤런트 마켓플레이스를 도입하여 스킬 기반 조직으로 전환했다. ✅ Fact 직원들은 잡(Job)·프로젝트·멘토십·러닝 콘텐츠를 스킬 기반으로 매칭받는다. 탤런트 마켓플레이스를 통해 성공적인 과제 수행 경험이 있는 직원은 조직 내 영구 이동 가능성이 132% 더 높아졌으며, 크로스펑셔널 프로젝트 배정이 67% 증가했다. ⚠️ 자사 보고: Novartis 및 Gloat 공개 자료 기반 수치.</t>
+          <t>글로벌 제약사 Novartis는 Gloat의 AI 탤런트 마켓플레이스를 도입하여 스킬 기반 조직으로 전환했다. ✅ Fact 직원들은 잡(Job)·프로젝트·멘토십·러닝 콘텐츠를 스킬 기반으로 매칭받는다. 탤런트 마켓플레이스를 통해 성공적인 과제 수행 경험이 있는 직원은 조직 내 영구 이동 가능성이 132% 더 높아졌으며, 크로스펑셔널 프로젝트 배정이 67% 증가했다. ⚠️ 자사 보고: Novartis 및 Gloat 공개 자료 기반 수치. sources/gloat-novartis-case-study-2024.md</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
@@ -10972,7 +10991,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="90" customHeight="1">
+    <row r="60" ht="140" customHeight="1">
       <c r="A60" s="7" t="n">
         <v>59</v>
       </c>
@@ -10993,7 +11012,7 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>SAP SuccessFactors의 첫 번째 HR Joule Agent인 Performance &amp; Goals Agent가 2025년 하반기 GA. 매니저에게 맞춤 인사이트·목표 진척 업데이트·개인화된 대화 포인트를 제공해 성과 대화의 질을 높인다. Josh Bersin(Tier 1)은 이를 "one of the most impressive array of enterprise-class AI announcements"로 평가. 2026년 상반기…</t>
+          <t>SAP SuccessFactors의 첫 번째 HR Joule Agent인 Performance &amp; Goals Agent가 2025년 하반기 GA. 매니저에게 맞춤 인사이트·목표 진척 업데이트·개인화된 대화 포인트를 제공해 성과 대화의 질을 높인다. Josh Bersin(Tier 1)은 이를 "one of the most impressive array of enterprise-class AI announcements"로 평가. 2026년 상반기 Career &amp; Talent Development Agent, HR Service Agent, People Intelligence Agent, Payroll Agent 등 4개 추가 에이전트 GA 예정. sources/sap-joule-performance-agent-bersin-2025-10.md</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr">
@@ -11009,7 +11028,13 @@
           <t>[Before]
 매니저가 SuccessFactors에서 직원별 목표·피드백·리뷰 데이터를 개별 조회 → 수동으로 대화 포인트 준비 /
 [After]
-1. md]]</t>
+1. SuccessFactors 목표 데이터
+2. Joule Performance Agent
+3. 피드백·리뷰 히스토리
+4. 맞춤 인사이트
+5. 목표 진척 업데이트
+6. 대화 포인트
+7. 성과 대화 실행</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
@@ -11119,7 +11144,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="90" customHeight="1">
+    <row r="61" ht="140" customHeight="1">
       <c r="A61" s="7" t="n">
         <v>60</v>
       </c>
@@ -11283,7 +11308,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="90" customHeight="1">
+    <row r="62" ht="140" customHeight="1">
       <c r="A62" s="7" t="n">
         <v>61</v>
       </c>
@@ -11304,7 +11329,7 @@
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>SK하이닉스가 2025 하반기 신입 채용에 'A! SK' (AI Interview with SK Hynix) 전형 신설. AI가 직무별 특화 문제를 출제하면 지원자가 영상 녹화 답변 제출. 자기소개서로 파악 어려운 커뮤니케이션·팀워크·상황 대처 능력을 종합 검증.</t>
+          <t>SK하이닉스가 2025 하반기 신입 채용에 'A!SK' (AI Interview with SK Hynix) 전형 신설. AI가 직무별 특화 문제를 출제하면 지원자가 영상 녹화 답변 제출. 자기소개서로 파악 어려운 커뮤니케이션·팀워크·상황 대처 능력을 종합 검증. 제출 영상은 미래 동료 구성원이 직접 평가하는 hybrid 모델. AI single decision 회피: bias mitigation + 한국 채용절차법 fit.</t>
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr">
@@ -11446,7 +11471,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="90" customHeight="1">
+    <row r="63" ht="140" customHeight="1">
       <c r="A63" s="7" t="n">
         <v>62</v>
       </c>
@@ -11467,7 +11492,7 @@
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>인도 3대 IT 서비스 기업 TCS·Infosys·Wipro는 AI 시대 전환에 맞춰 수십만에서 100만 명 이상 규모의 AI 리스킬링을 추진 중이다. ✅ Fact TCS는 275,000명이 "Ideate and Build with AI" 이니셔티브에 참여했고, Infosys는 AI 전환 프로그램에서 275,000명을 교육했으며, Wipro는 단 1분기 만에 180,000명에게 GenAI 기초 교육을 완료했다. 3사 합산 FY26 Q1 기준 …</t>
+          <t>인도 3대 IT 서비스 기업 TCS·Infosys·Wipro는 AI 시대 전환에 맞춰 수십만에서 100만 명 이상 규모의 AI 리스킬링을 추진 중이다. ✅ Fact TCS는 275,000명이 "Ideate and Build with AI" 이니셔티브에 참여했고, Infosys는 AI 전환 프로그램에서 275,000명을 교육했으며, Wipro는 단 1분기 만에 180,000명에게 GenAI 기초 교육을 완료했다. 3사 합산 FY26 Q1 기준 AI 교육 인원은 약 100만 명에 달한다. sources/aibase-india-it-ai-reskilling-2025.md</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
@@ -11592,7 +11617,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="90" customHeight="1">
+    <row r="64" ht="140" customHeight="1">
       <c r="A64" s="7" t="n">
         <v>63</v>
       </c>
@@ -11613,7 +11638,7 @@
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Workday가 2025-11에 $1.1B로 인수한 스웨덴 AI-native LMS 회사 Sana를 2026-03-17에 첫 통합 제품 "Sana for Workday"로 공개. Sana의 conversational interface가 Workday 신규 UI front door로 채택되고, Sana Learn은 AI-native LMS로 Workday Learning을 대체·보강. ⚠️ 벤더 주장: 코스 생성 시간 4개월 → 4일, enga…</t>
+          <t>Workday가 2025-11에 $1.1B로 인수한 스웨덴 AI-native LMS 회사 Sana를 2026-03-17에 첫 통합 제품 "Sana for Workday"로 공개. Sana의 conversational interface가 Workday 신규 UI front door로 채택되고, Sana Learn은 AI-native LMS로 Workday Learning을 대체·보강. ⚠️ 벤더 주장: 코스 생성 시간 4개월 → 4일, engagement 275% lift. ASOR 거버넌스 하에서 학습 에이전트가 사람·기존 에이전트와 통합 관리됨.</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
@@ -11771,7 +11796,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="90" customHeight="1">
+    <row r="65" ht="140" customHeight="1">
       <c r="A65" s="7" t="n">
         <v>64</v>
       </c>
@@ -11792,7 +11817,7 @@
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Docebo는 AI-native LMS/LXP (3,900+ 고객, 70개국, 30M+ 사용자). Josh Bersin(Tier 1)의 2025-06 독립 분석에서 "traditional → AI-native 전환 중"으로 분류된 학습 플랫폼 (). Bersin이 Project Harmony(neural search), dynamic content generation, virtual coaching 등 AI 기능을 독립적으로 확인. 가장 구체…</t>
+          <t>Docebo는 AI-native LMS/LXP (3,900+ 고객, 70개국, 30M+ 사용자). Josh Bersin(Tier 1)의 2025-06 독립 분석에서 "traditional → AI-native 전환 중"으로 분류된 학습 플랫폼 (bersin-ld-revolution-2025-06). Bersin이 Project Harmony(neural search), dynamic content generation, virtual coaching 등 AI 기능을 독립적으로 확인. 가장 구체적 고객 사례는 La-Z-Boy: ⚠️ 벤더 주장: 활성 LMS 사용자 179% YoY 증가, 과정 완료율 85% 증가. Disguise는 활성 learner 4x 증가, 학습 수익 45% 증가. Brooks Automation은 교육 시간·비용 20% 절감.</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr"/>
@@ -11937,7 +11962,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="90" customHeight="1">
+    <row r="66" ht="140" customHeight="1">
       <c r="A66" s="7" t="n">
         <v>65</v>
       </c>
@@ -11958,7 +11983,7 @@
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>Fujitsu는 73,000명(일본 기준)의 직원에 대한 스킬 기반 HR 전환을 추진하며, 내부 개발 AI 플랫폼 Kozuchi를 전사 배포했다. ✅ Fact Kozuchi는 월 69,000명 이상의 활성 사용자와 하루 약 380,000건의 사용량을 기록하고 있다. FY2020~FY2022 기간에 일본 직원의 약 25%(약 20,000명)가 자발적으로 내부 공모직에 지원했다.</t>
+          <t>Fujitsu는 73,000명(일본 기준)의 직원에 대한 스킬 기반 HR 전환을 추진하며, 내부 개발 AI 플랫폼 Kozuchi를 전사 배포했다. ✅ Fact Kozuchi는 월 69,000명 이상의 활성 사용자와 하루 약 380,000건의 사용량을 기록하고 있다. FY2020~FY2022 기간에 일본 직원의 약 25%(약 20,000명)가 자발적으로 내부 공모직에 지원했다. ⚠️ 자사 보고 sources/diginomica-fujitsu-hcm-ai-2025.md sources/unleash-fujitsu-chro-ai-2025.md</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr">
@@ -12082,7 +12107,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="90" customHeight="1">
+    <row r="67" ht="140" customHeight="1">
       <c r="A67" s="7" t="n">
         <v>66</v>
       </c>
@@ -12103,7 +12128,7 @@
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Hitachi는 2025년 초 HR AI 어시스턴트 "Skye"를 도입했다. ✅ Fact Skye는 사업부·국가·역할에 따라 문서를 추론하고 응답을 개인화하며, IT 서비스 티켓 생성·휴가 요청 처리 등 인텔리전트 액션도 수행한다. Hitachi의 접근이 특별한 이유는 문화 설계에 있다: Skye에 이름과 개성을 부여하여 직원들이 "또 다른 챗봇"이 아닌 "동료 AI"로 인식하도록 설계했다.</t>
+          <t>Hitachi는 2025년 초 HR AI 어시스턴트 "Skye"를 도입했다. ✅ Fact Skye는 사업부·국가·역할에 따라 문서를 추론하고 응답을 개인화하며, IT 서비스 티켓 생성·휴가 요청 처리 등 인텔리전트 액션도 수행한다. Hitachi의 접근이 특별한 이유는 문화 설계에 있다: Skye에 이름과 개성을 부여하여 직원들이 "또 다른 챗봇"이 아닌 "동료 AI"로 인식하도록 설계했다. sources/hrexecutive-hitachi-skye-2025.md</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
@@ -12232,7 +12257,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="90" customHeight="1">
+    <row r="68" ht="140" customHeight="1">
       <c r="A68" s="7" t="n">
         <v>67</v>
       </c>
@@ -12394,7 +12419,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="90" customHeight="1">
+    <row r="69" ht="140" customHeight="1">
       <c r="A69" s="7" t="n">
         <v>68</v>
       </c>
@@ -12415,7 +12440,7 @@
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>IBM Watson Recruitment: 2018 productized 후보자 매칭 AI. 정형·비정형 데이터 + soft trait으로 requisition 대비 score 산출. gender·race·age·ethnicity 억제 bias mitigation 내장. requisition 복잡도와 ideal-match profile flag.</t>
+          <t>IBM Watson Recruitment: 2018 productized 후보자 매칭 AI. 정형·비정형 데이터 + soft trait으로 requisition 대비 score 산출. gender·race·age·ethnicity 억제 bias mitigation 내장. requisition 복잡도와 ideal-match profile flag. ⚠️ 벤더 주장: 84% success prediction 정확도, 35% time-to-fill 감소, 50% turnover 감소, 30% recruitment efficiency 향상, 미국 underrepresented minority 채용 3년간 20% 증가.</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
@@ -12566,7 +12591,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="90" customHeight="1">
+    <row r="70" ht="140" customHeight="1">
       <c r="A70" s="7" t="n">
         <v>69</v>
       </c>
@@ -12743,7 +12768,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="90" customHeight="1">
+    <row r="71" ht="140" customHeight="1">
       <c r="A71" s="7" t="n">
         <v>70</v>
       </c>
@@ -12764,7 +12789,7 @@
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Meta(Facebook)는 2026년부터 모든 직원의 성과 평가에 AI 도구 채택·활용 수준을 공식 평가 항목으로 포함. 내부 AI 도구 Metamate(GPT-4 + Llama 기반 코딩·업무 어시스턴트)의 활용이 "core expectation". ⚠️ 자사 보고: Q4 2025 목표: 중앙 제품팀 코드 변경의 55%를 agent-assisted로, 중간~시니어 엔지니어 80%가 AI 도구 활용. "Level Up" 게임화 프로그램으로 …</t>
+          <t>Meta(Facebook)는 2026년부터 모든 직원의 성과 평가에 AI 도구 채택·활용 수준을 공식 평가 항목으로 포함. 내부 AI 도구 Metamate(GPT-4 + Llama 기반 코딩·업무 어시스턴트)의 활용이 "core expectation". ⚠️ 자사 보고: Q4 2025 목표: 중앙 제품팀 코드 변경의 55%를 agent-assisted로, 중간~시니어 엔지니어 80%가 AI 도구 활용. "Level Up" 게임화 프로그램으로 AI 채택 촉진.</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
@@ -12911,7 +12936,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="90" customHeight="1">
+    <row r="72" ht="140" customHeight="1">
       <c r="A72" s="7" t="n">
         <v>71</v>
       </c>
@@ -12932,7 +12957,10 @@
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>Moderna가 OpenAI Custom GPT로 구축한 Total Rewards 영역 직원 self-service 어시스턴트 2종: 1. US Benefits Assistant GPT: 직원이 의료 등 혜택을 선택할 때 도움. Moderna 내부 HR GPT 사용량 2위 (⚠️ 자사 보고) 2. Equity Compensation GPT: 직원들이 가장 적게 이해하던 프로그램이라는 인식에서 출발해 출시.</t>
+          <t>Moderna가 OpenAI Custom GPT로 구축한 Total Rewards 영역 직원 self-service 어시스턴트 2종:
+1. US Benefits Assistant GPT: 직원이 의료 등 혜택을 선택할 때 도움. Moderna 내부 HR GPT 사용량 2위 (⚠️ 자사 보고)
+2. Equity Compensation GPT: 직원들이 가장 적게 이해하던 프로그램이라는 인식에서 출발해 출시. ⚠️ 자사 보고: 출시 후 해당 영역 이메일·티켓 "a huge decrease"
+두 GPT 모두 전형적인 HR case deflection 패턴: 직원 자가 해결률을 높여 HR 팀 부담을 낮춤.</t>
         </is>
       </c>
       <c r="F72" s="7" t="inlineStr">
@@ -13065,7 +13093,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="90" customHeight="1">
+    <row r="73" ht="140" customHeight="1">
       <c r="A73" s="7" t="n">
         <v>72</v>
       </c>
@@ -13086,7 +13114,7 @@
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Moderna가 OpenAI Custom GPT 기반으로 구축한 HR 내부 도구. 직원 본인의 연말 성과 리뷰를 요약해주는 기능. Moderna 내부 통계(2025년 3~4월)에서 HR GPT 중 메시지·사용자 수 1위 (⚠️ 자사 보고, VP 발표 기준). HR Brew가 WorldatWork Total Rewards 컨퍼런스에서 취재.</t>
+          <t>Moderna가 OpenAI Custom GPT 기반으로 구축한 HR 내부 도구. 직원 본인의 연말 성과 리뷰를 요약해주는 기능. Moderna 내부 통계(2025년 3~4월)에서 HR GPT 중 메시지·사용자 수 1위 (⚠️ 자사 보고, VP 발표 기준). HR Brew가 WorldatWork Total Rewards 컨퍼런스에서 취재. 단일 Tier 2 소스 기반이므로 stub 경계.</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
@@ -13217,7 +13245,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="90" customHeight="1">
+    <row r="74" ht="140" customHeight="1">
       <c r="A74" s="7" t="n">
         <v>73</v>
       </c>
@@ -13374,7 +13402,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="90" customHeight="1">
+    <row r="75" ht="140" customHeight="1">
       <c r="A75" s="7" t="n">
         <v>74</v>
       </c>
@@ -13395,7 +13423,7 @@
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>포스코DX가 2026 그룹 조직개편과 함께 인사·구매·경영분석 사무 업무 영역 ~110개 AI 에이전트 개발 중. 2026 그룹DX전략실장(임치현 UNIST 교수 영입), AI·로봇 융합 연구소장(윤일용) 신설로 그룹 차원 AI 거버넌스 강화. 우리은행 175 에이전트 와 함께 KR 기업 AI 에이전트 portfolio 규모 트렌드의 제조업 reference.</t>
+          <t>포스코DX가 2026 그룹 조직개편과 함께 인사·구매·경영분석 사무 업무 영역 ~110개 AI 에이전트 개발 중. 2026 그룹DX전략실장(임치현 UNIST 교수 영입), AI·로봇 융합 연구소장(윤일용) 신설로 그룹 차원 AI 거버넌스 강화. 우리은행 175 에이전트 woori-bank-175-ai-agents와 함께 KR 기업 AI 에이전트 portfolio 규모 트렌드의 제조업 reference.</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
@@ -13544,7 +13572,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="90" customHeight="1">
+    <row r="76" ht="140" customHeight="1">
       <c r="A76" s="7" t="n">
         <v>75</v>
       </c>
@@ -13565,7 +13593,7 @@
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>SK 그룹이 2024년 하반기 신입사원 공채부터 적용한 생성형 AI 기반 채용 전 과정 자동화. 자사 계열사 (구 SK C&amp;C)와 합작 솔루션. 국내 최초 AICT(AI Competency Test)로 기존 코딩 테스트 폐지. 채용 전 단계를 생성형 AI가 처리하며, 1차 면접은 AI가 진행·평가·결과 보고서 작성까지 100% 자동화.</t>
+          <t>SK 그룹이 2024년 하반기 신입사원 공채부터 적용한 생성형 AI 기반 채용 전 과정 자동화. 자사 계열사 sk-ax (구 SK C&amp;C)와 skt 합작 솔루션. 국내 최초 AICT(AI Competency Test)로 기존 코딩 테스트 폐지. 채용 전 단계를 생성형 AI가 처리하며, 1차 면접은 AI가 진행·평가·결과 보고서 작성까지 100% 자동화. 초기 적용 계열사는 SK㈜ C&amp;C, SKT, SK 브로드밴드 3곳. 2025년 그룹 전사 확대 및 SaaS 대외 확산이 공식 목표.</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr">
@@ -13706,7 +13734,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="90" customHeight="1">
+    <row r="77" ht="140" customHeight="1">
       <c r="A77" s="7" t="n">
         <v>76</v>
       </c>
@@ -13727,7 +13755,7 @@
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>Tampa General Hospital (12,000 FTE, 대형 미국 의료시스템)이 Visier 인력 분석 플랫폼을 활용해 공석율·이직 원인을 데이터로 분석하고 에이전시 노동(파견 간호사) 의존도를 70% 줄였다. 절감 재원 $50M+를 직원 보상에 재투자해 공석율 10% 미만을 달성했다. Visier Outsmart 2025 컨퍼런스에서 Business Performance Impact Vizzie Award 수상. Visier 고객 …</t>
+          <t>Tampa General Hospital (12,000 FTE, 대형 미국 의료시스템)이 Visier 인력 분석 플랫폼을 활용해 공석율·이직 원인을 데이터로 분석하고 에이전시 노동(파견 간호사) 의존도를 70% 줄였다. 절감 재원 $50M+를 직원 보상에 재투자해 공석율 10% 미만을 달성했다. Visier Outsmart 2025 컨퍼런스에서 Business Performance Impact Vizzie Award 수상. Visier 고객 컨퍼런스 발표 기반으로 자사 보고 성격이 있으나, 독립 HIMSS Stage 7 인증(2025-06)이 병원의 분석 성숙도를 간접 검증.</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr">
@@ -13861,7 +13889,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="90" customHeight="1">
+    <row r="78" ht="140" customHeight="1">
       <c r="A78" s="7" t="n">
         <v>77</v>
       </c>
@@ -13882,7 +13910,7 @@
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>Workday가 2025년 9월 Rising에서 Illuminate Performance Review Agent를 발표. 다양한 시스템의 데이터를 종합해 매니저에게 성과 리뷰 초안(first draft)을 자동 생성. 2026년 GA 예정. 기존 Illuminate 에이전트에서는 계약 실행 시간 65% 단축, 스태핑 변경 최대 90% 감소, 감사 증거 수집 연 900시간 절약, 급여 컴플라이언스 4배 빠름 등의 성과를 공유.</t>
+          <t>Workday가 2025년 9월 Rising에서 Illuminate Performance Review Agent를 발표. 다양한 시스템의 데이터를 종합해 매니저에게 성과 리뷰 초안(first draft)을 자동 생성. 2026년 GA 예정. 기존 Illuminate 에이전트에서는 계약 실행 시간 65% 단축, 스태핑 변경 최대 90% 감소, 감사 증거 수집 연 900시간 절약, 급여 컴플라이언스 4배 빠름 등의 성과를 공유. sources/workday-illuminate-pr-2025-09.md</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr">
@@ -13897,7 +13925,11 @@
           <t>[Before]
 매니저가 직원별로 여러 시스템(HRIS·프로젝트 관리·피드백 도구)에서 데이터 수집 → 수동으로 리뷰 작성 /
 [After]
-1. md]]</t>
+1. Workday HRIS 데이터
+2. Performance Review Agent
+3. 타 시스템 데이터
+4. 리뷰 초안 생성
+5. 최종 리뷰 제출</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
@@ -14002,7 +14034,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="90" customHeight="1">
+    <row r="79" ht="140" customHeight="1">
       <c r="A79" s="7" t="n">
         <v>78</v>
       </c>
@@ -14023,7 +14055,7 @@
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>AtkinsRéalis ($8.6B 엔지니어링)가 Beamery로 skills-based 채용 전환. ⚠️ 벤더 주장: 신규 채용자가 25% 빨리 성과 마일스톤 도달, best-fit 후보 식별 30% 시간↓, 후보 engagement 40%↑. Flex (전자 제조)는 skills mapping을 89% 단축 (4~6개월→17일), 1,200+ JD를 40개 역할 아키텍처로 통합, 스킬 추론 90% 적합도. Forrester TEI: Bea…</t>
+          <t>AtkinsRéalis ($8.6B 엔지니어링)가 Beamery로 skills-based 채용 전환. ⚠️ 벤더 주장: 신규 채용자가 25% 빨리 성과 마일스톤 도달, best-fit 후보 식별 30% 시간↓, 후보 engagement 40%↑. Flex (전자 제조)는 skills mapping을 89% 단축 (4~6개월→17일), 1,200+ JD를 40개 역할 아키텍처로 통합, 스킬 추론 90% 적합도. Forrester TEI: Beamery 플랫폼 전체 467% ROI.</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr"/>
@@ -14160,7 +14192,7 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="90" customHeight="1">
+    <row r="80" ht="140" customHeight="1">
       <c r="A80" s="7" t="n">
         <v>79</v>
       </c>
@@ -14181,7 +14213,7 @@
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>Arca Continental Coca-Cola Southwest Beverages (AC-CCSWB, 미국 최대 코카콜라 보틀러 중 하나, 9,000+ 직원)이 Perceptyx Activate의 AI Intelligent Nudges를 통해 리더들에게 참여도 조사 결과 기반의 개인화 코칭 프롬프트를 제공했다. 2020~2025년 5년간 리더십 지수가 65% → 89.3%로 상승하고, 2024 연간 설문 주기에서 93%의 리더가 1,191개…</t>
+          <t>Arca Continental Coca-Cola Southwest Beverages (AC-CCSWB, 미국 최대 코카콜라 보틀러 중 하나, 9,000+ 직원)이 Perceptyx Activate의 AI Intelligent Nudges를 통해 리더들에게 참여도 조사 결과 기반의 개인화 코칭 프롬프트를 제공했다. 2020~2025년 5년간 리더십 지수가 65% → 89.3%로 상승하고, 2024 연간 설문 주기에서 93%의 리더가 1,191개 액션 플랜을 생성했다. 2025 Perceptyx EX Impact Award 수상 + 2025 Coca-Cola Candler Cup(글로벌 보틀러 최우수상) 수상.</t>
         </is>
       </c>
       <c r="F80" s="7" t="inlineStr">
@@ -14316,7 +14348,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="90" customHeight="1">
+    <row r="81" ht="140" customHeight="1">
       <c r="A81" s="7" t="n">
         <v>80</v>
       </c>
@@ -14337,7 +14369,7 @@
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>Deloitte가 2025-06-24에 발표한 Human Capital AI 솔루션 suite: Workforce Analyzer (AI가 직무·역할에 미치는 영향 평가) + Workforce Planner+ (AI 기반 인력 수급 분석·전략 정렬) + HR AI Maturity Model. Salesforce가 named customer로 확인됨 (Ruth Hickin, VP Workforce Innovation). ⚠️ 벤더 주장: 300…</t>
+          <t>Deloitte가 2025-06-24에 발표한 Human Capital AI 솔루션 suite: Workforce Analyzer (AI가 직무·역할에 미치는 영향 평가) + Workforce Planner+ (AI 기반 인력 수급 분석·전략 정렬) + HR AI Maturity Model. Salesforce가 named customer로 확인됨 (Ruth Hickin, VP Workforce Innovation). ⚠️ 벤더 주장: 300+ HR 워크플로를 agentic AI로 재설계.</t>
         </is>
       </c>
       <c r="F81" s="7" t="inlineStr"/>
@@ -14464,7 +14496,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="90" customHeight="1">
+    <row r="82" ht="140" customHeight="1">
       <c r="A82" s="7" t="n">
         <v>81</v>
       </c>
@@ -14485,7 +14517,7 @@
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>HireVue는 AI 비디오 면접 + 게임 기반 역량 평가 플랫폼. 주요 성과: ⚠️ 벤더 주장: time-to-hire 60~89% 단축, 만족도 17~25% 향상. Forrester TEI 연구에서 major financial institution 대상 134% ROI 보고. ★ 2020년 facial analysis 제거 (AI 윤리 논란 후 자발적 결정).</t>
+          <t>HireVue는 AI 비디오 면접 + 게임 기반 역량 평가 플랫폼. 주요 성과: ⚠️ 벤더 주장: time-to-hire 60~89% 단축, 만족도 17~25% 향상. Forrester TEI 연구에서 major financial institution 대상 134% ROI 보고. ★ 2020년 facial analysis 제거 (AI 윤리 논란 후 자발적 결정). DCI Consulting, ORCAA, Landers Workforce Science 등 외부 독��� 감사 기관에 알고리즘 bias audit 의뢰.</t>
         </is>
       </c>
       <c r="F82" s="7" t="inlineStr"/>
@@ -14608,7 +14640,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="90" customHeight="1">
+    <row r="83" ht="140" customHeight="1">
       <c r="A83" s="7" t="n">
         <v>82</v>
       </c>
@@ -14768,7 +14800,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="90" customHeight="1">
+    <row r="84" ht="140" customHeight="1">
       <c r="A84" s="7" t="n">
         <v>83</v>
       </c>
@@ -14789,7 +14821,7 @@
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>한국가스공사가 에너지 공공기관 최초 하이브리드 생성형 AI 플랫폼 도입 (2025-09 발주, 2026 구축). 사내 전용 LLM (보안 민감 영역) + 상용 초거대 LLM (전문지식) 라우팅. 임직원 문서 초안·규정 검토·단순 행정 자동화. 제논(GenON) 구축 사업 수주.</t>
+          <t>한국가스공사가 에너지 공공기관 최초 하이브리드 생성형 AI 플랫폼 도입 (2025-09 발주, 2026 구축). 사내 전용 LLM (보안 민감 영역) + 상용 초거대 LLM (전문지식) 라우팅. 임직원 문서 초안·규정 검토·단순 행정 자동화. 제논(GenON) 구축 사업 수주. 한국 공공기관 보안 vs 성능 trade-off 해법 표준 패턴.</t>
         </is>
       </c>
       <c r="F84" s="7" t="inlineStr">
@@ -14907,7 +14939,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="90" customHeight="1">
+    <row r="85" ht="140" customHeight="1">
       <c r="A85" s="7" t="n">
         <v>84</v>
       </c>
@@ -14928,7 +14960,7 @@
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>한국 인사혁신처는 2025년 3월 공무원 대상 "AI 활용가이드"를 배포하여 생성형 AI 프롬프트 작성 기법과 HR 업무 적용 사례를 안내했다. ✅ Fact 행정안전부·과학기술정보통신부는 삼성SDS·네이버클라우드의 AI 대화형 서비스를 정부 내부망에서 보안 운영하는 "범정부 AI 공통기반" 시범 운영을 시작했다.</t>
+          <t>한국 인사혁신처는 2025년 3월 공무원 대상 "AI 활용가이드"를 배포하여 생성형 AI 프롬프트 작성 기법과 HR 업무 적용 사례를 안내했다. ✅ Fact 행정안전부·과학기술정보통신부는 삼성SDS·네이버클라우드의 AI 대화형 서비스를 정부 내부망에서 보안 운영하는 "범정부 AI 공통기반" 시범 운영을 시작했다. sources/mpm-ai-guide-2025-03.md sources/mois-ai-common-infra-2025.md</t>
         </is>
       </c>
       <c r="F85" s="7" t="inlineStr">
@@ -14941,7 +14973,12 @@
           <t>[Before]
 공무원이 생성형 AI를 개인적·비공식적으로 사용하거나 외부 서비스 접근. /
 [After]
-1. md]]</t>
+1. 공무원
+2. 범정부 AI 공통기반\n내부망 보안 환경
+3. 삼성SDS·네이버클라우드 LLM
+4. 법령·지침·민원 RAG\n행정 문서 연계
+5. AI 응답 생성
+6. 공무원 검토·결재</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
@@ -15060,7 +15097,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="90" customHeight="1">
+    <row r="86" ht="140" customHeight="1">
       <c r="A86" s="7" t="n">
         <v>85</v>
       </c>
@@ -15081,7 +15118,7 @@
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>롯데그룹은 2024년부터 일부 계열사를 시작으로 "직무 기반 HR" 인사제도를 순차적으로 도입·확대하고 있다. ✅ Fact 직무 전문성과 성과에 따라 보상을 차등 지급하는 직무급제로 전환하며, 연차와 무관하게 직무 전문성에 따른 레벨업 심사를 허용한다. 2025년에는 롯데백화점(직원 95.3% 찬성)·롯데웰푸드 등으로 도입 범위를 확대했다.</t>
+          <t>롯데그룹은 2024년부터 일부 계열사를 시작으로 "직무 기반 HR" 인사제도를 순차적으로 도입·확대하고 있다. ✅ Fact 직무 전문성과 성과에 따라 보상을 차등 지급하는 직무급제로 전환하며, 연차와 무관하게 직무 전문성에 따른 레벨업 심사를 허용한다. 2025년에는 롯데백화점(직원 95.3% 찬성)·롯데웰푸드 등으로 도입 범위를 확대했다. sources/newdaily-lotte-hr-2025-04.md sources/sedaily-lotte-dept-store-2025.md</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr">
@@ -15184,7 +15221,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="90" customHeight="1">
+    <row r="87" ht="140" customHeight="1">
       <c r="A87" s="7" t="n">
         <v>86</v>
       </c>
@@ -15205,7 +15242,7 @@
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>Microsoft HR이 자사 제품 Viva + Microsoft 365 Copilot을 자체 HR 운영에 적용한 내부 배포 사례. 핵심은 Employee Self-Service Agent의 글로벌 phased rollout (UK→Canada→India→US→전 세계). Viva Glint 설문으로 Copilot 도입의 "employee thriving" 영향을 상관 측정. IBM AskHR과 마찬가지로 벤더 = 고객인 self-dogfoo…</t>
+          <t>Microsoft HR이 자사 제품 Viva + Microsoft 365 Copilot을 자체 HR 운영에 적용한 내부 배포 사례. 핵심은 Employee Self-Service Agent의 글로벌 phased rollout (UK→Canada→India→US→전 세계). Viva Glint 설문으로 Copilot 도입의 "employee thriving" 영향을 상관 측정. IBM AskHR과 마찬가지로 벤더 = 고객인 self-dogfooding 패턴.</t>
         </is>
       </c>
       <c r="F87" s="7" t="inlineStr"/>
@@ -15339,7 +15376,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="90" customHeight="1">
+    <row r="88" ht="140" customHeight="1">
       <c r="A88" s="7" t="n">
         <v>87</v>
       </c>
@@ -15485,7 +15522,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="90" customHeight="1">
+    <row r="89" ht="140" customHeight="1">
       <c r="A89" s="7" t="n">
         <v>88</v>
       </c>
@@ -15506,7 +15543,7 @@
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>T-Mobile은 Textio의 AI 기반 포용적 언어 플랫폼을 ~125명 리크루터 + 9,000명+ 채용 관리자에게 배포해, 성 중립적 어조 편집 시 여성 지원자 +17%, Textio Score 90+ 달성 시 채용 소요 기간 5일 단축을 확인했다. Workday ATS에 Textio를 직접 통합해 JD 작성 시 실시간 AI 제안을 받는 구조다. 기업 합병 통합 과정 중에 도입했으며, 2025년 3월 HR Brew가 Textio의 스킬 기…</t>
+          <t>T-Mobile은 Textio의 AI 기반 포용적 언어 플랫폼을 ~125명 리크루터 + 9,000명+ 채용 관리자에게 배포해, 성 중립적 어조 편집 시 여성 지원자 +17%, Textio Score 90+ 달성 시 채용 소요 기간 5일 단축을 확인했다. Workday ATS에 Textio를 직접 통합해 JD 작성 시 실시간 AI 제안을 받는 구조다. 기업 합병 통합 과정 중에 도입했으며, 2025년 3월 HR Brew가 Textio의 스킬 기반 면접 도구 출시를 별도 보도.</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr">
@@ -15647,7 +15684,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="90" customHeight="1">
+    <row r="90" ht="140" customHeight="1">
       <c r="A90" s="7" t="n">
         <v>89</v>
       </c>
@@ -15787,7 +15824,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="90" customHeight="1">
+    <row r="91" ht="140" customHeight="1">
       <c r="A91" s="7" t="n">
         <v>90</v>
       </c>
@@ -15954,7 +15991,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="90" customHeight="1">
+    <row r="92" ht="140" customHeight="1">
       <c r="A92" s="7" t="n">
         <v>91</v>
       </c>
@@ -16104,7 +16141,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="90" customHeight="1">
+    <row r="93" ht="140" customHeight="1">
       <c r="A93" s="7" t="n">
         <v>92</v>
       </c>
@@ -16125,7 +16162,7 @@
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>ADP는 Innovation Day 2025(2025-09-03)에서 ADP Assist의 새로운 AI 기능을 발표했다: ① 급여 이상 탐지 및 자동 수정 제안, ② 대화형 GenAI 분석(자연어 질문 → 즉시 차트/인사이트), ③ 규정 준수 자동화. 조기 도입 기업들이 급여 사이클당 최대 30분 절감을 보고했다(자사 보고). TechTarget(Tier 2)이 독립 보도. 플랫폼: Workforce Now, Global Payroll, Ly…</t>
+          <t>ADP는 Innovation Day 2025(2025-09-03)에서 ADP Assist의 새로운 AI 기능을 발표했다: ① 급여 이상 탐지 및 자동 수정 제안, ② 대화형 GenAI 분석(자연어 질문 → 즉시 차트/인사이트), ③ 규정 준수 자동화. 조기 도입 기업들이 급여 사이클당 최대 30분 절감을 보고했다(자사 보고). TechTarget(Tier 2)이 독립 보도. 플랫폼: Workforce Now, Global Payroll, Lyric HCM.</t>
         </is>
       </c>
       <c r="F93" s="7" t="inlineStr">
@@ -16273,7 +16310,7 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="90" customHeight="1">
+    <row r="94" ht="140" customHeight="1">
       <c r="A94" s="7" t="n">
         <v>93</v>
       </c>
@@ -16294,7 +16331,7 @@
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>디웨일이 운영하는 CLAP(클랩)는 중견·대기업 특화 AI 기반 성과관리 SaaS로, 주요 AI 기능은 주관식 평가 코멘트 AI 자동 요약, AI 피드백 생성, AI 원온원 미팅 내용 요약, AI 평가(서술형 리뷰 초안 작성), AI 성장 리포트 등이다. ⚠️ 자사 보고: 인지그룹 등 중견기업에 공급 사례를 확보했으며 2025년 시장 확대 중.</t>
+          <t>디웨일이 운영하는 CLAP(클랩)는 중견·대기업 특화 AI 기반 성과관리 SaaS로, 주요 AI 기능은 주관식 평가 코멘트 AI 자동 요약, AI 피드백 생성, AI 원온원 미팅 내용 요약, AI 평가(서술형 리뷰 초안 작성), AI 성장 리포트 등이다. ⚠️ 자사 보고: 인지그룹 등 중견기업에 공급 사례를 확보했으며 2025년 시장 확대 중. sources/clap-blog-hr-ai-trend-2026.md sources/sisajournal-clap-2025.md</t>
         </is>
       </c>
       <c r="F94" s="7" t="inlineStr">
@@ -16421,7 +16458,7 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="90" customHeight="1">
+    <row r="95" ht="140" customHeight="1">
       <c r="A95" s="7" t="n">
         <v>94</v>
       </c>
@@ -16442,7 +16479,7 @@
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>Culture Amp이 2025년 Q3부터 AI Coach를 전 플랫폼에 확장 배포. Engage(설문 분석) + Perform(성과 리뷰)에 과학 기반 대화형 AI 코칭을 제공하며, 6,800+ 기업·25M 직원 기반에 추가 비용 없이 제공. Asana Head of People Analytics가 "AI Coach puts an expert coach in every manager's pocket"으로 평가. 2026년 3월 Perform…</t>
+          <t>Culture Amp이 2025년 Q3부터 AI Coach를 전 플랫폼에 확장 배포. Engage(설문 분석) + Perform(성과 리뷰)에 과학 기반 대화형 AI 코칭을 제공하며, 6,800+ 기업·25M 직원 기반에 추가 비용 없이 제공. Asana Head of People Analytics가 "AI Coach puts an expert coach in every manager's pocket"으로 평가. 2026년 3월 Performance Culture Quadrant(PCQ) 발표: 1,800개 기업 데이터에서 문화-성과 연결 기업이 시장가치 47% 프리미엄을 보인다는 자체 연구 공개. sources/cultureamp-ai-coach-expansion-2025-10.md</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr">
@@ -16458,7 +16495,12 @@
           <t>[Before]
 매니저가 성과 리뷰를 빈 페이지에서 시작 → engagement 결과를 수동 해석 → 액션 플랜 없이 방치 /
 [After]
-1. md]]</t>
+1. Engagement 설문 결과
+2. AI Coach 분석
+3. 과거 피드백·동료 리뷰
+4. 개인화 액션 플랜
+5. 구조화 리뷰 가이드
+6. 성과 리뷰 제출</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr"/>
@@ -16563,7 +16605,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="90" customHeight="1">
+    <row r="96" ht="140" customHeight="1">
       <c r="A96" s="7" t="n">
         <v>95</v>
       </c>
@@ -16584,7 +16626,7 @@
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>그리팅(GreetingHR)은 국내 1위 채용 관리 솔루션(ATS/TRM)으로, 2025년 고용노동부 "채용관리 솔루션 지원사업" 공급기업으로 선정되어 중소기업 도입률이 전년 대비 158% 급증했다. ⚠️ 자사 보고: 그리팅 도입 시 채용 소요시간 약 65% 단축, 채용 비용 약 50% 절감을 주장한다. AI를 활용한 정교한 인재풀 구축과 기업 맞춤형 후보자 매칭이 핵심 차별점이다.</t>
+          <t>그리팅(GreetingHR)은 국내 1위 채용 관리 솔루션(ATS/TRM)으로, 2025년 고용노동부 "채용관리 솔루션 지원사업" 공급기업으로 선정되어 중소기업 도입률이 전년 대비 158% 급증했다. ⚠️ 자사 보고: 그리팅 도입 시 채용 소요시간 약 65% 단축, 채용 비용 약 50% 절감을 주장한다. AI를 활용한 정교한 인재풀 구축과 기업 맞춤형 후보자 매칭이 핵심 차별점이다. sources/greetinghr-ats-guide-2025.md sources/ezyeconomy-greetinghr-2025.md</t>
         </is>
       </c>
       <c r="F96" s="7" t="inlineStr">
@@ -16711,7 +16753,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="90" customHeight="1">
+    <row r="97" ht="140" customHeight="1">
       <c r="A97" s="7" t="n">
         <v>96</v>
       </c>
@@ -16865,7 +16907,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="90" customHeight="1">
+    <row r="98" ht="140" customHeight="1">
       <c r="A98" s="7" t="n">
         <v>97</v>
       </c>
@@ -17001,7 +17043,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="90" customHeight="1">
+    <row r="99" ht="140" customHeight="1">
       <c r="A99" s="7" t="n">
         <v>98</v>
       </c>
@@ -17145,7 +17187,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="90" customHeight="1">
+    <row r="100" ht="140" customHeight="1">
       <c r="A100" s="7" t="n">
         <v>99</v>
       </c>
@@ -17166,7 +17208,7 @@
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>adidas가 Qualtrics XM AI를 도입해 ⚠️ 벤더 주장: 수동 분석 95%↓, 매니저의 개인화 행동 계획 작성 70%↑. Dr. Sebastian Projahn (Sr. Director People Intelligence, adidas): *"We leveraged Qualtrics AI to democratize insights, reduce bias, and save time"*: 특히 매장·물류센터 매니저에게 즉시 인사이트 …</t>
+          <t>adidas가 Qualtrics XM AI를 도입해 ⚠️ 벤더 주장: 수동 분석 95%↓, 매니저의 개인화 행동 계획 작성 70%↑. Dr. Sebastian Projahn (Sr. Director People Intelligence, adidas): "We leveraged Qualtrics AI to democratize insights, reduce bias, and save time": 특히 매장·물류센터 매니저에게 즉시 인사이트 제공.</t>
         </is>
       </c>
       <c r="F100" s="7" t="inlineStr"/>
@@ -17303,7 +17345,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="90" customHeight="1">
+    <row r="101" ht="140" customHeight="1">
       <c r="A101" s="7" t="n">
         <v>100</v>
       </c>
@@ -17436,7 +17478,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="90" customHeight="1">
+    <row r="102" ht="140" customHeight="1">
       <c r="A102" s="7" t="n">
         <v>101</v>
       </c>
@@ -17457,7 +17499,7 @@
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>General Mills가 전통 EAP(Employee Assistance Program)의 1% 이용률 문제를 해결하기 위해 Spring Health의 AI 기반 정밀 정신건강 플랫폼을 도입. 14개월 내 28% 직원 등록, 이용률 26% (기존 대비 26배), 우울증 58% 증상 개선(평균 2.46 세션), 불안 49% 개선(1.4 세션), 전체 67% 개선을 보고. Spring Health는 AI를 활용해 직원-치료사 매칭·초기 평가·치…</t>
+          <t>General Mills가 전통 EAP(Employee Assistance Program)의 1% 이용률 문제를 해결하기 위해 Spring Health의 AI 기반 정밀 정신건강 플랫폼을 도입. 14개월 내 28% 직원 등록, 이용률 26% (기존 대비 26배), 우울증 58% 증상 개선(평균 2.46 세션), 불안 49% 개선(1.4 세션), 전체 67% 개선을 보고. Spring Health는 AI를 활용해 직원-치료사 매칭·초기 평가·치료 경로 최적화를 수행하며, 2026년 기준 50M+ lives 지원. sources/spring-health-general-mills-case.md</t>
         </is>
       </c>
       <c r="F102" s="7" t="inlineStr">
@@ -17587,7 +17629,7 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="90" customHeight="1">
+    <row r="103" ht="140" customHeight="1">
       <c r="A103" s="7" t="n">
         <v>102</v>
       </c>
@@ -17608,7 +17650,7 @@
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>UKG가 AI 기반 워크포스 스케줄링·인텔리전스 솔루션을 확대하며, 미국 최대 헬스케어 시스템의 90% 가까이가 UKG를 사용한다고 발표(2026-02). 대표 고객 사례로 KC CARE Health Center가 리텐션 92% 개선·효율성 60% 향상, Jetro Restaurant Depot이 UKG Rapid Hire로 연간 소싱·온보딩 비용 $1.8M 절감(2025), 연 $2.2M 절감 전망. 2025년 11월 Workforce In…</t>
+          <t>UKG가 AI 기반 워크포스 스케줄링·인텔리전스 솔루션을 확대하며, 미국 최대 헬스케어 시스템의 90% 가까이가 UKG를 사용한다고 발표(2026-02). 대표 고객 사례로 KC CARE Health Center가 리텐션 92% 개선·효율성 60% 향상, Jetro Restaurant Depot이 UKG Rapid Hire로 연간 소싱·온보딩 비용 $1.8M 절감(2025), 연 $2.2M 절감 전망. 2025년 11월 Workforce Intelligence Hub 출시: AI 기반 스케줄·타임·채용·성과·급여 데이터를 실시간 통합 뷰로 제공. sources/ukg-healthcare-scheduling-2026-02.md</t>
         </is>
       </c>
       <c r="F103" s="7" t="inlineStr">
@@ -17624,7 +17666,13 @@
           <t>[Before]
 매니저가 수동으로 교대표 작성 → 자격증·컴플라이언스·선호도 수동 확인 → 채용도 개별 프로세스 /
 [After]
-1. md]]</t>
+1. 자격증·규제·선호도 데이터
+2. AI 스케줄링 엔진
+3. 최적 교대표 추천
+4. 스케줄 배포
+5. Workforce Intelligence Hub
+6. 실시간 통합 뷰
+7. 타임·급여 데이터</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr"/>
@@ -17733,7 +17781,7 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="90" customHeight="1">
+    <row r="104" ht="140" customHeight="1">
       <c r="A104" s="7" t="n">
         <v>103</v>
       </c>
@@ -17754,7 +17802,8 @@
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>Viven AI: Eightfold 공동창업자 Ashutosh Garg·Varun Kacholia가 분사 창업한 신생 회사. 2025-10-15 stealth 탈출과 함께 Khosla Ventures·Foundation Capital 등으로부터 $35M seed funding 확보. 핵심 컨셉: "Digital Twin of unavailable coworkers": 부재중·휴직·시차 동료의 지식·전문성·맥락을 LLM 기반으로 재현해 다른 직…</t>
+          <t>Viven AI: Eightfold 공동창업자 Ashutosh Garg·Varun Kacholia가 분사 창업한 신생 회사. 2025-10-15 stealth 탈출과 함께 Khosla Ventures·Foundation Capital 등으로부터 $35M seed funding 확보. 핵심 컨셉: "Digital Twin of unavailable coworkers": 부재중·휴직·시차 동료의 지식·전문성·맥락을 LLM 기반으로 재현해 다른 직원이 query 가능. 비동기 협업의 "동료 부재 시 지식 단절" 문제 해결 시도.
+&gt; 📌 중요: PwC 자료에서 "Eightfold Digital Twin (2025)"으로 표기된 기능은 실제로는 본 분사 회사 Viven AI 제품. Eightfold 본체와 별개. Mastercard·다른 Eightfold 고객사에 deploy됐다는 증거 없음.</t>
         </is>
       </c>
       <c r="F104" s="7" t="inlineStr">
@@ -17877,7 +17926,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="90" customHeight="1">
+    <row r="105" ht="140" customHeight="1">
       <c r="A105" s="7" t="n">
         <v>104</v>
       </c>
@@ -17898,7 +17947,7 @@
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>Zapier (워크플로 자동화 SaaS, 100% 원격, 30개국 ~800명)은 Enboarder 플랫폼으로 온보딩 자동화를 구현해 수작업 온보딩 태스크 206,000분(86 근무 주) 절감, 채용 관리자 참여율 +10%, 신규 입사자의 온보딩 최우수 평가 가능성 2.5배 향상을 달성했다. 2022년 케이스 스터디; Enboarder는 이후 2025년 SmartRecruiters와 통합 파트너십을 맺고 AI 네이티브 온보딩 플랫폼으로 확장. …</t>
+          <t>Zapier (워크플로 자동화 SaaS, 100% 원격, 30개국 ~800명)은 Enboarder 플랫폼으로 온보딩 자동화를 구현해 수작업 온보딩 태스크 206,000분(86 근무 주) 절감, 채용 관리자 참여율 +10%, 신규 입사자의 온보딩 최우수 평가 가능성 2.5배 향상을 달성했다. 2022년 케이스 스터디; Enboarder는 이후 2025년 SmartRecruiters와 통합 파트너십을 맺고 AI 네이티브 온보딩 플랫폼으로 확장. Deloitte, KPMG, ING, T-Mobile, Cisco도 Enboarder 고객으로 확인.</t>
         </is>
       </c>
       <c r="F105" s="7" t="inlineStr">
@@ -18035,7 +18084,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="90" customHeight="1">
+    <row r="106" ht="140" customHeight="1">
       <c r="A106" s="7" t="n">
         <v>105</v>
       </c>
@@ -18056,7 +18105,7 @@
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>15Five가 2025년 5월 출시한 Kona는 AI 기반 매니저 효과성 코치로, 1:1 미팅에 자동 참여해 대화를 전사(transcribe)하고 요약·액션 아이템을 생성하며, 성과 리뷰·engagement 설문·이전 미팅 맥락을 통합 분석해 실시간 코칭 팁을 제공한다. ReUp Education이 초기 도입 고객으로 파일럿 → 전사 매니저 롤아웃을 완료했다.</t>
+          <t>15Five가 2025년 5월 출시한 Kona는 AI 기반 매니저 효과성 코치로, 1:1 미팅에 자동 참여해 대화를 전사(transcribe)하고 요약·액션 아이템을 생성하며, 성과 리뷰·engagement 설문·이전 미팅 맥락을 통합 분석해 실시간 코칭 팁을 제공한다. ReUp Education이 초기 도입 고객으로 파일럿 → 전사 매니저 롤아웃을 완료했다. sources/15five-kona-launch-2025-05.md</t>
         </is>
       </c>
       <c r="F106" s="7" t="inlineStr">
@@ -18072,7 +18121,13 @@
           <t>[Before]
 매니저가 1:1 미팅을 자유 형식으로 진행 → 노트 수동 작성 → 후속 조치 누락 빈번 → HR이 매니저 효과성 파악 어려움 /
 [After]
-1. md]]</t>
+1. 1:1 미팅 시작
+2. Kona 자동 참여·전사
+3. 요약·액션 아이템 생성
+4. engagement·성과 데이터 분석
+5. 실시간 코칭 팁 전달
+6. 행동 변화 자동 추적
+7. HR 대시보드 모니터링</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr">
@@ -18177,7 +18232,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="90" customHeight="1">
+    <row r="107" ht="140" customHeight="1">
       <c r="A107" s="7" t="n">
         <v>106</v>
       </c>
@@ -18331,7 +18386,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="90" customHeight="1">
+    <row r="108" ht="140" customHeight="1">
       <c r="A108" s="7" t="n">
         <v>107</v>
       </c>
@@ -18352,7 +18407,7 @@
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>Josh Bersin Co.가 2025년 5월에 발표한 AI-native 기업 학습 플랫폼. Sana Labs의 AI foundation을 기반으로, 기존 콘텐츠(PDF·Word·오디오·비디오·SCORM)를 자동으로 코스·assessment·simulation으로 변환. 외부 공개 고객: ✅ Workday internal leadership academy (Bersin 2025-06 follow-up에서 확인). Bersin Co.</t>
+          <t>Josh Bersin Co.가 2025년 5월에 발표한 AI-native 기업 학습 플랫폼. Sana Labs의 AI foundation을 기반으로, 기존 콘텐츠(PDF·Word·오디오·비디오·SCORM)를 자동으로 코스·assessment·simulation으로 변환. 외부 공개 고객: ✅ Workday internal leadership academy (Bersin 2025-06 follow-up에서 확인). Bersin Co. 자체 HR Academy 재전환 사례(8년 자료 → 5개월 만에 750 learning objects)와 함께 2건의 deployment 레퍼런스.</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr">
@@ -18500,7 +18555,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="90" customHeight="1">
+    <row r="109" ht="140" customHeight="1">
       <c r="A109" s="7" t="n">
         <v>108</v>
       </c>
@@ -18521,7 +18576,7 @@
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>Betterworks가 2026년 1월 NextGen AI-native 성과관리 플랫폼을 출시. 400+ 고객 우선순위 기능을 반영, Goal Intelligence (역할·팀·회사 우선순위 기반 SMART 목표 자동 추천), AI 기반 평가 편향 감소·일관성 향상, 부서·지역별 AI 기능 단계적 활성화를 지원. Colgate-Palmolive, Intuit, ATB Financial, Kuehne+Nagel 등이 고객. 2026 State …</t>
+          <t>Betterworks가 2026년 1월 NextGen AI-native 성과관리 플랫폼을 출시. 400+ 고객 우선순위 기능을 반영, Goal Intelligence (역할·팀·회사 우선순위 기반 SMART 목표 자동 추천), AI 기반 평가 편향 감소·일관성 향상, 부서·지역별 AI 기능 단계적 활성화를 지원. Colgate-Palmolive, Intuit, ATB Financial, Kuehne+Nagel 등이 고객. 2026 State of Performance 보고서에서 임원 vs 직원의 AI 성과관리 준비도 인식 6배 차이를 발견. sources/betterworks-nextgen-2026-01.md</t>
         </is>
       </c>
       <c r="F109" s="7" t="inlineStr">
@@ -18538,7 +18593,12 @@
           <t>[Before]
 연 1~2회 목표 설정 → 수동 리뷰 작성 → 편향 보정 없음 /
 [After]
-1. md]]</t>
+1. 역할·팀·회사 우선순위
+2. Goal Intelligence
+3. SMART 목표 추천
+4. 연속 피드백 수집
+5. AI 리뷰 편향 탐지
+6. 최종 평가 제출</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr"/>
@@ -18639,7 +18699,7 @@
         </is>
       </c>
     </row>
-    <row r="110" ht="90" customHeight="1">
+    <row r="110" ht="140" customHeight="1">
       <c r="A110" s="7" t="n">
         <v>109</v>
       </c>
@@ -18795,7 +18855,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="90" customHeight="1">
+    <row r="111" ht="140" customHeight="1">
       <c r="A111" s="7" t="n">
         <v>110</v>
       </c>
@@ -18816,7 +18876,7 @@
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>플렉스(flex)는 한국 올인원 HR SaaS 플랫폼으로, 6만+ 기업 가입·ARR 300억원 돌파, 기업가치 5,000억원 평가. 인사·급여·채용·성과관리·전자계약·비용관리를 단일 플랫폼에 통합. 2025년 OCR 기반 수기 근무표 자동변환 + 노동법·세법 AI 에이전트 상담 기능의 순차 도입을 발표하며, "SaaS → Service as a Software" 패러다임 전환을 선언.</t>
+          <t>플렉스(flex)는 한국 올인원 HR SaaS 플랫폼으로, 6만+ 기업 가입·ARR 300억원 돌파, 기업가치 5,000억원 평가. 인사·급여·채용·성과관리·전자계약·비용관리를 단일 플랫폼에 통합. 2025년 OCR 기반 수기 근무표 자동변환 + 노동법·세법 AI 에이전트 상담 기능의 순차 도입을 발표하며, "SaaS → Service as a Software" 패러다임 전환을 선언. sources/flex-korea-hr-saas-2025.md</t>
         </is>
       </c>
       <c r="F111" s="7" t="inlineStr">
@@ -18934,7 +18994,7 @@
         </is>
       </c>
     </row>
-    <row r="112" ht="90" customHeight="1">
+    <row r="112" ht="140" customHeight="1">
       <c r="A112" s="7" t="n">
         <v>111</v>
       </c>
@@ -19067,7 +19127,7 @@
         </is>
       </c>
     </row>
-    <row r="113" ht="90" customHeight="1">
+    <row r="113" ht="140" customHeight="1">
       <c r="A113" s="7" t="n">
         <v>112</v>
       </c>
@@ -19088,7 +19148,7 @@
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>Lattice는 성과관리·engagement·보상 통합 SaaS로, AI Performance Summarization (리뷰 주기 중 받은 피드백·리뷰를 자동 요약해 핵심 트렌드 도출), Goals AI Assistance (자연어로 목표 쿼리·요약·분석), AI Agent (Slack/Teams 내장, 개인별 이탈 리스크 탐지)를 제공한다. Ruggable VP of People이 "Lattice AI for engagement로 비즈니스…</t>
+          <t>Lattice는 성과관리·engagement·보상 통합 SaaS로, AI Performance Summarization (리뷰 주기 중 받은 피드백·리뷰를 자동 요약해 핵심 트렌드 도출), Goals AI Assistance (자연어로 목표 쿼리·요약·분석), AI Agent (Slack/Teams 내장, 개인별 이탈 리스크 탐지)를 제공한다. Ruggable VP of People이 "Lattice AI for engagement로 비즈니스의 다른 영역에서도 AI 필요성을 입증했다"고 평가. 2026년 상반기 AI Agent가 Slack/Teams 내 작동하는 업데이트 발표.</t>
         </is>
       </c>
       <c r="F113" s="7" t="inlineStr">
@@ -19211,7 +19271,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="90" customHeight="1">
+    <row r="114" ht="140" customHeight="1">
       <c r="A114" s="7" t="n">
         <v>113</v>
       </c>
@@ -19354,7 +19414,7 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="90" customHeight="1">
+    <row r="115" ht="140" customHeight="1">
       <c r="A115" s="7" t="n">
         <v>114</v>
       </c>
@@ -19498,7 +19558,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="90" customHeight="1">
+    <row r="116" ht="140" customHeight="1">
       <c r="A116" s="7" t="n">
         <v>115</v>
       </c>
@@ -19646,7 +19706,7 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="90" customHeight="1">
+    <row r="117" ht="140" customHeight="1">
       <c r="A117" s="7" t="n">
         <v>116</v>
       </c>
@@ -19667,7 +19727,7 @@
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>ServiceNow의 Now Assist는 HRSD(HR Service Delivery) 모듈에 통합된 GenAI 기능. HR 케이스 요약·해결 노트 생성·직원 셀프서비스 자동 응답을 제공. ⚠️ 벤더 주장: 54% helpfulness rate. Now Assist ACV $600M 달성 (2025년 말), QoQ 150%+ 딜 성장.</t>
+          <t>ServiceNow의 Now Assist는 HRSD(HR Service Delivery) 모듈에 통합된 GenAI 기능. HR 케이스 요약·해결 노트 생성·직원 셀프서비스 자동 응답을 제공. ⚠️ 벤더 주장: 54% helpfulness rate. Now Assist ACV $600M 달성 (2025년 말), QoQ 150%+ 딜 성장. HR 영역에서는 티켓 분류·라우팅·지식베이스 자동 유지에 특화: moderna-ask-hr-routing의 "routing" 기능과 유사하지만 ITSM DNA를 가진 접근법.</t>
         </is>
       </c>
       <c r="F117" s="7" t="inlineStr"/>
@@ -19790,7 +19850,7 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="90" customHeight="1">
+    <row r="118" ht="140" customHeight="1">
       <c r="A118" s="7" t="n">
         <v>117</v>
       </c>
@@ -19949,7 +20009,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="90" customHeight="1">
+    <row r="119" ht="140" customHeight="1">
       <c r="A119" s="7" t="n">
         <v>118</v>
       </c>
@@ -19970,7 +20030,7 @@
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>Visier는 People Analytics 전문 AI 플랫폼. 주력 AI 제품 Vee는 자연어로 workforce 데이터에 질문하면 즉시 인사이트를 제공하는 디지털 어시스턴트. 2025년 HR Tech에서 Visier Org Design 출시: AI 기반 조직 설계 + workforce planning 통합. 고객 Providence (헬스케어)는 Visier로 2,000+ 간호사(caregiver) proactive onboarding +…</t>
+          <t>Visier는 People Analytics 전문 AI 플랫폼. 주력 AI 제품 Vee는 자연어로 workforce 데이터에 질문하면 즉시 인사이트를 제공하는 디지털 어시스턴트. 2025년 HR Tech에서 Visier Org Design 출시: AI 기반 조직 설계 + workforce planning 통합. 고객 Providence (헬스케어)는 Visier로 2,000+ 간호사(caregiver) proactive onboarding + vacancy forecasting 달성.</t>
         </is>
       </c>
       <c r="F119" s="7" t="inlineStr"/>
@@ -20092,7 +20152,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="90" customHeight="1">
+    <row r="120" ht="140" customHeight="1">
       <c r="A120" s="7" t="n">
         <v>119</v>
       </c>
@@ -20113,7 +20173,7 @@
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>Workday HCM 플랫폼에 내장된 AI 기능으로, 조직의 직무 체계(job architecture)를 분석·생성·관리한다. Bersin의 2024-09 분석에서는 "skill gap·직무 통합 기회·역할 부적합 식별"(분석형)로, 2025-09 Workday press release에서는 "직무 사다리(job ladder)의 생성·관리 자동화"(구성형)로 묘사된다. 두 설명은 상호 모순은 아니며, 2024-09 이후 기능이 확장되었거나 측…</t>
+          <t>Workday HCM 플랫폼에 내장된 AI 기능으로, 조직의 직무 체계(job architecture)를 분석·생성·관리한다. Bersin의 2024-09 분석에서는 "skill gap·직무 통합 기회·역할 부적합 식별"(분석형)로, 2025-09 Workday press release에서는 "직무 사다리(job ladder)의 생성·관리 자동화"(구성형)로 묘사된다. 두 설명은 상호 모순은 아니며, 2024-09 이후 기능이 확장되었거나 측면이 다른 것으로 보이나 공식 확인은 없다.</t>
         </is>
       </c>
       <c r="F120" s="7" t="inlineStr">
@@ -20254,7 +20314,7 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="90" customHeight="1">
+    <row r="121" ht="140" customHeight="1">
       <c r="A121" s="7" t="n">
         <v>120</v>
       </c>
@@ -20408,7 +20468,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="90" customHeight="1">
+    <row r="122" ht="140" customHeight="1">
       <c r="A122" s="7" t="n">
         <v>121</v>
       </c>
@@ -20557,7 +20617,7 @@
         </is>
       </c>
     </row>
-    <row r="123" ht="90" customHeight="1">
+    <row r="123" ht="140" customHeight="1">
       <c r="A123" s="7" t="n">
         <v>122</v>
       </c>
@@ -20578,7 +20638,7 @@
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>더존비즈온(국내 ERP·급여 dominant player)이 자사 ONE AI 제품군에 포함시킨 연말정산 end-to-end 자동화 서비스. 대상자 선정부터 결과 안내까지 전 과정을 자동화. 국세청 간소화 자료 자동 다운로드·세액 예측·홈택스 자동신고·총괄현황판 등 제공. 2024-12 기준 1,000개 기업 추가 계약 보고(⚠ 벤더 주장).</t>
+          <t>더존비즈온(국내 ERP·급여 dominant player)이 자사 ONE AI 제품군에 포함시킨 연말정산 end-to-end 자동화 서비스. 대상자 선정부터 결과 안내까지 전 과정을 자동화. 국세청 간소화 자료 자동 다운로드·세액 예측·홈택스 자동신고·총괄현황판 등 제공. 2024-12 기준 1,000개 기업 추가 계약 보고(⚠ 벤더 주장). 중소·중견기업 타겟.</t>
         </is>
       </c>
       <c r="F123" s="7" t="inlineStr">
@@ -20733,7 +20793,7 @@
         </is>
       </c>
     </row>
-    <row r="124" ht="90" customHeight="1">
+    <row r="124" ht="140" customHeight="1">
       <c r="A124" s="7" t="n">
         <v>123</v>
       </c>
@@ -20754,7 +20814,7 @@
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>Eightfold AI는 skills-based talent intelligence 플랫폼으로, 채용·내부 이동·스킬 관리를 AI로 통합. 2025년 AI Interviewer (자동 1차 면접)과 Digital Twin (직원의 지식·스킬·경험을 캡처하는 개인화 LLM) 발표. ⚠️ 벤더 주장: AI Interviewer로 time to first interview 90% 감소, 3,000명 이상 후보자를 AI로 면접 처리. Deloitte…</t>
+          <t>Eightfold AI는 skills-based talent intelligence 플랫폼으로, 채용·내부 이동·스킬 관리를 AI로 통합. 2025년 AI Interviewer (자동 1차 면접)과 Digital Twin (직원의 지식·스킬·경험을 캡처하는 개인화 LLM) 발표. ⚠️ 벤더 주장: AI Interviewer로 time to first interview 90% 감소, 3,000명 이상 후보자를 AI로 면접 처리. Deloitte 전략적 제휴 확인.</t>
         </is>
       </c>
       <c r="F124" s="7" t="inlineStr">
@@ -20888,7 +20948,7 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="90" customHeight="1">
+    <row r="125" ht="140" customHeight="1">
       <c r="A125" s="7" t="n">
         <v>124</v>
       </c>
@@ -21024,7 +21084,7 @@
         </is>
       </c>
     </row>
-    <row r="126" ht="90" customHeight="1">
+    <row r="126" ht="140" customHeight="1">
       <c r="A126" s="7" t="n">
         <v>125</v>
       </c>
@@ -21161,7 +21221,7 @@
         </is>
       </c>
     </row>
-    <row r="127" ht="90" customHeight="1">
+    <row r="127" ht="140" customHeight="1">
       <c r="A127" s="7" t="n">
         <v>126</v>
       </c>
@@ -21302,7 +21362,7 @@
         </is>
       </c>
     </row>
-    <row r="128" ht="90" customHeight="1">
+    <row r="128" ht="140" customHeight="1">
       <c r="A128" s="7" t="n">
         <v>127</v>
       </c>
@@ -21323,7 +21383,7 @@
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>Paychex가 2026년 2월 Paycor 및 Paychex Flex 플랫폼에 에이전틱 AI 솔루션을 발표. Paycor Agentic Timesheet Approvals(타임카드 자동 스코어링·이상만 사람 검토), Paycor Auto-Shifts(근무시간 제한·휴식·공정근무법 기반 최적 교대 생성), Paychex Flex AI-Powered Time-Off(PTO 패턴 분석·반복 가용성 AI). 800,000 고객 규모. Nucleus…</t>
+          <t>Paychex가 2026년 2월 Paycor 및 Paychex Flex 플랫폼에 에이전틱 AI 솔루션을 발표. Paycor Agentic Timesheet Approvals(타임카드 자동 스코어링·이상만 사람 검토), Paycor Auto-Shifts(근무시간 제한·휴식·공정근무법 기반 최적 교대 생성), Paychex Flex AI-Powered Time-Off(PTO 패턴 분석·반복 가용성 AI). 800,000 고객 규모. Nucleus Research: 워크포스 관리 자동화 평균 ROI $12.24/달러. sources/paychex-agentic-workforce-2026-02.md</t>
         </is>
       </c>
       <c r="F128" s="7" t="inlineStr">
@@ -21339,7 +21399,14 @@
           <t>[Before]
 매니저가 타임카드 수동 검토 → 교대표 수동 작성 → PTO 개별 승인 /
 [After]
-1. md]]</t>
+1. 타임카드 제출
+2. Agentic Timesheet 스코어링
+3. 자동 승인
+4. 승인/수정
+5. 규칙: 근무시간·휴식·법규
+6. Auto-Shifts
+7. 최적 교대표
+8. 과거 PTO 데이터</t>
         </is>
       </c>
       <c r="H128" s="7" t="inlineStr"/>
@@ -21436,7 +21503,7 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="90" customHeight="1">
+    <row r="129" ht="140" customHeight="1">
       <c r="A129" s="7" t="n">
         <v>128</v>
       </c>
@@ -21457,7 +21524,7 @@
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>삼성 멀티캠퍼스의 CIC(Corporate Innovation Campus) 플랫폼은 삼성전자 사내 직원 대상 e-러닝 서비스로, 부서·직급·직무·관심 키워드·수강 이력을 분석해 맞춤형 교육 콘텐츠를 추천하는 AI 기능을 운영한다. 멀티캠퍼스는 별도로 외부 기업 대상 AI 직무 역량 교육 프로그램과 IT 업스킬링·리스킬링 서비스를 제공하며, 2025년 삼성청년SW·AI아카데미(SSAFY) 커리큘럼에서도 AI 역량 강화를 확대했다.</t>
+          <t>삼성 멀티캠퍼스의 CIC(Corporate Innovation Campus) 플랫폼은 삼성전자 사내 직원 대상 e-러닝 서비스로, 부서·직급·직무·관심 키워드·수강 이력을 분석해 맞춤형 교육 콘텐츠를 추천하는 AI 기능을 운영한다. 멀티캠퍼스는 별도로 외부 기업 대상 AI 직무 역량 교육 프로그램과 IT 업스킬링·리스킬링 서비스를 제공하며, 2025년 삼성청년SW·AI아카데미(SSAFY) 커리큘럼에서도 AI 역량 강화를 확대했다. sources/clap-blog-hr-ai-trend-2026.md</t>
         </is>
       </c>
       <c r="F129" s="7" t="inlineStr">
@@ -21470,9 +21537,7 @@
       <c r="G129" s="7" t="inlineStr">
         <is>
           <t>[Before]
-LMS에서 직원이 과정 목록을 수동 탐색 → 관련성 낮은 과정 수강 → 학습 효율 저하 /
-[After]
-1. md]]</t>
+LMS에서 직원이 과정 목록을 수동 탐색 → 관련성 낮은 과정 수강 → 학습 효율 저하 /</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr"/>
@@ -21565,7 +21630,7 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="90" customHeight="1">
+    <row r="130" ht="140" customHeight="1">
       <c r="A130" s="7" t="n">
         <v>129</v>
       </c>
@@ -21586,7 +21651,7 @@
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>PwC Korea가 SK하이닉스에 제안한 5-Agent agentic retention prediction 시스템. 5개 specialist 에이전트가 각기 다른 데이터 영역을 분석하고 hybrid 가중치 (AHP + Bayesian) + LLM·XAI 기반 explainability로 통합. 각 에이전트는 라틴어/그리스어 어원 명명: Structura(정형) · Cognita(관계) · Chronos(시계열) · Sentio(텍스트) · A…</t>
+          <t>PwC Korea가 SK하이닉스에 제안한 5-Agent agentic retention prediction 시스템. 5개 specialist 에이전트가 각기 다른 데이터 영역을 분석하고 hybrid 가중치 (AHP + Bayesian) + LLM·XAI 기반 explainability로 통합. 각 에이전트는 라틴어/그리스어 어원 명명: Structura(정형) · Cognita(관계) · Chronos(시계열) · Sentio(텍스트) · Agora(외부 시장). 결과는 3-tier 위험 등급 (Green/Yellow/Red) + 개인화 개입 권고. 2026-05 추진 계획, 실제 deployment·production metric 미공개.</t>
         </is>
       </c>
       <c r="F130" s="7" t="inlineStr">
@@ -21715,7 +21780,7 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="90" customHeight="1">
+    <row r="131" ht="140" customHeight="1">
       <c r="A131" s="7" t="n">
         <v>130</v>
       </c>
@@ -21736,7 +21801,7 @@
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>Syndio는 보상 공정성(pay equity) 전문 AI 플랫폼. 2025년 3월 Syndi라는 expert AI를 출시해 급여 보고 규제(EU Pay Transparency Directive·미국 주별 법률 등) 준수를 자동화. ⚠️ 벤더 주장: 300+ 고객, Fortune Most Admired 30%. "10페이지 법률 메모를 단일 actionable 답변으로" 대체한 사례 보고.</t>
+          <t>Syndio는 보상 공정성(pay equity) 전문 AI 플랫폼. 2025년 3월 Syndi라는 expert AI를 출시해 급여 보고 규제(EU Pay Transparency Directive·미국 주별 법률 등) 준수를 자동화. ⚠️ 벤더 주장: 300+ 고객, Fortune Most Admired 30%. "10페이지 법률 메모를 단일 actionable 답변으로" 대체한 사례 보고. EU AI Act 대응을 최전선에 내세운 벤더.</t>
         </is>
       </c>
       <c r="F131" s="7" t="inlineStr"/>
@@ -21859,7 +21924,7 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="90" customHeight="1">
+    <row r="132" ht="140" customHeight="1">
       <c r="A132" s="7" t="n">
         <v>131</v>
       </c>
@@ -22025,7 +22090,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="90" customHeight="1">
+    <row r="133" ht="140" customHeight="1">
       <c r="A133" s="7" t="n">
         <v>132</v>
       </c>

</xml_diff>

<commit_message>
fix(excel+html): Process Flow [Before] 제거 + 어색한 ':' 패턴 정리
사용자 피드백 2건:
1. Excel Process Flow에서 [Before] 제거 — Pain Point와 중복 (대부분 동일 내용)
2. 중간중간 ':' 어색한 패턴 점검·정리

수정 내용:
A) build_excel.build_process_flow:
   - Before 출력 부분 삭제 → After steps만 표시

B) extract_v3.extract_process (numbered step 결합 시):
   - bold + 본문 결합 시 본문 leading [—–-:：] 제거
   - 'Bold' + ': — body' → 'Bold: body' (이전: 'Bold: : body' 또는 'Bold:: body')

C) _remove_emdash_line (build_excel + build_html_v6 모두):
   - period·comma·) 직후 ' — '는 콜론 대신 공백 ('Co. — Galileo' → 'Co. Galileo')
   - '::' 또는 ': :' 패턴 자동 dedupe → ':'
   - '): :' → '): '

검증 (140 use cases):
- '::' 14 → 0
- ': :' 0 → 0
- '[Before]' 다수 → 0
- 'Co.:' 같은 period-then-colon 1 → 0
- ',:' comma-then-colon: 0

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/exports/hr-ai-usecase-collection.xlsx
+++ b/wiki/exports/hr-ai-usecase-collection.xlsx
@@ -1620,7 +1620,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="264" customHeight="1">
+    <row r="2" ht="216" customHeight="1">
       <c r="A2" s="8" t="n">
         <v>1</v>
       </c>
@@ -1641,8 +1641,8 @@
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>대한민국 고용노동부가 2024년 11월 시범 출시한 AI 노동법 상담 챗봇 (ai.moel.go.kr):
-노동자·사용자가 24/7 무료 노동법 상담.
+          <t>대한민국 고용노동부가 2024년 11월 시범 출시한 AI 노동법 상담 챗봇 (ai.moel.go.kr) 노동자·사용자가
+24/7 무료 노동법 상담.
 ✅ Fact:
 2025년 누적 117,000회 사용, 노동법 상담 시간 87.5% 단축 (정부 자체 측정), 야간·주말 사용 비중 37.7%, 32개 언어 지원 (외국인 노동자 대응).
 공인노무사회와 MOU 체결: 노동약자 보호 AI 혁신 협업.
@@ -1663,17 +1663,7 @@
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-한국 노동자·사용자가 노동법 (근로기준법·최저임금법·산업안전보건법·직장 내 괴롭힘 금지법 등) 관련 질문 시:
-(a) 고용노동부 콜센터 (1350, 평일 업무시간) (b) 공인노무사 유료 상담 (c) 인터넷 검색 (정확도 낮음) / Pain point:
-/ 시간·접근성 한계:
-콜센터 평일 업무시간만 → 야간·주말 근로자·외국인 노동자 접근 어려움 / 언어 장벽:
-외국인 노동자 (이주노동자 100만+)는 한국어 상담 어려움 / 유료 상담 부담:
-공인노무사 1건 30분 상담료 ~5만원 → 저소득 노동자 부담 / 노동법 복잡성:
-변수 다수 (근로계약 형태·근속·임금구조·교대제 등) → 자가 검색 정확도 낮음 / Trigger:
-윤석열 정부 노동약자 보호 정책 + GenAI 등장 + 32개 언어 LLM 가능성 +
-[After]
-1. 노동자·사용자가 ai.moel.go.kr 접속 (24/7, 무료, 32개 언어)
+          <t>1. 노동자·사용자가 ai.moel.go.kr 접속 (24/7, 무료, 32개 언어)
 2. 자연어 질문 입력 (예: "주 52시간 위반 신고는 어떻게?", "최저임금 미지급 시 대응 방법?")
 3. AI가 노동법 조문·판례·고시 기반 답변 생성 + 출처 인용
 4. 복잡 case는 공인노무사 추천 연계 (공인노무사회 MOU)
@@ -1779,8 +1769,9 @@
         <is>
           <t>• 한국 대기업 사내 ER/노무 AI 챗봇 도입 시 #1 reference:
 • "정부도 한다" 카드: CHRO·법무·노무팀 보수성 극복에 효과적
-• 정부 사례 정량 metric (117K 사용, 87.5% 단축, 37.7% 야간):
-한국 대기업 사내 챗봇 ROI 시뮬레이션 base
+• 정부 사례 정량 metric (117K 사용,
+87.5% 단축,
+37.7% 야간) 한국 대기업 사내 챗봇 ROI 시뮬레이션 base
 • vs HR Acuity hr-acuity-oliver-er-companion / Sodales
 sodales-spire-energy-labor-relations:</t>
         </is>
@@ -1799,7 +1790,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="280" customHeight="1">
+    <row r="3" ht="264" customHeight="1">
       <c r="A3" s="15" t="n">
         <v>2</v>
       </c>
@@ -1821,8 +1812,10 @@
       <c r="E3" s="16" t="inlineStr">
         <is>
           <t>HR Acuity는 미국 최대 ER 전용 case management 플랫폼.
-2024년 olivER™ AI Companion 출시 (2025년 본격화):
-ER 케이스의 intake → investigation → documentation → trend analysis 전 단계 자동화.
+2024년 olivER™ AI Companion 출시 (2025년 본격화) ER 케이스의 intake →
+investigation →
+documentation →
+trend analysis 전 단계 자동화.
 G2 Spring 2025 Enterprise HR Case Management 1위 + Fall 2025 Enterprise Investigation Management 1위,
 Brandon Hall Group 2025 Gold Award (Best Ethical AI &amp; Responsible Technology),
 Forrester TEI 520% ROI (벤더 commission),
@@ -1851,16 +1844,7 @@
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-미국 기업의 ER (employee relations) 처리는 ServiceNow·Jira 같은 범용 ticketing tool 또는 spreadsheet:
-case 분류·문서화 일관성 부재, audit trail 약함, 다국어 intake 한계 / Pain point:
-/ ER 전문성 부재 도구:
-일반 ticketing은 grievance·discipline·investigation 도메인 모름 → 변호사·노무사가 수작업 분류·요약 / Case 처리 시간:
-1건당 intake → investigation plan 작성 시간 over-burden / 익명 신고·다국어:
-글로벌 기업은 다국어 + 익명 hotline 필요.
-자체 구축 시 PII·legal hold 복잡 / 트렌드·hotspot 식별 어려움:
-[After]
-1. Case intake:
+          <t>1. Case intake:
 직원이 HR Acuity portal·Speakfully 익명 hotline·Workday Help integration으로 신고
 2. Investigation 지원:
 olivER가 case type 기반 AI 인터뷰 질문 자동 생성 (grievance·harassment·discipline 별 템플릿)
@@ -2009,7 +1993,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="184" customHeight="1">
+    <row r="4" ht="168" customHeight="1">
       <c r="A4" s="8" t="n">
         <v>3</v>
       </c>
@@ -2053,12 +2037,7 @@
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-230K 직원 대규모 finance enterprise, 정보보안·규제 제약으로 외부 LLM(ChatGPT) 직접 사용 불가 / Pain point:
-gen AI 효익 vs 금융정보보호·고객정보·내부거래 정보 제약 / Trigger:
-2023-24 ChatGPT 시장 도입 + 경쟁사(Goldman·Morgan Stanley) AI 배포 압박
-[After]
-1. 직원이 LLM Suite (private gateway) 접속
+          <t>1. 직원이 LLM Suite (private gateway) 접속
 2. 모델 선택 (OpenAI GPT-4 / Anthropic Claude: agnostic)
 3. 내부 데이터 활용 가능 (RAG with 회사 정책·문서)
 4. 사용 사례
@@ -2157,8 +2136,9 @@
       <c r="AK4" s="10" t="inlineStr">
         <is>
           <t>• KR 금융권 직격 reference (1순위):
-• KB·신한·우리·하나금융 모두 자체 LLM 플랫폼 구축 중 (신한 AI ONE, 하나 지식챗봇, 미래에셋 AI Assistant):
-JPMorgan LLM Suite의 model-agnostic gateway 아키텍처가 직접 reference
+• KB·신한·우리·하나금융 모두 자체 LLM 플랫폼 구축 중 (신한 AI ONE,
+하나 지식챗봇,
+미래에셋 AI Assistant) JPMorgan LLM Suite의 model-agnostic gateway 아키텍처가 직접 reference
 • 230K 직원 onboarding 8개월 모델:
 한국 대형 은행(KB 17K·신한 14K) 적용 시 6개월 미만 완료 가능성
 • AI 재배치 패러다임 (KR 핵심 어젠다):</t>
@@ -2182,7 +2162,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="216" customHeight="1">
+    <row r="5" ht="168" customHeight="1">
       <c r="A5" s="15" t="n">
         <v>4</v>
       </c>
@@ -2224,13 +2204,7 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-5만~10만 직원 KR 대기업 annual 조직문화 진단의 open-end 코멘트 코딩에 HRBP 팀 수주 투입:
-insight 도출 지연 / Pain point:
-글로벌 organization은 60+ 언어 응답 통합 분석 어려움 + theme·sentiment를 매니저별 actionable insight로 변환 어려움 / Trigger:
-Workday 2021-02 Peakon 인수 → 2024-12 Illuminate AI 통합 (Workday Illuminate 시리즈 일환)
-[After]
-1. 직원이 정기·수시 pulse 서베이 응답 (closed-end + open-end)
+          <t>1. 직원이 정기·수시 pulse 서베이 응답 (closed-end + open-end)
 2. Peakon Illuminate가 60+ 언어로 자연어 처리
 3. 자동 테마·sentiment·driver 추출 (1B+ 응답 학습 모델 기반)
 4. 매니저·HRBP에게 부서별 dashboard 제공: 강점·기회·이슈 자동 highlight
@@ -2359,7 +2333,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="216" customHeight="1">
+    <row r="6" ht="136" customHeight="1">
       <c r="A6" s="8" t="n">
         <v>5</v>
       </c>
@@ -2399,13 +2373,7 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-770K+ 글로벌 컨설팅 인력:
-직원 AI 역량 분포 편차 큰 / Pain point:
-컨설팅 비즈니스 자체가 AI를 사용·판매·구현해야 함 → 직원 AI literacy가 직접 매출 영향 / Trigger:
-ChatGPT 출시 직후 (2022-11) Sweet CEO가 즉각 mass reskilling 결단
-[After]
-1. 2022-11 시점 GenAI trained 직원 = 30명
+          <t>1. 2022-11 시점 GenAI trained 직원 = 30명
 2. mandatory GenAI fundamentals 모듈 전 직원 배포
 3. AI/data 전문 인력 채용·재배치 가속: 2023년 40K → 2025년 77K
 4. 매년 ~$1B L&amp;D 투자 (대부분 AI 비중)
@@ -2541,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="232" customHeight="1">
+    <row r="7" ht="184" customHeight="1">
       <c r="A7" s="15" t="n">
         <v>6</v>
       </c>
@@ -2583,14 +2551,7 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-ICT 직무·스킬 evolution 정량 데이터는 LinkedIn·Indeed·BLS 산발:
-글로벌 컨소시엄 합의 부재 / Pain point:
-HR·workforce planning 임원이 "AI가 우리 직무에 얼마나 영향을 주나"에 정량 답 부재 / Trigger:
-2024 multi-vendor 협업 출범:
-Cisco가 anchor
-[After]
-1. 6+ tech 대기업 협업 데이터 pooling
+          <t>1. 6+ tech 대기업 협업 데이터 pooling
 2. ICT 직무 mapping (BLS·O*NET 기반 + 회사 internal job architecture)
 3. AI 기술 스킬 포함 비율 측정 → 78% 결과
 4. fastest-growing ICT 직무 trend 분석 → top 10 중 7개 AI-related
@@ -2743,7 +2704,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="216" customHeight="1">
+    <row r="8" ht="200" customHeight="1">
       <c r="A8" s="8" t="n">
         <v>7</v>
       </c>
@@ -2784,12 +2745,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-270K 직원 IBM의 HR 운영 비용 baseline (CHRO LaMoreaux pre-AI era) / Pain point:
-HR 백오피스 transactional 업무가 budget 흡수, 전략 HR에 투자 여력 부족 / Trigger:
-AskHR·watsonx Orchestrate·cHaRlie·Predictive Attrition 누적 효과 (2018~2025) → 임계 도달
-[After]
-1. AskHR이 HR 정책 Q&amp;A·comp guidance·recognition·expense 80+ 태스크 자동 처리
+          <t>1. AskHR이 HR 정책 Q&amp;A·comp guidance·recognition·expense 80+ 태스크 자동 처리
 2. cHaRlie가 learning ops 백오피스 자율 처리
 3. Watson Recruitment·Predictive Attrition·watsonx Orchestrate TA Agent가
 채용·retention·comp 워크플로 자율화
@@ -2961,7 +2917,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="280" customHeight="1">
+    <row r="9" ht="216" customHeight="1">
       <c r="A9" s="15" t="n">
         <v>8</v>
       </c>
@@ -3008,17 +2964,7 @@
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-한국은 AI 거버넌스를 개인정보보호법(PIPA) 자동화된 결정 조항·차별금지법 등으로 산발 규율.
-HR AI 도입사도 자체 가이드라인에 의존 (ex.
-SK·삼성).
-/ Pain point: 채용 AI(마이다스 inAIR·SK AICT·원티드 AI Agent) 도입 가속화에도 불구하고 "이 AI가 합법인지",
-"지원자 권리는 어떻게 보장되는지",
-"차별 발생 시 책임은 누구인지" 가 회색 지대.
-/ Trigger:
-EU AI Act 발효(2024) + OECD AI 원칙 + 국내 마이다스 AI 면접 차별 논란(2020~) → 한국 정부가 2024년 입법 → 2025-01-21 공포 → 2026-01-22 시행.
-[After]
-1. AI 도입 전: 고영향 AI 분류 판정 (채용·인사평가·승진·해고 → 자동 분류)
+          <t>1. AI 도입 전: 고영향 AI 분류 판정 (채용·인사평가·승진·해고 → 자동 분류)
 2. 영향평가 (impact assessment): 차별·편향·정확도 등 사전 평가: 시행령 가이드라인 (2026 상반기 추가 고시 예정)
 3. 이용자 고지: 지원자·직원에게 "AI가 의사결정에 사용됨" 명시
 4. 인적 감독 (human oversight): 최종 결정에 사람의 검토·승인 단계 필수
@@ -3191,15 +3137,9 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-1.6M Walmart frontline 직원의 AI literacy baseline 매우 편차 큰 / Pain point:
-AI 도입 가속 vs frontline workforce 변화 압박:
-reskilling 없으면 mass 해고 사태 / Trigger:
-OpenAI Certification (2026 GA) launch 동시 vendor 파트너십 결단
-[After]
-1. Me@Walmart 디바이스 (Samsung Galaxy XCover Pro) 740K frontline 배포 →
+          <t>1. Me@Walmart 디바이스 (Samsung Galaxy XCover Pro) 740K frontline 배포 →
 학습 access 인프라
-2. OpenAI Certification 다층 모듈 (basics → prompt engineering): 무료 access
+2. OpenAI Certification 다층 모듈 (basics → prompt engineering) 무료 access
 3. ~50,000 직원이 AI/automation roles 재배치
 4. $1B 교육 commitment (2026까지)의 일부로 통합 운영</t>
         </is>
@@ -3208,8 +3148,8 @@
         <is>
           <t>• AI 시스템 배치: Walmart Academy (LMS 자체 운영) + OpenAI
 Academy 플랫폼 통합
-• 배포 환경: ChatGPT Enterprise rollout (Walmart 전사):
-Walmart-OpenAI 2025-10 partnership
+• 배포 환경: ChatGPT Enterprise rollout (Walmart
+전사) Walmart-OpenAI 2025-10 partnership
 • 연동·통합: Me@Walmart 앱 (frontline access 인프라,
 Walmart Global Tech 자체 빌드,
 2021 launch);
@@ -3249,10 +3189,10 @@
           <t>• Foundation model: OpenAI ChatGPT Enterprise (구체 GPT-4/4o/5 _미공개_);
 Google Gemini도 별도 인증 파트너 (multi-vendor,
 신규 발견)
-• 모델 유형: Generative LLM (ChatGPT Enterprise):
-직원 hands-on 사용
-• 제공 방식: 상용 API (OpenAI ChatGPT Enterprise, Google Gemini):
-multi-vendor
+• 모델 유형: Generative LLM (ChatGPT Enterprise) 직원
+hands-on 사용
+• 제공 방식: 상용 API (OpenAI ChatGPT Enterprise,
+Google Gemini) multi-vendor
 • 평가·가드레일: OpenAI Certifications (자체 평가 체계)</t>
         </is>
       </c>
@@ -3327,7 +3267,7 @@
       <c r="AK10" s="10" t="inlineStr">
         <is>
           <t>• KR retail/유통 frontline reskilling reference (1순위):
-• 이마트(이마트24·트레이더스 합산 ~10만)·롯데마트(~3만)·CJ대한통운(~2만)·쿠팡 fulfilment(~5만+):
+• 이마트(이마트24·트레이더스 합산 ~10만)·롯데마트(~3만)·CJ대한통운(~2만)·쿠팡 fulfilment(~5만+)
 모두 Walmart 모델 fit
 • 디바이스 + AI Certification + 배치 시나리오 통합 패키지
 • 벤더 파트너십 패턴:
@@ -3356,7 +3296,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="264" customHeight="1">
+    <row r="11" ht="184" customHeight="1">
       <c r="A11" s="15" t="n">
         <v>10</v>
       </c>
@@ -3388,9 +3328,9 @@
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>• Before:
-90%+ 기업이 여전히 Excel 기반 인력 계획 (Anaplan 조사):
-HR과 finance 시스템 단절, 시나리오 분석 수주~수개월 소요, 예측 오차 10%+
+          <t>• Before: 90%+ 기업이 여전히 Excel 기반 인력 계획 (Anaplan 조사) HR과 finance 시스템 단절,
+시나리오 분석 수주~수개월 소요,
+예측 오차 10%+
 • Pain point:
 "채용 동결·조직 개편·M&amp;A·인력 재배치 시나리오의 재무 영향이 즉시 분석 안 됨":
 CFO·CHRO 의사결정 지연
@@ -3401,15 +3341,7 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-90%+ 기업이 여전히 Excel 기반 인력 계획 (Anaplan 조사):
-HR과 finance 시스템 단절, 시나리오 분석 수주~수개월 소요, 예측 오차 10%+ / Pain point:
-"채용 동결·조직 개편·M&amp;A·인력 재배치 시나리오의 재무 영향이 즉시 분석 안 됨":
-CFO·CHRO 의사결정 지연 / Trigger:
-2025-12 Anaplan Role-Based AI Agents GA:
-HR·Finance·Sales·Supply Chain별 specialist agent 동시 launch
-[After]
-1. HCM (Workday/SAP) + ERP + finance 시스템을 Anaplan 플랫폼에 연동
+          <t>1. HCM (Workday/SAP) + ERP + finance 시스템을 Anaplan 플랫폼에 연동
 2. HR·CFO·CHRO가 자연어로 query (예:
 "지역별 이직률 추이는?", "보류 중인 채용 건은?", "headcount 5% 감축 시 인건비 영향?")
 3. AI agent가 실시간 데이터 분석 → 숨겨진 패턴·리스크 감지
@@ -3566,7 +3498,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="200" customHeight="1">
+    <row r="12" ht="136" customHeight="1">
       <c r="A12" s="8" t="n">
         <v>11</v>
       </c>
@@ -3606,14 +3538,7 @@
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-HR Q&amp;A 챗봇은 정보 조회까지만:
-"내 매니저에게 휴가 알리는 메시지 어떻게 쓰지" 같은 outbound 작업은 수동 / Pain point:
-HR 챗봇이 Q&amp;A에 머물러 ROI 한계:
-agentic 수준 도약 필요 / Trigger:
-Cisco의 "AI agents + nudges" 전사 bureaucracy 감소 이니셔티브 (Jeetu Patel 주도)
-[After]
-1. 직원이 AI Assistant에 "다음주 휴가 가능한지 + 매니저에게 알려줘" 한 번에 요청
+          <t>1. 직원이 AI Assistant에 "다음주 휴가 가능한지 + 매니저에게 알려줘" 한 번에 요청
 2. Assistant가 PTO 잔여 + 부서 calendar 조회
 3. 매니저용 time-off notification 메시지 자동 작성 (직원 검토·전송)
 4. HR 정책 위배 시 alert + 사람 escalation</t>
@@ -3626,7 +3551,7 @@
 • 연동·통합: HR tools (PTO 입력,
 401k 조회 등) 통합;
 구체 시스템명 _미공개_
-• 인증·권한: "purpose-built with security" (벤더 주장):
+• 인증·권한: "purpose-built with security" (벤더 주장)
 구체 모델 _미공개_</t>
         </is>
       </c>
@@ -3728,9 +3653,8 @@
           <t>• KR Ask-HR RFP의 mature reference (1순위):
 • 한국 대기업 사내 챗봇은 대부분 Q&amp;A 단계 (LG CNS·삼성SDS·SK C&amp;C·신한 AI ONE·하나 지식챗봇)
 • Cisco의 "Q&amp;A → drafting + action" agentic 진화는 KR 차세대 챗봇 RFP의 standard
-• 2026 Q3-Q4 KR 컨설팅 deck:
-Moderna Ask HR (routing) + IBM AskHR (80+ 태스크) + Cisco AI Assistant (agentic outbound):
-3-tier maturity ladder</t>
+• 2026 Q3-Q4 KR 컨설팅 deck: Moderna Ask HR (routing) + IBM AskHR (80+
+태스크) + Cisco AI Assistant (agentic outbound) 3-tier maturity ladder</t>
         </is>
       </c>
       <c r="AL12" s="10" t="inlineStr">
@@ -3772,8 +3696,9 @@
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>IBM이 2023년 launch한 cHaRlie (Cognitive HR Learning EM Assistant):
-Enterprise Learning Operations &amp; Administration 팀을 위한 watsonx Orchestrate 기반 백오피스 에이전트.
+          <t>IBM이 2023년 launch한 cHaRlie (Cognitive HR Learning EM Assistant)
+Enterprise Learning Operations &amp; Administration 팀을 위한 watsonx
+Orchestrate 기반 백오피스 에이전트.
 학습 enrollment 모니터링·저조 alert·event 홍보·pre-event comms·virtual class 출석
 자동 로깅.
 ⚠️ 자사 보고:
@@ -3793,13 +3718,7 @@
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-L&amp;D operations 팀이 enrollment 추적·홍보·출석 캡처·event 운영을 manual로 처리:
-270K 직원 규모에서 병목 / Pain point:
-직원 facing AI(tutor·content)는 ROI 모호, 학습 ops 백오피스는 ROI 명확하지만 자동화 후순위 / Trigger:
-watsonx Orchestrate dogfooding + L&amp;D 운영 효율 압박
-[After]
-1. cHaRlie가 enrollment 모니터링 → 저조 시 admin alert
+          <t>1. cHaRlie가 enrollment 모니터링 → 저조 시 admin alert
 2. event 홍보 메시지 자동 생성·배포
 3. virtual class 출석 자동 캡처 (100% 정확도)
 4. pre-event comms 자동 발송
@@ -4006,13 +3925,7 @@
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-230K 직원 중 AI literacy 분포 편차 큰:
-데이터 사이언티스트는 풍부, 운영·영업·고객서비스 직원은 baseline / Pain point:
-회사 LLM Suite를 도입해도 사용 모르면 ROI 없음 / Trigger:
-LLM Suite launch 동시 추진 (2024-08)
-[After]
-1. 전 직원 baseline AI fundamentals 모듈 의무
+          <t>1. 전 직원 baseline AI fundamentals 모듈 의무
 2. Prompt engineering 모듈 (LLM Suite 활용 직군 의무)
 3. 컴플라이언스 모듈 (금융정보·고객정보 처리 가이드)
 4. 직무별 use case curriculum (analyst·trader·banker·HR·legal·ops 별)
@@ -4207,13 +4120,7 @@
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-한국·글로벌 대기업 모두 직원 self-update profile에 의존:
-outdated·incomplete / Pain point:
-스킬 inventory 부정확하면 internal mobility·workforce planning·learning 추천 모두 약화 / Trigger:
-Microsoft가 M365 Copilot 위에 People Skills 출시 (2025-04, Bersin "HR tech market 변경"으로 평가)
-[After]
-1. M365 Copilot이 일상 활동 (이메일·문서·미팅) 텔레메트리 수집
+          <t>1. M365 Copilot이 일상 활동 (이메일·문서·미팅) 텔레메트리 수집
 2. OpenAI 모델로 LinkedIn 16K taxonomy 매핑 → 추론 스킬 프로파일 자동 생성
 3. 직원 검토·승인 (HITL: 추론 결과 거부·수정 가능)
 4. 매니저 Skills Agent 활용: "이 프로젝트에 맞는 사내 talent" search
@@ -4383,7 +4290,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="232" customHeight="1">
+    <row r="16" ht="216" customHeight="1">
       <c r="A16" s="8" t="n">
         <v>15</v>
       </c>
@@ -4428,15 +4335,7 @@
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Moderna는 5,000명 규모의 바이오텍이지만 급성장기 동안 HR 인력만으로 늘어나는 직원 문의를 처리하기 어려워짐.
-❓ 구체 before 수치(월간 HR 티켓 수·평균 응답 시간·HR 인력 대비 직원 비율) 미공개:
-이 baseline 부재가 이 use case의 최대 약점 / Franklin의 프레이밍:
-기존의 "workforce planning"(HR 독립)과 "technology planning"(IT 독립)이 "work의 흐름 자체를 설계"하지 못했다.
-개별 HR 프로세스 개선이 아니라 업무·정보·의사결정 흐름 전체 재설계가 목적:
-/ 기술적으로는, 전사 ChatGPT Enterprise 위에 각 부서가 GPT를 남발할 경우 HR 도메인 질문이 품질 낮은 일반 GPT로 향할 위험 → HR
-[After]
-1. 직원이 "Ask HR" 중앙 GPT에 자연어 질문 입력
+          <t>1. 직원이 "Ask HR" 중앙 GPT에 자연어 질문 입력
 2. Ask HR GPT가 질문 도메인 분류: performance, career, benefits 등
 3. 해당 영역의 specialized GPT로 routing
 4. Specialized GPT가 답변 제공
@@ -4620,18 +4519,7 @@
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-사내 익명 신고는 (a) 외부 hotline 위탁 (NAVEX·Convercent 등) (b) 자체 portal:
-case management는 별도 도구.
-AI 분석·precedent 검색은 사람이 수작업 / Pain point:
-/ 익명 신고 → ER case 단절:
-hotline은 신고만 받고, ER team이 별도 시스템에 옮겨 처리 → 정보 분산 / 다국어 지원 한계:
-글로벌 기업의 200+ 언어 신고 자동 번역 없으면 처리 지연 / 유사사례 (precedent) 검색:
-과거 case 검색 수작업 → 일관성 결여 + investigation 시간 over-burden / AI 안전성:
-ER 데이터는 PII + legal hold + GDPR 영역 → 일반 LLM 사용 불가 / Trigger:
-Ge
-[After]
-1. 직원이 AllVoices portal·Slack·Teams·이메일 익명 신고 (200+ 언어 자동 인식)
+          <t>1. 직원이 AllVoices portal·Slack·Teams·이메일 익명 신고 (200+ 언어 자동 인식)
 2. Intake: Vera가 신고 내용 구조화 + 유사 precedent 자동 검색 표면화
 3. Investigation 지원: 인터뷰 질문 자동 생성 + 메시지 초안 작성 + case timeline 자동 작성
 4. Insight: 부서·매니저별 trend·hotspot dashboard + 위험 신호 alert
@@ -4816,12 +4704,7 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-annual·biannual 서베이로는 1.5M frontline 직원의 daily 변화 포착 불가 / Pain point:
-high-turnover frontline (creator·warehouse·delivery)의 sentiment·attrition 신호를 연 1~2회로 잡으면 늦음 / Trigger:
-People Science 데이터 사이언스 팀의 high-frequency listening 실험
-[After]
-1. 직원 로그인 시 1개 질문 자동 출현 (5초 답변)
+          <t>1. 직원 로그인 시 1개 질문 자동 출현 (5초 답변)
 2. 응답 + non-response 모두 데이터로 수집
 3. ML 모델이 행동(non-response trend)·태도(응답 sentiment) 변화 추적
 4. attrition·engagement 이벤트 사전 예측
@@ -4971,7 +4854,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="312" customHeight="1">
+    <row r="19" ht="248" customHeight="1">
       <c r="A19" s="15" t="n">
         <v>18</v>
       </c>
@@ -5019,17 +4902,7 @@
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-미국 employer의 OE(연 1회 plan 선택)는 직원 stress 최고점:
-정책 복잡(의료·치과·생명·FSA·HSA·HDHP), 문서 검증(QLE:
-qualifying life event:
-결혼·출산·이혼시 plan 변경)·승인 워크플로 수작업 / Pain point:
-HR/벤처사 콜센터에 OE 시즌 콜 급증, 직원당 평균 통화 시간 길고 같은 질문 반복, document 검증은 사람 reviewer가 1건씩 처리 / Trigger:
-GenAI 등장으로 chat·문서 처리 자동화 가능.
-Businessolver 1998년 설립 이후 축적된 25년+ 도메인 데이터 + Sofia AI 엔진을 agentic으로 재구성 / 비교 reference:
-는 single-tenant Custom GPT, Sof
-[After]
-1. 직원이 chat·portal·전화로 문의
+          <t>1. 직원이 chat·portal·전화로 문의
 2. Answer Agent:
 자연어 질문 (의료 plan 비교·HSA 적격성·deductible 계산 등) 즉시 답변: 세션 내 multi-turn
 3. 직원이 QLE 증빙 (출생증명서·결혼증명서·이혼판결문 등) 업로드
@@ -5155,8 +5028,7 @@
 Moderna는 단일 GPT (Custom GPT × 2종), Sofia는 specialist agent 멀티.
 SaaS 벤더와 self-build의 차이
 • Vs Nayya nayya-benefits-decision-support:
-Nayya는 decision support (어느 plan을 선택할지 추천), Sofia는 operations (선택 후 admin·문서 처리·Q&amp;A):
-보완적 포지션
+Nayya는 decision support (어느 plan을 선택할지 추천), Sofia는 operations (선택 후 admin·문서 처리·Q&amp;A) 보완적 포지션
 • 한국 적용: 복지포인트 관리·flex benefit·연말정산 자료 검증 등 한국 EX·HR운영 도메인에 3-agent pattern 적용 가능 (Intake = 증빙 OCR/검증,
 Answer = 정책 Q&amp;A,
 Insights = 사용 패턴)</t>
@@ -5221,14 +5093,7 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-컨설팅사가 HR AI 컨설팅을 "case-by-case" 진행:
-표준화·재사용 자산 부족 / Pain point:
-HR transformation 프로젝트마다 workflow 재설계 압도적:
-300+ workflow library가 필요 / Trigger:
-agentic AI 부상 + Big-4 컨설팅 경쟁 압박 (PwC·KPMG·EY 동반 발표)
-[After]
-1. Zora AI 플랫폼이 ready-to-deploy agents 제공 (HR 포함 6 영역)
+          <t>1. Zora AI 플랫폼이 ready-to-deploy agents 제공 (HR 포함 6 영역)
 2. Workforce Analyzer가 클라이언트 workforce 세그먼트별 AI 영향평가
 3. Workforce Planner+가 시나리오 기반 인력 재배치 계획
 4. 300+ HR workflow library에서 use case 매칭
@@ -5242,7 +5107,7 @@
 pre-built integrations로 "deploy
 rapidly on existing technologies"
 • 배포 환경: NVIDIA AI Enterprise stack (cloud-agnostic);
-Oracle 파트너십 (별도 발표): 구체 hyperscaler 선택은 클라이언트 옵션
+Oracle 파트너십 (별도 발표) 구체 hyperscaler 선택은 클라이언트 옵션
 • 연동·통합: Pre-built integrations;
 구체 connector 목록 _미공개_;
 Oracle Fusion Cloud Apps 통합 (Deloitte-Oracle 파트너십)
@@ -5274,7 +5139,7 @@
           <t>• Foundation model: NVIDIA Llama Nemotron (reasoning
 models)
 • 모델 유형: Agentic LLM (reasoning + generative +
-predictive): finance·human
+predictive) finance·human
 capital·supply
 chain·procurement·sales·customer
 service agents
@@ -5389,7 +5254,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="312" customHeight="1">
+    <row r="21" ht="280" customHeight="1">
       <c r="A21" s="15" t="n">
         <v>20</v>
       </c>
@@ -5436,18 +5301,7 @@
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-사내 윤리·컴플라이언스 신고는 hotline (NAVEX·Convercent) 또는 자체 portal:
-익명 신고 단발 처리, 패턴 분석·예측 기능 부족, 글로벌 GRC 통합 부재 / Pain point:
-/ 익명 신고 단발 처리:
-1건씩 처리 → 패턴·systemic risk 식별 어려움 / EU Whistleblower Directive (2023~):
-EU 50인+ 기업 의무:
-신고 mechanism 구축 + 조치 timeline 의무 / 집단 신고 mechanism 부재:
-1인 신고는 retaliation risk → 다수 직원이 함께 신고하는 mechanism 필요 / GRC 통합:
-ESG·board governance·내부감사와 연결 안 됨 → C-suite 가시성 부족 / Trigger:
-D
-[After]
-1. 직원이 Vault portal·VaultTalk·GoTogether 익명 신고 (1인 또는 집단)
+          <t>1. 직원이 Vault portal·VaultTalk·GoTogether 익명 신고 (1인 또는 집단)
 2. EthicsChat AI: 신고 전 AI 자문: "이게 신고 대상인가?", "어떤 채널?", "어떤 증거?" 가이드
 3. AI pattern recognition:
 신고 내용 분석 + 과거 case·부서·매니저 패턴 결합 → misconduct predictive risk score
@@ -5626,13 +5480,7 @@
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-IBM 내부 이동은 직원 본인 search에 의존 → silo·visibility 격차로 매칭 비효율 / Pain point:
-280K 글로벌 조직에서 internal posting 게시판은 잘 작동 안 함:
-직원이 본인 옆 부서 외 기회를 모름 / Trigger:
-핵심 인재 retention 위기 + 외부 talent marketplace 시장 형성 (Gloat·Eightfold) 전 자체 구축
-[After]
-1. 직원이 opt-in (~15% 참여)
+          <t>1. 직원이 opt-in (~15% 참여)
 2. AI가 스킬·경력·성과·근무지·digital footprint 분석 → 개인 프로파일 생성
 3. 신규 internal posting 발생 시 매칭 직원에게 personalized 추천
 4. peer 이동 패턴 학습 (A→B 5건 누적 시 유사 프로파일에 동일 추천)
@@ -5794,7 +5642,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="232" customHeight="1">
+    <row r="23" ht="184" customHeight="1">
       <c r="A23" s="15" t="n">
         <v>22</v>
       </c>
@@ -5836,15 +5684,7 @@
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-KB국민은행 영업점 직원 인사이동은 매년 manual 조정:
-수천 직원 개인 사정 (출퇴근·육아·자격) 종합 어려움 / Pain point:
-17,000+ KB 직원 base, 영업점 1,000+ 곳:
-manual 인사 운영 한계 + 직원 만족도 격차 / Trigger:
-2020 'HR Deep Change' 프로젝트 launch:
-공공·금융권 최초 large-scale AI 인사 배치
-[After]
-1. 직원 master data + 영업점 수요 + 정성 데이터 (출퇴근·자격증·육아 고충 등) 입력
+          <t>1. 직원 master data + 영업점 수요 + 정성 데이터 (출퇴근·자격증·육아 고충 등) 입력
 2. ML 알고리즘이 다변량 최적화: 수십 변수 simultaneous
 3. 후보 배치안 생성 → HR 검토·조정
 4. 매니저·직원 통보
@@ -5942,7 +5782,7 @@
         <is>
           <t>• KR 대기업 인사이동 AI reference (1순위):
 • 한국에서 가장 잘 문서화된 large-scale 인사이동 AI 사례
-• 5년+ 운영 (2020~2025): stability proof
+• 5년+ 운영 (2020~2025) stability proof
 • 2025 PB·RM 확장 + 57% 두 달 사용은 adoption 성공 정량 증거</t>
         </is>
       </c>
@@ -6022,16 +5862,7 @@
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Mastercard는 2019년부터 "Project Possible"이라는 수동 internal gig 프로그램 운영: HR이
-spreadsheet로 직원 ↔ gig 매칭, scale 한계 / Pain point: / 30,000+ global 직원의 스킬
-inventory invisible: 어느 부서에 어떤 스킬을 가진 직원이 있는지 매니저도 모름 / 직원이 internal
-mobility 경로 모름 → external offer로 이탈 / cross-functional·cross-regional
-collaboration 기회 손실 / Trigger: Project Possible의 success → AI 자동 매칭으로 scale
-up 결정.
-Gloat 도입 (2022)
-[After]
-1. 직원 onboarding: 자기 스킬·관심사·career goal 입력 (또는 LinkedIn/자체 데이터에서 자동 추출)
+          <t>1. 직원 onboarding: 자기 스킬·관심사·career goal 입력 (또는 LinkedIn/자체 데이터에서 자동 추출)
 2. 매니저가 internal job/gig/project/mentor 요청: 등록 (필요 스킬·기간·시간 commitment)
 3. AI 매칭 엔진: 직원 ↔ opportunity 자동 추천 (스킬 fit·career fit·가용성)
 4. 직원이 관심 표시 → 매니저 검토 → 24h 내 인터뷰 스케줄 (벤더 발표 평균)
@@ -6169,7 +6000,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="328" customHeight="1">
+    <row r="25" ht="248" customHeight="1">
       <c r="A25" s="15" t="n">
         <v>24</v>
       </c>
@@ -6216,17 +6047,7 @@
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-NAVEX EthicsPoint은 1990년대부터 hotline service의 사실상 표준:
-2024년까지는 신고 intake·case 분류는 사람이 처리, AI 분석·자동 번역 부분적 / Pain point:
-/ 다국어 신고 처리 시간:
-글로벌 enterprise 30+ 언어 신고 → 사람 번역사 처리 시간 over-burden / Case 분류·라우팅 지연:
-1건씩 사람이 분류 → 우선순위 case 누락 risk / 컴플라이언스 training content 노화:
-정책 변경 시 training material 갱신 수작업 / 대화형 자문 부재:
-컴플라이언스 담당자가 정책 question 시 검색 수작업 / Trigger:
-GenAI 시대 + HR Acuity·AllVoices·Vault 등 AI-n
-[After]
-1. 직원이 EthicsPoint hotline (전화·web·SMS) 익명 신고: 30+ 언어
+          <t>1. 직원이 EthicsPoint hotline (전화·web·SMS) 익명 신고: 30+ 언어
 2. AI 자동 번역 → 영어·통합 언어로 normalize
 3. AI classification:
 case type (harassment·fraud·SOX·safety) + severity + urgency 자동 분류
@@ -6240,7 +6061,7 @@
       <c r="H25" s="16" t="inlineStr">
         <is>
           <t>• AI 시스템 배치: NCA (Compliance Assistant) +
-EthicsPoint AI (intake·routing): 모두
+EthicsPoint AI (intake·routing) 모두
 platform 내장
 • 사용자 접점: hotline 전화·web·mobile·SMS·이메일 (다국어),
 컴플라이언스 담당자 dashboard</t>
@@ -6376,7 +6197,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="216" customHeight="1">
+    <row r="26" ht="120" customHeight="1">
       <c r="A26" s="8" t="n">
         <v>25</v>
       </c>
@@ -6406,12 +6227,7 @@
       <c r="F26" s="10" t="inlineStr"/>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-130k+ 직원 스킬 보유 현황은 자가 신고·이력서 기반 단편적이며,
-매니저는 후보자 스킬을 일일이 확인해 internal mobility 후보 search.
-스킬 갭 진단은 부서별 수기·연 1회 수준 /
-[After]
-1. HR이 41개 future-ready skills · 11개 capability를 정의해 taxonomy 등록
+          <t>1. HR이 41개 future-ready skills · 11개 capability를 정의해 taxonomy 등록
 2. LLM(skills inference)이 직원 프로필·learning 이력·과제 이력을 읽어 skill별 0~5 proficiency
 자동 산출 (60~70% 추론)
 3. MySkills 플랫폼이 직원에게 본인 스킬 그래프·갭·추천 학습/이동 기회 제시
@@ -6577,10 +6393,7 @@
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개_ (Chipotle의 이전 채용 플로우 세부) /
-[After]
-1. 지원자가 Chipotle 채용 채널에서 "Ava Cado" 와 대화 시작 (multilingual chat: 영·스·불·독)
+          <t>1. 지원자가 Chipotle 채용 채널에서 "Ava Cado" 와 대화 시작 (multilingual chat: 영·스·불·독)
 2. Ava Cado가 Candidate screening + applicant 정보 수집
 3. Ava Cado가 인터뷰 스케줄링 (매장 매니저와 연동)
 4. 매장 General Manager가 인터뷰 진행 + 채용 결정
@@ -6763,10 +6576,7 @@
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-전통적 IT 지원 프로세스, 수동 데이터 분석, 역량 개발 개인 주도. /
-[After]
-1. Fact ChatGPT Enterprise: 50,000명 배포로 AI 역량 구축.
+          <t>1. Fact ChatGPT Enterprise: 50,000명 배포로 AI 역량 구축.
 2. Fact Microsoft 365 Copilot: 17,500명 배포.
 84%의 10,000명 사용자가 "Copilot 없이 돌아가기 싫다"고 응답.
 3. Fact ChatIT: Microsoft Teams 기반 AI IT 지원 어시스턴트 (Azure + Copilot Studio
@@ -6938,8 +6748,7 @@
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>[After]
-1. 9,000명 임원 서베이 89개국
+          <t>1. 9,000명 임원 서베이 89개국
 2. 3축 긴장 분석
 3. Workforce: 사람+에이전트
 4. Workplace: 물리+디지털
@@ -7094,18 +6903,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Hitachi는 다수의 사업부(BU)와 다국가 운영 환경에서 HR 정책·복리후생·시스템이 BU·국가별로 상이.
-직원이 자기에게 맞는 정책을 찾으려면 어느 문서를, 어떤 버전으로, 어느 부서에 물어야 하는지 파악이 어려움.
-❓ 구체 수치(월간 HR 문의 건수·평균 해결 시간) 미공개 / Pain point:
-(1) 정책 탐색의 복잡성:
-BU·국가·역할별로 적용되는 정책이 다르기 때문에 "하나의 답"이 없음 → 직원 불만·프로세스 지연.
-(2) HR 팀에 반복 문의 집중:
-같은 유형의 질문(복리후생·휴가·IT 요청)이 반복적으로 HR에 유입 → HR의 전략적 업무 시간 잠식 / Trigger:
-Hitachi가 "문화 설계" 관점에서 AI를 도입하기로 결정:
-단순 챗봇이 아니라 이름(Skye)과 개성을 부여
-[After]
-1. Fact Skye가 정책 문서를 추론하여 사업부·국가·역할에 맞게 개인화된 응답 제공.
+          <t>1. Fact Skye가 정책 문서를 추론하여 사업부·국가·역할에 맞게 개인화된 응답 제공.
 2. Fact IT 서비스 티켓 생성, 휴가 요청 처리 등 지능적 액션 수행.
 3. Fact 채용·온보딩·리텐션 영역의 유스케이스 개발 진행 중.</t>
         </is>
@@ -7284,15 +7082,7 @@
       </c>
       <c r="G31" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-IBM 글로벌 280K 직원 분기 승진 cycle은 HR Business Partner 수작업 spreadsheet: 부서별
-eligible employees 식별·매니저별 promotion criteria 안내·결정 후
-compensation/title/org 시스템 수동 갱신 / Pain point: / 분기당 10주 소요: HRBP 시간의 상당 비중
-/ 매니저 10,000명 × 부서·지역 별 승진 정책 차이 → 일관성 결여, 매니저 confusion / 승진 결정 후
-compensation·org chart·title 갱신을 여러 시스템에 수동 입력 / Trigger: IBM 자체 AI/agentic
-transformation (AskHR 6년 운영 후 specialist agent 확장 단계)
-[After]
-1. HiRo가 분기 시작 시 자동으로 HR 시스템들 (HRMS·평가·comp)에서 eligible employees 데이터 통합
+          <t>1. HiRo가 분기 시작 시 자동으로 HR 시스템들 (HRMS·평가·comp)에서 eligible employees 데이터 통합
 2. 매니저별·부서별 promotion criteria 맞춤 작성 (LLM 기반)
 3. 10,000명 매니저에게 자동 발송 + 매니저용 simplified UI (criteria + eligible list + 승진 추천
 데이터)
@@ -7317,8 +7107,8 @@
       </c>
       <c r="K31" s="16" t="inlineStr">
         <is>
-          <t>• Foundation model: IBM watsonx (Granite 모델 자체 제품):
-구체 model variant·버전 _부분 미공개_</t>
+          <t>• Foundation model: IBM watsonx (Granite 모델 자체 제품) 구체
+model variant·버전 _부분 미공개_</t>
         </is>
       </c>
       <c r="L31" s="16" t="inlineStr">
@@ -7477,10 +7267,7 @@
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-직원이 개별적으로 외부 AI 도구 또는 전통적 검색·작성 도구를 사용. 성과 리뷰는 관리자가 수동으로 직접 작성. /
-[After]
-1. 직원 요청 문서 요약·이메일·리뷰 초안 등
+          <t>1. 직원 요청 문서 요약·이메일·리뷰 초안 등
 2. LLM Suite 내부 보안 포털
 3. AI 응답 생성
 4. 직원 검토·편집
@@ -7673,8 +7460,8 @@
 • Pain point:
 • 매니저 시간 over-burden:
 매장 매니저가 주 8~15시간을 스케줄 작성·조정에 사용 → 매장 운영·고객 서비스 시간 감소
-• 시급직 turnover 60~150%/년 (US retail 평균):
-schedule 불만이 turnover 1대 사유
+• 시급직 turnover 60~150%/년 (US retail 평균) schedule 불만이
+turnover 1대 사유
 • labor cost over/under:
 수요 예측 없으면 trafic 낮은 시간대에도 인력 배치 → 비용 over-spend
 • Trigger: 미국 retail의 hourly worker 부족 + Schedule
@@ -7684,16 +7471,7 @@
       </c>
       <c r="G33" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-시급직 매니저가 매주 spreadsheet로 직원 shift 작성:
-수요 예측 부재, 노동 시간 over/under, 결근 1회당 대체 인력 찾기 30~60분 소요 / Pain point:
-/ 매니저 시간 over-burden:
-매장 매니저가 주 8~15시간을 스케줄 작성·조정에 사용 → 매장 운영·고객 서비스 시간 감소 / 시급직 turnover 60~150%/년 (US retail 평균):
-schedule 불만이 turnover 1대 사유 / labor cost over/under:
-수요 예측 없으면 trafic 낮은 시간대에도 인력 배치 → 비용 over-spend / Trigger:
-미국 retail의 hourly worker 부족 + Schedule Fairness 법규 강화 (NYC·SF·Se
-[After]
-1. 수요 예측:
+          <t>1. 수요 예측:
 POS·트래픽·날씨·이벤트 데이터 → AI가 시간대별 labor demand 예측 (95% accuracy: Forrester study에서 검증)
 2. 자동 스케줄 생성: demand × 직원 가용성·skill·preferences·labor law 제약 → 매장별 shift 최적화
 3. 직원 모바일: shift 확인·교체·gig swap·휴가 신청 self-service
@@ -7838,7 +7616,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="216" customHeight="1">
+    <row r="34" ht="184" customHeight="1">
       <c r="A34" s="8" t="n">
         <v>33</v>
       </c>
@@ -7881,14 +7659,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-LG 그룹 5만+ 임직원이 사내 정책·프로젝트 자료 검색을 sharepoint·이메일·시니어 문의로 처리:
-정보 fragmented / Pain point:
-글로벌 commercial LLM (ChatGPT·Claude) 사용은 데이터 주권·보안 이슈로 제약.
-한국어·LG 도메인 fit 부족 / Trigger:
-LG AI연구원이 EXAONE 자체 LLM 개발 → 그룹 dogfooding 명분 → 1년 베타(2024-08~2025) 후 production 정식 launch
-[After]
-1. 직원이 ChatEXAONE web/모바일 access (그룹 SSO)
+          <t>1. 직원이 ChatEXAONE web/모바일 access (그룹 SSO)
 2. 자연어로 query: 사내 규정·프로젝트 자료·기술 문서 등
 3. EXAONE이 multi-format 이해 (PPTX·PDF·CSV·도표·수식)
 4. 응답 + 출처 표시; SQL 생성·22개 언어 코드 지원
@@ -7897,11 +7668,10 @@
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>• Core HRIS: 각 LG 계열사 HRIS (Workday·SAP 혼재):
-별도, ChatEXAONE은 horizontal 플랫폼
+          <t>• Core HRIS: 각 LG 계열사 HRIS (Workday·SAP 혼재) 별도,
+ChatEXAONE은 horizontal 플랫폼
 • AI 시스템 배치: LG AI연구원이 운영, 계열사에 share
-• 배포 환경: LG cloud / on-prem (보안 민감 영역):
-구체 _미공개_
+• 배포 환경: LG cloud / on-prem (보안 민감 영역) 구체 _미공개_
 • 연동·통합: 그룹 SSO + 사내 문서 RAG 코퍼스
 • 사용자 접점: Web + 모바일 + IDE plugin (코드 지원)
 • 인증·권한: LG 그룹 SSO</t>
@@ -8031,7 +7801,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="200" customHeight="1">
+    <row r="35" ht="168" customHeight="1">
       <c r="A35" s="15" t="n">
         <v>34</v>
       </c>
@@ -8075,13 +7845,7 @@
       </c>
       <c r="G35" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-기업 LMS·LXP의 AI coaching은 generic feedback 위주.
-1:1 코칭은 임원 한정 (비용 ~$200~500/h) / Pain point:
-중간 관리자·일반 직원 soft skill (어려운 대화·feedback·negotiation) 학습 기회 부족 → role-play 환경 부재 / Trigger:
-2024 LinkedIn Learning AI Coaching launch → 2025 Microsoft Copilot 통합 가속
-[After]
-1. 학습자가 LinkedIn Learning Premium·Enterprise tier 구독
+          <t>1. 학습자가 LinkedIn Learning Premium·Enterprise tier 구독
 2. 강의 중 AI Coach와 대화형 Q&amp;A·요약·심화 질문 가능
 3. 2025 확장: role-play scenario: feedback 대화·면접·negotiation을 AI character와 모의
 4. AI가 응답 평가·improvement 제안
@@ -8187,8 +7951,8 @@
       <c r="AK35" s="16" t="inlineStr">
         <is>
           <t>• KR L&amp;D 컨설팅 reference:
-• LinkedIn Premium·Enterprise 기존 도입 KR 대기업 (대부분 매출 1조+):
-AI Coaching 추가 활성화 즉시 가능
+• LinkedIn Premium·Enterprise 기존 도입 KR 대기업 (대부분 매출 1조+) AI Coaching 추가
+활성화 즉시 가능
 • Microsoft 365 도입사와 cross-sell:
 Microsoft People Skills microsoft-people-skills-inferred-ontology 통합
 • Soft skill 학습 카테고리 reference:</t>
@@ -8248,10 +8012,7 @@
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-HR 정책 관련 문의를 HR 팀이 직접 처리. 스킬 데이터는 사일로화. /
-[After]
-1. Fact Workday HCM을 단일 HR 시스템으로 운영 (2018년 이후).
+          <t>1. Fact Workday HCM을 단일 HR 시스템으로 운영 (2018년 이후).
 2. Fact Workday Skills Cloud로 스킬 데이터 통합 관리 (2020년 이후).
 3. Fact GenAI 파일럿: 고볼륨 정책(휴가, 복리후생 옵션 등) Q&amp;A를 AI가 처리.
 300명 파일럿 중 12–15%의 정책 문의를 GenAI가 응답.</t>
@@ -8415,14 +8176,11 @@
       </c>
       <c r="G37" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-인력의 67% 코어 직원, 8% 내부 유연 인력, 25% 계약직(Agency). /
-[After]
-1. Fact AI 기반 유연 스케줄링으로 내부 유연 인력(Float Pool·Gig Nurses) 확대:
+          <t>1. Fact AI 기반 유연 스케줄링으로 내부 유연 인력(Float Pool·Gig Nurses) 확대:
 코어 69%, 유연+기그 23%, 계약직 8%로 재편.
 2. Fact "Win From Within" 프로그램 20개 병원으로 확대: 예비 간호사에게 학비 지원·파트타임 역할 제공,
 2026년 봄 340명+ 등록.
-3. Fact Microsoft·Epic 협력으로 Dragon Copilot AI 문서화 도구 도입 (2025년 2월 파일럿): 문서
+3. Fact Microsoft·Epic 협력으로 Dragon Copilot AI 문서화 도구 도입 (2025년 2월 파일럿) 문서
 정확도 30%→90% 향상.</t>
         </is>
       </c>
@@ -8565,7 +8323,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="232" customHeight="1">
+    <row r="38" ht="200" customHeight="1">
       <c r="A38" s="8" t="n">
         <v>37</v>
       </c>
@@ -8607,14 +8365,7 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-5만~10만 직원 KR 대기업 annual 서베이 open-end 코멘트 코딩에 HRBP 팀이 수주 투입 / Pain point:
-open-end NLP 분석은 sentiment·테마 추출에 manual 작업 압도적:
-insight 도출 지연 / Trigger:
-Glint Copilot 통합:
-Microsoft가 LinkedIn(Glint owner)을 M365 ecosystem 통합
-[After]
-1. 서베이 데이터 → Glint Copilot 자동 처리
+          <t>1. 서베이 데이터 → Glint Copilot 자동 처리
 2. 반복 테마 탐지 + sentiment slice (속성별: 부서·재임기간·매니저 등)
 3. benchmark 비교 (산업·규모)
 4. Team/Executive 요약 리포트에 "Copilot Highlights" 자동 생성: 강점·기회·점수 변화·benchmark
@@ -8624,8 +8375,8 @@
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>• Core HRIS: Microsoft Viva (M365 ecosystem):
-Glint이 LinkedIn → MS Viva 통합
+          <t>• Core HRIS: Microsoft Viva (M365 ecosystem) Glint이 LinkedIn →
+MS Viva 통합
 • AI 시스템 배치: Viva Glint 내장 Copilot
 • 배포 환경: Microsoft Azure cloud (M365 표준)
 • 연동·통합: M365 (Outlook·Teams·Power BI),
@@ -8747,8 +8498,8 @@
       <c r="AK38" s="10" t="inlineStr">
         <is>
           <t>• KR 대기업 annual 조직문화 진단의 직접 reference:
-• 삼성·SK·LG·현대 모두 매년 1~2회 engagement survey (5자리 인원):
-open-end 코멘트 코딩에 HRBP 팀 수주 투입
+• 삼성·SK·LG·현대 모두 매년 1~2회 engagement survey (5자리 인원) open-end 코멘트 코딩에
+HRBP 팀 수주 투입
 • Glint Copilot은 이 ROI 격차 즉시 해소: 이미 M365 도입사는 추가 도입 부담 적음
 • 한국 기업 sentiment 한국어 NLP 품질 검증 필수:
 Korean Glint Copilot의 존댓말·dialect·industry-specific term 처리 POC 4주</t>
@@ -8807,10 +8558,7 @@
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-HR·재무·구매 문의가 100개 이상의 개별 이메일 사서함으로 분산. 고객이 어떤 채널에 연락해야 할지 혼란. /
-[After]
-1. Fact "My Services" 단일 포털로 모든 HR·재무·구매 요청을 통합 접수.
+          <t>1. Fact "My Services" 단일 포털로 모든 HR·재무·구매 요청을 통합 접수.
 2. Fact ServiceNow AI 에이전트가 인테이크·라우팅·해결 자동화.
 3. Fact 이메일·챗봇·음성·전화를 포함하는 현대적 디지털 인터랙션 레이어 구축.</t>
         </is>
@@ -8970,8 +8718,9 @@
       <c r="E40" s="10" t="inlineStr">
         <is>
           <t>Spire Inc.는 미주리주 St.
-Louis 기반 미국 5위 천연가스 utility (1.7M 고객, 3개 주, 10+ 노조 운영):
-미국 최대급 단일 unionized utility.
+Louis 기반 미국 5위 천연가스 utility (1.7M 고객,
+3개 주,
+10+ 노조 운영) 미국 최대급 단일 unionized utility.
 Sodales Labour Relations Management (SAP SuccessFactors 통합 endorsed
 app)을 도입해 incident·grievance·discipline·appeals를 실시간 추적하고 다중 노조별 case
 관리·CBA(단체협약) 중앙화·노조 규칙 기반 워크플로우 자동화를 운영.
@@ -8999,17 +8748,7 @@
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Spire는 10+ 노조와 동시 운영:
-각 노조별 단체협약(CBA)·grievance procedure·timeline·escalation 절차가 모두 상이.
-매니저·HR이 spreadsheet·이메일로 1건씩 처리, 노조별 일관성 부재 + audit trail 약함 / Pain point:
-/ 다중 노조 복잡성:
-10+ CBA 문서 manual 검색 → grievance 처리 시 잘못된 절차 적용 risk / 근태·LMS·comp 데이터 silo:
-각 시스템에서 case 정보 수집 시간 over-burden / 컴플라이언스 audit 추적 어려움:
-사건 처리 이력 분산 → 외부 audit·노조 측 조회 시 bottleneck / Trigger:
-SAP SuccessFactors 도입 + Sodales의
-[After]
-1. 직원·매니저가 conversational AI 챗봇으로 grievance/incident/disciplinary report 신고
+          <t>1. 직원·매니저가 conversational AI 챗봇으로 grievance/incident/disciplinary report 신고
 2. Sodales가 자동으로 SAP Employee Central·LMS·근태에서 관련 데이터 auto-populate
 3. AI가 case 자동 요약 + 조사 추천 (grievance type·노조 식별·timeline 생성)
 4. 다중 노조별 grievance 트래킹: 노조별 CBA·timeline·escalation 프로토콜 내장
@@ -9198,10 +8937,7 @@
       </c>
       <c r="G41" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-채용 소요시간 약 60일, 수동 이력서 검토, 전통적 교육 방식. /
-[After]
-1. Fact Workday HCM으로 2.3M 직원 HR 단일 통합 관리.
+          <t>1. Fact Workday HCM으로 2.3M 직원 HR 단일 통합 관리.
 2. Fact Paradox Olivia 대화형 ATS로 프론트라인 채용 자동화: 채용 소요시간 60일→18일 단축.
 3. Fact 2025년 6월, 1.5M 직원 대상 AI 도구 모음 공개.
 4. Fact 2025년 9월, OpenAI와 AI 인증 교육 프로그램 파트너십 발표 (2026년 시작 예정).
@@ -9348,7 +9084,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="184" customHeight="1">
+    <row r="42" ht="168" customHeight="1">
       <c r="A42" s="8" t="n">
         <v>41</v>
       </c>
@@ -9384,11 +9120,7 @@
       <c r="F42" s="10" t="inlineStr"/>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-매장 associate가 가격·재고·통로 위치·근무 schedule을 종이 매뉴얼·Telxon 단말기·매니저 호출로 확인.
-신규 정책·프로모션은 매장별 매니저가 구두 전달 /
-[After]
-1. associate가 회사 지급 모바일 단말로 Ask Sam 앱을 음성 호출 ("What aisle is hand soap?")
+          <t>1. associate가 회사 지급 모바일 단말로 Ask Sam 앱을 음성 호출 ("What aisle is hand soap?")
 2. 음성→텍스트 변환 후 Walmart 내부 KB(상품·매장·정책·schedule)에서 답변 검색
 3. 결과를 음성·텍스트로 반환, 위치는 매장 지도 overlay
 4. 본인 schedule 조회·교대 요청은 WFM 시스템 연동,
@@ -9576,17 +9308,7 @@
       </c>
       <c r="G43" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-Waymo는 ServiceNow 같은 범용 ITSM/HR ticketing 도구로 ER case 처리:
-grievance·discipline·investigation도 일반 ticket으로 처리 / Pain point:
-/ ER 도메인 부재:
-ServiceNow는 ER (grievance·investigation·legal hold·noncompete) 도메인 모름:
-case 분류·workflow가 일반 IT ticket과 동일 / Role-based access 한계:
-ER case는 매니저·HR·legal 권한 분리 필요.
-일반 ticket은 해당 분리 약함 / Audit trail 부족:
-ER case는 SOX·legal hold·investigation 이력 필요 → 일반 ticket의 audit
-[After]
-1. 직원이 HR Acuity portal로 ER case 신고: case type 자동 분류
+          <t>1. 직원이 HR Acuity portal로 ER case 신고: case type 자동 분류
 2. HR/People Relations team이 ER 전용 workflow로 처리: investigation plan·인터뷰 질문 등
 ER 템플릿
 3. Role-based access: 매니저·HR·legal 권한 분리
@@ -9755,10 +9477,7 @@
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-HR 정책·셀프서비스 문의를 직원이 이메일·전화로 HR 팀에 직접 요청. /
-[After]
-1. Fact ROB가 계좌 정보 업데이트, 정책 안내, 커리어 정보 탐색 등의 셀프서비스 프로세스 안내.
+          <t>1. Fact ROB가 계좌 정보 업데이트, 정책 안내, 커리어 정보 탐색 등의 셀프서비스 프로세스 안내.
 2. Fact 대화 중 감성 지능으로 추가 인간 지원 필요 여부 식별 → HR 담당자 연결.
 3. Fact 직원 대화를 통해 지속적으로 개선.</t>
         </is>
@@ -9901,7 +9620,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="200" customHeight="1">
+    <row r="45" ht="168" customHeight="1">
       <c r="A45" s="15" t="n">
         <v>44</v>
       </c>
@@ -9924,8 +9643,7 @@
         <is>
           <t>싱가포르 최대 은행 DBS Bank는 인사 전 영역에 AI를 내재화한 아시아 금융권 선도 사례다.
 ✅ Fact 핵심 세 가지:
-(1) AI 채용 플랫폼 JIM(Jobs Intelligence Maestro):
-이력서 스크리닝·면접 일정·초기 평가 자동화로 채용 소요시간을 32일→8일 단축, (2) 이탈 예측 모델:
+(1) AI 채용 플랫폼 JIM(Jobs Intelligence Maestro) 이력서 스크리닝·면접 일정·초기 평가 자동화로 채용 소요시간을 32일→8일 단축, (2) 이탈 예측 모델:
 학습·보상·휴가 패턴 등 다변수 분석으로 이탈 징후 조기 감지, (3) iGrow 커리어 어드바이저:
 10,000개 이상 내부 과정 기반 개인화 커리어 경로 추천.
 sources/emerj-dbs-ai-cases.md sources/adriantan-dbs-ai-recruiting.md</t>
@@ -9942,10 +9660,7 @@
       </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-채용 담당자가 수동으로 이력서 검토·면접 일정 조율·초기 평가 진행. 32일 소요. /
-[After]
-1. 지원자
+          <t>1. 지원자
 2. JIM AI 채용 이력서·일정·평가
 3. 면접 진행
 4. 채용 결정 인간
@@ -10119,10 +9834,7 @@
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-지식노동자가 직접 문서 작성, 수동 검색, 개별 도구 사용. /
-[After]
-1. 직원 입력 텍스트·문서
+          <t>1. 직원 입력 텍스트·문서
 2. GS AI Assistant 사내 방화벽 내
 3. AI 응답 생성
 4. 직원 검토</t>
@@ -10145,7 +9857,7 @@
         <is>
           <t>지식노동자 자연어 요청에 대한 LLM 멀티모델 답변 (GPT-4o/o3-mini,
 Gemini 2.0,
-Claude 3.7 라우팅): 문서 요약·리서치 노트·규제 문서 분석·코드·다국어 번역.
+Claude 3.7 라우팅) 문서 요약·리서치 노트·규제 문서 분석·코드·다국어 번역.
 사내 방화벽 격리</t>
         </is>
       </c>
@@ -10296,13 +10008,7 @@
       </c>
       <c r="G47" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-270K 직원 대상 retention 관리는 사후 exit interview 의존:
-떠난 후에야 원인 파악 / Pain point:
-핵심인재 이탈 비용 (replacement cost 연봉의 1~3배) + 외부 채용 시장 경쟁 격화 / Trigger:
-2010년대 HR analytics 부상 + Watson 자사 활용 dogfooding 명분
-[After]
-1. ML 모델이 월간 데이터 갱신 → flight risk score 산출
+          <t>1. ML 모델이 월간 데이터 갱신 → flight risk score 산출
 2. 위험군 매니저에게 alert + 권장 action menu (raise / promotion / training / mentoring)
 3. AI 보상 추천: 매니저에게 per-employee salary 인상 권고 + supporting factors (flight
 risk·성과·시장)
@@ -10476,10 +10182,7 @@
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-서류 → 인적성(SSAT 류) → 면접관 면접 → 합격 (한국 대기업 전형) /
-[After]
-1. 지원자가 성향파악 과제 수행 (행동 성향 분석)
+          <t>1. 지원자가 성향파악 과제 수행 (행동 성향 분석)
 2. 전략게임: 수행 (시뮬레이션 기반 문제 해결 능력)
 3. 영상면접: (AI 분석)
 4. AI가 3개 과제 종합해 성과역량 예측 점수 산출
@@ -10518,8 +10221,8 @@
           <t>• 모델 유형: predictive (성과역량 예측) + recognition
 (영상·음성) + simulation (게임 행동)
 • 제공 방식: 자체 모델 (마이다스아이티 R&amp;D)
-• 평가·가드레일: KAIST 연구진 *Nature Scientific Reports* (2025-07):
-채용 1년 후 업무 성과 예측 통계적 유의성 검증.
+• 평가·가드레일: KAIST 연구진 *Nature Scientific Reports*
+(2025-07) 채용 1년 후 업무 성과 예측 통계적 유의성 검증.
 단 편향 부재 별도 검증 미공개</t>
         </is>
       </c>
@@ -10631,7 +10334,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="280" customHeight="1">
+    <row r="49" ht="184" customHeight="1">
       <c r="A49" s="15" t="n">
         <v>48</v>
       </c>
@@ -10679,15 +10382,7 @@
       </c>
       <c r="G49" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-미국 직원이 OE 시즌에 plan 선택:
-평균 17분 소요, 의료 plan만 5~10개 옵션, voluntary benefit (accident·hospital·critical illness·disability)은 추가 5~15개.
-정보 비대칭으로 직원이 "안전하게" 비싼 PPO 선택 → 본인부담 over-pay / Pain point:
-직원당 plan mismatch로 연 평균 $750~$1,500 over-pay (Nayya 자사 조사).
-voluntary benefit 가입율 낮음 (직원 정보 부족) / Trigger:
-미국 의료비 인플레이션 + HDHP/HSA 채택 증가 → 직원이 "올바른 선택"하기 어려운 환경 → AI 추천 수요
-[After]
-1. 직원이 Nayya portal·MetLife channel 로그인
+          <t>1. 직원이 Nayya portal·MetLife channel 로그인
 2. 데이터 통합:
 직원이 본인 정보 (가족 구성·예상 의료 사용·소득) + Nayya가 보유한 외부 데이터 (지역 의료 비용·청구 패턴) 결합
 3. AI engine이 plan별 expected total cost (premium + deductible + copay + 본인부담)
@@ -10825,7 +10520,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="216" customHeight="1">
+    <row r="50" ht="152" customHeight="1">
       <c r="A50" s="8" t="n">
         <v>49</v>
       </c>
@@ -10867,14 +10562,7 @@
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-풀무원 ~7K 직원이 HR 정책 문의를 HR 팀 전화·이메일로 처리:
-HR 팀 단순 반복 응대 부담 / Pain point:
-한국 중견기업 HR 팀 ~10명 규모:
-직원당 daily 문의 부담, 정책 변경 시 안내 누락 / Trigger:
-2024 한국 ChatGPT 도입 가속 + 풀무원 디지털 전환 명분
-[After]
-1. 직원이 두리번 chatbot에 자연어 query (PC, 모바일 확장 예정)
+          <t>1. 직원이 두리번 chatbot에 자연어 query (PC, 모바일 확장 예정)
 2. 두리번이 인사 정보 문서 RAG 검색 (근태·복리후생·학습·평가·승진·보상)
 3. 출처 표시 + 답변 생성 (hallucination 최소화 design)
 4. 복잡 case는 HR 팀 escalation
@@ -11006,7 +10694,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="312" customHeight="1">
+    <row r="51" ht="248" customHeight="1">
       <c r="A51" s="15" t="n">
         <v>50</v>
       </c>
@@ -11052,17 +10740,7 @@
       </c>
       <c r="G51" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-SAP SuccessFactors는 conventional HCM 위주, AI 기능은 모듈별 산발 (Joule 초기 release).
-Workday Illuminate에 비해 agentic 카테고리 catch-up 필요.
-/ Pain point:
-대규모 SAP HCM 고객(IBM·Disney·한국 제조 대기업)이 AI 에이전트 carve-out을 별도 벤더로 가는 것을 막아야 함.
-SAP suite 안에 native agent 생태계 형성이 시급.
-/ Trigger:
-Workday Illuminate (2024~2025), Workday × Sana 인수, Workday ASOR(2026-02) 등 경쟁 압박.
-SAP가 Joule 통합 가속화로 대응.
-[After]
-1. 직원/매니저
+          <t>1. 직원/매니저
 2. Joule Orchestrator
 3. Performance &amp; Goals Agent
 4. Career &amp; Talent Dev Agent
@@ -11277,10 +10955,7 @@
       </c>
       <c r="G52" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-직원이 내부 성장 기회를 인식하지 못함 → 50% 퇴직 사유 /
-[After]
-1. 직원이 프로필(스킬·관심·포부) 작성
+          <t>1. 직원이 프로필(스킬·관심·포부) 작성
 2. Gloat AI가 스킬·관심과 조직 내 기회를 매칭
 3. 제공되는 기회 유형: gig work(단기 프로젝트), career transitions(역할 이동), mentorship(멘토링)
 4. 직원이 자율적으로 참여 선택</t>
@@ -11424,7 +11099,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="216" customHeight="1">
+    <row r="53" ht="184" customHeight="1">
       <c r="A53" s="15" t="n">
         <v>52</v>
       </c>
@@ -11464,14 +11139,7 @@
       </c>
       <c r="G53" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-신한은행 직원이 다수의 산발 AI 도구 (A.I 몰리·OCR·R비서) 별도 사용:
-UX 분산 / Pain point:
-14,000+ 직원 base에서 AI 도구 fragmentation으로 ROI 약화 / Trigger:
-2024-09 통합 launch:
-단일 인터페이스 + 모바일·태블릿 음성 지원
-[After]
-1. 직원이 AI ONE 단일 인터페이스 접속
+          <t>1. 직원이 AI ONE 단일 인터페이스 접속
 2. 40+ 업무비서 중 task 선택 (또는 음성 지시)
 3. AI-STUDIO (분석)·AI-OCR (문서 인식)·R비서 (자동화) 통합 호출
 4. 모바일·태블릿 Speech-to-AI 지원
@@ -11598,7 +11266,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="184" customHeight="1">
+    <row r="54" ht="136" customHeight="1">
       <c r="A54" s="8" t="n">
         <v>53</v>
       </c>
@@ -11638,12 +11306,7 @@
       </c>
       <c r="G54" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-SK C&amp;C 신입·주니어 채용 시 수천 건 지원서 review에 HR + 사업부 SME 다수 인력 1주 투입 / Pain point:
-한국 대졸 정기공채 (3월·9월) 시즌 압박 + 직무 적합성 판단 표준화 어려움 / Trigger:
-2025년 SKT-SK AX 'A.Biz' 합작 launch + 신입 공채 시즌 적용
-[After]
-1. 자기소개서 input → A.Biz HR이 키워드 추출 (경력·핵심 역량)
+          <t>1. 자기소개서 input → A.Biz HR이 키워드 추출 (경력·핵심 역량)
 2. 직무 적합성 + 리스크 요인 score
 3. 4시간 내 결과 (수천 건)
 4. AI 면접 (영상 응답 분석) + 맞춤 면접 질문 자동 생성
@@ -11788,7 +11451,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="200" customHeight="1">
+    <row r="55" ht="120" customHeight="1">
       <c r="A55" s="15" t="n">
         <v>54</v>
       </c>
@@ -11828,13 +11491,7 @@
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-SK 그룹 25개 멤버사가 각각 별도 HR 시스템·챗봇 운영:
-그룹 표준 부재 / Pain point:
-그룹 차원 AI 거버넌스·비용·표준 보안 통제 어려움 + 멤버사별 중복 투자 / Trigger:
-SKT 'A.Biz' B2B launch 자체 dogfooding + 그룹 차원 AI 가속 명령
-[After]
-1. SKT-SK AX가 'A.Biz' 단일 platform 제공
+          <t>1. SKT-SK AX가 'A.Biz' 단일 platform 제공
 2. 멤버사 HR 담당자가 agent builder no-code로 자체 챗봇·자동화 구축
 3. 일반 멤버사: A.Biz 표준 LLM 호출
 4. 국가핵심기술 보유사 (SK하이닉스·SK온·SK실트론): 자체 LLM 'A.X' + SK AX 산업특화 AI 사용으로 격리 보안
@@ -11954,7 +11611,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="232" customHeight="1">
+    <row r="56" ht="136" customHeight="1">
       <c r="A56" s="8" t="n">
         <v>55</v>
       </c>
@@ -11995,15 +11652,8 @@
       </c>
       <c r="G56" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-우리은행 ~13K 직원이 다수 산발 시스템 (코어뱅킹·CRM·콜센터·내부통제) 사용.
-AI 도입은 부서별 산발 PoC / Pain point:
-KB국민은행 (인사이동 AI), 신한 AI ONE 등 경쟁 은행 AI 가속 → 우리은행 차별화 시급 / Trigger:
-2026 신년 신경 그룹장 발표:
-금융권 최초 전사 AI 에이전트 도입 결단
-[After]
-1. 575개 사업부 nominate: 된 AI 에이전트 후보 수집
-2. 평가 기준 적용:: 업무 적합성·ROI·실행 가능성·리스크 (구체 framework _미공개_)
+          <t>1. 575개 사업부 nominate: 된 AI 에이전트 후보 수집
+2. 평가 기준 적용: 업무 적합성·ROI·실행 가능성·리스크 (구체 framework _미공개_)
 3. 5대 영역 29개 업무 → 175개 에이전트 선정: (체계적 portfolio prune)
 4. 삼성SDS 우선협상대상자 (2026-04-07) → 구축 계약
 5. 2026-12 1차 97개 production, 2026 초 78개 추가
@@ -12159,7 +11809,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="248" customHeight="1">
+    <row r="57" ht="184" customHeight="1">
       <c r="A57" s="15" t="n">
         <v>56</v>
       </c>
@@ -12202,17 +11852,7 @@
       </c>
       <c r="G57" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-엔터프라이즈가 AI 에이전트를 부서별·도구별로 산발 도입.
-누가 만들었는지, 어떤 권한을 갖는지, 누가 책임지는지가 불투명.
-shadow AI 리스크 누적.
-/ Pain point: AI 에이전트가 빠르게 늘어나는데 거버넌스·감사·권한 통제가 부재.
-Deloitte 2026 HC Trends에 따르면 임원 60%가 AI를 의사결정에 사용하지만 5%만 잘 관리 중.
-/ Trigger:
-2026-Q1 EU AI Act high-risk 의무 발효 임박 + 한국 AI 기본법(2026-01-22 시행) 등 글로벌 규제 압력.
-엔터프라이즈가 "AI 거버넌스" 카테고리 솔루션 시급히 요구.
-[After]
-1. 신규 AI 에이전트 등록 시 ASOR에 owner·purpose·scope 명시
+          <t>1. 신규 AI 에이전트 등록 시 ASOR에 owner·purpose·scope 명시
 2. ASOR이 권한·조직도·스킬 매핑 자동 적용 (Workday IAM 연계)
 3. 에이전트 활동 로그·outcome 분석 (사람 직원 분석과 동일 dashboard)
 4. 권한 변경·비활성화·감사 추적 (Workday change history)</t>
@@ -12226,7 +11866,7 @@
 • 배포 환경: Workday cloud (multi-tenant)
 • 연동·통합: 1st-party Workday Illuminate agents +
 3rd-party (Salesforce Agentforce,
-OpenAI, Microsoft, Anthropic 등): 표준
+OpenAI, Microsoft, Anthropic 등) 표준
 프로토콜(MCP·a2a) 기반
 • 사용자 접점: Workday admin console + 권한 변경은 기존
 Workday self-service 워크플로
@@ -12316,8 +11956,7 @@
       <c r="AK57" s="16" t="inlineStr">
         <is>
           <t>• KR 적용 1순위:
-이미 Workday 도입한 한국 대기업(LG·SK·CJ 등 일부):
-AI 거버넌스 솔루션 도입 즉시 reference로 사용 가능
+이미 Workday 도입한 한국 대기업(LG·SK·CJ 등 일부) AI 거버넌스 솔루션 도입 즉시 reference로 사용 가능
 • 확장 어젠다:
 Workday 미사용 KR 대기업에는 "Workday ASOR이 만든 카테고리"로 자체 구축 또는 다른 거버넌스 솔루션 도입 논의 진입점
 • 2026 Q3-Q4 제안서 핵심 슬라이드:
@@ -12340,7 +11979,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="264" customHeight="1">
+    <row r="58" ht="232" customHeight="1">
       <c r="A58" s="8" t="n">
         <v>57</v>
       </c>
@@ -12385,16 +12024,7 @@
       </c>
       <c r="G58" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Amazon PXT(People eXperience and Technology) 조직은 10,000+ HR 전문 인력이 채용·HR
-운영·기술·분석 업무를 수행.
-1.5M+ 매장 직원 + 수십만 기업 직원의 HR 서비스 수요를 사람이 직접 처리 / Pain point:
-$100B+ AI 투자를 진행하면서 HR 기능도 자동화 가능 영역으로 식별됨.
-채용 심사·정책 질의·분석 리포팅 등이 AI copilot으로 대체 가능하다는 판단 / Trigger: CEO Andy Jassy의
-"모든 client experience·employee process·backend operation에 AI를 주입"하라는 전사 방침
-→ HR 조직도 예외 없음 / ⚠️ 핵심 갈등: 동시에 250,000명 계절직 warehouse 채용은
-[After]
-1. PXT가 internal AI 시스템 (이미 CS·warehouse 자동화에 사용 중)을 talent
+          <t>1. PXT가 internal AI 시스템 (이미 CS·warehouse 자동화에 사용 중)을 talent
 management·recruiting·employee engagement 플랫폼에 통합
 2. Recruiting screening·티켓 라우팅·정책 Q&amp;A·성과 데이터 합성 등 반복 업무 자동화
 3. AI로 처리되는 영역에서 매니저·HRBP 역할 축소 → 14k 포지션 redundant 판정
@@ -12404,8 +12034,8 @@
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>• Core HRIS: Amazon 자체 (구체 _미공개_):
-Workday/SAP 도입 여부 공식 확인 안 됨
+          <t>• Core HRIS: Amazon 자체 (구체 _미공개_) Workday/SAP 도입 여부
+공식 확인 안 됨
 • AI 시스템 배치: 자사 보고: PXT 조직이 internal AI
 시스템(CS·warehouse 자동화에 사용 중)을 talent
 management·recruiting·employee
@@ -12429,8 +12059,8 @@
       </c>
       <c r="K58" s="10" t="inlineStr">
         <is>
-          <t>• 모델 유형: generative + predictive + automation (RPA):
-Recruiting screening·티켓·정책 Q&amp;A
+          <t>• 모델 유형: generative + predictive + automation
+(RPA) Recruiting screening·티켓·정책 Q&amp;A
 • 제공 방식: 자사 보고: Amazon internal build</t>
         </is>
       </c>
@@ -12547,7 +12177,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="216" customHeight="1">
+    <row r="59" ht="168" customHeight="1">
       <c r="A59" s="15" t="n">
         <v>58</v>
       </c>
@@ -12590,11 +12220,7 @@
       </c>
       <c r="G59" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-Twilio는 double-digit 성장 속에 매니저 effectiveness 70% 수준.
-Manager 역량개발은 이벤트성 워크숍·LMS 과정 위주로 1:1 코칭은 임원에 한정 /
-[After]
-1. 매니저가 BetterUp Manage 플랫폼에서 Whole Person Assessment 수행 (resilience·growth
+          <t>1. 매니저가 BetterUp Manage 플랫폼에서 Whole Person Assessment 수행 (resilience·growth
 mindset·risk tolerance 등)
 2. 시스템이 strengths·focus area 식별 → AI가 scenario 질문(예:
 "low-performer 대화") 통해 맥락 수집
@@ -12641,8 +12267,7 @@
 • 커스터마이징 기법: 벤더 주장:
 BetterUp 코칭 IP·과학 자문 (Martin Seligman 등) prompt·rubric
 • 평가·가드레일: 벤더 주장:
-95% user satisfaction (Inc.com, BetterUp 자체 측정):
-독립 검증 부재</t>
+95% user satisfaction (Inc.com, BetterUp 자체 측정) 독립 검증 부재</t>
         </is>
       </c>
       <c r="L59" s="16" t="inlineStr">
@@ -12749,7 +12374,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="264" customHeight="1">
+    <row r="60" ht="184" customHeight="1">
       <c r="A60" s="8" t="n">
         <v>59</v>
       </c>
@@ -12784,15 +12409,7 @@
       </c>
       <c r="G60" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Deloitte 470,000 직원이 150개국에서 회계·감사·컨설팅·세무 업무 수행.
-각 직무별 AI 도구가 파편화돼 있거나 부재.
-지식 검색·문서 초안·분석에 사람의 반복 작업 시간이 과도 / Pain point: 경쟁
-컨설팅사(Accenture·PwC·McKinsey)가 각각 AI를 전사 배포하는 상황에서 "consulting firms의 AI 군비
-경쟁"이 Deloitte의 채택 가속화 요인 / Trigger: Anthropic Claude가 엔터프라이즈 보안·규정 준수를
-충족하면서도 "회계사·개발자별 특화 버전"을 제공할 수 있다는 판단 → 역대 최대 엔터프라이즈 배포 결정
-[After]
-1. Deloitte가 Anthropic Claude Enterprise를 글로벌 SSO로 470k 계정에 프로비저닝
+          <t>1. Deloitte가 Anthropic Claude Enterprise를 글로벌 SSO로 470k 계정에 프로비저닝
 2. Claude Center of Excellence가 부서별 use case·implementation framework 제공,
 15,000명 certification 프로그램 운영
 3. 직원이 Claude로 문서 합성·코드 생성·클라이언트 자료 분석 수행, 산출물은 Trustworthy AI framework로 검증
@@ -12937,7 +12554,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="200" customHeight="1">
+    <row r="61" ht="120" customHeight="1">
       <c r="A61" s="15" t="n">
         <v>60</v>
       </c>
@@ -12977,13 +12594,7 @@
       </c>
       <c r="G61" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-자동차 부품사 33K 직원: 매뉴얼·도면·기술 문서 fragmented.
-보안 민감 (R&amp;D 영업비밀) / Pain point:
-글로벌 commercial LLM 사용은 영업비밀·도면 leakage risk → 사내 LLM 필요 / Trigger:
-2025 현대차 그룹 AI 가속 + 모비스 R&amp;D 효율 압박
-[After]
-1. 직원이 MoAI 자연어 query (사전 탑재 프롬프트 템플릿 활용)
+          <t>1. 직원이 MoAI 자연어 query (사전 탑재 프롬프트 템플릿 활용)
 2. MoAI가 1,000만 건 사내문서 RAG 검색
 3. 답변 + 출처 표시
 4. 7개 업무 영역 (R&amp;D·IT·품질·영업·생산 + 2개)
@@ -13150,10 +12761,7 @@
       </c>
       <c r="G62" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개_ (IBM 내부 HR service center의 기존 운영) /
-[After]
-1. IBM 직원이 AskHR에 자연어 질문/요청 입력
+          <t>1. IBM 직원이 AskHR에 자연어 질문/요청 입력
 2. AskHR이 80+ 자동화된 HR 태스크 중 해당 작업 식별
 3. 처리 유형에 따라
 4. 해결 안 되면 human HR specialist에 에스컬레이션</t>
@@ -13328,12 +12936,7 @@
       </c>
       <c r="G63" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-recruiter가 JD 작성·후보자 search·일정 조율·feedback 수집을 manual·다중 시스템 hop으로 처리 / Pain point:
-high-volume 채용에서 recruiter productivity 한계 + diverse sourcing 가시성 부족 / Trigger:
-agentic AI 부상 + IBM 자체 채용 효율화 압박 (2025 8,000 layoff와 동시에 핵심 직무 채용 가속)
-[After]
-1. 매니저가 자연어로 채용 요청 ("senior Python engineer in Bangalore for watsonx team")
+          <t>1. 매니저가 자연어로 채용 요청 ("senior Python engineer in Bangalore for watsonx team")
 2. Agent가 JD 초안 생성 → hiring manager 공유·승인
 3. 후보자 매칭 (사내 + ThisWay Global 8,500+ community)
 4. 자격자 신규 지원 시 매니저 alert
@@ -13509,20 +13112,14 @@
         <is>
           <t>• Before:
 잡코리아 채용 담당자는 공고 작성·후보자 search·매칭을 별도 도구·매뉴얼 process
-• Pain point: 한국 채용 시장 vendor 경쟁 (사람인·잡코리아·원티드): 차별화 압박
+• Pain point: 한국 채용 시장 vendor 경쟁 (사람인·잡코리아·원티드) 차별화 압박
 • Trigger:
 2025-10 wantedlab-ai-recruiting-agent launch + 잡코리아 시장 점유 방어</t>
         </is>
       </c>
       <c r="G64" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-잡코리아 채용 담당자는 공고 작성·후보자 search·매칭을 별도 도구·매뉴얼 process / Pain point:
-한국 채용 시장 vendor 경쟁 (사람인·잡코리아·원티드):
-차별화 압박 / Trigger:
-2025-10 launch + 잡코리아 시장 점유 방어
-[After]
-1. 채용 담당자가 탤런트 에이전트에 자연어로 의도 입력 ("Python backend 시니어 + 핀테크 경력 + 서울")
+          <t>1. 채용 담당자가 탤런트 에이전트에 자연어로 의도 입력 ("Python backend 시니어 + 핀테크 경력 + 서울")
 2. 에이전트가 공고 맥락 분석 → 후보자 매칭 + 추천 사유
 3. 채용 담당자가 후보자 contact·면접 진행
 4. 통합 채용 솔루션으로 ATS 기능 흡수</t>
@@ -13638,7 +13235,7 @@
         <is>
           <t>• KR 채용 시장 vendor 경쟁 reference:
 • 잡코리아 '하이어링 센터' (2026-03) + 원티드 wantedlab-ai-recruiting-agent
-(2025-10) + 사람인 '커리어 매칭 에이전트' (2026 출시 예정): 한국 ATS·채용 vendor 3사 AI
+(2025-10) + 사람인 '커리어 매칭 에이전트' (2026 출시 예정) 한국 ATS·채용 vendor 3사 AI
 agent 경쟁 본격화
 • 글로벌 Eightfold AI Interviewer + IBM watsonx Orchestrate TA Agent
 ibm-watsonx-orchestrate-ta-agent와 비교
@@ -13661,7 +13258,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="168" customHeight="1">
+    <row r="65" ht="120" customHeight="1">
       <c r="A65" s="15" t="n">
         <v>64</v>
       </c>
@@ -13682,7 +13279,7 @@
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
-          <t>한국전력의 HR-Bot (솔트룩스 기반): 24/7 채용 상담·단순 반복 채용업무 자동화.
+          <t>한국전력의 HR-Bot (솔트룩스 기반) 24/7 채용 상담·단순 반복 채용업무 자동화.
 별도 AI 인사추천 시스템은 직원 역량·업무 이력 분석으로 적재적소 배치 지원: 공공기관 최초 사례.
 2024년 한전 경영평가에서 인사혁신 부문 가점.
 2025년 12월~2026년 3월 사내 규정·법규·문서 작성용 생성형 AI 시스템 전 직원 개방 예정.</t>
@@ -13699,12 +13296,7 @@
       </c>
       <c r="G65" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-한전 23,000+ 직원, 공공기관 특성상 인사이동·채용 manual + 정량 자료 의존 / Pain point:
-공공기관 인사이동의 표준화 어려움 + 채용 상담 volume 大 / Trigger:
-2024 공공기관 AI 도입 가속 + 한전 경영평가 인사혁신 부문 (정부 평가 KPI)
-[After]
-1. 지원자가 HR-Bot 24/7 챗봇 access
+          <t>1. 지원자가 HR-Bot 24/7 챗봇 access
 2. 채용 상담·FAQ·일정 안내 자동 응답
 3. 단순 반복 채용업무 자동화 (서류 접수·일정 조율)
 4. 복잡 케이스 사람 HR escalation</t>
@@ -13739,8 +13331,8 @@
       <c r="K65" s="16" t="inlineStr">
         <is>
           <t>• 모델 유형: 챗봇 NLP + recommendation
-• 제공 방식: 솔트룩스 vendor (한국 NLP):
-single vendor lock-in risk
+• 제공 방식: 솔트룩스 vendor (한국 NLP) single vendor
+lock-in risk
 • 평가·가드레일: KR AI 기본법 (2026-01) 고영향 AI:
 인적감독 의무 자동 충족 검증 _미공개_</t>
         </is>
@@ -13842,7 +13434,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="216" customHeight="1">
+    <row r="66" ht="184" customHeight="1">
       <c r="A66" s="8" t="n">
         <v>65</v>
       </c>
@@ -13883,14 +13475,7 @@
       </c>
       <c r="G66" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-미래에셋증권 직원이 사내 매뉴얼·노하우 문서 search 시 sharepoint·이메일 산발:
-정보 접근 비효율 / Pain point:
-부서별 specific knowledge가 사내 walking encyclopedia (시니어)에 의존:
-시니어 퇴직·부재 시 손실 / Trigger:
-2024 한국 자체 LLM 시장 성숙 + 금융 데이터 주권 압박
-[After]
-1. 직원·부서가 본인 업무 매뉴얼·노하우 문서 업로드
+          <t>1. 직원·부서가 본인 업무 매뉴얼·노하우 문서 업로드
 2. AI Assistant 플랫폼이 RAG indexing
 3. No-code 빌더: 로 부서·직원 전용 챗봇 자체 생성
 4. 직원·부서원이 자연어로 챗봇 query
@@ -13901,7 +13486,7 @@
         <is>
           <t>• Core HRIS: 미래에셋증권 사내 시스템 (구체 _미공개_)
 • AI 시스템 배치: 자체 AI Assistant 플랫폼 (네이버클라우드 협업)
-• 배포 환경: 네이버클라우드 (NCP): 한국 데이터 주권 driver
+• 배포 환경: 네이버클라우드 (NCP) 한국 데이터 주권 driver
 • 연동·통합: 사내 SSO + 부서별 매뉴얼·노하우 문서 upload
 • 사용자 접점: web 기반 No-code 챗봇 빌더 + 직원 자연어 query
 • 인증·권한: 사내 SSO + 부서별 RBAC</t>
@@ -13926,8 +13511,8 @@
       </c>
       <c r="K66" s="10" t="inlineStr">
         <is>
-          <t>• Foundation model: 네이버 하이퍼클로바X 대시 (HyperCLOVA X Dash):
-한국어 specialized
+          <t>• Foundation model: 네이버 하이퍼클로바X 대시 (HyperCLOVA X Dash) 한국어
+specialized
 • 모델 유형: LLM (요약·QA)
 • 제공 방식: Naver Cloud Platform via 협업
 • 커스터마이징 기법: RAG + No-code 빌더 (부서별)
@@ -14006,8 +13591,8 @@
       <c r="AK66" s="10" t="inlineStr">
         <is>
           <t>• KR 금융권 자체 LLM 활용 reference (1순위):
-• JPMorgan LLM Suite jpmorgan-llm-suite-redeployment (외부 LLM private gateway) vs 미래에셋 (한국 자체 LLM):
-양 방향 비교
+• JPMorgan LLM Suite jpmorgan-llm-suite-redeployment (외부 LLM private
+gateway) vs 미래에셋 (한국 자체 LLM) 양 방향 비교
 • KB·신한·하나·미래에셋 모두 자체 LLM 플랫폼 구축:
 미래에셋은 Hyperclova X 선택, 신한 shinhan-bank-ai-one-platform은 자체 통합, 하나 hana-bank-knowledge-chatbot은 자체 GenAI
 • No-code 빌더 패턴:
@@ -14069,10 +13654,7 @@
       </c>
       <c r="G67" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-직무 중심의 경직된 인사 관리. 내부 이동 기회가 제한적이고 관리자 추천에 의존. /
-[After]
-1. Fact Gloat 탤런트 마켓플레이스로 직원에게 잡·프로젝트·멘토·러닝 기회를 AI 기반으로 개인화 추천.
+          <t>1. Fact Gloat 탤런트 마켓플레이스로 직원에게 잡·프로젝트·멘토·러닝 기회를 AI 기반으로 개인화 추천.
 2. Fact 스킬 온톨로지 기반으로 직원의 현재 스킬과 희망 스킬을 분석, 성장 기회 연결.
 3. Fact "기존 접근법 대비 2개월 만에 4년치 품질 데이터 수집."</t>
         </is>
@@ -14252,10 +13834,7 @@
       </c>
       <c r="G68" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-매니저가 SuccessFactors에서 직원별 목표·피드백·리뷰 데이터를 개별 조회 → 수동으로 대화 포인트 준비 /
-[After]
-1. Joule Performance &amp; Goals Agent가 목표 진척·피드백 데이터를 자동 통합
+          <t>1. Joule Performance &amp; Goals Agent가 목표 진척·피드백 데이터를 자동 통합
 2. 맞춤 인사이트·대화 포인트 생성
 3. 매니저가 리뷰</t>
         </is>
@@ -14401,11 +13980,7 @@
       <c r="F69" s="16" t="inlineStr"/>
       <c r="G69" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-Siemens가 디지털 전환을 추진하나 data analytics·digital twin·automation 인력은 외부 채용 의존,
-기존 직원 reskilling은 부서별 단발 교육 /
-[After]
-1. Siemens가 Future Skills Initiative 발표 (300k 직원 대상, 41개 capability 영역 정의)
+          <t>1. Siemens가 Future Skills Initiative 발표 (300k 직원 대상, 41개 capability 영역 정의)
 2. Germany Qualification Opportunities Act 활용해 정부 25% 비용 분담,
 외부 파트너와 cost-sharing
 3. 직원·파트너에게 vocational training (digitalization·sustainability) 콘텐츠 제공
@@ -14555,7 +14130,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="264" customHeight="1">
+    <row r="70" ht="168" customHeight="1">
       <c r="A70" s="8" t="n">
         <v>69</v>
       </c>
@@ -14597,14 +14172,7 @@
       </c>
       <c r="G70" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-SK하이닉스 신입 채용은 자기소개서 + 인적성 + 면접:
-직무 적합 soft skill (커뮤니케이션·팀워크) 측정 어려움 / Pain point:
-반도체 기술사무직 신입 채용 volume 크지만 면접관 시간 한정 + soft skill 평가 표준화 어려움 / Trigger:
-2025 하반기 신입 공채:
-A!SK 전형 신설 (마이다스 inAIR 차별 논란 후 자체 hybrid 설계)
-[After]
-1. 서류 + AI 종합 역량 Report (Phase 1):
+          <t>1. 서류 + AI 종합 역량 Report (Phase 1):
 학력·전공·직무 연관성 검토 → AI가 정량·정성 역량 점수화 + 직무역량-JD 매칭율 → 면접관 참고 Report 자동 생성
 2. SKCT (인적성 검사): 온라인 역량 검사
 3. A!SK 전형 (AI 화상 면접): AI 인프라 기반 화상 면접: 문제은행식 직무별 맞춤 출제
@@ -14633,8 +14201,8 @@
 AI 면접 영상,
 JD-역량 매칭,
 (고도화) 석박사 Lab·논문 + LinkedIn 코멘트 자동 크롤링
-• 데이터 거버넌스: AI single decision 회피 (peer + HR + 면접관 hybrid):
-KR AI 기본법 인적감독 best practice
+• 데이터 거버넌스: AI single decision 회피 (peer + HR + 면접관
+hybrid) KR AI 기본법 인적감독 best practice
 • 민감정보 처리: AI 영상 분석의 표정·억양·외모 신호 사용 여부 _미공개_</t>
         </is>
       </c>
@@ -14642,7 +14210,7 @@
         <is>
           <t>직무별 AI 영상면접 질문 출제 + 지원자 영상 답변 평가 + 정량·정성 통합
 AI 종합 역량 Report (서류·SKCT·면접·논문·LinkedIn 크롤
-통합): 미래 동료 peer + 면접관용</t>
+통합) 미래 동료 peer + 면접관용</t>
         </is>
       </c>
       <c r="K70" s="10" t="inlineStr">
@@ -14759,7 +14327,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="216" customHeight="1">
+    <row r="71" ht="200" customHeight="1">
       <c r="A71" s="15" t="n">
         <v>70</v>
       </c>
@@ -14799,12 +14367,7 @@
       </c>
       <c r="G71" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-TCS·Infosys·Wipro·Tech Mahindra 합산 200만+ IT 인력이 manual testing·infra 운영·기본
-코딩 중심.
-AI 역량은 small subset에 한정, 클라이언트의 GenAI 프로젝트 수요 대응 곤란 /
-[After]
-1. NVIDIA와 4사 파트너십 체결 → NVIDIA AI Enterprise·Omniverse 기반 커리큘럼 표준화
+          <t>1. NVIDIA와 4사 파트너십 체결 → NVIDIA AI Enterprise·Omniverse 기반 커리큘럼 표준화
 2. 직원이 사내 LMS (Infosys Springboard·TCS iEvolve 등)에서 AI 기초·Agent·Physical AI
 단계별 수강
 3. TCS는 25k 엔지니어를 Microsoft Azure OpenAI 별도 트랙,
@@ -14930,7 +14493,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="248" customHeight="1">
+    <row r="72" ht="200" customHeight="1">
       <c r="A72" s="8" t="n">
         <v>71</v>
       </c>
@@ -14975,19 +14538,10 @@
       </c>
       <c r="G72" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Workday Learning은 기존 LMS 카테고리에 속해 conventional course management 위주.
-AI-native 경쟁자(Sana·Bersin Galileo·Docebo Shape) 대비 콘텐츠 생성·개인화·대화형 UX 격차 누적.
-/ Pain point: 기업 학습 콘텐츠 제작 비용·시간이 ROI를 짓누르는 구조 (코스 1개당 수개월·수천만원).
-직원 engagement도 낮음 (LMS 평균 완료율 30~50%).
-/ Trigger:
-Bersin이 발표한 "AI Transforms $400B of Corporate Learning" 보고서 + Sana의 빠른 시장 침투 (Klarna 등).
-Workday가 자체 개발 대신 acquisition으로 catch-up.
-[After]
-1. HRD가 Sana for Workday 대화창에 학습 목적·대상 입력
+          <t>1. HRD가 Sana for Workday 대화창에 학습 목적·대상 입력
 2. 벤더 주장: AI가 4일 내 멀티모달 코스 초안 생성 (텍스트·비디오·음성)
 3. HRD가 검토·수정 → 배포
-4. 직원이 conversational interface로 수강 (Sana Learn): 질문·요약·실습 양방향
+4. 직원이 conversational interface로 수강 (Sana Learn) 질문·요약·실습 양방향
 5. ASOR이 학습 에이전트 활동 거버넌스 적용</t>
         </is>
       </c>
@@ -15000,7 +14554,7 @@
 • 배포 환경: Workday cloud (multi-tenant)
 • 연동·통합: Workday HCM 마스터 데이터 + ASOR 거버넌스 + 30+
 언어 지원
-• 사용자 접점: 대화형 UI (web + mobile): Sana 기존 UX 차용
+• 사용자 접점: 대화형 UI (web + mobile) Sana 기존 UX 차용
 • 인증·권한: Workday IAM + ASOR 에이전트 정책</t>
         </is>
       </c>
@@ -15139,7 +14693,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="200" customHeight="1">
+    <row r="73" ht="184" customHeight="1">
       <c r="A73" s="15" t="n">
         <v>72</v>
       </c>
@@ -15176,12 +14730,7 @@
       <c r="F73" s="16" t="inlineStr"/>
       <c r="G73" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-La-Z-Boy (10k+ 글로벌 직원, 가구 제조·소매)가 15년 된 LMS 사용.
-잦은 crash·낮은 engagement,
-신상품·VOC 트레이닝 콘텐츠 제작에 instructional designer 수개월 소요 /
-[After]
-1. L&amp;D 팀이 Docebo Learning Suite로 마이그레이션, 글로벌 dealer·corporate 대상 통합 카탈로그 구성
+          <t>1. L&amp;D 팀이 Docebo Learning Suite로 마이그레이션, 글로벌 dealer·corporate 대상 통합 카탈로그 구성
 2. Docebo AI가 기존 콘텐츠·정책 문서 학습해 신규 과정 outline·퀴즈·요약 자동 생성
 3. AI virtual coach (beta)가 학습자 질문에 답변,
 use case template로 instructor 콘텐츠 제작 가속
@@ -15225,8 +14774,8 @@
 • 제공 방식: Docebo 자체 통합 (SaaS)
 • 커스터마이징 기법: Use-case instructional templates,
 Collaborative content design (AI 보조)
-• 평가·가드레일: SME가 AI 생성 콘텐츠 검토·승인 (HITL):
-자동 quality scoring 미공개</t>
+• 평가·가드레일: SME가 AI 생성 콘텐츠 검토·승인 (HITL) 자동 quality
+scoring 미공개</t>
         </is>
       </c>
       <c r="L73" s="16" t="inlineStr">
@@ -15370,11 +14919,8 @@
       </c>
       <c r="G74" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-직무(Job) 중심의 경직된 HR 관리. 내부 이동 기회 제한. /
-[After]
-1. Fact 모든 직무 역할에 스킬을 할당하여 지역별 스킬 갭 파악 → 업스킬링·리스킬링 프로그램 실행.
-2. Fact Fujitsu Learning Experience(온디맨드 학습 플랫폼): 직원이 커리어 목표를 설정하고 자율적으로 학습.
+          <t>1. Fact 모든 직무 역할에 스킬을 할당하여 지역별 스킬 갭 파악 → 업스킬링·리스킬링 프로그램 실행.
+2. Fact Fujitsu Learning Experience(온디맨드 학습 플랫폼) 직원이 커리어 목표를 설정하고 자율적으로 학습.
 3. Fact 내부 공모제: FY2020~FY2022에 일본 73,000명 중 약 25%(20,000명)가 자발적 지원.
 4. Fact Kozuchi AI 플랫폼 전사 배포: 업무 AI 보조, 월 69,000명 활성 사용자, 일 380,000건 사용.</t>
         </is>
@@ -15493,7 +15039,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="152" customHeight="1">
+    <row r="75" ht="136" customHeight="1">
       <c r="A75" s="15" t="n">
         <v>74</v>
       </c>
@@ -15530,12 +15076,7 @@
       </c>
       <c r="G75" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-현대제철 ~12K 직원이 매뉴얼·기술 문서·경영지원 정책을 분산 search / Pain point:
-철강 제조 도메인 매뉴얼 양 거대 + 신입 학습 곡선 길음 / Trigger:
-2024 한국 기업 사내 AI 플랫폼 도입 가속
-[After]
-1. 사내문서검색: 매뉴얼·기술·경영 문서 RAG
+          <t>1. 사내문서검색: 매뉴얼·기술·경영 문서 RAG
 2. 경영지원챗봇: HR·재무·총무 정책 Q&amp;A
 3. 2025-10 확장: 임직원 AI·로봇 역량 강화 프로그램</t>
         </is>
@@ -15708,12 +15249,7 @@
       </c>
       <c r="G76" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-recruiter 수동 screening 시 무의식적 bias + volume 한계 / Pain point:
-high-volume 채용에서 quality·diversity·speed 동시 달성 어려움 / Trigger:
-2014-2018 Amazon biased model 사건 등 industry bias 우려 부상
-[After]
-1. requisition 등록 → Watson이 자동 복잡도·ideal-profile 분석
+          <t>1. requisition 등록 → Watson이 자동 복잡도·ideal-profile 분석
 2. 후보자 지원 시 정형/비정형(이력서·LinkedIn·소셜) + soft trait 분석
 3. requisition 대비 success score 산출 (gender·race·age·ethnicity 억제)
 4. recruiter에게 ranked shortlist + supporting factor 제공
@@ -15760,7 +15296,7 @@
 • 제공 방식: IBM 자체 호스팅 (Watson Cloud)
 • 커스터마이징 기법: 과거 채용 데이터 학습, requisition 복잡도 분석
 • 평가·가드레일: protected attribute 억제.
-모델 age (2018): LLM 시대 후 fit 약화.
+모델 age (2018) LLM 시대 후 fit 약화.
 "soft trait" explainability 부족</t>
         </is>
       </c>
@@ -15870,7 +15406,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="232" customHeight="1">
+    <row r="77" ht="168" customHeight="1">
       <c r="A77" s="15" t="n">
         <v>76</v>
       </c>
@@ -15893,14 +15429,7 @@
       <c r="F77" s="16" t="inlineStr"/>
       <c r="G77" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-투자은행·자산관리·리테일금융의 인건비가 총비용의 50%+:
-금융 산업에서 AI 자동화의 ROI가 가장 큰 이유 / Pain point:
-(1) AI 역량 인력 확보 경쟁 치열, (2) 기존 HR 프로세스(채용·온보딩·분석)에 과도한 인력 투입, (3) 데이터 보안·규제 준수 하에서 AI 도입이 다른 산업보다 복잡 / Trigger:
-2024~2025 금융 산업 전반에서 "AI 도입을 안 하면 경쟁에서 뒤처진다"는 공감대 형성.
-JPMorgan CEO Dimon의 "모든 프로세스에 AI 주입" 방침이 HR에도 적용
-[After]
-1. 사용자는 portal 내에서 모델 선택 (GS는 GPT/Gemini/Claude/OSS 중) →
+          <t>1. 사용자는 portal 내에서 모델 선택 (GS는 GPT/Gemini/Claude/OSS 중) →
 문서 요약·이메일 초안·Excel/data 분석·번역 요청
 2. 모든 prompt·response는 firewall 내 audit trail에 기록, 모델 swap 시 재학습 불필요
 3. JPM은 8회 메이저 업그레이드로 custom assistant·문서 분석·시각화·모바일·접근성 기능 추가;
@@ -16072,7 +15601,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="280" customHeight="1">
+    <row r="78" ht="200" customHeight="1">
       <c r="A78" s="8" t="n">
         <v>77</v>
       </c>
@@ -16118,15 +15647,7 @@
       </c>
       <c r="G78" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Meta 직원들의 AI 도구 채택률이 불균형: 일부 엔지니어만 적극 활용, 나머지는 기존 방식 유지.
-자발적 채택만으로는 전사 AI transformation 속도가 부족 / Pain point: Moderna(모든 직원에게
-ChatGPT Enterprise 배포)·Deloitte(470k Claude)·PwC(65k upskilling) 등 경쟁사가 전사
-AI 배포를 가속화하는 상황에서, Meta가 "AI-first 기업"이라는 포지셔닝을 유지하려면 채택을 기대가 아닌 의무로 전환 필요
-/ Trigger: 내부 데이터에서 AI 도구 활용 직원의 생산성이 높다는 신호 → "AI 채택을 성과 평가에 공식 반영"이라는 가장
-과감한 정책 결정
-[After]
-1. CHRO Janelle Gale 메모(2025-11)로 2026 review 사이클부터 "AI-driven impact"를 모든
+          <t>1. CHRO Janelle Gale 메모(2025-11)로 2026 review 사이클부터 "AI-driven impact"를 모든
 직급·직군의 core expectation으로 공식화
 2. 직원이 자기 평가에 AI를 활용한 productivity·dev cycle·team performance 기여 사례 명시
 3. 매니저가 AI usage·outcome을 PSC rubric에 반영해 평가,
@@ -16138,10 +15659,10 @@
       </c>
       <c r="H78" s="10" t="inlineStr">
         <is>
-          <t>• Core HRIS: Meta 사내 PSC (Performance Summary Cycle):
-자체 (구체 _미공개_)
-• AI 시스템 배치: Metamate (사내 코딩·업무 어시스턴트):
-Llama + GPT-4 hybrid (Fortune 2024-12)
+          <t>• Core HRIS: Meta 사내 PSC (Performance Summary
+Cycle) 자체 (구체 _미공개_)
+• AI 시스템 배치: Metamate (사내 코딩·업무 어시스턴트) Llama +
+GPT-4 hybrid (Fortune 2024-12)
 • 연동·통합: 코드 commit 시스템 (engineering KPI
 tracking: agent-assisted % 측정), PSC
 rubric, People Analytics dashboard
@@ -16323,11 +15844,7 @@
       </c>
       <c r="G79" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개_: 아마 HR 팀 직접 문의, 또는 기존 benefits portal의 FAQ 수준.
-이 전제는 소스에 없음, 추측 금지: 단순히 "미공개" /
-[After]
-1. 직원이 혜택·equity 관련 질문을 GPT에 입력
+          <t>1. 직원이 혜택·equity 관련 질문을 GPT에 입력
 2. GPT가 정책·FAQ·개인 상황 반영하여 답변
 3. 해결되지 않으면 HR로 escalate (이 escalation 경로는 미공개)</t>
         </is>
@@ -16496,10 +16013,7 @@
       </c>
       <c r="G80" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개_ /
-[After]
-1. 직원이 본인의 성과 data·프로젝트·목표 달성을 GPT에 입력/연결
+          <t>1. 직원이 본인의 성과 data·프로젝트·목표 달성을 GPT에 입력/연결
 2. GPT가 연말 리뷰 초안 요약
 3. 직원이 검토·편집 후 제출 (추정 흐름 아님,
 소스에 구체 단계 미공개: 위 흐름은 "self-review 요약"이라는 기능 정의에서 직접 읽히는 부분만)</t>
@@ -16511,7 +16025,7 @@
 Enterprise 기반으로 추정 (Moderna 전사 인프라가 그쪽
 기반이므로) (, )
 • 배포 환경: OpenAI 클라우드
-• 사용자 접점: ChatGPT Enterprise UI (Custom GPT 형식):
+• 사용자 접점: ChatGPT Enterprise UI (Custom GPT 형식)
 Moderna 전사 기본값</t>
         </is>
       </c>
@@ -16626,7 +16140,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="200" customHeight="1">
+    <row r="81" ht="120" customHeight="1">
       <c r="A81" s="15" t="n">
         <v>80</v>
       </c>
@@ -16663,14 +16177,7 @@
       </c>
       <c r="G81" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-국민연금공단 ~7K 직원, 5,000만+ 국민 가입자:
-상담·규정 응대 부담 거대 / Pain point:
-공공기관 디지털 전환 + 정부 AI 정책 (한국 AI 기본법 2026-01) 대응 / Trigger:
-2025-09 AI·혁신 추진단 출범:
-기관 차원 AI 거버넌스 강화
-[After]
-1. AI 사원
+          <t>1. AI 사원
 2. AI 규정비서
 3. AI 수어 영상안내
 4. AI·혁신 추진단</t>
@@ -16783,7 +16290,7 @@
           <t>• KR 공공기관·연기금 reference:
 • 한국전력 HR-Bot korea-electric-power-hr-bot (공공기관 첫 AI 인사추천)
 • 인사혁신처/행정안전부 korea-gov-ai-hr-public-sector (정부 AI HR)
-• 국민연금공단 (CAIO + 추진단 + 다중 솔루션): KR 공공섹터 비교표 필수</t>
+• 국민연금공단 (CAIO + 추진단 + 다중 솔루션) KR 공공섹터 비교표 필수</t>
         </is>
       </c>
       <c r="AL81" s="16" t="inlineStr">
@@ -16800,7 +16307,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="184" customHeight="1">
+    <row r="82" ht="136" customHeight="1">
       <c r="A82" s="8" t="n">
         <v>81</v>
       </c>
@@ -16840,13 +16347,7 @@
       </c>
       <c r="G82" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-포스코 그룹 ~30K 직원 사무 영역 (인사·구매·경영분석)에 단순 반복 업무 다수 / Pain point:
-철강 산업 DX 전환 + 그룹 차원 AI 통합 부재 (계열사별 분산) / Trigger:
-2026 그룹 조직개편:
-그룹DX전략실 + AI·로봇 융합 연구소 신설로 거버넌스 강화
-[After]
-1. 110개 AI 에이전트가 인사·구매·경영분석 사무 업무 자동화
+          <t>1. 110개 AI 에이전트가 인사·구매·경영분석 사무 업무 자동화
 2. 그룹DX전략실 (임치현 실장)이 portfolio 거버넌스
 3. AI·로봇 융합 연구소 (윤일용 소장)이 R&amp;D 연계
 4. 계열사 (포스코·포스코홀딩스·포스코이앤씨 등) 공통 활용</t>
@@ -16881,7 +16382,7 @@
           <t>• 모델 유형: generative + automation (RPA) +
 classifier
 • 제공 방식: 포스코DX internal build
-• 평가·가드레일: "개발 중" (announced): production 후 검증 필요</t>
+• 평가·가드레일: "개발 중" (announced) production 후 검증 필요</t>
         </is>
       </c>
       <c r="L82" s="10" t="inlineStr">
@@ -17034,17 +16535,12 @@
       </c>
       <c r="G83" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개_.
-일반적으로 알려진 한국 대기업 공채 플로우 (서류→인적성→코딩/필기→면접→합격 통보)는 일반 지식이며 SK 특정 프로세스는 소스에 세부
-없음 /
-[After]
-1. 서류 지원:: 지원자가 온라인 지원
-2. 서류 심사:: 생성형 AI 자동 스크리닝 (LLM 기반, 시간당 1,000명)
-3. 필기 시험 (AICT):: 생성형 AI 활용 능력 평가
-4. 1차 면접:: ★ AI 100% 자동화 (진행·평가·결과 보고서 작성 모두 AI)
+          <t>1. 서류 지원: 지원자가 온라인 지원
+2. 서류 심사: 생성형 AI 자동 스크리닝 (LLM 기반, 시간당 1,000명)
+3. 필기 시험 (AICT): 생성형 AI 활용 능력 평가
+4. 1차 면접: ★ AI 100% 자동화 (진행·평가·결과 보고서 작성 모두 AI)
 5. (후속 면접은 사람 또는 혼합: 소스에 명시 없음): 6. 합격/불합격 고지: AI 자동
-6. OT 안내:: AI 자동</t>
+6. OT 안내: AI 자동</t>
         </is>
       </c>
       <c r="H83" s="16" t="inlineStr">
@@ -17213,10 +16709,7 @@
       </c>
       <c r="G84" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-에이전시 노동에 의존, 공석 원인 분석 없이 임시 충원 반복 /
-[After]
-1. Visier로 공석율·이직 패턴·에이전시 비용 연동 분석
+          <t>1. Visier로 공석율·이직 패턴·에이전시 비용 연동 분석
 2. 인력 투자 우선순위 결정
 3. 보상 재투자로 내부 충원율 제고</t>
         </is>
@@ -17380,10 +16873,7 @@
       </c>
       <c r="G85" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-매니저가 직원별로 여러 시스템(HRIS·프로젝트 관리·피드백 도구)에서 데이터 수집 → 수동으로 리뷰 작성 /
-[After]
-1. Performance Review Agent가 타 시스템 데이터를 자동 수집
+          <t>1. Performance Review Agent가 타 시스템 데이터를 자동 수집
 2. 리뷰 초안 자동 생성
 3. 매니저가 검토·수정·확정</t>
         </is>
@@ -17396,8 +16886,8 @@
       <c r="I85" s="16" t="inlineStr"/>
       <c r="J85" s="16" t="inlineStr">
         <is>
-          <t>매니저용 직원별 성과 리뷰 first draft (Workday HCM + 타 시스템 데이터 자동 통합):
-매니저 검토·수정 후 제출</t>
+          <t>매니저용 직원별 성과 리뷰 first draft (Workday HCM + 타
+시스템 데이터 자동 통합) 매니저 검토·수정 후 제출</t>
         </is>
       </c>
       <c r="K85" s="16" t="inlineStr"/>
@@ -17538,17 +17028,7 @@
       </c>
       <c r="G86" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Yelp의 ER documentation 분산:
-case 기록·investigation note·resolution이 여러 도구·spreadsheet에 흩어짐 / Pain point:
-/ Documentation 분산:
-ER team이 case 검색·trend 분석 시 1건씩 수작업 / Case 분류 복잡성:
-grievance type 분류 기준 일관성 없음 → analytics 부정확 / Advanced analytics 부재:
-부서·매니저별 trend dashboard 부재 / Trigger:
-ER team 성장 + case management 전문 도구 필요성.
-HR Acuity가 ER 전용 leader로 등장
-[After]
-1. ER team이 HR Acuity portal로 모든 case 단일 기록
+          <t>1. ER team이 HR Acuity portal로 모든 case 단일 기록
 2. Case 분류·investigation note·resolution 통합 documentation
 3. Advanced analytics: 부서·매니저·case type별 dashboard
 4. Rachel Greer Head of ER team이 운영 + HR Acuity 커뮤니티 활동</t>
@@ -17669,7 +17149,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="168" customHeight="1">
+    <row r="87" ht="120" customHeight="1">
       <c r="A87" s="15" t="n">
         <v>86</v>
       </c>
@@ -17702,10 +17182,7 @@
       <c r="F87" s="16" t="inlineStr"/>
       <c r="G87" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-정적 직무 기술서·수동 skills 매핑 (4~6개월 소요), 부서별 분절된 skills 데이터 /
-[After]
-1. 기존 직무 기술서·HRIS·프로젝트 이력 등 fragmented data 업로드
+          <t>1. 기존 직무 기술서·HRIS·프로젝트 이력 등 fragmented data 업로드
 2. Beamery Skills Inference 엔진이 role별 핵심 skill 추출 ( 벤더 주장 90% 정확도)
 3. Dynamic Job Architecture 자동 생성: role/family/proficiency level 매핑
 4. HRBP·HR tech 팀이 taxonomy 검토·승인
@@ -17811,8 +17288,7 @@
 Flex의 "1,200 JD→40역할" 통합은 workday-illuminate-job-architecture와 같은 도메인이지만 실제 deployment + metric이 있음
 • Forrester 467% ROI: HireVue의 134%를 크게 상회, Tier 1 독립 검증
 • J&amp;J(MIT CISR, 스킬 추론)과의 비교:
-J&amp;J는 학술 검증(정확도), Beamery는 Forrester(ROI):
-검증 축이 다름</t>
+J&amp;J는 학술 검증(정확도), Beamery는 Forrester(ROI) 검증 축이 다름</t>
         </is>
       </c>
       <c r="AL87" s="16" t="inlineStr">
@@ -17881,10 +17357,7 @@
       </c>
       <c r="G88" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-연간 설문 → 데이터 취합 → HR 분석 → 리더 브리핑 → 자체 액션 플랜 수립 (완결율 저조) /
-[After]
-1. 연간 설문 완료
+          <t>1. 연간 설문 완료
 2. AI가 각 리더의 팀 결과 + AC-CCSWB 리더십 원칙·코드 기반으로 개인화 Intelligent Nudge 생성
 3. 리더가 본인 팀 피드백과 가장 관련 높은 Nudge 주제 선택 (개인화)
 4. 1:1 코칭·개발 집중 → 액션 플랜 자동 추적</t>
@@ -18016,7 +17489,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="168" customHeight="1">
+    <row r="89" ht="104" customHeight="1">
       <c r="A89" s="15" t="n">
         <v>88</v>
       </c>
@@ -18048,10 +17521,7 @@
       <c r="F89" s="16" t="inlineStr"/>
       <c r="G89" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-역할별 AI 영향도를 수기 워크숍·인터뷰로 6~12개월에 걸쳐 평가 /
-[After]
-1. 조직의 job catalog·task inventory를 Workforce Analyzer에 로드
+          <t>1. 조직의 job catalog·task inventory를 Workforce Analyzer에 로드
 2. GenAI 엔진이 role별 task 분해·AI 자동화/증강 가능성 점수화
 3. 시나리오 모델링: task automation 비율·재배치 영향·skills gap 시뮬레이션
 4. Workforce Planner+ 모듈이 우선순위·도입 로드맵 추천
@@ -18174,7 +17644,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="184" customHeight="1">
+    <row r="90" ht="120" customHeight="1">
       <c r="A90" s="8" t="n">
         <v>89</v>
       </c>
@@ -18207,10 +17677,7 @@
       <c r="F90" s="10" t="inlineStr"/>
       <c r="G90" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-AI 채용 알고리즘이 inference time에 학습되거나 bias 점검 없이 운영 /
-[After]
-1. HireVue의 competency·game-based 알고리즘은 lab에서 학습·테스트 후 lock
+          <t>1. HireVue의 competency·game-based 알고리즘은 lab에서 학습·테스트 후 lock
 (static·deterministic)
 2. 외부 감사기관(DCI Consulting Group)이 인종·성별·교차 카테고리별 disparate impact 분석
 3. NYC Local Law 144 등 규제 요건에 맞춰 bias audit table 생성 (~300건)
@@ -18332,7 +17799,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="184" customHeight="1">
+    <row r="91" ht="152" customHeight="1">
       <c r="A91" s="15" t="n">
         <v>90</v>
       </c>
@@ -18368,13 +17835,7 @@
       </c>
       <c r="G91" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-1. HR 담당자가 각 신규입사자에게 개별 이메일·서류 안내
-2. ServiceNow·Jira·Okta 등 다수 시스템에 수작업 등록
-3. HR 문의는 담당자 직접 응답: 평균 5일+ 소요
-4. 온보딩 완료까지 최대 15일 /
-[After]
-1. Skye가 입사 확정 시점에 개인화 온보딩 여정 자동 개시
+          <t>1. Skye가 입사 확정 시점에 개인화 온보딩 여정 자동 개시
 2. ServiceNow·Jira·Okta·Teams·Google Chat 등 200+ 시스템 자동 연동·프로비저닝
 3. HR 문의 → Skye가 1차 처리 (20+ 유스케이스 대응); 복잡 건만 담당자 에스컬레이션
 4. 온보딩 완료: 기존 대비 4일 단축</t>
@@ -18508,7 +17969,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="184" customHeight="1">
+    <row r="92" ht="120" customHeight="1">
       <c r="A92" s="8" t="n">
         <v>91</v>
       </c>
@@ -18546,13 +18007,7 @@
       </c>
       <c r="G92" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-가스공사 ~3K 직원이 문서 초안·규정 검토를 manual / Pain point:
-공공기관 보안 민감 영역 (에너지 인프라) + 성능 우수한 상용 LLM 활용 동시 필요 / Trigger:
-2025-09 발주:
-제논 우선협상자, 2026 구축
-[After]
-1. 직원 query → 보안 민감도 자동 분류
+          <t>1. 직원 query → 보안 민감도 자동 분류
 2. 보안 민감 영역 → 사내 LLM
 3. 일반 영역 (전문지식) → 상용 LLM (외부 API)
 4. 답변 통합 → 직원 활용</t>
@@ -18693,10 +18148,7 @@
       </c>
       <c r="G93" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-공무원이 생성형 AI를 개인적·비공식적으로 사용하거나 외부 서비스 접근. /
-[After]
-1. 공무원
+          <t>1. 공무원
 2. 범정부 AI 공통기반 내부망 보안 환경
 3. 삼성SDS·네이버클라우드 LLM
 4. 법령·지침·민원 RAG 행정 문서 연계
@@ -18706,7 +18158,7 @@
       </c>
       <c r="H93" s="16" t="inlineStr">
         <is>
-          <t>• 배포 환경: Fact 정부 내부망(망분리 환경): 보안 격리 운영.
+          <t>• 배포 환경: Fact 정부 내부망(망분리 환경) 보안 격리 운영.
 • 연동·통합: Fact 정부 보유 법령·지침·민원 데이터 연계.</t>
         </is>
       </c>
@@ -18720,8 +18172,9 @@
       </c>
       <c r="J93" s="16" t="inlineStr">
         <is>
-          <t>공무원용 보고서·민원 답변·보도자료 초안 (망분리 환경 내 삼성SDS·네이버클라우드 LLM + 법령·지침·민원 RAG):
-공무원 최종 검토·결재</t>
+          <t>공무원용 보고서·민원 답변·보도자료 초안 (망분리 환경 내
+삼성SDS·네이버클라우드 LLM + 법령·지침·민원 RAG) 공무원 최종
+검토·결재</t>
         </is>
       </c>
       <c r="K93" s="16" t="inlineStr">
@@ -18867,10 +18320,7 @@
       </c>
       <c r="G94" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-연공서열 중심 보상 체계. 직급별 일률적 급여. /
-[After]
-1. Fact 직무 가치와 성과에 따른 차등 보상(직무급제).
+          <t>1. Fact 직무 가치와 성과에 따른 차등 보상(직무급제).
 2. Fact 연차 무관 직무 전문성 기반 레벨업 심사 신청 허용.
 3. Fact 도입 순서: 롯데바이오로직스(2024-05) → 대홍기획·롯데이노베이트(시범) → 롯데백화점·롯데웰푸드(2025).</t>
         </is>
@@ -18953,7 +18403,7 @@
 SAP Joule 등)를 도입하면 효율화 가능: AI 도입 확대 시 연계 제안 기회.
 • 한계: AI HR 사례라기보다는 전통적 HR 제도 개혁 사례.
 AI 요소가 확인될 경우 업데이트 필요.
-현재 confidence가 낮음(0.35): 소스가 국내 언론 Tier 4 수준.</t>
+현재 confidence가 낮음(0.35) 소스가 국내 언론 Tier 4 수준.</t>
         </is>
       </c>
       <c r="AL94" s="10" t="inlineStr">
@@ -19002,10 +18452,7 @@
       <c r="F95" s="16" t="inlineStr"/>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-직원이 HR/IT 문의 시 다중 portal·ticket 시스템을 거치며 응답 지연 /
-[After]
-1. 직원이 M365 Copilot 비즈니스 채팅에서 "Employee Self-Service" 선택
+          <t>1. 직원이 M365 Copilot 비즈니스 채팅에서 "Employee Self-Service" 선택
 2. 자연어로 질문 입력 (휴가 신청·급여·복리후생·장비 요청 등)
 3. Agent가 SharePoint 정책 KB·Workday/SAP/ServiceNow connector 조회
 4. authoritative 응답 또는 action form 제시 (휴가신청·transfer 요청 등)
@@ -19139,7 +18586,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="168" customHeight="1">
+    <row r="96" ht="120" customHeight="1">
       <c r="A96" s="8" t="n">
         <v>95</v>
       </c>
@@ -19170,10 +18617,7 @@
       <c r="F96" s="10" t="inlineStr"/>
       <c r="G96" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-컨설턴트가 ad-hoc 외부 강의·자율학습으로 AI 역량 습득, 일관성·실무 적용 부족 /
-[After]
-1. PwC가 My AI 프로그램 출범: Responsible AI·prompting·leadership 커리큘럼 설계
+          <t>1. PwC가 My AI 프로그램 출범: Responsible AI·prompting·leadership 커리큘럼 설계
 2. ChatPwC (사내 GenAI tool) 액세스 부여: risk-free playground 제공
 3. GenAI Super User Network (약 350명 자원자)가 팀별 워크숍·prompting party 진행
 4. 직원이 hackathon·게임쇼식 경쟁·라이브 실습에 참여
@@ -19331,10 +18775,7 @@
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-리크루터·채용 관리자가 개별적으로 JD 작성 → 편향 언어 미감지 → 다양성 지원자 풀 제한 /
-[After]
-1. JD를 Workday ATS에서 직접 작성 (Textio 인라인 통합)
+          <t>1. JD를 Workday ATS에서 직접 작성 (Textio 인라인 통합)
 2. Textio AI가 실시간 언어 점수(Textio Score) + 개선 제안 표시
 3. Textio Score 기준 이상(T-Mobile 기준 미공개)이어야 게시 허용
 4. 리크루팅 이메일·고용 브랜드 콘텐츠에도 동일 도구 적용</t>
@@ -19470,7 +18911,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="168" customHeight="1">
+    <row r="98" ht="104" customHeight="1">
       <c r="A98" s="8" t="n">
         <v>97</v>
       </c>
@@ -19493,10 +18934,7 @@
       <c r="F98" s="10" t="inlineStr"/>
       <c r="G98" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-채용 매니저가 JD를 자유 작성, gendered language·전형적 표현으로 다양성 후보 풀 제한 /
-[After]
-1. 채용 매니저/리크루터가 Workday ATS에서 JD 작성 시작
+          <t>1. 채용 매니저/리크루터가 Workday ATS에서 JD 작성 시작
 2. Textio 플러그인이 실시간으로 단어·구문 분석 (수백만 hiring docs 학습)
 3. 편향·가독성 기반 Textio Score 산출 + 대안 표현 제안
 4. 작성자가 제안 수용/거절하며 점수 ≥90 목표
@@ -19651,10 +19089,7 @@
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-회의 기록 수작업, 이메일·회의 정보 수동 파악, PPT 초안 수작업 /
-[After]
-1. 400명 파일럿 → 사용 패턴 분석 (Viva Insights 연동)
+          <t>1. 400명 파일럿 → 사용 패턴 분석 (Viva Insights 연동)
 2. 파일럿 결과 검증 후 10,000명 배포
 3. Microsoft 기술 지원으로 개인 활동 패턴 기반 Copilot 사용 자동 추천 시스템 구축
 4. 상시 사용 현황 모니터링 (Viva Insights)</t>
@@ -19680,15 +19115,14 @@
       <c r="J99" s="16" t="inlineStr">
         <is>
           <t>회의 트랜스크립트 요약 + 이메일·회의 따라잡기 응답 + PPT 초안 + 개인
-활동 패턴 기반 Copilot 사용 자동 추천 (Viva Insights 분석):
+활동 패턴 기반 Copilot 사용 자동 추천 (Viva Insights 분석)
 1인당 월 5.6시간 절감</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
         <is>
           <t>• Foundation model: 벤더 주장:
-GPT-4 계열 (Microsoft/OpenAI):
-Microsoft 공식 사양이나 버전 미명시
+GPT-4 계열 (Microsoft/OpenAI) Microsoft 공식 사양이나 버전 미명시
 • 제공 방식: Microsoft Azure OpenAI Service (상용
 API)</t>
         </is>
@@ -19801,7 +19235,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="264" customHeight="1">
+    <row r="100" ht="184" customHeight="1">
       <c r="A100" s="8" t="n">
         <v>99</v>
       </c>
@@ -19843,16 +19277,7 @@
       </c>
       <c r="G100" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-Accenture 733,000+ 직원이 전통적 e-learning + classroom 방식으로 교육.
-⚠️ 자사 보고:
-과정 완료율이 낮고 교육 시간이 길어 실무 적용까지의 gap이 큼 / Pain point:
-글로벌 컨설팅 업계에서 "직원 역량이 곧 매출"인 구조:
-교육 효율이 직접적 비즈니스 성과와 연결.
-AI 기술 역량이 부족하면 고객 프로젝트에 배정 불가 / Trigger:
-경쟁사(Deloitte Claude 470k, PwC 65k upskilling) 대비 "자사에 먼저 적용 → 고객에 판매" 전략 실행
-[After]
-1. 직원 skills profile·role·우선순위 영역을 LearnVantage에 입력
+          <t>1. 직원 skills profile·role·우선순위 영역을 LearnVantage에 입력
 2. AI recommendation 엔진이 Accenture·Stanford Online·Udacity 등 콘텐츠 큐레이션
 3. 개인화된 learning journey + Nanodegree/academy track 추천
 4. 일상 워크플로 내 AI coaching·real-time feedback 제공
@@ -20007,12 +19432,7 @@
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-1. 급여 담당자가 급여 실행 전 수작업으로 데이터 검토
-2. 이상 발견 시 수작업 조사 + 수정
-3. 분석 리포트는 수동 쿼리/Excel 집계 /
-[After]
-1. AI가 급여 실행 전 이상 자동 탐지 + 수정 제안 생성
+          <t>1. AI가 급여 실행 전 이상 자동 탐지 + 수정 제안 생성
 2. 급여 담당자가 제안 검토·승인(HITL)
 3. 자연어로 "초과근무 비용 트렌드는?" → 즉시 차트·인사이트 생성
 4. 규정 변경 자동 모니터링 + 컴플라이언스 태스크 자동 실행</t>
@@ -20155,7 +19575,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="280" customHeight="1">
+    <row r="102" ht="264" customHeight="1">
       <c r="A102" s="8" t="n">
         <v>101</v>
       </c>
@@ -20205,18 +19625,7 @@
       </c>
       <c r="G102" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-국내 중견·대기업의 성과 평가 시즌(월별·분기·연간)마다 관리자가 수동으로 주관식 평가 코멘트 작성 + HR이 수백~수천 건의 평가
-내용을 수동 취합·정리.
-원온원 미팅 노트도 수기 기록.
-❓ 구체 시간/비용 baseline 미공개 (관리자당 평가 작성 시간, HR 취합 소요 시간 등) / Pain point:
-(1) 형식적·부정확한 평가 코멘트:
-관리자가 시간 압박으로 "복붙"하거나 피상적으로 작성 → 직원 개발에 도움 안 됨.
-(2) HR 행정 부담: 평가 시즌에 HR 인력이 취합·정리에 과도 투입.
-(3) 원온원 미팅 내용이 기록되지 않거나 비체계적 → 지속적 성과 관리 연결 부족 / Trigger:
-국내 중견기업(인지그룹 등)이 SaaS 기반 성과관리 도구를 탐색하면서 "AI가 코멘트를 자동 요약
-[After]
-1. Fact 주관식 평가 코멘트 AI 자동 요약·정제 + 비속어·불필요 표현 필터링.
+          <t>1. Fact 주관식 평가 코멘트 AI 자동 요약·정제 + 비속어·불필요 표현 필터링.
 2. Fact AI 피드백 생성.
 3. Fact AI 원온원: 미팅 내용 자동 요약.
 4. Fact AI 평가: 서술형 리뷰 초안 작성.
@@ -20380,10 +19789,7 @@
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-매니저가 성과 리뷰를 빈 페이지에서 시작 → engagement 결과를 수동 해석 → 액션 플랜 없이 방치 /
-[After]
-1. AI Coach가 과거 피드백·동료 리뷰를 자동 통합
+          <t>1. AI Coach가 과거 피드백·동료 리뷰를 자동 통합
 2. 구조화된 리뷰 가이드 제공
 3. engagement 결과 기반 개인화 액션 플랜
 4. 매니저에게 대화형 코칭</t>
@@ -20535,10 +19941,7 @@
       </c>
       <c r="G104" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-HR 담당자가 수동으로 이력서 검토, 이메일·전화로 면접 일정 조율, 엑셀로 지원자 관리. /
-[After]
-1. Fact 채용 홈페이지 제작, 지원자 통합 관리, 협업 평가, 면접 일정 조율, 채용 데이터 분석 대시보드를 단일 플랫폼에서 제공.
+          <t>1. Fact 채용 홈페이지 제작, 지원자 통합 관리, 협업 평가, 면접 일정 조율, 채용 데이터 분석 대시보드를 단일 플랫폼에서 제공.
 2. Fact AI를 활용한 인재풀 구축·후보자 매칭(키워드 스크리닝을 넘어선 정교한 매칭).
 3. Fact 공정 채용·법규 준수 기능(2025 고용노동부 공정 채용 지침 방향 반영).</t>
         </is>
@@ -20645,7 +20048,7 @@
 중소기업 클라이언트 비용 절감 방안으로 제시 가능.
 • 한계: 구체 AI 기능 설명과 성과 수치가 벤더 마케팅 주장 수준.
 Tier 1·2 독립 검증 없음.
-Confidence가 낮음(0.30): 추가 독립 검증 소스 필요.
+Confidence가 낮음(0.30) 추가 독립 검증 소스 필요.
 • 원티드랩과 비교: 원티드랩은 대기업/전문직 수시 채용, 그리팅은 중소기업 ATS: 타겟 세그먼트 차별화 명확.
 (→ wantedlab-ai-recruiting-agent 연계)</t>
         </is>
@@ -20664,7 +20067,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="264" customHeight="1">
+    <row r="105" ht="216" customHeight="1">
       <c r="A105" s="15" t="n">
         <v>104</v>
       </c>
@@ -20701,16 +20104,7 @@
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-HSBC(275,000 직원)의 TA(채용)와 TM(인재관리)이 사일로화되어 운영.
-채용은 전통적 CV 기반, 내부 이동은 가시성 부족으로 외부 채용에 과도 의존 / Pain point:
-글로벌 은행의 skills transformation 압박:
-디지털·AI 역량 인력 확보가 시급하지만 기존 채용 방식으로는 속도·품질 부족.
-⚠️ Fortune Europe 보도: HSBC가 다른 유럽 은행보다 30% 더 많은 AI 채용 공고를 게시 (인력 전환 가속화 필요
-반증) / Trigger: SAP SuccessFactors(Core HRIS)만으로는 skills-based hiring +
-internal mobility 모두를 커버하기 어렵다는 판단 → Eightfold(TA) + Gloat(TM) + Acce
-[After]
-1. HSBC middleware가 HRIS·ATS·LMS·skills 데이터를 통합
+          <t>1. HSBC middleware가 HRIS·ATS·LMS·skills 데이터를 통합
 2. Eightfold이 1.6B+ profile 기반 skills inferencing 수행 (기반 skill graph)
 3. Gloat marketplace에 inferred skills로 직원·기회 매칭
 4. 직원이 project·gig·job·mentorship 검색·지원 (인도 tech팀 우선 → 14만 확장)
@@ -20838,7 +20232,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="168" customHeight="1">
+    <row r="106" ht="88" customHeight="1">
       <c r="A106" s="8" t="n">
         <v>105</v>
       </c>
@@ -20874,12 +20268,7 @@
       </c>
       <c r="G106" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-LG U+ 직원이 이메일·문서·코드를 manual 처리 / Pain point:
-통신사 코드 base 거대 + glob·다국적 파트너 이메일 다언어 / Trigger:
-2025 한국 통신사 사내 AI 가속
-[After]
-1. 이메일 자동 번역
+          <t>1. 이메일 자동 번역
 2. 파일 요약 (PDF·Word 등)
 3. 코드 리뷰 + 오류 사전 탐지
 4. 사내 코드 분석</t>
@@ -20970,8 +20359,7 @@
         <is>
           <t>• KR 통신 3사 비교:
 SKT (A.Biz sk-group-aibiz-25-companies:
-SK 그룹 외부 비공개) / KT (Mi:dm B2B, 사내 미공개) / LG U+ (지혜):
-KR 통신 vendor 사내 AI deck reference
+SK 그룹 외부 비공개) / KT (Mi:dm B2B, 사내 미공개) / LG U+ (지혜) KR 통신 vendor 사내 AI deck reference
 • 반면교사: 파일럿 단계 + HR 특화 미공개: 일반 코드·문서 copilot 위주</t>
         </is>
       </c>
@@ -20989,7 +20377,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="168" customHeight="1">
+    <row r="107" ht="136" customHeight="1">
       <c r="A107" s="15" t="n">
         <v>106</v>
       </c>
@@ -21023,10 +20411,7 @@
       <c r="F107" s="16" t="inlineStr"/>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-내부 후보자가 지원해도 결과 통보 없이 발표로 알게 되는 등 candidate experience 미흡 /
-[After]
-1. 직원이 MyGrowth 포털에서 profile 생성·skills 입력 (200,000+ skills)
+          <t>1. 직원이 MyGrowth 포털에서 profile 생성·skills 입력 (200,000+ skills)
 2. Phenom AI가 inferred skills로 jobs·gigs·learning·mentor 매칭
 3. 개인 dashboard에서 추천 기회·learning(29,000+ 콘텐츠)·mentor 1,000+ 표시
 4. 직원이 gig/job/mentor 신청 → 매니저·HR에 routing
@@ -21145,7 +20530,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="168" customHeight="1">
+    <row r="108" ht="120" customHeight="1">
       <c r="A108" s="8" t="n">
         <v>107</v>
       </c>
@@ -21178,10 +20563,7 @@
       <c r="F108" s="10" t="inlineStr"/>
       <c r="G108" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-분기/연간 engagement 설문 후 manager가 보고서 수기 분석 (160+ hours/cycle) /
-[After]
-1. 직원이 Continuous Listening 설문 응답: Qualtrics가 conversational AI로 follow-up 질문
+          <t>1. 직원이 Continuous Listening 설문 응답: Qualtrics가 conversational AI로 follow-up 질문
 2. Qualtrics Assist for EX가 sentiment·테마 분석, manager별 personalized insight 생성
 3. 매니저별 dashboard에 팀 specific feedback + action recommendation 제시
 4. xFlow workflow가 HRIS·ticketing 시스템과 연동해 자동 alert·action
@@ -21316,7 +20698,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="152" customHeight="1">
+    <row r="109" ht="104" customHeight="1">
       <c r="A109" s="15" t="n">
         <v>108</v>
       </c>
@@ -21353,12 +20735,7 @@
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-보험사 직원이 약관·특약·사내 규정 search 시 sharepoint·시니어 문의 의존 / Pain point:
-보험 약관·특약 양 거대 + 빈번한 변경 → 신입·경력 모두 학습 부담 / Trigger:
-2026 삼성생명 중심 그룹 AI센터 (126명) 인접 인프라 활용
-[After]
-1. 직원이 RAG 챗봇 query
+          <t>1. 직원이 RAG 챗봇 query
 2. 보험 약관·특약·사내 규정 RAG 검색
 3. 답변 + 출처 표시</t>
         </is>
@@ -21505,10 +20882,7 @@
       </c>
       <c r="G110" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-전통 EAP → 직원이 전화로 접수 → 치료사 무작위 배정 → 이용률 1% /
-[After]
-1. Spring Health 앱/웹에서 AI 기반 정신건강 평가(wellness assessment) 완료
+          <t>1. Spring Health 앱/웹에서 AI 기반 정신건강 평가(wellness assessment) 완료
 2. AI가 최적 치료 경로(therapy/coaching/자가관리) 추천
 3. 정밀 매칭으로 치료사 배정
 4. 이용률 26%</t>
@@ -21666,10 +21040,7 @@
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-매니저가 수동으로 교대표 작성 → 자격증·컴플라이언스·선호도 수동 확인 → 채용도 개별 프로세스 /
-[After]
-1. AI가 자격증·규제·선호도·노동법 제약을 반영한 최적 스케줄 자동 생성
+          <t>1. AI가 자격증·규제·선호도·노동법 제약을 반영한 최적 스케줄 자동 생성
 2. Workforce Intelligence Hub에서 스케줄·타임·채용·급여 데이터 실시간 통합 뷰
 3. UKG Rapid Hire로 AI-first 채용</t>
         </is>
@@ -21782,7 +21153,7 @@
         </is>
       </c>
     </row>
-    <row r="112" ht="216" customHeight="1">
+    <row r="112" ht="200" customHeight="1">
       <c r="A112" s="8" t="n">
         <v>111</v>
       </c>
@@ -21832,14 +21203,7 @@
       </c>
       <c r="G112" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-글로벌 enterprise에서 시차·휴가·휴직·퇴사 동료의 contextual knowledge 단절:
-Slack search·Confluence·이메일 검색에 의존 / Pain point:
-knowledge worker 1명 평균 19% 시간을 "정보 search"에 투입 (McKinsey Digital).
-부재 동료의 "왜 이렇게 결정했나"·"이 고객은 어떻게 대응?" 같은 contextual Q&amp;A 답 부재 / Trigger:
-Eightfold 공동창업자가 Talent Intelligence 영역에서 Knowledge Twin으로 영역 확장 (2025-10 stealth exit + $35M Khosla seed)
-[After]
-1. 직원이 자기 활동 (이메일·문서·미팅·decision log)을 Viven AI에 학습 동의 (opt-in)
+          <t>1. 직원이 자기 활동 (이메일·문서·미팅·decision log)을 Viven AI에 학습 동의 (opt-in)
 2. AI가 직원별 "Digital Twin" 지식 모델 구축: RAG + agentic
 3. 다른 동료가 "X에게 물어보고 싶었던 것"을 Twin에게 query
 4. Twin이 X의 과거 발언·결정·전문성 기반 답변 (출처 표시)
@@ -21991,10 +21355,7 @@
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-HR 담당자가 각 신규입사자에게 개별 수작업 이메일·체크리스트 전달; 채용 관리자 참여율 낮음 /
-[After]
-1. 입사 확정 시점에 Enboarder가 자동화된 온보딩 여정 개시
+          <t>1. 입사 확정 시점에 Enboarder가 자동화된 온보딩 여정 개시
 2. 채용 관리자에게 개인화된 액션·넛지 자동 전송
 3. 신규 입사자에게 단계별 콘텐츠(기대치 설정·리소스 안내·관계 구축·커뮤니케이션) 자동 전달
 4. 완료율·목표 달성률·Time-to-productivity 자동 추적</t>
@@ -22165,10 +21526,7 @@
       </c>
       <c r="G114" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-매니저가 1:1 미팅을 자유 형식으로 진행 → 노트 수동 작성 → 후속 조치 누락 빈번 → HR이 매니저 효과성 파악 어려움 /
-[After]
-1. Kona가 1:1 미팅에 자동 참여
+          <t>1. Kona가 1:1 미팅에 자동 참여
 2. 대화 전사·요약·액션 아이템 생성
 3. engagement·성과 데이터 기반 실시간 코칭 팁 전달
 4. 매니저 행동 변화 자동 추적</t>
@@ -22316,12 +21674,7 @@
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-1. 각 자회사 개별적으로 AI 툴 도입: 중앙 파악 없음
-2. 내부 파악: 145개 AI 시스템
-3. 신규 AI 도입 시 리스크 평가 체계 없음; 감사 수행 시 수 주 소요 /
-[After]
-1. Holistic AI 플랫폼을 통해 전사 AI 시스템 500~600개 탐지·등록
+          <t>1. Holistic AI 플랫폼을 통해 전사 AI 시스템 500~600개 탐지·등록
 2. 중앙화된 리스크 레지스트리: 시스템별 리스크 카테고리·완화 전략 경영진 가시화
 3. AI 라이프사이클 전반 연속 모니터링
 4. NYC LL144 대응: 채용 AEDT에 대한 독립 바이어스 감사 수행·공개</t>
@@ -22329,7 +21682,7 @@
       </c>
       <c r="H115" s="16" t="inlineStr">
         <is>
-          <t>• AI 시스템 배치: Holistic AI 플랫폼 (SaaS): 전사 AI 거버넌스 레이어
+          <t>• AI 시스템 배치: Holistic AI 플랫폼 (SaaS) 전사 AI 거버넌스 레이어
 • 사용자 접점: 경영진 대시보드, 리크루터용 고객사 컴플라이언스 대시보드 (실시간)</t>
         </is>
       </c>
@@ -22459,7 +21812,7 @@
       </c>
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>Josh Bersin Co.: Galileo Learn</t>
+          <t>Josh Bersin Co. Galileo Learn</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
@@ -22493,10 +21846,7 @@
       </c>
       <c r="G116" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-전통적 LMS/LXP: 코스 수동 제작, 업데이트 느림, 다국어 번역 별도 작업 /
-[After]
-1. 기존 콘텐츠(문서·영상·SCORM)를 플랫폼에 업로드
+          <t>1. 기존 콘텐츠(문서·영상·SCORM)를 플랫폼에 업로드
 2. AI가 "with your guidance" 자동으로 코스·assessment·polls·exercises·시뮬레이션 생성
 3. Galileo agent가 업무 중 사이드 패널로 학습 제공 (Workflow-embedded)
 4. AI 튜터·"AI Josh" avatar persona와 대화형 학습</t>
@@ -22678,10 +22028,7 @@
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-연 1~2회 목표 설정 → 수동 리뷰 작성 → 편향 보정 없음 /
-[After]
-1. Goal Intelligence가 역할·팀·회사 맥락 기반 SMART 목표 추천
+          <t>1. Goal Intelligence가 역할·팀·회사 맥락 기반 SMART 목표 추천
 2. 연속 피드백 수집
 3. AI가 리뷰 편향 탐지·일관성 향상
 4. 부서·지역별 단계적 AI 활성화</t>
@@ -22786,7 +22133,7 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="168" customHeight="1">
+    <row r="118" ht="152" customHeight="1">
       <c r="A118" s="8" t="n">
         <v>117</v>
       </c>
@@ -22824,10 +22171,7 @@
       </c>
       <c r="G118" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-5년 전 300명 과학자 한정 LMS, role-기반 정적 커리큘럼 /
-[After]
-1. 직원이 Degreed에서 skill profile·proficiency 입력 (97% 활성화)
+          <t>1. 직원이 Degreed에서 skill profile·proficiency 입력 (97% 활성화)
 2. AI가 role·proficiency 기반 personalized learning path 추천
 3. 직원이 micro-learning·course·role-play·coaching 소비 (월 64% 재방문)
 4. Career Hub talent marketplace가 skill 매칭으로 internal mobility/gig 제공
@@ -22998,10 +22342,7 @@
       </c>
       <c r="G119" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-수기 근무표 → 엑셀 입력 → 급여 수동 계산 → 노동법 변경 시 수동 반영 /
-[After]
-1. OCR이 수기 근무표를 앱 내 스케줄로 자동 변환
+          <t>1. OCR이 수기 근무표를 앱 내 스케줄로 자동 변환
 2. AI 에이전트가 노동법·세법 이슈 상담
 3. 근태 데이터 기반 연장·야간·휴일 가산임금 자동 산출</t>
         </is>
@@ -23101,7 +22442,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="152" customHeight="1">
+    <row r="120" ht="104" customHeight="1">
       <c r="A120" s="8" t="n">
         <v>119</v>
       </c>
@@ -23136,12 +22477,7 @@
       </c>
       <c r="G120" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-GS칼텍스 ~3K 직원이 정유·안전 매뉴얼·정책을 manual search / Pain point:
-정유 산업 안전 critical + 매뉴얼 양 거대 / Trigger:
-2025 한국 기업 사내 AI 플랫폼 가속
-[After]
-1. AIU 플랫폼
+          <t>1. AIU 플랫폼
 2. 직원 자연어 query
 3. 안전·실무 정보 응답</t>
         </is>
@@ -23225,8 +22561,8 @@
       <c r="AK120" s="10" t="inlineStr">
         <is>
           <t>• 정유·에너지 산업 reference (GS칼텍스·SK이노베이션·S-Oil 등)
-• 현대모비스 MoAI hyundai-mobis-moai-platform (자동차) + 가스공사 kogas-hybrid-genai-platform (가스) + GS칼텍스 (정유):
-한국 에너지·제조 사내 AI plat 비교
+• 현대모비스 MoAI hyundai-mobis-moai-platform (자동차) + 가스공사
+kogas-hybrid-genai-platform (가스) + GS칼텍스 (정유) 한국 에너지·제조 사내 AI plat 비교
 • 반면교사: 자사 보고만, 외부 검증·HR 비중 미공개: POC 4주 자체 측정 권장</t>
         </is>
       </c>
@@ -23284,10 +22620,7 @@
       </c>
       <c r="G121" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-매니저가 직원별 피드백·리뷰를 수동으로 읽고 종합 → 목표 대시보드 수동 확인 /
-[After]
-1. AI Performance Summarization이 현 주기 피드백·리뷰를 자동 요약
+          <t>1. AI Performance Summarization이 현 주기 피드백·리뷰를 자동 요약
 2. 핵심 트렌드 도출
 3. Goals AI가 자연어 쿼리로 목표 진척 분석
 4. AI Agent가 이탈 리스크 신호 탐지</t>
@@ -23392,7 +22725,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="152" customHeight="1">
+    <row r="122" ht="88" customHeight="1">
       <c r="A122" s="8" t="n">
         <v>121</v>
       </c>
@@ -23423,10 +22756,7 @@
       <c r="F122" s="10" t="inlineStr"/>
       <c r="G122" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개_ (전통적 HR 서류 심사 + 매뉴얼 면접 질문 준비) /
-[After]
-1. 채용 시 지원자의 자기소개서·인적성검사 데이터 (수만 건)가 인사 시스템에 제출
+          <t>1. 채용 시 지원자의 자기소개서·인적성검사 데이터 (수만 건)가 인사 시스템에 제출
 2. 에이전틱 AI가 기존 인사 문서도 함께 분석
 3. AI가 적합 인재를 추천
 4. AI가 지원자별 맞춤 면접 질문을 자동 생성
@@ -23545,7 +22875,7 @@
         </is>
       </c>
     </row>
-    <row r="123" ht="168" customHeight="1">
+    <row r="123" ht="104" customHeight="1">
       <c r="A123" s="15" t="n">
         <v>122</v>
       </c>
@@ -23576,10 +22906,7 @@
       <c r="F123" s="16" t="inlineStr"/>
       <c r="G123" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-후보자가 career site에서 긴 지원 form 작성, 리크루터가 수동 스크리닝/스케줄링 /
-[After]
-1. 후보자가 career site/모바일에서 Olivia chatbot과 대화 시작
+          <t>1. 후보자가 career site/모바일에서 Olivia chatbot과 대화 시작
 2. Olivia가 knockout 질문 (자격·근무가능시간·work auth)으로 스크리닝
 3. 통과 후보에게 FAQ (급여·복지·문화: 500+ Q&amp;A) 응답 + interview slot 제안
 4. 채용 매니저 캘린더와 동기화하여 interview 자동 예약
@@ -23733,10 +23060,7 @@
       </c>
       <c r="G124" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-직무 데이터 수작업 분류 → 직무체계 설계 → 수개월 소요 /
-[After]
-1. Orgvue Henshaw Roles AI가 8,000개 직위 자동 분석
+          <t>1. Orgvue Henshaw Roles AI가 8,000개 직위 자동 분석
 2. 83개 역할 클러스터로 자동 분류 (분 단위)
 3. OD 팀이 클러스터 결과 검토·수정 (HITL)
 4. 검증된 클러스터 기반으로 조직설계·인력계획 가속</t>
@@ -23857,7 +23181,7 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="184" customHeight="1">
+    <row r="125" ht="120" customHeight="1">
       <c r="A125" s="15" t="n">
         <v>124</v>
       </c>
@@ -23889,10 +23213,7 @@
       <c r="F125" s="16" t="inlineStr"/>
       <c r="G125" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-HR 케이스가 분류·라우팅·해결까지 다단계 manual ticket 처리 /
-[After]
-1. 직원이 ServiceNow employee portal/Teams에서 HR 요청 제출
+          <t>1. 직원이 ServiceNow employee portal/Teams에서 HR 요청 제출
 2. Now Assist가 case 내용 분석 → criticality 분류 (non-critical/critical)
 3. Non-critical case는 HR knowledge base·catalog 조회하여 자동 해결
 4. Hiring 영역에서는 Schedule Interview agent·Create Job Requisition agent가
@@ -24055,10 +23376,7 @@
       </c>
       <c r="G126" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개_ (기존 직무 이동·프로젝트 배치 메커니즘 세부는 기사에 없음) /
-[After]
-1. 직원이 professional profile + purpose statement (관심·포부) 작성
+          <t>1. 직원이 professional profile + purpose statement (관심·포부) 작성
 2. Gloat AI가 직원 스킬과 등록된 프로젝트·역할 기회를 매칭
 3. 직원에게 기회 추천 (단기 프로젝트·장기 역할 모두)
 4. 매니저 허가 불필요: (본업 수행 전제)
@@ -24081,8 +23399,8 @@
           <t>• 입력 데이터 소스: - 직원 self-reported 프로필 (스킬·관심·purpose)
 • 데이터 규모: 2019-12 기준 30,000+ 직원 ·
 1,750명 HR 초기 pilot
-• 전처리·정제: 스킬 ontology로 정규화 (Gloat 핵심 기능):
-구체 구현 미공개</t>
+• 전처리·정제: 스킬 ontology로 정규화 (Gloat 핵심 기능) 구체 구현
+미공개</t>
         </is>
       </c>
       <c r="J126" s="10" t="inlineStr">
@@ -24223,10 +23541,7 @@
       <c r="F127" s="16" t="inlineStr"/>
       <c r="G127" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-HRBP·매니저가 People analytics 질문에 데이터 팀 ticket 의존, 답변 수일 소요 /
-[After]
-1. 사용자가 Visier People 또는 Microsoft Teams에서 Vee와 자연어로 채팅
+          <t>1. 사용자가 Visier People 또는 Microsoft Teams에서 Vee와 자연어로 채팅
 2. Vee가 자연어 질문을 Visier query로 변환
 3. 조직의 people data로 query 실행 (proprietary customer data는 LLM 학습 미사용)
 4. narrative 답변·차트·요약·자동 보고서 생성
@@ -24388,10 +23703,7 @@
       </c>
       <c r="G128" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개. Bersin·PR 모두 기존 workflow를 기술하지 않음_ /
-[After]
-1. After (To-be) (PR 기준): 에이전트가 "job ladder의 생성과 관리를 자동화" (구체 단계 미공개)</t>
+          <t>1. After (To-be) (PR 기준): 에이전트가 "job ladder의 생성과 관리를 자동화" (구체 단계 미공개)</t>
         </is>
       </c>
       <c r="H128" s="10" t="inlineStr">
@@ -24537,7 +23849,7 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="280" customHeight="1">
+    <row r="129" ht="264" customHeight="1">
       <c r="A129" s="15" t="n">
         <v>128</v>
       </c>
@@ -24582,15 +23894,7 @@
       </c>
       <c r="G129" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-SK하이닉스 38K 직원의 인사 데이터가 HRMS·평가·교육·프로젝트·자격증·외부 교육 등 다수 시스템에 분산.
-매니저가 internal mobility·project staffing·후계자 후보 검색 시 여러 시스템 + 인적 네트워크 의존 /
-Pain point: / 사내 talent visibility 부족: 매니저가 "양산공정 + 머신러닝 경험 5년+ 영어 가능자"를
-사내에서 찾기 어려움 / 직원 본인도 자기 career path·내부 기회 잘 모름 / 핵심 인재 retention·project
-staffing·후계자 풀 식별 모두 동일한 root cause (skill·경력 visibility 부재) / Trigger:
-2024-25 SK 그룹 차원 AI 적극 도입 흐름
-[After]
-1. 데이터 통합 layer:
+          <t>1. 데이터 통합 layer:
 HRMS·평가·교육 LMS·프로젝트 시스템·자격 DB·외부 교육 이력 등에서 직원별 데이터 자동 수집 → ETL → 단일 직원 프로필
 2. One Resume 생성: 정형 데이터 (인사 기본·역할·근속·평가·교육) + 비정형 데이터 (프로젝트 기여·자격·관심사) 결합
 3. AI 구성원 검색 (talent search):
@@ -24713,7 +24017,7 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="168" customHeight="1">
+    <row r="130" ht="104" customHeight="1">
       <c r="A130" s="8" t="n">
         <v>129</v>
       </c>
@@ -24736,10 +24040,7 @@
       <c r="F130" s="10" t="inlineStr"/>
       <c r="G130" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-졸업생 trainee 채용에 3개월 소요, in-person 면접 no-show율 높음 /
-[After]
-1. 지원자가 온라인 지원 → ATS에서 HireVue 초대 발송
+          <t>1. 지원자가 온라인 지원 → ATS에서 HireVue 초대 발송
 2. 후보자가 mobile/web으로 on-demand video 인터뷰 녹화 (graduate 90% 응답률)
 3. HireVue가 응답·언어 사용 (콜로키얼/슬랭 포함) 평가하여 점수 산출
 4. 채용팀이 score·video 검토 후 최종 라운드 후보 shortlist
@@ -24866,7 +24167,7 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="232" customHeight="1">
+    <row r="131" ht="200" customHeight="1">
       <c r="A131" s="15" t="n">
         <v>130</v>
       </c>
@@ -24908,19 +24209,14 @@
       </c>
       <c r="G131" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-_미공개 (기업별 상이)_.
-일반적 한국 기업의 기존 연말정산 플로우는 HR 담당자가 직원별로 국세청 간소화 자료 수집·입력·검증하는 수작업이나,
-소스에 기업별 구체 기술은 없음 (🚫 일반 지식) /
-[After]
-1. 대상자 선정:: ONE AI가 직원 DB에서 연말정산 대상자 자동 식별
-2. 안내:: 대상자에게 일정·필요 자료 자동 고지
-3. 자료 입력:: 국세청 간소화 서비스에서 PDF 자동 다운로드, 시스템에 반영
-4. 검토:: 연말정산 데이터 검증 + 세액 예측
-5. 추가 증빙 수집:: 원챔버 연동으로 직원이 추가 증빙 업로드
-6. 결과 안내:: 세액 계산 결과를 직원·HR에 자동 통보
-7. 신고 처리:: 홈택스 자동신고 + 요약보고서·지급명세서 자동 작성·신고
-8. HR 모니터링:: 총괄현황판으로 전사 진행상황 실시간 관리</t>
+          <t>1. 대상자 선정: ONE AI가 직원 DB에서 연말정산 대상자 자동 식별
+2. 안내: 대상자에게 일정·필요 자료 자동 고지
+3. 자료 입력: 국세청 간소화 서비스에서 PDF 자동 다운로드, 시스템에 반영
+4. 검토: 연말정산 데이터 검증 + 세액 예측
+5. 추가 증빙 수집: 원챔버 연동으로 직원이 추가 증빙 업로드
+6. 결과 안내: 세액 계산 결과를 직원·HR에 자동 통보
+7. 신고 처리: 홈택스 자동신고 + 요약보고서·지급명세서 자동 작성·신고
+8. HR 모니터링: 총괄현황판으로 전사 진행상황 실시간 관리</t>
         </is>
       </c>
       <c r="H131" s="16" t="inlineStr">
@@ -25056,7 +24352,7 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="184" customHeight="1">
+    <row r="132" ht="168" customHeight="1">
       <c r="A132" s="8" t="n">
         <v>131</v>
       </c>
@@ -25095,10 +24391,7 @@
       </c>
       <c r="G132" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-채용·내부이동·후계 별도 시스템, 정적 직무 기술서·resume keyword 매칭 /
-[After]
-1. 회사 HRIS·ATS·LMS 데이터를 Eightfold에 연결
+          <t>1. 회사 HRIS·ATS·LMS 데이터를 Eightfold에 연결
 2. Capabilities Matrix가 직원 skill·capability·aspiration·work pattern 모델링 (1.6B+
 profile 기반)
 3. Job Intelligence Engine이 role 정의·job architecture 자동 생성·refresh
@@ -25229,7 +24522,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="168" customHeight="1">
+    <row r="133" ht="104" customHeight="1">
       <c r="A133" s="15" t="n">
         <v>132</v>
       </c>
@@ -25252,10 +24545,7 @@
       <c r="F133" s="16" t="inlineStr"/>
       <c r="G133" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-Pandemic 후 1만 명 cabin crew 재채용 필요, 전통 face-to-face 채용으로는 timeline 불가 /
-[After]
-1. 글로벌 후보자가 Emirates 채용 페이지에서 지원 → HireVue 초대
+          <t>1. 글로벌 후보자가 Emirates 채용 페이지에서 지원 → HireVue 초대
 2. 후보자가 English 어학 평가 (15분 객관식) 응시: 가장 큰 탈락 관문
 3. situational prompt에 대한 video 응답 녹화 (수초간 준비)
 4. HireVue가 verbal·written 응답을 채점 ( 벤더 주장 non-verbal cues 포함)
@@ -25369,7 +24659,7 @@
         </is>
       </c>
     </row>
-    <row r="134" ht="168" customHeight="1">
+    <row r="134" ht="104" customHeight="1">
       <c r="A134" s="8" t="n">
         <v>133</v>
       </c>
@@ -25397,10 +24687,7 @@
       </c>
       <c r="G134" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-내부이동이 매니저 referral·HR 큐레이션에 의존, 직원 가시성·career path 불투명 /
-[After]
-1. 직원이 Fuel50에서 Talent DNA (Talents/Skills/Values/Agility/Fit) 작성
+          <t>1. 직원이 Fuel50에서 Talent DNA (Talents/Skills/Values/Agility/Fit) 작성
 2. AI가 ethically-enhanced 매칭으로 gigs·projects·mentorships·lateral moves 추천
 3. 직원이 즉시 검색·지원 가능, 매니저 추천 불필요
 4. 매니저는 gig 게시·applicant 풀 관리·프로젝트 talent pool 구축
@@ -25493,8 +24780,7 @@
           <t>• "내부 이동의 재무 가치를 정량화"한 유일 사례:
 다른 talent marketplace(Gloat·Phenom)는 시간·비용으로 측정하지만 Fuel50은 근속 연장으로 측정
 • Onboarding &amp; Transitions 카테고리 4번째 사례:
-Unilever(Gloat) + Schneider(Gloat) + Merck KGaA(Phenom) + Lennox(Fuel50):
-3개 벤더 비교 가능</t>
+Unilever(Gloat) + Schneider(Gloat) + Merck KGaA(Phenom) + Lennox(Fuel50) 3개 벤더 비교 가능</t>
         </is>
       </c>
       <c r="AL134" s="10" t="inlineStr">
@@ -25515,7 +24801,7 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="168" customHeight="1">
+    <row r="135" ht="104" customHeight="1">
       <c r="A135" s="15" t="n">
         <v>134</v>
       </c>
@@ -25538,10 +24824,7 @@
       <c r="F135" s="16" t="inlineStr"/>
       <c r="G135" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-매장 매니저가 종이/이메일로 지원 처리, 지원 시간 10분, 시간 부족으로 채용 누수 /
-[After]
-1. 후보자가 매장 sign·광고·Alexa/Google Assistant (Apply Thru)로 시작
+          <t>1. 후보자가 매장 sign·광고·Alexa/Google Assistant (Apply Thru)로 시작
 2. 텍스트 번호 발송 → Olivia가 즉시 conversational 스크리닝 시작
 3. 기본 work history·available shift 질문 (지원 시간 10분→2분)
 4. 통과 후보에게 매장 매니저 캘린더 기반 interview slot 제시
@@ -25660,7 +24943,7 @@
         </is>
       </c>
     </row>
-    <row r="136" ht="136" customHeight="1">
+    <row r="136" ht="120" customHeight="1">
       <c r="A136" s="8" t="n">
         <v>135</v>
       </c>
@@ -25700,10 +24983,7 @@
       </c>
       <c r="G136" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-매니저가 타임카드 수동 검토 → 교대표 수동 작성 → PTO 개별 승인 /
-[After]
-1. Agentic Timesheet Approvals가 타임카드를 임계값 기반 자동 스코어링
+          <t>1. Agentic Timesheet Approvals가 타임카드를 임계값 기반 자동 스코어링
 2. 정상은 자동 승인, 이상만 사람에게 플래그
 3. Auto-Shifts가 규칙(근무시간·휴식·공정근무) 기반 최적 교대 생성
 4. AI Time-Off가 과거 PTO 패턴 분석·피크 예측</t>
@@ -25843,10 +25123,7 @@
       </c>
       <c r="G137" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-LMS에서 직원이 과정 목록을 수동 탐색 → 관련성 낮은 과정 수강 → 학습 효율 저하 /
-[After]
-1. CIC가 부서·직급·직무·관심 키워드·수강 이력을 분석
+          <t>1. CIC가 부서·직급·직무·관심 키워드·수강 이력을 분석
 2. 맞춤형 교육 콘텐츠 자동 추천</t>
         </is>
       </c>
@@ -25941,7 +25218,7 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="248" customHeight="1">
+    <row r="138" ht="152" customHeight="1">
       <c r="A138" s="8" t="n">
         <v>137</v>
       </c>
@@ -25984,15 +25261,7 @@
       </c>
       <c r="G138" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-핵심 인재 이탈은 사후 면담 + 단편적 정형 데이터(근속·평가) 위주 분석.
-미묘한 행동 변화·외부 시장 신호·관계 패턴 unintegrated.
-매니저 "감"에 의존 / Pain point:
-SK하이닉스 38K 직원 중 반도체 핵심 인재 (R&amp;D·tech 전문가) 이탈 비용 거대.
-사후 대응으론 retention 불가 / Trigger:
-2024-25 SK 그룹 차원 AI 적극 도입 + PwC Korea 컨설팅 제안
-[After]
-1. 5개 specialist 에이전트가 각자 영역 데이터 분석
+          <t>1. 5개 specialist 에이전트가 각자 영역 데이터 분석
 2. 각 에이전트가 개별 퇴사 확률값 산출 → 이진 분류 (퇴사·재직)
 3. Hybrid 가중치 엔진: AHP (분석적 계층 과정): HR 전문가 도메인 지식 정량화
 4. 위험 등급 산출: Green / Yellow / Red
@@ -26119,7 +25388,7 @@
         </is>
       </c>
     </row>
-    <row r="139" ht="168" customHeight="1">
+    <row r="139" ht="104" customHeight="1">
       <c r="A139" s="15" t="n">
         <v>138</v>
       </c>
@@ -26151,10 +25420,7 @@
       <c r="F139" s="16" t="inlineStr"/>
       <c r="G139" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-보상 결정 시 매니저·HR이 spreadsheet·외부 market data로 ad-hoc 판단, equity 위반 사후 발견 /
-[After]
-1. 회사가 compensation·workforce·HRIS data를 Syndio에 연결
+          <t>1. 회사가 compensation·workforce·HRIS data를 Syndio에 연결
 2. PayEQ가 protected class 그룹별 pay gap 분석·통계적 검증
 3. 매니저가 Teams/Slack/ATS에서 offer·raise 결정 시 Syndi 호출
 4. Syndi agentic AI가 internal equity·budget·market 균형 추천 + 설명 제공
@@ -26275,7 +25541,7 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="152" customHeight="1">
+    <row r="140" ht="136" customHeight="1">
       <c r="A140" s="8" t="n">
         <v>139</v>
       </c>
@@ -26312,10 +25578,7 @@
       </c>
       <c r="G140" s="10" t="inlineStr">
         <is>
-          <t>[Before]
-채용 담당자가 키워드·필터로 후보자를 검색, 검색 결과를 수동으로 검토 /
-[After]
-1. 채용 담당자가 자연어로 원하는 후보자 프로필 입력 (예: "AI 스타트업 경험 있는 백엔드 5년차 이상")
+          <t>1. 채용 담당자가 자연어로 원하는 후보자 프로필 입력 (예: "AI 스타트업 경험 있는 백엔드 5년차 이상")
 2. 기본 탐색: 조건에 맞는 후보자를 빠르고 넓게 추출
 3. 고급 탐색: AI 에이전트가 각 후보의 자기소개서·프로젝트 경험 등 정성 데이터 분석
 4. AI가 역량·경험 판단 + 추천 사유 제시
@@ -26451,7 +25714,7 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="168" customHeight="1">
+    <row r="141" ht="120" customHeight="1">
       <c r="A141" s="15" t="n">
         <v>140</v>
       </c>
@@ -26489,10 +25752,7 @@
       </c>
       <c r="G141" s="16" t="inlineStr">
         <is>
-          <t>[Before]
-engagement 설문 결과를 People 팀이 quarterly로 분석·매니저에게 PPT 배포, action 지연 /
-[After]
-1. Workday HCM 내 engagement·pulse·feedback·exit data가 Illuminate에 자동 공급
+          <t>1. Workday HCM 내 engagement·pulse·feedback·exit data가 Illuminate에 자동 공급
 2. Employee Sentiment Agent가 feedback 데이터를 continuous 분석
 3. 팀·코호트별 sentiment trend·driver·이상 신호 추출
 4. 매니저 Workday 워크플로에 proactive insight 푸시
@@ -38344,7 +37604,7 @@
         <is>
           <t>• 자체 통합 platform 'AI ONE': 40+ AI를 단일 인터페이스 + Speech-to-AI 모바일/태블릿
 • AI 인사이동 알고리즘: 2020~ 운영, 신한·KB 한국 large-scale 인사 AI 양대 reference
-• 그룹사 확산: 신한카드 'AINa' (AI 5025 프로젝트): 그룹 차원 LLM 활용
+• 그룹사 확산: 신한카드 'AINa' (AI 5025 프로젝트) 그룹 차원 LLM 활용
 • 자체 GenAI: 외부 모델 의존 축소: 데이터 주권 강조</t>
         </is>
       </c>
@@ -38485,8 +37745,7 @@
           <t>세계 2위 메모리 반도체 기업.
 SK 그룹 핵심 멤버사이자 국가핵심기술 보유사.
 HR AI는 채용 + 그룹 표준 결합:
-(1) A!SK AI 영상면접 hybrid (AI + 미래 동료 평가):
-2025 신설, (2) SK 그룹 'A.Biz' 표준 사용 with 자체 LLM 'A.X' 격리 환경.</t>
+(1) A!SK AI 영상면접 hybrid (AI + 미래 동료 평가) 2025 신설, (2) SK 그룹 'A.Biz' 표준 사용 with 자체 LLM 'A.X' 격리 환경.</t>
         </is>
       </c>
       <c r="H19" s="16" t="inlineStr">
@@ -38548,7 +37807,7 @@
 • 주의점:
 • Unilever FLEX의 "매니저 승인 불필요" 원칙이 한국 연공 문화에서 작동할지 미검증
 • DEI 효과(여성 직원 참여율) 부분은 한국 적용 시 별도 설계 필요
-• 현재 wiki의 주요 소스가 2019년 기준 (76개월 stale): 최신 data로 업데이트하지 않으면 제안서 사용 시 리스크
+• 현재 wiki의 주요 소스가 2019년 기준 (76개월 stale) 최신 data로 업데이트하지 않으면 제안서 사용 시 리스크
 • 반면교사 리스크:</t>
         </is>
       </c>

</xml_diff>